<commit_message>
Weekly indices update 2026-09-16
</commit_message>
<xml_diff>
--- a/tracker_auto.xlsx
+++ b/tracker_auto.xlsx
@@ -2770,47 +2770,47 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>25402.28</v>
+        <v>25369.23</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>-0.0233</v>
+        <v>-0.008100000000000001</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>-0.0326</v>
+        <v>-0.0339</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>-0.0393</v>
+        <v>-0.0368</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>0.0197</v>
+        <v>0.0174</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>0.0704</v>
+        <v>0.0794</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>0.0372</v>
+        <v>0.0359</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>0.12</v>
+        <v>0.1186</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>0.0696</v>
+        <v>0.08740000000000001</v>
       </c>
       <c r="L46" s="3" t="n">
-        <v>0.1652</v>
+        <v>0.167</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>0.1691</v>
+        <v>0.1685</v>
       </c>
       <c r="N46" s="3" t="n">
-        <v>0.1018</v>
+        <v>0.1038</v>
       </c>
       <c r="O46" s="3" t="n">
-        <v>0.09480000000000001</v>
+        <v>0.0946</v>
       </c>
     </row>
     <row r="47">
@@ -2821,47 +2821,47 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>8090.28</v>
+        <v>8088.8</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>-0.0274</v>
+        <v>-0.0083</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>-0.0293</v>
+        <v>-0.0295</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>-0.0633</v>
+        <v>-0.0572</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>-0.0423</v>
+        <v>-0.0406</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>0.0145</v>
+        <v>0.0149</v>
       </c>
       <c r="I47" s="3" t="n">
-        <v>-0.0073</v>
+        <v>-0.0074</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>0.035</v>
+        <v>0.0348</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>0.0245</v>
+        <v>0.0346</v>
       </c>
       <c r="L47" s="3" t="n">
-        <v>0.0409</v>
+        <v>0.0421</v>
       </c>
       <c r="M47" s="3" t="n">
-        <v>0.0312</v>
+        <v>0.0311</v>
       </c>
       <c r="N47" s="3" t="n">
-        <v>0.0409</v>
+        <v>0.0425</v>
       </c>
       <c r="O47" s="3" t="n">
-        <v>0.0645</v>
+        <v>0.0644</v>
       </c>
     </row>
     <row r="48">
@@ -2872,47 +2872,47 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>10658.13</v>
+        <v>10680.53</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>-0.0142</v>
+        <v>0.001</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>-0.0154</v>
+        <v>-0.0133</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>-0.0086</v>
+        <v>-0.0037</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>0.0156</v>
+        <v>0.0164</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>0.0245</v>
+        <v>0.0364</v>
       </c>
       <c r="I48" s="3" t="n">
-        <v>0.0732</v>
+        <v>0.07539999999999999</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>0.0473</v>
+        <v>0.0495</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>0.1489</v>
+        <v>0.1615</v>
       </c>
       <c r="L48" s="3" t="n">
-        <v>0.1347</v>
+        <v>0.136</v>
       </c>
       <c r="M48" s="3" t="n">
-        <v>0.1139</v>
+        <v>0.1145</v>
       </c>
       <c r="N48" s="3" t="n">
-        <v>0.08689999999999999</v>
+        <v>0.08939999999999999</v>
       </c>
       <c r="O48" s="3" t="n">
-        <v>0.0474</v>
+        <v>0.0476</v>
       </c>
     </row>
     <row r="49">

</xml_diff>

<commit_message>
Manual indices update 2026-09-17
</commit_message>
<xml_diff>
--- a/tracker_auto.xlsx
+++ b/tracker_auto.xlsx
@@ -524,47 +524,47 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>23118.6</v>
+        <v>23217.6</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>-0.0219</v>
+        <v>-0.0091</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-0.0399</v>
+        <v>-0.0358</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>-0.0512</v>
+        <v>-0.0441</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>-0.0363</v>
+        <v>-0.036</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>-0.0196</v>
+        <v>-0.0236</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>-0.1152</v>
+        <v>-0.1114</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.0353</v>
+        <v>0.0397</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>-0.07780000000000001</v>
+        <v>-0.0801</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>-0.0451</v>
+        <v>-0.0436</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>0.0461</v>
+        <v>0.0476</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>0.0557</v>
+        <v>0.0572</v>
       </c>
       <c r="O2" s="3" t="n">
-        <v>0.1017</v>
+        <v>0.1021</v>
       </c>
     </row>
     <row r="3">
@@ -575,47 +575,47 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>74329.63</v>
+        <v>74314.59</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>-0.0058</v>
+        <v>-0.007900000000000001</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>-0.0341</v>
+        <v>-0.0343</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>-0.0437</v>
+        <v>-0.0378</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>-0.0366</v>
+        <v>-0.04</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>-0.031</v>
+        <v>0.0014</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>-0.1278</v>
+        <v>-0.128</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>0.0331</v>
+        <v>0.0329</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>-0.0977</v>
+        <v>-0.1013</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>-0.0536</v>
+        <v>-0.05429999999999999</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>0.0309</v>
+        <v>0.0321</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>0.0473</v>
+        <v>0.0472</v>
       </c>
       <c r="O3" s="3" t="n">
-        <v>0.1002</v>
+        <v>0.1001</v>
       </c>
     </row>
     <row r="4">
@@ -626,47 +626,47 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>70281.14999999999</v>
+        <v>70368.60000000001</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>-0.0366</v>
+        <v>-0.0341</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>-0.0472</v>
+        <v>-0.046</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>-0.0565</v>
+        <v>-0.0551</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>-0.0211</v>
+        <v>-0.0262</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.0809</v>
+        <v>0.0716</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.0132</v>
+        <v>0.0145</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.1646</v>
+        <v>0.166</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>0.0245</v>
+        <v>0.0198</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>-0.0346</v>
+        <v>-0.0344</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>0.1513</v>
+        <v>0.1516</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>0.1007</v>
+        <v>0.1028</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>0.1189</v>
+        <v>0.119</v>
       </c>
     </row>
     <row r="5">
@@ -677,47 +677,47 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>24193</v>
+        <v>24282.95</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>-0.0246</v>
+        <v>-0.0139</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>-0.0413</v>
+        <v>-0.0377</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>-0.0522</v>
+        <v>-0.0461</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>-0.0334</v>
+        <v>-0.0342</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>-0.0018</v>
+        <v>-0.0067</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>-0.0935</v>
+        <v>-0.0902</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0.0576</v>
+        <v>0.06150000000000001</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>-0.0599</v>
+        <v>-0.0626</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>-0.043</v>
+        <v>-0.04190000000000001</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>0.0636</v>
+        <v>0.06480000000000001</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>0.0619</v>
+        <v>0.0634</v>
       </c>
       <c r="O5" s="3" t="n">
-        <v>0.1042</v>
+        <v>0.1045</v>
       </c>
     </row>
     <row r="6">
@@ -728,47 +728,47 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>31555.6</v>
+        <v>31669.65</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>-0.0228</v>
+        <v>-0.0149</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-0.0433</v>
+        <v>-0.0398</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-0.0541</v>
+        <v>-0.04650000000000001</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>-0.0289</v>
+        <v>-0.029</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.0203</v>
+        <v>0.0149</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>-0.0533</v>
+        <v>-0.0498</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.06759999999999999</v>
+        <v>0.07150000000000001</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>-0.0159</v>
+        <v>-0.019</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>-0.0174</v>
+        <v>-0.0155</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>0.09630000000000001</v>
+        <v>0.0975</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>0.0989</v>
+        <v>0.1005</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>0.1124</v>
+        <v>0.1128</v>
       </c>
     </row>
     <row r="7">
@@ -779,47 +779,47 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>33339.3</v>
+        <v>33426.35</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>-0.0315</v>
+        <v>-0.0252</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-0.0473</v>
+        <v>-0.04480000000000001</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>-0.0573</v>
+        <v>-0.0527</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>-0.0257</v>
+        <v>-0.0284</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.053</v>
+        <v>0.045</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>-0.0182</v>
+        <v>-0.0156</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>0.1192</v>
+        <v>0.1222</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>0.0027</v>
+        <v>-0.0011</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>-0.0209</v>
+        <v>-0.0199</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>0.1218</v>
+        <v>0.1227</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>0.09669999999999999</v>
+        <v>0.09859999999999999</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>0.1118</v>
+        <v>0.112</v>
       </c>
     </row>
     <row r="8">
@@ -830,47 +830,47 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>18089.82</v>
+        <v>18143.16</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>-0.0262</v>
+        <v>-0.0166</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-0.0433</v>
+        <v>-0.0405</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-0.0505</v>
+        <v>-0.0458</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>-0.0252</v>
+        <v>-0.0269</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.0247</v>
+        <v>0.0168</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>-0.0675</v>
+        <v>-0.06469999999999999</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.0833</v>
+        <v>0.08650000000000001</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>-0.0318</v>
+        <v>-0.0352</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>-0.0236</v>
+        <v>-0.023</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>0.08779999999999999</v>
+        <v>0.0888</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>0.0867</v>
+        <v>0.08839999999999999</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>0.124</v>
+        <v>0.1243</v>
       </c>
     </row>
     <row r="9">
@@ -881,47 +881,47 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>16087.45</v>
+        <v>16120.65</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>-0.0282</v>
+        <v>-0.0206</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-0.0457</v>
+        <v>-0.0438</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-0.0487</v>
+        <v>-0.0462</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>-0.0236</v>
+        <v>-0.0262</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>0.0475</v>
+        <v>0.0355</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>-0.0455</v>
+        <v>-0.0436</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>0.1038</v>
+        <v>0.1061</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>-0.0142</v>
+        <v>-0.0184</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>-0.0189</v>
+        <v>-0.0191</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>0.1006</v>
+        <v>0.1013</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>0.1037</v>
+        <v>0.106</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>0.1329</v>
+        <v>0.1331</v>
       </c>
     </row>
     <row r="10">
@@ -932,44 +932,44 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>22358.8</v>
+        <v>22368.8</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>-0.0317</v>
+        <v>-0.0271</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>-0.05</v>
+        <v>-0.0496</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>-0.0453</v>
+        <v>-0.0463</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>-0.0138</v>
+        <v>-0.0183</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.0978</v>
+        <v>0.07820000000000001</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>0.0037</v>
+        <v>0.004099999999999999</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.1507</v>
+        <v>0.1512</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>0.03240000000000001</v>
+        <v>0.0265</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>0.0038</v>
+        <v>0.0023</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0.1367</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0.1449</v>
+        <v>0.148</v>
       </c>
       <c r="O10" s="3" t="n">
         <v>0.1599</v>
@@ -983,47 +983,47 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>17892.8</v>
+        <v>17863.3</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>-0.0342</v>
+        <v>-0.0309</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>-0.0261</v>
+        <v>-0.0277</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>-0.0211</v>
+        <v>-0.0245</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>0.0301</v>
+        <v>0.021</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0.2017</v>
+        <v>0.1788</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>0.07240000000000001</v>
+        <v>0.0706</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>0.2523</v>
+        <v>0.2502</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>0.03700000000000001</v>
+        <v>0.0277</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>-0.0177</v>
+        <v>-0.0193</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>0.133</v>
+        <v>0.1322</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>0.1385</v>
+        <v>0.1397</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>0.1372</v>
+        <v>0.137</v>
       </c>
     </row>
     <row r="12">
@@ -1034,47 +1034,47 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>20750.7</v>
+        <v>20744.9</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>-0.0326</v>
+        <v>-0.0284</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>-0.04190000000000001</v>
+        <v>-0.04219999999999999</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>-0.0371</v>
+        <v>-0.0389</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0.0011</v>
+        <v>-0.005</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.1319</v>
+        <v>0.1112</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>0.0264</v>
+        <v>0.0261</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0.1841</v>
+        <v>0.1838</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>0.0332</v>
+        <v>0.0261</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>-0.0043</v>
+        <v>-0.0058</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0.135</v>
+        <v>0.1348</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.1428</v>
+        <v>0.1454</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>0.1524</v>
+        <v>0.1523</v>
       </c>
     </row>
     <row r="13">
@@ -1085,47 +1085,47 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>22477.45</v>
+        <v>22532</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>-0.0272</v>
+        <v>-0.0186</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>-0.0415</v>
+        <v>-0.0392</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>-0.0474</v>
+        <v>-0.0438</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>-0.0226</v>
+        <v>-0.025</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>0.0373</v>
+        <v>0.028</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>-0.0584</v>
+        <v>-0.0561</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>0.095</v>
+        <v>0.09759999999999999</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>-0.0318</v>
+        <v>-0.0358</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>-0.0307</v>
+        <v>-0.0304</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>0.08359999999999999</v>
+        <v>0.08439999999999999</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>0.0828</v>
+        <v>0.08439999999999999</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>0.1163</v>
+        <v>0.1165</v>
       </c>
     </row>
     <row r="14">
@@ -1136,47 +1136,47 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>35169.62</v>
+        <v>35276.25</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>-0.027</v>
+        <v>-0.018</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>-0.0395</v>
+        <v>-0.0366</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>-0.04849999999999999</v>
+        <v>-0.0442</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>-0.0214</v>
+        <v>-0.0235</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0.0362</v>
+        <v>0.0276</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>-0.0607</v>
+        <v>-0.0579</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>0.09279999999999999</v>
+        <v>0.09609999999999999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>-0.0352</v>
+        <v>-0.0387</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>-0.0348</v>
+        <v>-0.034</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0.0788</v>
+        <v>0.07980000000000001</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>0.0793</v>
+        <v>0.081</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>0.1151</v>
+        <v>0.1154</v>
       </c>
     </row>
     <row r="15">
@@ -1187,47 +1187,47 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>19233</v>
+        <v>19298.7</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>-0.0233</v>
+        <v>-0.0104</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>-0.0489</v>
+        <v>-0.0457</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>-0.06179999999999999</v>
+        <v>-0.0515</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>-0.0257</v>
+        <v>-0.0251</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>0.0048</v>
+        <v>0.0015</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>-0.0898</v>
+        <v>-0.0867</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>0.0505</v>
+        <v>0.0541</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>-0.0636</v>
+        <v>-0.06509999999999999</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>-0.0467</v>
+        <v>-0.045</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>0.0779</v>
+        <v>0.079</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>0.0713</v>
+        <v>0.0727</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>0.1073</v>
+        <v>0.1076</v>
       </c>
     </row>
     <row r="16">
@@ -1238,44 +1238,44 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>5426</v>
+        <v>5430.65</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>-0.0322</v>
+        <v>-0.0221</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>-0.05139999999999999</v>
+        <v>-0.0506</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>-0.06</v>
+        <v>-0.0527</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>-0.0115</v>
+        <v>-0.0188</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>0.0276</v>
+        <v>0.0196</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>-0.0741</v>
+        <v>-0.0733</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>0.0781</v>
+        <v>0.079</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>-0.0552</v>
+        <v>-0.0579</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.06570000000000001</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0.0614</v>
+        <v>0.0616</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>0.06</v>
+        <v>0.0608</v>
       </c>
       <c r="O16" s="3" t="n">
         <v>0.0922</v>
@@ -1289,47 +1289,47 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>25338.29</v>
+        <v>25503.07</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>-0.0226</v>
+        <v>-0.0176</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>-0.029</v>
+        <v>-0.0227</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>-0.04219999999999999</v>
+        <v>-0.0352</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>-0.0646</v>
+        <v>-0.0611</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>-0.0224</v>
+        <v>-0.0218</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>-0.0114</v>
+        <v>-0.0049</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>0.0307</v>
+        <v>0.0374</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>0.1222</v>
+        <v>0.1224</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>0.0358</v>
+        <v>0.0395</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>0.2273</v>
+        <v>0.2297</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>0.2406</v>
+        <v>0.2453</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>0.1679</v>
+        <v>0.1686</v>
       </c>
     </row>
     <row r="18">
@@ -1340,47 +1340,47 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>37404.52</v>
+        <v>37368.99</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>-0.04</v>
+        <v>-0.0462</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>-0.0512</v>
+        <v>-0.0521</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>-0.0418</v>
+        <v>-0.0466</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>-0.0394</v>
+        <v>-0.0434</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>0.0315</v>
+        <v>0.0153</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>-0.0398</v>
+        <v>-0.0407</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>0.1035</v>
+        <v>0.1025</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>-0.0287</v>
+        <v>-0.0339</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>-0.0906</v>
+        <v>-0.0926</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>0.09810000000000001</v>
+        <v>0.0977</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>0.09029999999999999</v>
+        <v>0.09279999999999999</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>0.1619</v>
+        <v>0.1617</v>
       </c>
     </row>
     <row r="19">
@@ -1391,47 +1391,47 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>28180.28</v>
+        <v>28238.7</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>-0.0331</v>
+        <v>-0.0208</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>-0.0541</v>
+        <v>-0.0522</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>-0.0684</v>
+        <v>-0.06059999999999999</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>-0.0233</v>
+        <v>-0.031</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>0.0336</v>
+        <v>0.0214</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>-0.07969999999999999</v>
+        <v>-0.07780000000000001</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>0.0781</v>
+        <v>0.0803</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>-0.062</v>
+        <v>-0.0645</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>-0.0725</v>
+        <v>-0.07099999999999999</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>0.0694</v>
+        <v>0.0701</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>0.0663</v>
+        <v>0.06759999999999999</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>0.1174</v>
+        <v>0.1176</v>
       </c>
     </row>
     <row r="20">
@@ -1442,47 +1442,47 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>29731.75</v>
+        <v>29703.5</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>-0.04</v>
+        <v>-0.0462</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>-0.0517</v>
+        <v>-0.0526</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>-0.0426</v>
+        <v>-0.0474</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>-0.04219999999999999</v>
+        <v>-0.0462</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>0.0264</v>
+        <v>0.0103</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>-0.0455</v>
+        <v>-0.0464</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>0.0983</v>
+        <v>0.09720000000000001</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>-0.0346</v>
+        <v>-0.0397</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>-0.09660000000000001</v>
+        <v>-0.09859999999999999</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>0.0892</v>
+        <v>0.0888</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>0.0806</v>
+        <v>0.08310000000000001</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>0.1508</v>
+        <v>0.1506</v>
       </c>
     </row>
     <row r="21">
@@ -1493,47 +1493,47 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>54486.9</v>
+        <v>54665.6</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>-0.0381</v>
+        <v>-0.0364</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>-0.053</v>
+        <v>-0.0499</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>-0.0301</v>
+        <v>-0.0304</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>0.0242</v>
+        <v>0.0178</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>0.1468</v>
+        <v>0.1335</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>0.083</v>
+        <v>0.0866</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>0.2248</v>
+        <v>0.2288</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>0.0595</v>
+        <v>0.0567</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>-0.0471</v>
+        <v>-0.0508</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>0.148</v>
+        <v>0.1491</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>0.1138</v>
+        <v>0.1157</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>0.191</v>
+        <v>0.1913</v>
       </c>
     </row>
     <row r="22">
@@ -1544,47 +1544,47 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>25743.7</v>
+        <v>25954.05</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>-0.0293</v>
+        <v>-0.0202</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>-0.0529</v>
+        <v>-0.0452</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>-0.0596</v>
+        <v>-0.0509</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>-0.0161</v>
+        <v>-0.0108</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>0.018</v>
+        <v>0.0182</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>-0.0492</v>
+        <v>-0.0415</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>0.07440000000000001</v>
+        <v>0.0832</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>-0.038</v>
+        <v>-0.0355</v>
       </c>
       <c r="L22" s="3" t="n">
-        <v>-0.0795</v>
+        <v>-0.0764</v>
       </c>
       <c r="M22" s="3" t="n">
-        <v>0.0885</v>
+        <v>0.09140000000000001</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>0.07389999999999999</v>
+        <v>0.0767</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>0.116</v>
+        <v>0.1169</v>
       </c>
     </row>
     <row r="23">
@@ -1595,44 +1595,44 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>10132.65</v>
+        <v>10115.98</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>-0.08539999999999999</v>
+        <v>-0.0771</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>-0.059</v>
+        <v>-0.06059999999999999</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>-0.0679</v>
+        <v>-0.0722</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>0.0029</v>
+        <v>-0.0364</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>0.1431</v>
+        <v>0.1298</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>0.1858</v>
+        <v>0.1838</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>0.2694</v>
+        <v>0.2673</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>0.1346</v>
+        <v>0.1252</v>
       </c>
       <c r="L23" s="3" t="n">
-        <v>0.162</v>
+        <v>0.1664</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>0.4147999999999999</v>
+        <v>0.4136</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>0.5065999999999999</v>
+        <v>0.508</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -1648,47 +1648,47 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>11200.17</v>
+        <v>11361.33</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>-0.0302</v>
+        <v>-0.0112</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>-0.0524</v>
+        <v>-0.0388</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>-0.0664</v>
+        <v>-0.04940000000000001</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>-0.0472</v>
+        <v>-0.0501</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>-0.0445</v>
+        <v>-0.038</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>-0.0368</v>
+        <v>-0.023</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>0.0433</v>
+        <v>0.0583</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>0.1578</v>
+        <v>0.1694</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>0.1097</v>
+        <v>0.1181</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>0.1819</v>
+        <v>0.1874</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>0.276</v>
+        <v>0.2874</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>0.1065</v>
+        <v>0.1081</v>
       </c>
     </row>
     <row r="25">
@@ -1699,47 +1699,47 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>78319.77</v>
+        <v>79018.42</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>-0.0173</v>
+        <v>-0.0001</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>-0.0384</v>
+        <v>-0.0299</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>-0.0295</v>
+        <v>-0.021</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>-0.0214</v>
+        <v>-0.0176</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>0.0234</v>
+        <v>0.0242</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>-0.0574</v>
+        <v>-0.049</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>0.1171</v>
+        <v>0.127</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>0.0232</v>
+        <v>0.0275</v>
       </c>
       <c r="L25" s="3" t="n">
-        <v>0.04389999999999999</v>
+        <v>0.04650000000000001</v>
       </c>
       <c r="M25" s="3" t="n">
-        <v>0.073</v>
+        <v>0.0761</v>
       </c>
       <c r="N25" s="3" t="n">
-        <v>0.09050000000000001</v>
+        <v>0.0916</v>
       </c>
       <c r="O25" s="3" t="n">
-        <v>0.1154</v>
+        <v>0.1163</v>
       </c>
     </row>
     <row r="26">
@@ -1750,47 +1750,47 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>32043.48</v>
+        <v>32297.32</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>-0.0147</v>
+        <v>0.0026</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>-0.0334</v>
+        <v>-0.0258</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>-0.0064</v>
+        <v>-0.001</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>-0.0245</v>
+        <v>-0.016</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>0.04480000000000001</v>
+        <v>0.0438</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>-0.0518</v>
+        <v>-0.0443</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>0.1279</v>
+        <v>0.1368</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>0.0192</v>
+        <v>0.0193</v>
       </c>
       <c r="L26" s="3" t="n">
-        <v>0.0247</v>
+        <v>0.0263</v>
       </c>
       <c r="M26" s="3" t="n">
-        <v>0.049</v>
+        <v>0.0517</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>0.07290000000000001</v>
+        <v>0.07400000000000001</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>0.0989</v>
+        <v>0.09970000000000001</v>
       </c>
     </row>
     <row r="27">
@@ -1801,47 +1801,47 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>32088.15</v>
+        <v>32325.83</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>-0.0241</v>
+        <v>-0.004500000000000001</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>-0.0463</v>
+        <v>-0.0392</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>-0.0431</v>
+        <v>-0.0362</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>-0.0458</v>
+        <v>-0.0374</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>-0.0172</v>
+        <v>-0.0176</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>-0.08400000000000001</v>
+        <v>-0.07719999999999999</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>0.0746</v>
+        <v>0.0825</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>-0.0413</v>
+        <v>-0.0379</v>
       </c>
       <c r="L27" s="3" t="n">
-        <v>0.0323</v>
+        <v>0.0359</v>
       </c>
       <c r="M27" s="3" t="n">
-        <v>0.0793</v>
+        <v>0.0819</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>0.0745</v>
+        <v>0.0747</v>
       </c>
       <c r="O27" s="3" t="n">
-        <v>0.1273</v>
+        <v>0.1281</v>
       </c>
     </row>
     <row r="28">
@@ -1852,47 +1852,47 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>17149.92</v>
+        <v>17200.12</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>-0.025</v>
+        <v>-0.0249</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>-0.0216</v>
+        <v>-0.0188</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>-0.0351</v>
+        <v>-0.0339</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>-0.0483</v>
+        <v>-0.0551</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>-0.0464</v>
+        <v>-0.0478</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>-0.0252</v>
+        <v>-0.0224</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>-0.0027</v>
+        <v>0.0002</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>-0.004099999999999999</v>
+        <v>-0.0097</v>
       </c>
       <c r="L28" s="3" t="n">
-        <v>-0.0491</v>
+        <v>-0.0493</v>
       </c>
       <c r="M28" s="3" t="n">
-        <v>0.1995</v>
+        <v>0.2004</v>
       </c>
       <c r="N28" s="3" t="n">
-        <v>0.2247</v>
+        <v>0.2276</v>
       </c>
       <c r="O28" s="3" t="n">
-        <v>0.1406</v>
+        <v>0.1409</v>
       </c>
     </row>
     <row r="29">
@@ -1903,47 +1903,47 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>907.58</v>
+        <v>916.55</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>-0.08699999999999999</v>
+        <v>-0.057</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>-0.0992</v>
+        <v>-0.09029999999999999</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>-0.0907</v>
+        <v>-0.0949</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>-0.0004</v>
+        <v>0.0138</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>0.1499</v>
+        <v>0.1302</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>-0.0683</v>
+        <v>-0.0591</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>0.2561</v>
+        <v>0.2685</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>-0.09669999999999999</v>
+        <v>-0.0974</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>-0.1171</v>
+        <v>-0.1156</v>
       </c>
       <c r="M29" s="3" t="n">
-        <v>0.1192</v>
+        <v>0.1228</v>
       </c>
       <c r="N29" s="3" t="n">
-        <v>0.1439</v>
+        <v>0.1515</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>0.1523</v>
+        <v>0.1534</v>
       </c>
     </row>
     <row r="30">
@@ -1954,47 +1954,47 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>35815.54</v>
+        <v>35999</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>-0.0367</v>
+        <v>-0.0275</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>-0.0723</v>
+        <v>-0.0675</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>-0.0839</v>
+        <v>-0.07829999999999999</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>0.0016</v>
+        <v>0.013</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>0.075</v>
+        <v>0.0602</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>-0.04099999999999999</v>
+        <v>-0.0361</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>0.1355</v>
+        <v>0.1413</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>0.0105</v>
+        <v>0.0012</v>
       </c>
       <c r="L30" s="3" t="n">
-        <v>0.028</v>
+        <v>0.0306</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>0.1873</v>
+        <v>0.1891</v>
       </c>
       <c r="N30" s="3" t="n">
-        <v>0.2205</v>
+        <v>0.2217</v>
       </c>
       <c r="O30" s="3" t="n">
-        <v>0.1138</v>
+        <v>0.1144</v>
       </c>
     </row>
     <row r="31">
@@ -2005,47 +2005,47 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>20469.86</v>
+        <v>20511.22</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>-0.0408</v>
+        <v>-0.0366</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>-0.0602</v>
+        <v>-0.0583</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>-0.0579</v>
+        <v>-0.0582</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>-0.015</v>
+        <v>-0.02</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>0.0611</v>
+        <v>0.0534</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>0.019</v>
+        <v>0.0211</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>0.117</v>
+        <v>0.1193</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>0.04769999999999999</v>
+        <v>0.0395</v>
       </c>
       <c r="L31" s="3" t="n">
-        <v>0.0208</v>
+        <v>0.0212</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>0.168</v>
+        <v>0.1686</v>
       </c>
       <c r="N31" s="3" t="n">
-        <v>0.1534</v>
+        <v>0.1563</v>
       </c>
       <c r="O31" s="3" t="n">
-        <v>0.1368</v>
+        <v>0.137</v>
       </c>
     </row>
     <row r="32">
@@ -2056,47 +2056,47 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>11770.22</v>
+        <v>11767.56</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>-0.0255</v>
+        <v>-0.0231</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>-0.0287</v>
+        <v>-0.0289</v>
       </c>
       <c r="F32" s="3" t="n">
         <v>-0.0534</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>-0.05139999999999999</v>
+        <v>-0.0559</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>0.0113</v>
+        <v>-0.0005</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>-0.0668</v>
+        <v>-0.067</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>0.0471</v>
+        <v>0.04679999999999999</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>-0.0124</v>
+        <v>-0.0227</v>
       </c>
       <c r="L32" s="3" t="n">
-        <v>-0.0144</v>
+        <v>-0.0154</v>
       </c>
       <c r="M32" s="3" t="n">
-        <v>0.133</v>
+        <v>0.1328</v>
       </c>
       <c r="N32" s="3" t="n">
-        <v>0.1357</v>
+        <v>0.1367</v>
       </c>
       <c r="O32" s="3" t="n">
-        <v>0.1352</v>
+        <v>0.1351</v>
       </c>
     </row>
     <row r="33">
@@ -2107,47 +2107,47 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>19454.88</v>
+        <v>19425.8</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>-0.0196</v>
+        <v>-0.0185</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>-0.0379</v>
+        <v>-0.0394</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>-0.0125</v>
+        <v>-0.009399999999999999</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>0.0584</v>
+        <v>0.05889999999999999</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>0.1321</v>
+        <v>0.1281</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>0.1188</v>
+        <v>0.1171</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>0.1512</v>
+        <v>0.1495</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>0.1168</v>
+        <v>0.1145</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>0.0588</v>
+        <v>0.057</v>
       </c>
       <c r="M33" s="3" t="n">
-        <v>0.1916</v>
+        <v>0.1908</v>
       </c>
       <c r="N33" s="3" t="n">
-        <v>0.1285</v>
+        <v>0.1305</v>
       </c>
       <c r="O33" s="3" t="n">
-        <v>0.1054</v>
+        <v>0.1053</v>
       </c>
     </row>
     <row r="34">
@@ -2158,47 +2158,47 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>19331.94</v>
+        <v>19440.19</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>-0.03700000000000001</v>
+        <v>-0.0486</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>-0.0396</v>
+        <v>-0.0342</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>-0.0206</v>
+        <v>-0.0273</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>-0.0143</v>
+        <v>-0.0186</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>0.0984</v>
+        <v>0.1057</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>0.1453</v>
+        <v>0.1517</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>0.145</v>
+        <v>0.1514</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>0.2942</v>
+        <v>0.2907</v>
       </c>
       <c r="L34" s="3" t="n">
-        <v>0.1737</v>
+        <v>0.174</v>
       </c>
       <c r="M34" s="3" t="n">
-        <v>0.2263</v>
+        <v>0.2284</v>
       </c>
       <c r="N34" s="3" t="n">
-        <v>0.1831</v>
+        <v>0.1901</v>
       </c>
       <c r="O34" s="3" t="n">
-        <v>0.201</v>
+        <v>0.2016</v>
       </c>
     </row>
     <row r="35">
@@ -2209,47 +2209,47 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>9703.540000000001</v>
+        <v>9735.99</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>-0.0323</v>
+        <v>-0.0254</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>-0.0552</v>
+        <v>-0.0521</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>-0.0609</v>
+        <v>-0.0568</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>0.0273</v>
+        <v>0.0254</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>0.1282</v>
+        <v>0.109</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>-0.0157</v>
+        <v>-0.0124</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>0.1867</v>
+        <v>0.1907</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>-0.0428</v>
+        <v>-0.0488</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>-0.0472</v>
+        <v>-0.04679999999999999</v>
       </c>
       <c r="M35" s="3" t="n">
-        <v>0.1103</v>
+        <v>0.1114</v>
       </c>
       <c r="N35" s="3" t="n">
-        <v>0.1191</v>
+        <v>0.1206</v>
       </c>
       <c r="O35" s="3" t="n">
-        <v>0.1167</v>
+        <v>0.1171</v>
       </c>
     </row>
     <row r="36">
@@ -2260,47 +2260,47 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>14021.65</v>
+        <v>14073.22</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>-0.0278</v>
+        <v>-0.0304</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>-0.0276</v>
+        <v>-0.024</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>-0.0406</v>
+        <v>-0.0391</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>-0.0562</v>
+        <v>-0.0561</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>-0.0005999999999999999</v>
+        <v>-0.0001</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>-0.0023</v>
+        <v>0.0014</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>0.03700000000000001</v>
+        <v>0.0408</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>0.0663</v>
+        <v>0.0614</v>
       </c>
       <c r="L36" s="3" t="n">
-        <v>0.0133</v>
+        <v>0.012</v>
       </c>
       <c r="M36" s="3" t="n">
-        <v>0.1356</v>
+        <v>0.1368</v>
       </c>
       <c r="N36" s="3" t="n">
-        <v>0.1178</v>
+        <v>0.1221</v>
       </c>
       <c r="O36" s="3" t="n">
-        <v>0.1397</v>
+        <v>0.1401</v>
       </c>
     </row>
     <row r="37">
@@ -2311,47 +2311,47 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>74387.52</v>
+        <v>75597.22</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>-0.0201</v>
+        <v>0.005500000000000001</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>-0.026</v>
+        <v>-0.0101</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>-0.07780000000000001</v>
+        <v>-0.0529</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>-0.0926</v>
+        <v>-0.0762</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>-0.0623</v>
+        <v>-0.0466</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>-0.1862</v>
+        <v>-0.1729</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>-0.0095</v>
+        <v>0.0066</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>-0.1999</v>
+        <v>-0.1847</v>
       </c>
       <c r="L37" s="3" t="n">
-        <v>-0.1574</v>
+        <v>-0.1479</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>-0.0321</v>
+        <v>-0.0269</v>
       </c>
       <c r="N37" s="3" t="n">
-        <v>0.0351</v>
+        <v>0.0395</v>
       </c>
       <c r="O37" s="3" t="n">
-        <v>0.08710000000000001</v>
+        <v>0.0888</v>
       </c>
     </row>
     <row r="38">
@@ -2362,47 +2362,47 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>5400.02</v>
+        <v>5381.66</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>-0.0142</v>
+        <v>-0.0283</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>0.0033</v>
+        <v>-0.0001</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>-0.0417</v>
+        <v>-0.0379</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>-0.08539999999999999</v>
+        <v>-0.0873</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>-0.0014</v>
+        <v>-0.0071</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>0.0509</v>
+        <v>0.0473</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>0.038</v>
+        <v>0.0344</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>0.0206</v>
+        <v>0.008399999999999999</v>
       </c>
       <c r="L38" s="3" t="n">
-        <v>-0.0789</v>
+        <v>-0.08960000000000001</v>
       </c>
       <c r="M38" s="3" t="n">
-        <v>0.1363</v>
+        <v>0.1348</v>
       </c>
       <c r="N38" s="3" t="n">
-        <v>0.1363</v>
+        <v>0.1386</v>
       </c>
       <c r="O38" s="3" t="n">
-        <v>0.1205</v>
+        <v>0.1201</v>
       </c>
     </row>
     <row r="39">
@@ -2413,47 +2413,47 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>5858.52</v>
+        <v>5878.62</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>-0.0239</v>
+        <v>-0.0137</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>-0.0459</v>
+        <v>-0.04269999999999999</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>-0.0588</v>
+        <v>-0.052</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>-0.0143</v>
+        <v>-0.0163</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>0.0296</v>
+        <v>0.0204</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>-0.0669</v>
+        <v>-0.06370000000000001</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>0.0859</v>
+        <v>0.08960000000000001</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>-0.029</v>
+        <v>-0.031</v>
       </c>
       <c r="L39" s="3" t="n">
-        <v>-0.0225</v>
+        <v>-0.021</v>
       </c>
       <c r="M39" s="3" t="n">
-        <v>0.08960000000000001</v>
+        <v>0.09080000000000001</v>
       </c>
       <c r="N39" s="3" t="n">
-        <v>0.0693</v>
+        <v>0.0706</v>
       </c>
       <c r="O39" s="3" t="n">
-        <v>0.1286</v>
+        <v>0.129</v>
       </c>
     </row>
     <row r="40">
@@ -2464,47 +2464,47 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>16620.01</v>
+        <v>16737.03</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>-0.0225</v>
+        <v>-0.0142</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>-0.0268</v>
+        <v>-0.0199</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>-0.035</v>
+        <v>-0.0289</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>-0.04219999999999999</v>
+        <v>-0.0362</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>-0.0259</v>
+        <v>-0.0252</v>
       </c>
       <c r="I40" s="3" t="n">
-        <v>-0.1118</v>
+        <v>-0.1055</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>0.004699999999999999</v>
+        <v>0.0118</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>-0.0225</v>
+        <v>-0.0239</v>
       </c>
       <c r="L40" s="3" t="n">
-        <v>-0.0684</v>
+        <v>-0.0658</v>
       </c>
       <c r="M40" s="3" t="n">
-        <v>0.1137</v>
+        <v>0.1162</v>
       </c>
       <c r="N40" s="3" t="n">
-        <v>0.0873</v>
+        <v>0.0919</v>
       </c>
       <c r="O40" s="3" t="n">
-        <v>0.1416</v>
+        <v>0.1424</v>
       </c>
     </row>
     <row r="41">
@@ -2515,47 +2515,47 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>65774.78</v>
+        <v>65837.55</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>-0.0248</v>
+        <v>-0.03</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>-0.0187</v>
+        <v>-0.0177</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>-0.0339</v>
+        <v>-0.0354</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>-0.0645</v>
+        <v>-0.0711</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>0.0387</v>
+        <v>0.035</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>0.062</v>
+        <v>0.063</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>0.07240000000000001</v>
+        <v>0.07339999999999999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>0.0698</v>
+        <v>0.0614</v>
       </c>
       <c r="L41" s="3" t="n">
-        <v>-0.0493</v>
+        <v>-0.0528</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>0.1227</v>
+        <v>0.1229</v>
       </c>
       <c r="N41" s="3" t="n">
-        <v>0.1312</v>
+        <v>0.1337</v>
       </c>
       <c r="O41" s="3" t="n">
-        <v>0.167</v>
+        <v>0.1671</v>
       </c>
     </row>
     <row r="42">
@@ -2566,47 +2566,47 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>42683.53</v>
+        <v>42008.16</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>-0.011</v>
+        <v>0.006</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>-0.0525</v>
+        <v>-0.0674</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>-0.0575</v>
+        <v>-0.0558</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>0.0379</v>
+        <v>0.0129</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>0.0366</v>
+        <v>-0.0073</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>-0.2092</v>
+        <v>-0.2217</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>0.0259</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>-0.1591</v>
+        <v>-0.1795</v>
       </c>
       <c r="L42" s="3" t="n">
-        <v>-0.1563</v>
+        <v>-0.163</v>
       </c>
       <c r="M42" s="3" t="n">
-        <v>-0.0189</v>
+        <v>-0.024</v>
       </c>
       <c r="N42" s="3" t="n">
-        <v>-0.0183</v>
+        <v>-0.0203</v>
       </c>
       <c r="O42" s="3" t="n">
-        <v>0.1327</v>
+        <v>0.1309</v>
       </c>
     </row>
     <row r="43">
@@ -2617,47 +2617,47 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>7585.73</v>
+        <v>7551.81</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>-0.0114</v>
+        <v>-0.0111</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>-0.0131</v>
+        <v>-0.0175</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>-0.0257</v>
+        <v>-0.025</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>0.009899999999999999</v>
+        <v>0.0178</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>0.1295</v>
+        <v>0.1399</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>0.1081</v>
+        <v>0.1032</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>0.1619</v>
+        <v>0.1567</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>0.1467</v>
+        <v>0.143</v>
       </c>
       <c r="L43" s="3" t="n">
-        <v>0.1608</v>
+        <v>0.158</v>
       </c>
       <c r="M43" s="3" t="n">
-        <v>0.1945</v>
+        <v>0.1925</v>
       </c>
       <c r="N43" s="3" t="n">
-        <v>0.1115</v>
+        <v>0.1125</v>
       </c>
       <c r="O43" s="3" t="n">
-        <v>0.135</v>
+        <v>0.1345</v>
       </c>
     </row>
     <row r="44">
@@ -2668,44 +2668,44 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>28937.84</v>
+        <v>28945.06</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>-0.0193</v>
+        <v>-0.0162</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>-0.0176</v>
+        <v>-0.0174</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>-0.0369</v>
+        <v>-0.035</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>-0.0344</v>
+        <v>-0.0245</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>0.1678</v>
+        <v>0.1851</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>0.1461</v>
+        <v>0.1463</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>0.2189</v>
+        <v>0.2192</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>0.1912</v>
+        <v>0.1924</v>
       </c>
       <c r="L44" s="3" t="n">
-        <v>0.2172</v>
+        <v>0.2209</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>0.2393</v>
+        <v>0.2391</v>
       </c>
       <c r="N44" s="3" t="n">
-        <v>0.1329</v>
+        <v>0.1356</v>
       </c>
       <c r="O44" s="3" t="n">
         <v>0.1964</v>
@@ -2719,47 +2719,47 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
-        <v>63662.9</v>
+        <v>64136.25</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>-0.0227</v>
+        <v>-0.0174</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>-0.0399</v>
+        <v>-0.0328</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>-0.0803</v>
+        <v>-0.0493</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>-0.08929999999999999</v>
+        <v>-0.0974</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>0.1525</v>
+        <v>0.2017</v>
       </c>
       <c r="I45" s="3" t="n">
-        <v>0.2647</v>
+        <v>0.2741</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>0.2467</v>
+        <v>0.256</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>0.4178</v>
+        <v>0.4319</v>
       </c>
       <c r="L45" s="3" t="n">
-        <v>0.318</v>
+        <v>0.3313</v>
       </c>
       <c r="M45" s="3" t="n">
-        <v>0.2379</v>
+        <v>0.2408</v>
       </c>
       <c r="N45" s="3" t="n">
-        <v>0.1587</v>
+        <v>0.1603</v>
       </c>
       <c r="O45" s="3" t="n">
-        <v>0.1445</v>
+        <v>0.1453</v>
       </c>
     </row>
     <row r="46">
@@ -2770,47 +2770,47 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>25369.23</v>
+        <v>25677.47</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>-0.008100000000000001</v>
+        <v>0.0125</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>-0.0339</v>
+        <v>-0.0221</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>-0.0368</v>
+        <v>-0.0173</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>0.0174</v>
+        <v>0.026</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>0.0794</v>
+        <v>0.1243</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>0.0359</v>
+        <v>0.04849999999999999</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>0.1186</v>
+        <v>0.1322</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>0.08740000000000001</v>
+        <v>0.0992</v>
       </c>
       <c r="L46" s="3" t="n">
-        <v>0.167</v>
+        <v>0.1711</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>0.1685</v>
+        <v>0.1777</v>
       </c>
       <c r="N46" s="3" t="n">
-        <v>0.1038</v>
+        <v>0.1064</v>
       </c>
       <c r="O46" s="3" t="n">
-        <v>0.0946</v>
+        <v>0.0949</v>
       </c>
     </row>
     <row r="47">
@@ -2821,47 +2821,47 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>8088.8</v>
+        <v>8160.39</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>-0.0083</v>
+        <v>0.0054</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>-0.0295</v>
+        <v>-0.0209</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>-0.0572</v>
+        <v>-0.04099999999999999</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>-0.0406</v>
+        <v>-0.0363</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>0.0149</v>
+        <v>0.0451</v>
       </c>
       <c r="I47" s="3" t="n">
-        <v>-0.0074</v>
+        <v>0.0013</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>0.0348</v>
+        <v>0.04389999999999999</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>0.0346</v>
+        <v>0.048</v>
       </c>
       <c r="L47" s="3" t="n">
-        <v>0.0421</v>
+        <v>0.044</v>
       </c>
       <c r="M47" s="3" t="n">
-        <v>0.0311</v>
+        <v>0.039</v>
       </c>
       <c r="N47" s="3" t="n">
-        <v>0.0425</v>
+        <v>0.0443</v>
       </c>
       <c r="O47" s="3" t="n">
-        <v>0.0644</v>
+        <v>0.0639</v>
       </c>
     </row>
     <row r="48">
@@ -2872,47 +2872,47 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>10680.53</v>
+        <v>10708.15</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>0.001</v>
+        <v>0.009399999999999999</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>-0.0133</v>
+        <v>-0.0107</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>-0.0037</v>
+        <v>-0.0019</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>0.0164</v>
+        <v>0.0297</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>0.0364</v>
+        <v>0.0641</v>
       </c>
       <c r="I48" s="3" t="n">
-        <v>0.07539999999999999</v>
+        <v>0.07820000000000001</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>0.0495</v>
+        <v>0.0522</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>0.1615</v>
+        <v>0.1629</v>
       </c>
       <c r="L48" s="3" t="n">
-        <v>0.136</v>
+        <v>0.1353</v>
       </c>
       <c r="M48" s="3" t="n">
-        <v>0.1145</v>
+        <v>0.1186</v>
       </c>
       <c r="N48" s="3" t="n">
-        <v>0.08939999999999999</v>
+        <v>0.08990000000000001</v>
       </c>
       <c r="O48" s="3" t="n">
-        <v>0.0476</v>
+        <v>0.0463</v>
       </c>
     </row>
     <row r="49">
@@ -2923,47 +2923,47 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>24697.35</v>
+        <v>24604.29</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>-0.0229</v>
+        <v>-0.014</v>
       </c>
       <c r="E49" s="3" t="n">
+        <v>-0.0377</v>
+      </c>
+      <c r="F49" s="3" t="n">
         <v>-0.034</v>
       </c>
-      <c r="F49" s="3" t="n">
-        <v>-0.0297</v>
-      </c>
       <c r="G49" s="3" t="n">
-        <v>0.0158</v>
+        <v>0.0284</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>-0.051</v>
+        <v>-0.0351</v>
       </c>
       <c r="I49" s="3" t="n">
-        <v>-0.0364</v>
+        <v>-0.04</v>
       </c>
       <c r="J49" s="3" t="n">
-        <v>-0.0037</v>
+        <v>-0.0074</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>-0.0659</v>
+        <v>-0.08560000000000001</v>
       </c>
       <c r="L49" s="3" t="n">
-        <v>0.1908</v>
+        <v>0.1805</v>
       </c>
       <c r="M49" s="3" t="n">
-        <v>0.1073</v>
+        <v>0.1113</v>
       </c>
       <c r="N49" s="3" t="n">
-        <v>-0.0018</v>
+        <v>-0.0026</v>
       </c>
       <c r="O49" s="3" t="n">
-        <v>0.005699999999999999</v>
+        <v>0.0044</v>
       </c>
     </row>
     <row r="50">
@@ -2974,47 +2974,47 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>4478.55</v>
+        <v>4460.16</v>
       </c>
       <c r="D50" s="3" t="n">
-        <v>-0.0206</v>
+        <v>-0.0194</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>-0.0317</v>
+        <v>-0.0357</v>
       </c>
       <c r="F50" s="3" t="n">
-        <v>-0.0554</v>
+        <v>-0.0562</v>
       </c>
       <c r="G50" s="3" t="n">
-        <v>-0.09179999999999999</v>
+        <v>-0.0974</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>-0.0386</v>
+        <v>-0.0269</v>
       </c>
       <c r="I50" s="3" t="n">
-        <v>-0.0327</v>
+        <v>-0.0367</v>
       </c>
       <c r="J50" s="3" t="n">
-        <v>0.0064</v>
+        <v>0.0023</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>-0.009899999999999999</v>
+        <v>-0.02</v>
       </c>
       <c r="L50" s="3" t="n">
-        <v>0.1899</v>
+        <v>0.1872</v>
       </c>
       <c r="M50" s="3" t="n">
-        <v>0.06480000000000001</v>
+        <v>0.0617</v>
       </c>
       <c r="N50" s="3" t="n">
-        <v>-0.0161</v>
+        <v>-0.0169</v>
       </c>
       <c r="O50" s="3" t="n">
-        <v>0.0329</v>
+        <v>0.0318</v>
       </c>
     </row>
     <row r="51">
@@ -3025,47 +3025,47 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v>95.93000000000001</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>0.0117</v>
+        <v>0.0086</v>
       </c>
       <c r="E51" s="3" t="n">
         <v>0.0058</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>0.0051</v>
+        <v>0.0025</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>0.011</v>
+        <v>0.0113</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>0.0383</v>
+        <v>0.0288</v>
       </c>
       <c r="I51" s="3" t="n">
-        <v>0.0687</v>
+        <v>0.06860000000000001</v>
       </c>
       <c r="J51" s="3" t="n">
         <v>0.0167</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>0.0886</v>
+        <v>0.0915</v>
       </c>
       <c r="L51" s="3" t="n">
-        <v>0.06950000000000001</v>
+        <v>0.0694</v>
       </c>
       <c r="M51" s="3" t="n">
-        <v>0.0493</v>
+        <v>0.0491</v>
       </c>
       <c r="N51" s="3" t="n">
-        <v>0.0546</v>
+        <v>0.0545</v>
       </c>
       <c r="O51" s="3" t="n">
-        <v>0.0368</v>
+        <v>0.0365</v>
       </c>
     </row>
     <row r="52">
@@ -3076,47 +3076,47 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>4362.7</v>
+        <v>4355.9</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>-0.0121</v>
+        <v>-0.002</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>-0.0154</v>
+        <v>-0.017</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>-0.0125</v>
+        <v>-0.0023</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>0.0009</v>
+        <v>0.0312</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>-0.1078</v>
+        <v>-0.0532</v>
       </c>
       <c r="I52" s="3" t="n">
-        <v>0.0086</v>
+        <v>0.006999999999999999</v>
       </c>
       <c r="J52" s="3" t="n">
-        <v>-0.0613</v>
+        <v>-0.06280000000000001</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>0.1827</v>
+        <v>0.1831</v>
       </c>
       <c r="L52" s="3" t="n">
-        <v>0.3005</v>
+        <v>0.3036</v>
       </c>
       <c r="M52" s="3" t="n">
-        <v>0.3134</v>
+        <v>0.3116</v>
       </c>
       <c r="N52" s="3" t="n">
-        <v>0.2007</v>
+        <v>0.2002</v>
       </c>
       <c r="O52" s="3" t="n">
-        <v>0.1282</v>
+        <v>0.1275</v>
       </c>
     </row>
     <row r="53">
@@ -3127,47 +3127,47 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>65.06999999999999</v>
+        <v>64.45999999999999</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>-0.04219999999999999</v>
+        <v>0.0027</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>-0.0173</v>
+        <v>-0.0267</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>-0.0158</v>
+        <v>0.008</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>-0.0795</v>
+        <v>-0.0272</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>-0.1575</v>
+        <v>-0.09089999999999999</v>
       </c>
       <c r="I53" s="3" t="n">
-        <v>-0.0721</v>
+        <v>-0.081</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>-0.1287</v>
+        <v>-0.137</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>0.5322</v>
+        <v>0.5449000000000001</v>
       </c>
       <c r="L53" s="3" t="n">
-        <v>0.4546</v>
+        <v>0.4513</v>
       </c>
       <c r="M53" s="3" t="n">
-        <v>0.4112</v>
+        <v>0.4055</v>
       </c>
       <c r="N53" s="3" t="n">
-        <v>0.2391</v>
+        <v>0.2366</v>
       </c>
       <c r="O53" s="3" t="n">
-        <v>0.1323</v>
+        <v>0.1288</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Manual indices update 2026-09-18
</commit_message>
<xml_diff>
--- a/tracker_auto.xlsx
+++ b/tracker_auto.xlsx
@@ -524,44 +524,44 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>23217.6</v>
+        <v>23270.6</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>-0.0091</v>
+        <v>-0.008800000000000001</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-0.0358</v>
+        <v>-0.0336</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>-0.0441</v>
+        <v>-0.0366</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>-0.036</v>
+        <v>-0.0371</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>-0.0236</v>
+        <v>0.0117</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>-0.1114</v>
+        <v>-0.1094</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.0397</v>
+        <v>0.0421</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>-0.0801</v>
+        <v>-0.08130000000000001</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>-0.0436</v>
+        <v>-0.0432</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>0.0476</v>
+        <v>0.0495</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>0.0572</v>
+        <v>0.0576</v>
       </c>
       <c r="O2" s="3" t="n">
         <v>0.1021</v>
@@ -575,47 +575,47 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>74314.59</v>
+        <v>74294.96000000001</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>-0.007900000000000001</v>
+        <v>-0.006500000000000001</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>-0.0343</v>
+        <v>-0.0346</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>-0.0378</v>
+        <v>-0.034</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>-0.04</v>
+        <v>-0.0327</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>0.0014</v>
+        <v>-0.0032</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>-0.128</v>
+        <v>-0.1282</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>0.0329</v>
+        <v>0.0326</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>-0.1013</v>
+        <v>-0.105</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>-0.05429999999999999</v>
+        <v>-0.0536</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>0.0321</v>
+        <v>0.032</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>0.0472</v>
+        <v>0.0471</v>
       </c>
       <c r="O3" s="3" t="n">
-        <v>0.1001</v>
+        <v>0.1005</v>
       </c>
     </row>
     <row r="4">
@@ -626,47 +626,47 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>70368.60000000001</v>
+        <v>71144</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>-0.0341</v>
+        <v>-0.0191</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>-0.046</v>
+        <v>-0.0355</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>-0.0551</v>
+        <v>-0.0426</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>-0.0262</v>
+        <v>-0.02</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.0716</v>
+        <v>0.1191</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.0145</v>
+        <v>0.0257</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.166</v>
+        <v>0.1789</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>0.0198</v>
+        <v>0.0289</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>-0.0344</v>
+        <v>-0.0277</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>0.1516</v>
+        <v>0.1563</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>0.1028</v>
+        <v>0.1052</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>0.119</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="5">
@@ -677,47 +677,47 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>24282.95</v>
+        <v>24377.75</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>-0.0139</v>
+        <v>-0.0108</v>
       </c>
       <c r="E5" s="3" t="n">
+        <v>-0.034</v>
+      </c>
+      <c r="F5" s="3" t="n">
         <v>-0.0377</v>
       </c>
-      <c r="F5" s="3" t="n">
-        <v>-0.0461</v>
-      </c>
       <c r="G5" s="3" t="n">
-        <v>-0.0342</v>
+        <v>-0.0339</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>-0.0067</v>
+        <v>0.0307</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>-0.0902</v>
+        <v>-0.0866</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0.06150000000000001</v>
+        <v>0.06570000000000001</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>-0.0626</v>
+        <v>-0.062</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>-0.04190000000000001</v>
+        <v>-0.0404</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>0.06480000000000001</v>
+        <v>0.0673</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>0.0634</v>
+        <v>0.06419999999999999</v>
       </c>
       <c r="O5" s="3" t="n">
-        <v>0.1045</v>
+        <v>0.1047</v>
       </c>
     </row>
     <row r="6">
@@ -728,47 +728,47 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>31669.65</v>
+        <v>31892.3</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>-0.0149</v>
+        <v>-0.009000000000000001</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-0.0398</v>
+        <v>-0.033</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-0.04650000000000001</v>
+        <v>-0.0339</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>-0.029</v>
+        <v>-0.0269</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.0149</v>
+        <v>0.0545</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>-0.0498</v>
+        <v>-0.0432</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.07150000000000001</v>
+        <v>0.079</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>-0.019</v>
+        <v>-0.0158</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>-0.0155</v>
+        <v>-0.0125</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>0.0975</v>
+        <v>0.0998</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>0.1005</v>
+        <v>0.102</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>0.1128</v>
+        <v>0.113</v>
       </c>
     </row>
     <row r="7">
@@ -779,47 +779,47 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>33426.35</v>
+        <v>33705.7</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>-0.0252</v>
+        <v>-0.0154</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-0.04480000000000001</v>
+        <v>-0.0368</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>-0.0527</v>
+        <v>-0.04019999999999999</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>-0.0284</v>
+        <v>-0.0257</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.045</v>
+        <v>0.0877</v>
       </c>
       <c r="I7" s="3" t="n">
+        <v>-0.0074</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>0.1315</v>
+      </c>
+      <c r="K7" s="3" t="n">
+        <v>0.0044</v>
+      </c>
+      <c r="L7" s="3" t="n">
         <v>-0.0156</v>
       </c>
-      <c r="J7" s="3" t="n">
-        <v>0.1222</v>
-      </c>
-      <c r="K7" s="3" t="n">
-        <v>-0.0011</v>
-      </c>
-      <c r="L7" s="3" t="n">
-        <v>-0.0199</v>
-      </c>
       <c r="M7" s="3" t="n">
-        <v>0.1227</v>
+        <v>0.1261</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>0.09859999999999999</v>
+        <v>0.1004</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>0.112</v>
+        <v>0.1124</v>
       </c>
     </row>
     <row r="8">
@@ -830,47 +830,47 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>18143.16</v>
+        <v>18233.33</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>-0.0166</v>
+        <v>-0.0116</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-0.0405</v>
+        <v>-0.0357</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-0.0458</v>
+        <v>-0.0365</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>-0.0269</v>
+        <v>-0.0257</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.0168</v>
+        <v>0.05599999999999999</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>-0.06469999999999999</v>
+        <v>-0.0601</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.08650000000000001</v>
+        <v>0.0919</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>-0.0352</v>
+        <v>-0.0332</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>-0.023</v>
+        <v>-0.0208</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>0.0888</v>
+        <v>0.09179999999999999</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>0.08839999999999999</v>
+        <v>0.08939999999999999</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>0.1243</v>
+        <v>0.1246</v>
       </c>
     </row>
     <row r="9">
@@ -881,47 +881,47 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>16120.65</v>
+        <v>16224.6</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>-0.0206</v>
+        <v>-0.0127</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-0.0438</v>
+        <v>-0.03759999999999999</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-0.0462</v>
+        <v>-0.0359</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>-0.0262</v>
+        <v>-0.0241</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>0.0355</v>
+        <v>0.0762</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>-0.0436</v>
+        <v>-0.0374</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>0.1061</v>
+        <v>0.1132</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>-0.0184</v>
+        <v>-0.0146</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>-0.0191</v>
+        <v>-0.0158</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>0.1013</v>
+        <v>0.105</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>0.106</v>
+        <v>0.1074</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>0.1331</v>
+        <v>0.1334</v>
       </c>
     </row>
     <row r="10">
@@ -932,47 +932,47 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>22368.8</v>
+        <v>22568.85</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>-0.0271</v>
+        <v>-0.0146</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>-0.0496</v>
+        <v>-0.0411</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>-0.0463</v>
+        <v>-0.0341</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>-0.0183</v>
+        <v>-0.0142</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.07820000000000001</v>
+        <v>0.1223</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>0.004099999999999999</v>
+        <v>0.0131</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.1512</v>
+        <v>0.1615</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>0.0265</v>
+        <v>0.0338</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>0.0023</v>
+        <v>0.0075</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>0.1367</v>
+        <v>0.1417</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0.148</v>
+        <v>0.15</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>0.1599</v>
+        <v>0.1605</v>
       </c>
     </row>
     <row r="11">
@@ -983,47 +983,47 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>17863.3</v>
+        <v>18009.25</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>-0.0309</v>
+        <v>-0.023</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>-0.0277</v>
+        <v>-0.0198</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>-0.0245</v>
+        <v>-0.0184</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>0.021</v>
+        <v>0.0225</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0.1788</v>
+        <v>0.2207</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>0.0706</v>
+        <v>0.0794</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>0.2502</v>
+        <v>0.2604</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>0.0277</v>
+        <v>0.0308</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>-0.0193</v>
+        <v>-0.0144</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>0.1322</v>
+        <v>0.1374</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>0.1397</v>
+        <v>0.1415</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>0.137</v>
+        <v>0.1373</v>
       </c>
     </row>
     <row r="12">
@@ -1034,47 +1034,47 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>20744.9</v>
+        <v>20924.9</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>-0.0284</v>
+        <v>-0.0176</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>-0.04219999999999999</v>
+        <v>-0.0338</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>-0.0389</v>
+        <v>-0.0287</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>-0.005</v>
+        <v>-0.0017</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.1112</v>
+        <v>0.1547</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>0.0261</v>
+        <v>0.035</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0.1838</v>
+        <v>0.194</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>0.0261</v>
+        <v>0.0319</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>-0.0058</v>
+        <v>-0.0008</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0.1348</v>
+        <v>0.1399</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.1454</v>
+        <v>0.1473</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>0.1523</v>
+        <v>0.1528</v>
       </c>
     </row>
     <row r="13">
@@ -1085,47 +1085,47 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>22532</v>
+        <v>22654.65</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>-0.0186</v>
+        <v>-0.013</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>-0.0392</v>
+        <v>-0.0339</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>-0.0438</v>
+        <v>-0.0348</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>-0.025</v>
+        <v>-0.0238</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>0.028</v>
+        <v>0.0673</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>-0.0561</v>
+        <v>-0.051</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>0.09759999999999999</v>
+        <v>0.1036</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>-0.0358</v>
+        <v>-0.0337</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>-0.0304</v>
+        <v>-0.0278</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>0.08439999999999999</v>
+        <v>0.0876</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>0.08439999999999999</v>
+        <v>0.08560000000000001</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>0.1165</v>
+        <v>0.1168</v>
       </c>
     </row>
     <row r="14">
@@ -1136,47 +1136,47 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>35276.25</v>
+        <v>35439.31</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>-0.018</v>
+        <v>-0.0132</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>-0.0366</v>
+        <v>-0.0321</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>-0.0442</v>
+        <v>-0.0356</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>-0.0235</v>
+        <v>-0.0233</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0.0276</v>
+        <v>0.06570000000000001</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>-0.0579</v>
+        <v>-0.0535</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>0.09609999999999999</v>
+        <v>0.1012</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>-0.0387</v>
+        <v>-0.0373</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>-0.034</v>
+        <v>-0.0318</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0.07980000000000001</v>
+        <v>0.0828</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>0.081</v>
+        <v>0.08199999999999999</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>0.1154</v>
+        <v>0.1156</v>
       </c>
     </row>
     <row r="15">
@@ -1187,47 +1187,47 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>19298.7</v>
+        <v>19378.85</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>-0.0104</v>
+        <v>-0.0064</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>-0.0457</v>
+        <v>-0.0417</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>-0.0515</v>
+        <v>-0.0411</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>-0.0251</v>
+        <v>-0.0231</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>0.0015</v>
+        <v>0.0362</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>-0.0867</v>
+        <v>-0.08289999999999999</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>0.0541</v>
+        <v>0.0585</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>-0.06509999999999999</v>
+        <v>-0.0619</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>-0.045</v>
+        <v>-0.0445</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>0.079</v>
+        <v>0.0795</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>0.0727</v>
+        <v>0.0735</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>0.1076</v>
+        <v>0.1078</v>
       </c>
     </row>
     <row r="16">
@@ -1238,47 +1238,47 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>5430.65</v>
+        <v>5457.8</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>-0.0221</v>
+        <v>-0.0131</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>-0.0506</v>
+        <v>-0.0458</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>-0.0527</v>
+        <v>-0.0418</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>-0.0188</v>
+        <v>-0.0147</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>0.0196</v>
+        <v>0.0565</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>-0.0733</v>
+        <v>-0.06860000000000001</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>0.079</v>
+        <v>0.08439999999999999</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>-0.0579</v>
+        <v>-0.0559</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>-0.06570000000000001</v>
+        <v>-0.06309999999999999</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0.0616</v>
+        <v>0.0634</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>0.0608</v>
+        <v>0.0619</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>0.0922</v>
+        <v>0.0925</v>
       </c>
     </row>
     <row r="17">
@@ -1289,47 +1289,47 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>25503.07</v>
+        <v>25570.99</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>-0.0176</v>
+        <v>-0.015</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>-0.0227</v>
+        <v>-0.0201</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>-0.0352</v>
+        <v>-0.0268</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>-0.0611</v>
+        <v>-0.06</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>-0.0218</v>
+        <v>0.0106</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>-0.0049</v>
+        <v>-0.0023</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>0.0374</v>
+        <v>0.0401</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>0.1224</v>
+        <v>0.1174</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>0.0395</v>
+        <v>0.0431</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>0.2297</v>
+        <v>0.2281</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>0.2453</v>
+        <v>0.2458</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>0.1686</v>
+        <v>0.1679</v>
       </c>
     </row>
     <row r="18">
@@ -1340,47 +1340,47 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>37368.99</v>
+        <v>37906.17</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>-0.0462</v>
+        <v>-0.0251</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>-0.0521</v>
+        <v>-0.0385</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>-0.0466</v>
+        <v>-0.031</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>-0.0434</v>
+        <v>-0.0334</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>0.0153</v>
+        <v>0.06950000000000001</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>-0.0407</v>
+        <v>-0.0269</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>0.1025</v>
+        <v>0.1183</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>-0.0339</v>
+        <v>-0.0205</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>-0.0926</v>
+        <v>-0.0864</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>0.0977</v>
+        <v>0.1024</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>0.09279999999999999</v>
+        <v>0.0958</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>0.1617</v>
+        <v>0.1627</v>
       </c>
     </row>
     <row r="19">
@@ -1391,47 +1391,47 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>28238.7</v>
+        <v>28353.18</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>-0.0208</v>
+        <v>-0.0132</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>-0.0522</v>
+        <v>-0.0483</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>-0.06059999999999999</v>
+        <v>-0.0472</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>-0.031</v>
+        <v>-0.0271</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>0.0214</v>
+        <v>0.05889999999999999</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>-0.07780000000000001</v>
+        <v>-0.0741</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>0.0803</v>
+        <v>0.08470000000000001</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>-0.0645</v>
+        <v>-0.06280000000000001</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>-0.07099999999999999</v>
+        <v>-0.06900000000000001</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>0.0701</v>
+        <v>0.07139999999999999</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>0.06759999999999999</v>
+        <v>0.06849999999999999</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>0.1176</v>
+        <v>0.1181</v>
       </c>
     </row>
     <row r="20">
@@ -1442,47 +1442,47 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>29703.5</v>
+        <v>30130.5</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>-0.0462</v>
+        <v>-0.0251</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>-0.0526</v>
+        <v>-0.039</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>-0.0474</v>
+        <v>-0.0318</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>-0.0462</v>
+        <v>-0.0363</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>0.0103</v>
+        <v>0.0643</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>-0.0464</v>
+        <v>-0.0327</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>0.09720000000000001</v>
+        <v>0.113</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>-0.0397</v>
+        <v>-0.0264</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>-0.09859999999999999</v>
+        <v>-0.0924</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>0.0888</v>
+        <v>0.0935</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>0.08310000000000001</v>
+        <v>0.0861</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>0.1506</v>
+        <v>0.1516</v>
       </c>
     </row>
     <row r="21">
@@ -1493,47 +1493,47 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>54665.6</v>
+        <v>55090.4</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>-0.0364</v>
+        <v>-0.0286</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>-0.0499</v>
+        <v>-0.0426</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>-0.0304</v>
+        <v>-0.0242</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>0.0178</v>
+        <v>0.0221</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>0.1335</v>
+        <v>0.1809</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>0.0866</v>
+        <v>0.095</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>0.2288</v>
+        <v>0.2383</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>0.0567</v>
+        <v>0.0593</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>-0.0508</v>
+        <v>-0.0442</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>0.1491</v>
+        <v>0.1512</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>0.1157</v>
+        <v>0.1174</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>0.1913</v>
+        <v>0.1914</v>
       </c>
     </row>
     <row r="22">
@@ -1544,47 +1544,47 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>25954.05</v>
+        <v>26101</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>-0.0202</v>
+        <v>-0.0131</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>-0.0452</v>
+        <v>-0.0398</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>-0.0509</v>
+        <v>-0.0411</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>-0.0108</v>
+        <v>-0.0091</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>0.0182</v>
+        <v>0.0548</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>-0.0415</v>
+        <v>-0.036</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>0.0832</v>
+        <v>0.08929999999999999</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>-0.0355</v>
+        <v>-0.0292</v>
       </c>
       <c r="L22" s="3" t="n">
-        <v>-0.0764</v>
+        <v>-0.07519999999999999</v>
       </c>
       <c r="M22" s="3" t="n">
-        <v>0.09140000000000001</v>
+        <v>0.09210000000000002</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>0.0767</v>
+        <v>0.0779</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>0.1169</v>
+        <v>0.1174</v>
       </c>
     </row>
     <row r="23">
@@ -1595,44 +1595,44 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>10115.98</v>
+        <v>10274.17</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>-0.0771</v>
+        <v>-0.0534</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>-0.06059999999999999</v>
+        <v>-0.0459</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>-0.0722</v>
+        <v>-0.0697</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>-0.0364</v>
+        <v>-0.025</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>0.1298</v>
+        <v>0.1916</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>0.1838</v>
+        <v>0.2023</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>0.2673</v>
+        <v>0.2871</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>0.1252</v>
+        <v>0.1205</v>
       </c>
       <c r="L23" s="3" t="n">
-        <v>0.1664</v>
+        <v>0.1847</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>0.4136</v>
+        <v>0.4221</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>0.508</v>
+        <v>0.5123</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -1648,47 +1648,47 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>11361.33</v>
+        <v>11343.39</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>-0.0112</v>
+        <v>-0.0165</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>-0.0388</v>
+        <v>-0.0403</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>-0.04940000000000001</v>
+        <v>-0.0413</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>-0.0501</v>
+        <v>-0.0579</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>-0.038</v>
+        <v>-0.0108</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>-0.023</v>
+        <v>-0.0245</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>0.0583</v>
+        <v>0.0566</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>0.1694</v>
+        <v>0.1379</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>0.1181</v>
+        <v>0.1205</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>0.1874</v>
+        <v>0.174</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>0.2874</v>
+        <v>0.2868</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>0.1081</v>
+        <v>0.1073</v>
       </c>
     </row>
     <row r="25">
@@ -1699,47 +1699,47 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>79018.42</v>
+        <v>78686.11</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>-0.0001</v>
+        <v>-0.0074</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>-0.0299</v>
+        <v>-0.0339</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>-0.021</v>
+        <v>-0.0211</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>-0.0176</v>
+        <v>-0.0282</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>0.0242</v>
+        <v>0.0556</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>-0.049</v>
+        <v>-0.053</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>0.127</v>
+        <v>0.1223</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>0.0275</v>
+        <v>0.0168</v>
       </c>
       <c r="L25" s="3" t="n">
-        <v>0.04650000000000001</v>
+        <v>0.04389999999999999</v>
       </c>
       <c r="M25" s="3" t="n">
-        <v>0.0761</v>
+        <v>0.0767</v>
       </c>
       <c r="N25" s="3" t="n">
-        <v>0.0916</v>
+        <v>0.0906</v>
       </c>
       <c r="O25" s="3" t="n">
-        <v>0.1163</v>
+        <v>0.1157</v>
       </c>
     </row>
     <row r="26">
@@ -1750,47 +1750,47 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>32297.32</v>
+        <v>32161.16</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>0.0026</v>
+        <v>-0.005</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>-0.0258</v>
+        <v>-0.0299</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>-0.001</v>
+        <v>-0.0029</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>-0.016</v>
+        <v>-0.0249</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>0.0438</v>
+        <v>0.0761</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>-0.0443</v>
+        <v>-0.0483</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>0.1368</v>
+        <v>0.132</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>0.0193</v>
+        <v>0.0113</v>
       </c>
       <c r="L26" s="3" t="n">
-        <v>0.0263</v>
+        <v>0.0233</v>
       </c>
       <c r="M26" s="3" t="n">
-        <v>0.0517</v>
+        <v>0.0532</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>0.07400000000000001</v>
+        <v>0.0731</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>0.09970000000000001</v>
+        <v>0.0989</v>
       </c>
     </row>
     <row r="27">
@@ -1801,47 +1801,47 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>32325.83</v>
+        <v>32397.43</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>-0.004500000000000001</v>
+        <v>-0.007900000000000001</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>-0.0392</v>
+        <v>-0.0371</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>-0.0362</v>
+        <v>-0.03</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>-0.0374</v>
+        <v>-0.0417</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>-0.0176</v>
+        <v>0.023</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>-0.07719999999999999</v>
+        <v>-0.07519999999999999</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>0.0825</v>
+        <v>0.0849</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>-0.0379</v>
+        <v>-0.0382</v>
       </c>
       <c r="L27" s="3" t="n">
-        <v>0.0359</v>
+        <v>0.0371</v>
       </c>
       <c r="M27" s="3" t="n">
-        <v>0.0819</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>0.0747</v>
+        <v>0.0751</v>
       </c>
       <c r="O27" s="3" t="n">
-        <v>0.1281</v>
+        <v>0.1284</v>
       </c>
     </row>
     <row r="28">
@@ -1852,47 +1852,47 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>17200.12</v>
+        <v>17308.14</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>-0.0249</v>
+        <v>-0.0201</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>-0.0188</v>
+        <v>-0.0126</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>-0.0339</v>
+        <v>-0.0256</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>-0.0551</v>
+        <v>-0.0555</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>-0.0478</v>
+        <v>-0.0197</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>-0.0224</v>
+        <v>-0.0162</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>0.0002</v>
+        <v>0.006500000000000001</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>-0.0097</v>
+        <v>-0.0108</v>
       </c>
       <c r="L28" s="3" t="n">
-        <v>-0.0493</v>
+        <v>-0.0434</v>
       </c>
       <c r="M28" s="3" t="n">
-        <v>0.2004</v>
+        <v>0.1977</v>
       </c>
       <c r="N28" s="3" t="n">
-        <v>0.2276</v>
+        <v>0.229</v>
       </c>
       <c r="O28" s="3" t="n">
-        <v>0.1409</v>
+        <v>0.1405</v>
       </c>
     </row>
     <row r="29">
@@ -1903,47 +1903,47 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>916.55</v>
+        <v>929.86</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>-0.057</v>
+        <v>-0.0431</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>-0.09029999999999999</v>
+        <v>-0.0771</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>-0.0949</v>
+        <v>-0.06849999999999999</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>0.0138</v>
+        <v>0.0215</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>0.1302</v>
+        <v>0.192</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>-0.0591</v>
+        <v>-0.0454</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>0.2685</v>
+        <v>0.2869</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>-0.0974</v>
+        <v>-0.08810000000000001</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>-0.1156</v>
+        <v>-0.1119</v>
       </c>
       <c r="M29" s="3" t="n">
-        <v>0.1228</v>
+        <v>0.1337</v>
       </c>
       <c r="N29" s="3" t="n">
-        <v>0.1515</v>
+        <v>0.1548</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>0.1534</v>
+        <v>0.1535</v>
       </c>
     </row>
     <row r="30">
@@ -1954,47 +1954,47 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>35999</v>
+        <v>36354.4</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>-0.0275</v>
+        <v>-0.0139</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>-0.0675</v>
+        <v>-0.0583</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>-0.07829999999999999</v>
+        <v>-0.07190000000000001</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>0.013</v>
+        <v>0.0222</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>0.0602</v>
+        <v>0.1182</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>-0.0361</v>
+        <v>-0.0266</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>0.1413</v>
+        <v>0.1525</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>0.0012</v>
+        <v>0.005600000000000001</v>
       </c>
       <c r="L30" s="3" t="n">
-        <v>0.0306</v>
+        <v>0.0343</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>0.1891</v>
+        <v>0.19</v>
       </c>
       <c r="N30" s="3" t="n">
-        <v>0.2217</v>
+        <v>0.224</v>
       </c>
       <c r="O30" s="3" t="n">
-        <v>0.1144</v>
+        <v>0.1152</v>
       </c>
     </row>
     <row r="31">
@@ -2005,47 +2005,47 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>20511.22</v>
+        <v>20788.01</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>-0.0366</v>
+        <v>-0.0179</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>-0.0583</v>
+        <v>-0.0455</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>-0.0582</v>
+        <v>-0.0438</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>-0.02</v>
+        <v>-0.0095</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>0.0534</v>
+        <v>0.1035</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>0.0211</v>
+        <v>0.0349</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>0.1193</v>
+        <v>0.1344</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>0.0395</v>
+        <v>0.0499</v>
       </c>
       <c r="L31" s="3" t="n">
-        <v>0.0212</v>
+        <v>0.0285</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>0.1686</v>
+        <v>0.1746</v>
       </c>
       <c r="N31" s="3" t="n">
-        <v>0.1563</v>
+        <v>0.1593</v>
       </c>
       <c r="O31" s="3" t="n">
-        <v>0.137</v>
+        <v>0.1381</v>
       </c>
     </row>
     <row r="32">
@@ -2056,44 +2056,44 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>11767.56</v>
+        <v>11847.6</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>-0.0231</v>
+        <v>-0.018</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>-0.0289</v>
+        <v>-0.0223</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>-0.0534</v>
+        <v>-0.0429</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>-0.0559</v>
+        <v>-0.0525</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>-0.0005</v>
+        <v>0.0352</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>-0.067</v>
+        <v>-0.06059999999999999</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>0.04679999999999999</v>
+        <v>0.0539</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>-0.0227</v>
+        <v>-0.0196</v>
       </c>
       <c r="L32" s="3" t="n">
-        <v>-0.0154</v>
+        <v>-0.0137</v>
       </c>
       <c r="M32" s="3" t="n">
-        <v>0.1328</v>
+        <v>0.1364</v>
       </c>
       <c r="N32" s="3" t="n">
-        <v>0.1367</v>
+        <v>0.1382</v>
       </c>
       <c r="O32" s="3" t="n">
         <v>0.1351</v>
@@ -2107,47 +2107,47 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>19425.8</v>
+        <v>19729.57</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>-0.0185</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>-0.0394</v>
+        <v>-0.0243</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>-0.009399999999999999</v>
+        <v>0.004</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>0.05889999999999999</v>
+        <v>0.065</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>0.1281</v>
+        <v>0.1744</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>0.1171</v>
+        <v>0.1346</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>0.1495</v>
+        <v>0.1674</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>0.1145</v>
+        <v>0.1331</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>0.057</v>
+        <v>0.0653</v>
       </c>
       <c r="M33" s="3" t="n">
-        <v>0.1908</v>
+        <v>0.1993</v>
       </c>
       <c r="N33" s="3" t="n">
-        <v>0.1305</v>
+        <v>0.1339</v>
       </c>
       <c r="O33" s="3" t="n">
-        <v>0.1053</v>
+        <v>0.1067</v>
       </c>
     </row>
     <row r="34">
@@ -2158,47 +2158,47 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>19440.19</v>
+        <v>19622.27</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>-0.0486</v>
+        <v>-0.0335</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>-0.0342</v>
+        <v>-0.0252</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>-0.0273</v>
+        <v>-0.0123</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>-0.0186</v>
+        <v>-0.009399999999999999</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>0.1057</v>
+        <v>0.1534</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>0.1517</v>
+        <v>0.1625</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>0.1514</v>
+        <v>0.1622</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>0.2907</v>
+        <v>0.3094</v>
       </c>
       <c r="L34" s="3" t="n">
-        <v>0.174</v>
+        <v>0.1818</v>
       </c>
       <c r="M34" s="3" t="n">
-        <v>0.2284</v>
+        <v>0.2372</v>
       </c>
       <c r="N34" s="3" t="n">
-        <v>0.1901</v>
+        <v>0.1922</v>
       </c>
       <c r="O34" s="3" t="n">
-        <v>0.2016</v>
+        <v>0.2011</v>
       </c>
     </row>
     <row r="35">
@@ -2209,47 +2209,47 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>9735.99</v>
+        <v>9818</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>-0.0254</v>
+        <v>-0.0157</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>-0.0521</v>
+        <v>-0.0441</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>-0.0568</v>
+        <v>-0.04650000000000001</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>0.0254</v>
+        <v>0.0285</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>0.109</v>
+        <v>0.1603</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>-0.0124</v>
+        <v>-0.004099999999999999</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>0.1907</v>
+        <v>0.2007</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>-0.0488</v>
+        <v>-0.0444</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>-0.04679999999999999</v>
+        <v>-0.0429</v>
       </c>
       <c r="M35" s="3" t="n">
-        <v>0.1114</v>
+        <v>0.114</v>
       </c>
       <c r="N35" s="3" t="n">
-        <v>0.1206</v>
+        <v>0.1224</v>
       </c>
       <c r="O35" s="3" t="n">
-        <v>0.1171</v>
+        <v>0.1179</v>
       </c>
     </row>
     <row r="36">
@@ -2260,47 +2260,47 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>14073.22</v>
+        <v>14161.71</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>-0.0304</v>
+        <v>-0.0215</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>-0.024</v>
+        <v>-0.0179</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>-0.0391</v>
+        <v>-0.0303</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>-0.0561</v>
+        <v>-0.0545</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>-0.0001</v>
+        <v>0.032</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>0.0014</v>
+        <v>0.0077</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>0.0408</v>
+        <v>0.0473</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>0.0614</v>
+        <v>0.0663</v>
       </c>
       <c r="L36" s="3" t="n">
-        <v>0.012</v>
+        <v>0.0153</v>
       </c>
       <c r="M36" s="3" t="n">
-        <v>0.1368</v>
+        <v>0.1407</v>
       </c>
       <c r="N36" s="3" t="n">
-        <v>0.1221</v>
+        <v>0.1235</v>
       </c>
       <c r="O36" s="3" t="n">
-        <v>0.1401</v>
+        <v>0.1398</v>
       </c>
     </row>
     <row r="37">
@@ -2311,47 +2311,47 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>75597.22</v>
+        <v>75619.97</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>0.005500000000000001</v>
+        <v>0.0086</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>-0.0101</v>
+        <v>-0.0098</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>-0.0529</v>
+        <v>-0.0452</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>-0.0762</v>
+        <v>-0.07780000000000001</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>-0.0466</v>
+        <v>-0.0215</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>-0.1729</v>
+        <v>-0.1727</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>0.0066</v>
+        <v>0.0069</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>-0.1847</v>
+        <v>-0.1833</v>
       </c>
       <c r="L37" s="3" t="n">
-        <v>-0.1479</v>
+        <v>-0.1483</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>-0.0269</v>
+        <v>-0.0287</v>
       </c>
       <c r="N37" s="3" t="n">
         <v>0.0395</v>
       </c>
       <c r="O37" s="3" t="n">
-        <v>0.0888</v>
+        <v>0.08929999999999999</v>
       </c>
     </row>
     <row r="38">
@@ -2362,44 +2362,44 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>5381.66</v>
+        <v>5418.38</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>-0.0283</v>
+        <v>-0.0243</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>-0.0001</v>
+        <v>0.0067</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>-0.0379</v>
+        <v>-0.0308</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>-0.0873</v>
+        <v>-0.0969</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>-0.0071</v>
+        <v>0.0118</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>0.0473</v>
+        <v>0.0545</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>0.0344</v>
+        <v>0.0415</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>0.008399999999999999</v>
+        <v>0.0186</v>
       </c>
       <c r="L38" s="3" t="n">
-        <v>-0.08960000000000001</v>
+        <v>-0.0885</v>
       </c>
       <c r="M38" s="3" t="n">
-        <v>0.1348</v>
+        <v>0.1334</v>
       </c>
       <c r="N38" s="3" t="n">
-        <v>0.1386</v>
+        <v>0.1401</v>
       </c>
       <c r="O38" s="3" t="n">
         <v>0.1201</v>
@@ -2413,47 +2413,47 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>5878.62</v>
+        <v>5907.25</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>-0.0137</v>
+        <v>-0.0092</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>-0.04269999999999999</v>
+        <v>-0.038</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>-0.052</v>
+        <v>-0.04219999999999999</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>-0.0163</v>
+        <v>-0.0144</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>0.0204</v>
+        <v>0.06059999999999999</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>-0.06370000000000001</v>
+        <v>-0.0591</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>0.08960000000000001</v>
+        <v>0.0949</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>-0.031</v>
+        <v>-0.0292</v>
       </c>
       <c r="L39" s="3" t="n">
-        <v>-0.021</v>
+        <v>-0.0188</v>
       </c>
       <c r="M39" s="3" t="n">
-        <v>0.09080000000000001</v>
+        <v>0.09329999999999999</v>
       </c>
       <c r="N39" s="3" t="n">
-        <v>0.0706</v>
+        <v>0.0716</v>
       </c>
       <c r="O39" s="3" t="n">
-        <v>0.129</v>
+        <v>0.1291</v>
       </c>
     </row>
     <row r="40">
@@ -2464,47 +2464,47 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>16737.03</v>
+        <v>16713.77</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>-0.0142</v>
+        <v>-0.0156</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>-0.0199</v>
+        <v>-0.0213</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>-0.0289</v>
+        <v>-0.03240000000000001</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>-0.0362</v>
+        <v>-0.0375</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>-0.0252</v>
+        <v>-0.0068</v>
       </c>
       <c r="I40" s="3" t="n">
-        <v>-0.1055</v>
+        <v>-0.1068</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>0.0118</v>
+        <v>0.0104</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>-0.0239</v>
+        <v>-0.0314</v>
       </c>
       <c r="L40" s="3" t="n">
-        <v>-0.0658</v>
+        <v>-0.06709999999999999</v>
       </c>
       <c r="M40" s="3" t="n">
-        <v>0.1162</v>
+        <v>0.1158</v>
       </c>
       <c r="N40" s="3" t="n">
-        <v>0.0919</v>
+        <v>0.0915</v>
       </c>
       <c r="O40" s="3" t="n">
-        <v>0.1424</v>
+        <v>0.1416</v>
       </c>
     </row>
     <row r="41">
@@ -2515,47 +2515,47 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>65837.55</v>
+        <v>66188.71000000001</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>-0.03</v>
+        <v>-0.022</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>-0.0177</v>
+        <v>-0.0125</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>-0.0354</v>
+        <v>-0.0285</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>-0.0711</v>
+        <v>-0.0712</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>0.035</v>
+        <v>0.0552</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>0.063</v>
+        <v>0.06860000000000001</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>0.07339999999999999</v>
+        <v>0.0791</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>0.0614</v>
+        <v>0.06320000000000001</v>
       </c>
       <c r="L41" s="3" t="n">
-        <v>-0.0528</v>
+        <v>-0.0512</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>0.1229</v>
+        <v>0.1224</v>
       </c>
       <c r="N41" s="3" t="n">
-        <v>0.1337</v>
+        <v>0.1348</v>
       </c>
       <c r="O41" s="3" t="n">
-        <v>0.1671</v>
+        <v>0.1668</v>
       </c>
     </row>
     <row r="42">
@@ -2566,47 +2566,47 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>42008.16</v>
+        <v>42106.33</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>0.006</v>
+        <v>0.0092</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>-0.0674</v>
+        <v>-0.0653</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>-0.0558</v>
+        <v>-0.035</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>0.0129</v>
+        <v>0.0275</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>-0.0073</v>
+        <v>0.0291</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>-0.2217</v>
+        <v>-0.2199</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.012</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>-0.1795</v>
+        <v>-0.1829</v>
       </c>
       <c r="L42" s="3" t="n">
-        <v>-0.163</v>
+        <v>-0.1626</v>
       </c>
       <c r="M42" s="3" t="n">
-        <v>-0.024</v>
+        <v>-0.0211</v>
       </c>
       <c r="N42" s="3" t="n">
-        <v>-0.0203</v>
+        <v>-0.0198</v>
       </c>
       <c r="O42" s="3" t="n">
-        <v>0.1309</v>
+        <v>0.1305</v>
       </c>
     </row>
     <row r="43">
@@ -2617,47 +2617,47 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>7551.81</v>
+        <v>7637.76</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>-0.0111</v>
+        <v>0.0061</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>-0.0175</v>
+        <v>-0.0063</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>-0.025</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>0.0178</v>
+        <v>0.0183</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>0.1399</v>
+        <v>0.1561</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>0.1032</v>
+        <v>0.1157</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>0.1567</v>
+        <v>0.1699</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>0.143</v>
+        <v>0.1572</v>
       </c>
       <c r="L43" s="3" t="n">
-        <v>0.158</v>
+        <v>0.1644</v>
       </c>
       <c r="M43" s="3" t="n">
-        <v>0.1925</v>
+        <v>0.1971</v>
       </c>
       <c r="N43" s="3" t="n">
-        <v>0.1125</v>
+        <v>0.115</v>
       </c>
       <c r="O43" s="3" t="n">
-        <v>0.1345</v>
+        <v>0.1358</v>
       </c>
     </row>
     <row r="44">
@@ -2668,47 +2668,47 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>28945.06</v>
+        <v>29446.98</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>-0.0162</v>
+        <v>0.0118</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>-0.0174</v>
+        <v>-0.0003</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>-0.035</v>
+        <v>-0.0015</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>-0.0245</v>
+        <v>-0.0315</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>0.1851</v>
+        <v>0.2091</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>0.1463</v>
+        <v>0.1662</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>0.2192</v>
+        <v>0.2404</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>0.1924</v>
+        <v>0.2156</v>
       </c>
       <c r="L44" s="3" t="n">
-        <v>0.2209</v>
+        <v>0.2312</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>0.2391</v>
+        <v>0.2461</v>
       </c>
       <c r="N44" s="3" t="n">
-        <v>0.1356</v>
+        <v>0.1394</v>
       </c>
       <c r="O44" s="3" t="n">
-        <v>0.1964</v>
+        <v>0.1991</v>
       </c>
     </row>
     <row r="45">
@@ -2719,47 +2719,47 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
-        <v>64136.25</v>
+        <v>65018.95</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>-0.0174</v>
+        <v>0.0157</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>-0.0328</v>
+        <v>-0.0195</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>-0.0493</v>
+        <v>-0.004699999999999999</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>-0.0974</v>
+        <v>-0.08749999999999999</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>0.2017</v>
+        <v>0.2182</v>
       </c>
       <c r="I45" s="3" t="n">
-        <v>0.2741</v>
+        <v>0.2916</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>0.256</v>
+        <v>0.2733</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>0.4319</v>
+        <v>0.4352</v>
       </c>
       <c r="L45" s="3" t="n">
-        <v>0.3313</v>
+        <v>0.3371</v>
       </c>
       <c r="M45" s="3" t="n">
-        <v>0.2408</v>
+        <v>0.2508</v>
       </c>
       <c r="N45" s="3" t="n">
-        <v>0.1603</v>
+        <v>0.1634</v>
       </c>
       <c r="O45" s="3" t="n">
-        <v>0.1453</v>
+        <v>0.1471</v>
       </c>
     </row>
     <row r="46">
@@ -2770,47 +2770,47 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>25677.47</v>
+        <v>25532.82</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>0.0125</v>
+        <v>-0.0014</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>-0.0221</v>
+        <v>-0.0276</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>-0.0173</v>
+        <v>-0.0214</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>0.026</v>
+        <v>0.0219</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>0.1243</v>
+        <v>0.1409</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>0.04849999999999999</v>
+        <v>0.0426</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>0.1322</v>
+        <v>0.1258</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>0.0992</v>
+        <v>0.0785</v>
       </c>
       <c r="L46" s="3" t="n">
-        <v>0.1711</v>
+        <v>0.1683</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>0.1777</v>
+        <v>0.177</v>
       </c>
       <c r="N46" s="3" t="n">
-        <v>0.1064</v>
+        <v>0.1051</v>
       </c>
       <c r="O46" s="3" t="n">
-        <v>0.0949</v>
+        <v>0.0941</v>
       </c>
     </row>
     <row r="47">
@@ -2821,47 +2821,47 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>8160.39</v>
+        <v>8116.7</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>0.0054</v>
+        <v>-0.0077</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>-0.0209</v>
+        <v>-0.0261</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>-0.04099999999999999</v>
+        <v>-0.0453</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>-0.0363</v>
+        <v>-0.0362</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>0.0451</v>
+        <v>0.0588</v>
       </c>
       <c r="I47" s="3" t="n">
-        <v>0.0013</v>
+        <v>-0.004</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>0.04389999999999999</v>
+        <v>0.0383</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>0.048</v>
+        <v>0.0334</v>
       </c>
       <c r="L47" s="3" t="n">
-        <v>0.044</v>
+        <v>0.0442</v>
       </c>
       <c r="M47" s="3" t="n">
-        <v>0.039</v>
+        <v>0.0369</v>
       </c>
       <c r="N47" s="3" t="n">
-        <v>0.0443</v>
+        <v>0.0432</v>
       </c>
       <c r="O47" s="3" t="n">
-        <v>0.0639</v>
+        <v>0.0635</v>
       </c>
     </row>
     <row r="48">
@@ -2872,47 +2872,47 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>10708.15</v>
+        <v>10726.4</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>0.009399999999999999</v>
+        <v>0.0071</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>-0.0107</v>
+        <v>-0.009000000000000001</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>-0.0019</v>
+        <v>-0.0016</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>0.0297</v>
+        <v>0.035</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>0.0641</v>
+        <v>0.0815</v>
       </c>
       <c r="I48" s="3" t="n">
-        <v>0.07820000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>0.0522</v>
+        <v>0.05400000000000001</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>0.1629</v>
+        <v>0.1624</v>
       </c>
       <c r="L48" s="3" t="n">
-        <v>0.1353</v>
+        <v>0.1401</v>
       </c>
       <c r="M48" s="3" t="n">
-        <v>0.1186</v>
+        <v>0.1188</v>
       </c>
       <c r="N48" s="3" t="n">
-        <v>0.08990000000000001</v>
+        <v>0.0902</v>
       </c>
       <c r="O48" s="3" t="n">
-        <v>0.0463</v>
+        <v>0.0462</v>
       </c>
     </row>
     <row r="49">
@@ -2923,47 +2923,47 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>24604.29</v>
+        <v>24750.78</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>-0.014</v>
+        <v>-0.0022</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>-0.0377</v>
+        <v>-0.0319</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>-0.034</v>
+        <v>-0.0292</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>0.0284</v>
+        <v>0.0345</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>-0.0351</v>
+        <v>-0.0208</v>
       </c>
       <c r="I49" s="3" t="n">
-        <v>-0.04</v>
+        <v>-0.0343</v>
       </c>
       <c r="J49" s="3" t="n">
-        <v>-0.0074</v>
+        <v>-0.0015</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>-0.08560000000000001</v>
+        <v>-0.06759999999999999</v>
       </c>
       <c r="L49" s="3" t="n">
-        <v>0.1805</v>
+        <v>0.1837</v>
       </c>
       <c r="M49" s="3" t="n">
-        <v>0.1113</v>
+        <v>0.1121</v>
       </c>
       <c r="N49" s="3" t="n">
-        <v>-0.0026</v>
+        <v>-0.0014</v>
       </c>
       <c r="O49" s="3" t="n">
-        <v>0.0044</v>
+        <v>0.0051</v>
       </c>
     </row>
     <row r="50">
@@ -3025,47 +3025,47 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>95.93000000000001</v>
+        <v>95.87</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>0.0086</v>
+        <v>0.0019</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>0.0058</v>
+        <v>0.0052</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>0.0025</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>0.0113</v>
+        <v>0.0162</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>0.0288</v>
+        <v>0.03</v>
       </c>
       <c r="I51" s="3" t="n">
-        <v>0.06860000000000001</v>
+        <v>0.068</v>
       </c>
       <c r="J51" s="3" t="n">
-        <v>0.0167</v>
+        <v>0.0161</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>0.0915</v>
+        <v>0.0906</v>
       </c>
       <c r="L51" s="3" t="n">
-        <v>0.0694</v>
+        <v>0.0698</v>
       </c>
       <c r="M51" s="3" t="n">
-        <v>0.0491</v>
+        <v>0.0482</v>
       </c>
       <c r="N51" s="3" t="n">
-        <v>0.0545</v>
+        <v>0.0544</v>
       </c>
       <c r="O51" s="3" t="n">
-        <v>0.0365</v>
+        <v>0.0366</v>
       </c>
     </row>
     <row r="52">
@@ -3076,47 +3076,47 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>4355.9</v>
+        <v>4421.4</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>-0.002</v>
+        <v>0.0028</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>-0.017</v>
+        <v>-0.0022</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>-0.0023</v>
+        <v>-0.0151</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>0.0312</v>
+        <v>0.0467</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>-0.0532</v>
+        <v>-0.0326</v>
       </c>
       <c r="I52" s="3" t="n">
-        <v>0.006999999999999999</v>
+        <v>0.0221</v>
       </c>
       <c r="J52" s="3" t="n">
-        <v>-0.06280000000000001</v>
+        <v>-0.0487</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>0.1831</v>
+        <v>0.2134</v>
       </c>
       <c r="L52" s="3" t="n">
-        <v>0.3036</v>
+        <v>0.3117</v>
       </c>
       <c r="M52" s="3" t="n">
-        <v>0.3116</v>
+        <v>0.3181</v>
       </c>
       <c r="N52" s="3" t="n">
-        <v>0.2002</v>
+        <v>0.2037</v>
       </c>
       <c r="O52" s="3" t="n">
-        <v>0.1275</v>
+        <v>0.1291</v>
       </c>
     </row>
     <row r="53">
@@ -3127,47 +3127,47 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>64.45999999999999</v>
+        <v>67.66</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>0.0027</v>
+        <v>0.0481</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>-0.0267</v>
+        <v>0.0217</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>0.008</v>
+        <v>0.0293</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>-0.0272</v>
+        <v>0.0212</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>-0.09089999999999999</v>
+        <v>-0.0245</v>
       </c>
       <c r="I53" s="3" t="n">
-        <v>-0.081</v>
+        <v>-0.0353</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>-0.137</v>
+        <v>-0.0941</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>0.5449000000000001</v>
+        <v>0.6223</v>
       </c>
       <c r="L53" s="3" t="n">
-        <v>0.4513</v>
+        <v>0.4937</v>
       </c>
       <c r="M53" s="3" t="n">
-        <v>0.4055</v>
+        <v>0.4292</v>
       </c>
       <c r="N53" s="3" t="n">
-        <v>0.2366</v>
+        <v>0.2485</v>
       </c>
       <c r="O53" s="3" t="n">
-        <v>0.1288</v>
+        <v>0.1344</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Weekly indices update 2026-09-18
</commit_message>
<xml_diff>
--- a/tracker_auto.xlsx
+++ b/tracker_auto.xlsx
@@ -830,47 +830,47 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>18233.33</v>
+        <v>18351.23</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>-0.0116</v>
+        <v>-0.0016</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-0.0357</v>
+        <v>-0.0295</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-0.0365</v>
+        <v>-0.0271</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>-0.0257</v>
+        <v>-0.0164</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.05599999999999999</v>
+        <v>0.0574</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>-0.0601</v>
+        <v>-0.05400000000000001</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.0919</v>
+        <v>0.0989</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>-0.0332</v>
+        <v>-0.0304</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>-0.0208</v>
+        <v>-0.0163</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>0.09179999999999999</v>
+        <v>0.0941</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>0.08939999999999999</v>
+        <v>0.09080000000000001</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>0.1246</v>
+        <v>0.1257</v>
       </c>
     </row>
     <row r="9">
@@ -1289,47 +1289,47 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>25570.99</v>
+        <v>25660.26</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>-0.015</v>
+        <v>-0.0034</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>-0.0201</v>
+        <v>-0.0166</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>-0.0268</v>
+        <v>-0.0191</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>-0.06</v>
+        <v>-0.0539</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>0.0106</v>
+        <v>0.0042</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>-0.0023</v>
+        <v>0.0012</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>0.0401</v>
+        <v>0.0438</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>0.1174</v>
+        <v>0.1197</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>0.0431</v>
+        <v>0.0461</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>0.2281</v>
+        <v>0.2293</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>0.2458</v>
+        <v>0.2465</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>0.1679</v>
+        <v>0.1682</v>
       </c>
     </row>
     <row r="18">
@@ -1340,47 +1340,47 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>37906.17</v>
+        <v>38277.74</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>-0.0251</v>
+        <v>-0.008699999999999999</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>-0.0385</v>
+        <v>-0.0291</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>-0.031</v>
+        <v>-0.0107</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>-0.0334</v>
+        <v>-0.0236</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>0.06950000000000001</v>
+        <v>0.0762</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>-0.0269</v>
+        <v>-0.0174</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>0.1183</v>
+        <v>0.1293</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>-0.0205</v>
+        <v>-0.015</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>-0.0864</v>
+        <v>-0.07969999999999999</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>0.1024</v>
+        <v>0.1059</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>0.0958</v>
+        <v>0.09789999999999999</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>0.1627</v>
+        <v>0.164</v>
       </c>
     </row>
     <row r="19">
@@ -1391,47 +1391,47 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>28353.18</v>
+        <v>28332.96</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>-0.0132</v>
+        <v>-0.0073</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>-0.0483</v>
+        <v>-0.049</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>-0.0472</v>
+        <v>-0.0453</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>-0.0271</v>
+        <v>-0.0197</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>0.05889999999999999</v>
+        <v>0.0475</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>-0.0741</v>
+        <v>-0.0747</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>0.08470000000000001</v>
+        <v>0.0839</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>-0.06280000000000001</v>
+        <v>-0.065</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>-0.06900000000000001</v>
+        <v>-0.0633</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>0.07139999999999999</v>
+        <v>0.0711</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>0.06849999999999999</v>
+        <v>0.0683</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>0.1181</v>
+        <v>0.1183</v>
       </c>
     </row>
     <row r="20">
@@ -1595,44 +1595,44 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>10274.17</v>
+        <v>10363.48</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>-0.0534</v>
+        <v>-0.0382</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>-0.0459</v>
+        <v>-0.03759999999999999</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>-0.0697</v>
+        <v>-0.0474</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>-0.025</v>
+        <v>-0.0231</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>0.1916</v>
+        <v>0.2108</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>0.2023</v>
+        <v>0.2128</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>0.2871</v>
+        <v>0.2983</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>0.1205</v>
+        <v>0.1363</v>
       </c>
       <c r="L23" s="3" t="n">
-        <v>0.1847</v>
+        <v>0.1952</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>0.4221</v>
+        <v>0.4257</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>0.5123</v>
+        <v>0.5146000000000001</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -1648,47 +1648,47 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>11343.39</v>
+        <v>11418.56</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>-0.0165</v>
+        <v>-0.0039</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>-0.0403</v>
+        <v>-0.0339</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>-0.0413</v>
+        <v>-0.0348</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>-0.0579</v>
+        <v>-0.0457</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>-0.0108</v>
+        <v>-0.0245</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>-0.0245</v>
+        <v>-0.018</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>0.0566</v>
+        <v>0.0636</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>0.1379</v>
+        <v>0.1473</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>0.1205</v>
+        <v>0.1241</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>0.174</v>
+        <v>0.1764</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>0.2868</v>
+        <v>0.2883</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>0.1073</v>
+        <v>0.1084</v>
       </c>
     </row>
     <row r="25">
@@ -1699,47 +1699,47 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>78686.11</v>
+        <v>79111.42</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>-0.0074</v>
+        <v>-0.0044</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>-0.0339</v>
+        <v>-0.0287</v>
       </c>
       <c r="F25" s="3" t="n">
+        <v>-0.0154</v>
+      </c>
+      <c r="G25" s="3" t="n">
         <v>-0.0211</v>
       </c>
-      <c r="G25" s="3" t="n">
-        <v>-0.0282</v>
-      </c>
       <c r="H25" s="3" t="n">
-        <v>0.0556</v>
+        <v>0.06179999999999999</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>-0.053</v>
+        <v>-0.0479</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>0.1223</v>
+        <v>0.1284</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>0.0168</v>
+        <v>0.018</v>
       </c>
       <c r="L25" s="3" t="n">
-        <v>0.04389999999999999</v>
+        <v>0.0412</v>
       </c>
       <c r="M25" s="3" t="n">
-        <v>0.0767</v>
+        <v>0.0785</v>
       </c>
       <c r="N25" s="3" t="n">
-        <v>0.0906</v>
+        <v>0.0917</v>
       </c>
       <c r="O25" s="3" t="n">
-        <v>0.1157</v>
+        <v>0.1166</v>
       </c>
     </row>
     <row r="26">
@@ -1750,47 +1750,47 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>32161.16</v>
+        <v>32304.13</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>-0.005</v>
+        <v>-0.0053</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>-0.0299</v>
+        <v>-0.0256</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>-0.0029</v>
+        <v>0.003</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>-0.0249</v>
+        <v>-0.0188</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>0.0761</v>
+        <v>0.08650000000000001</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>-0.0483</v>
+        <v>-0.0441</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>0.132</v>
+        <v>0.1371</v>
       </c>
       <c r="K26" s="3" t="n">
         <v>0.0113</v>
       </c>
       <c r="L26" s="3" t="n">
-        <v>0.0233</v>
+        <v>0.0206</v>
       </c>
       <c r="M26" s="3" t="n">
-        <v>0.0532</v>
+        <v>0.0547</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>0.0731</v>
+        <v>0.07400000000000001</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>0.0989</v>
+        <v>0.09970000000000001</v>
       </c>
     </row>
     <row r="27">
@@ -1801,47 +1801,47 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>32397.43</v>
+        <v>32642.69</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>-0.007900000000000001</v>
+        <v>-0.0014</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>-0.0371</v>
+        <v>-0.0298</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>-0.03</v>
+        <v>-0.0191</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>-0.0417</v>
+        <v>-0.0319</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>0.023</v>
+        <v>0.0378</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>-0.07519999999999999</v>
+        <v>-0.0682</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>0.0849</v>
+        <v>0.0931</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>-0.0382</v>
+        <v>-0.0358</v>
       </c>
       <c r="L27" s="3" t="n">
-        <v>0.0371</v>
+        <v>0.0338</v>
       </c>
       <c r="M27" s="3" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.0876</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>0.0751</v>
+        <v>0.0767</v>
       </c>
       <c r="O27" s="3" t="n">
-        <v>0.1284</v>
+        <v>0.1294</v>
       </c>
     </row>
     <row r="28">
@@ -1852,47 +1852,47 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>17308.14</v>
+        <v>17385.42</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>-0.0201</v>
+        <v>-0.009399999999999999</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>-0.0126</v>
+        <v>-0.008199999999999999</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>-0.0256</v>
+        <v>-0.0124</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>-0.0555</v>
+        <v>-0.0505</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>-0.0197</v>
+        <v>-0.0217</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>-0.0162</v>
+        <v>-0.0118</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>0.006500000000000001</v>
+        <v>0.011</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>-0.0108</v>
+        <v>-0.0059</v>
       </c>
       <c r="L28" s="3" t="n">
-        <v>-0.0434</v>
+        <v>-0.0381</v>
       </c>
       <c r="M28" s="3" t="n">
-        <v>0.1977</v>
+        <v>0.1993</v>
       </c>
       <c r="N28" s="3" t="n">
-        <v>0.229</v>
+        <v>0.23</v>
       </c>
       <c r="O28" s="3" t="n">
-        <v>0.1405</v>
+        <v>0.1409</v>
       </c>
     </row>
     <row r="29">
@@ -1903,47 +1903,47 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>929.86</v>
+        <v>940.97</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>-0.0431</v>
+        <v>-0.005</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>-0.0771</v>
+        <v>-0.06610000000000001</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>-0.06849999999999999</v>
+        <v>-0.05690000000000001</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>0.0215</v>
+        <v>0.0443</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>0.192</v>
+        <v>0.2177</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>-0.0454</v>
+        <v>-0.034</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>0.2869</v>
+        <v>0.3023</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>-0.08810000000000001</v>
+        <v>-0.0765</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>-0.1119</v>
+        <v>-0.1056</v>
       </c>
       <c r="M29" s="3" t="n">
-        <v>0.1337</v>
+        <v>0.138</v>
       </c>
       <c r="N29" s="3" t="n">
-        <v>0.1548</v>
+        <v>0.1574</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>0.1535</v>
+        <v>0.1566</v>
       </c>
     </row>
     <row r="30">
@@ -1954,47 +1954,47 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>36354.4</v>
+        <v>36314.06</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>-0.0139</v>
+        <v>-0.0064</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>-0.0583</v>
+        <v>-0.0594</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>-0.07190000000000001</v>
+        <v>-0.07049999999999999</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>0.0222</v>
+        <v>0.0268</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>0.1182</v>
+        <v>0.1076</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>-0.0266</v>
+        <v>-0.0276</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>0.1525</v>
+        <v>0.1513</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>0.005600000000000001</v>
+        <v>0.0032</v>
       </c>
       <c r="L30" s="3" t="n">
-        <v>0.0343</v>
+        <v>0.0356</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>0.19</v>
+        <v>0.1894</v>
       </c>
       <c r="N30" s="3" t="n">
-        <v>0.224</v>
+        <v>0.2236</v>
       </c>
       <c r="O30" s="3" t="n">
-        <v>0.1152</v>
+        <v>0.1159</v>
       </c>
     </row>
     <row r="31">
@@ -2005,47 +2005,47 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>20788.01</v>
+        <v>20923.37</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>-0.0179</v>
+        <v>-0.0024</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>-0.0455</v>
+        <v>-0.0393</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>-0.0438</v>
+        <v>-0.0329</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>-0.0095</v>
+        <v>-0.0024</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>0.1035</v>
+        <v>0.1002</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>0.0349</v>
+        <v>0.0416</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>0.1344</v>
+        <v>0.1418</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>0.0499</v>
+        <v>0.05400000000000001</v>
       </c>
       <c r="L31" s="3" t="n">
-        <v>0.0285</v>
+        <v>0.036</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>0.1746</v>
+        <v>0.1769</v>
       </c>
       <c r="N31" s="3" t="n">
-        <v>0.1593</v>
+        <v>0.1608</v>
       </c>
       <c r="O31" s="3" t="n">
-        <v>0.1381</v>
+        <v>0.1392</v>
       </c>
     </row>
     <row r="32">
@@ -2056,47 +2056,47 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>11847.6</v>
+        <v>11982.33</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>-0.018</v>
+        <v>-0.0005999999999999999</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>-0.0223</v>
+        <v>-0.0112</v>
       </c>
       <c r="F32" s="3" t="n">
+        <v>-0.0246</v>
+      </c>
+      <c r="G32" s="3" t="n">
         <v>-0.0429</v>
       </c>
-      <c r="G32" s="3" t="n">
-        <v>-0.0525</v>
-      </c>
       <c r="H32" s="3" t="n">
-        <v>0.0352</v>
+        <v>0.03700000000000001</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>-0.06059999999999999</v>
+        <v>-0.05</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>0.0539</v>
+        <v>0.0659</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>-0.0196</v>
+        <v>-0.0091</v>
       </c>
       <c r="L32" s="3" t="n">
-        <v>-0.0137</v>
+        <v>-0.0059</v>
       </c>
       <c r="M32" s="3" t="n">
-        <v>0.1364</v>
+        <v>0.1406</v>
       </c>
       <c r="N32" s="3" t="n">
-        <v>0.1382</v>
+        <v>0.1407</v>
       </c>
       <c r="O32" s="3" t="n">
-        <v>0.1351</v>
+        <v>0.1371</v>
       </c>
     </row>
     <row r="33">
@@ -2107,47 +2107,47 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>19729.57</v>
+        <v>19830.73</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0074</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>-0.0243</v>
+        <v>-0.0193</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>0.004</v>
+        <v>0.0123</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>0.065</v>
+        <v>0.0626</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>0.1744</v>
+        <v>0.1585</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>0.1346</v>
+        <v>0.1404</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>0.1674</v>
+        <v>0.1734</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>0.1331</v>
+        <v>0.124</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>0.0653</v>
+        <v>0.0751</v>
       </c>
       <c r="M33" s="3" t="n">
-        <v>0.1993</v>
+        <v>0.2012</v>
       </c>
       <c r="N33" s="3" t="n">
-        <v>0.1339</v>
+        <v>0.135</v>
       </c>
       <c r="O33" s="3" t="n">
-        <v>0.1067</v>
+        <v>0.1073</v>
       </c>
     </row>
     <row r="34">
@@ -2158,47 +2158,47 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>19622.27</v>
+        <v>19918.59</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>-0.0335</v>
+        <v>0.0042</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>-0.0252</v>
+        <v>-0.0105</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>-0.0123</v>
+        <v>0.0028</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>-0.009399999999999999</v>
+        <v>0.0048</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>0.1534</v>
+        <v>0.154</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>0.1625</v>
+        <v>0.18</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>0.1622</v>
+        <v>0.1797</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>0.3094</v>
+        <v>0.3248</v>
       </c>
       <c r="L34" s="3" t="n">
-        <v>0.1818</v>
+        <v>0.1956</v>
       </c>
       <c r="M34" s="3" t="n">
-        <v>0.2372</v>
+        <v>0.2432</v>
       </c>
       <c r="N34" s="3" t="n">
-        <v>0.1922</v>
+        <v>0.1957</v>
       </c>
       <c r="O34" s="3" t="n">
-        <v>0.2011</v>
+        <v>0.2025</v>
       </c>
     </row>
     <row r="35">
@@ -2260,47 +2260,47 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>14161.71</v>
+        <v>14258.59</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>-0.0215</v>
+        <v>-0.0014</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>-0.0179</v>
+        <v>-0.0112</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>-0.0303</v>
+        <v>-0.0177</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>-0.0545</v>
+        <v>-0.04480000000000001</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>0.032</v>
+        <v>0.0259</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>0.0077</v>
+        <v>0.0146</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>0.0473</v>
+        <v>0.0545</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>0.0663</v>
+        <v>0.073</v>
       </c>
       <c r="L36" s="3" t="n">
-        <v>0.0153</v>
+        <v>0.023</v>
       </c>
       <c r="M36" s="3" t="n">
+        <v>0.1432</v>
+      </c>
+      <c r="N36" s="3" t="n">
+        <v>0.1249</v>
+      </c>
+      <c r="O36" s="3" t="n">
         <v>0.1407</v>
-      </c>
-      <c r="N36" s="3" t="n">
-        <v>0.1235</v>
-      </c>
-      <c r="O36" s="3" t="n">
-        <v>0.1398</v>
       </c>
     </row>
     <row r="37">
@@ -2311,47 +2311,47 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>75619.97</v>
+        <v>75444.25</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>0.0086</v>
+        <v>0.0092</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>-0.0098</v>
+        <v>-0.0121</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>-0.0452</v>
+        <v>-0.04219999999999999</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>-0.07780000000000001</v>
+        <v>-0.0781</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>-0.0215</v>
+        <v>-0.0268</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>-0.1727</v>
+        <v>-0.1746</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>0.0069</v>
+        <v>0.0046</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>-0.1833</v>
+        <v>-0.1881</v>
       </c>
       <c r="L37" s="3" t="n">
-        <v>-0.1483</v>
+        <v>-0.1489</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>-0.0287</v>
+        <v>-0.0295</v>
       </c>
       <c r="N37" s="3" t="n">
-        <v>0.0395</v>
+        <v>0.039</v>
       </c>
       <c r="O37" s="3" t="n">
-        <v>0.08929999999999999</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="38">
@@ -2413,47 +2413,47 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>5907.25</v>
+        <v>5950.87</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>-0.0092</v>
+        <v>0.0027</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>-0.038</v>
+        <v>-0.0309</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>-0.04219999999999999</v>
+        <v>-0.0322</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>-0.0144</v>
+        <v>-0.0012</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>0.06059999999999999</v>
+        <v>0.06269999999999999</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>-0.0591</v>
+        <v>-0.0522</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>0.0949</v>
+        <v>0.103</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>-0.0292</v>
+        <v>-0.0269</v>
       </c>
       <c r="L39" s="3" t="n">
-        <v>-0.0188</v>
+        <v>-0.0132</v>
       </c>
       <c r="M39" s="3" t="n">
-        <v>0.09329999999999999</v>
+        <v>0.0958</v>
       </c>
       <c r="N39" s="3" t="n">
-        <v>0.0716</v>
+        <v>0.0731</v>
       </c>
       <c r="O39" s="3" t="n">
-        <v>0.1291</v>
+        <v>0.1303</v>
       </c>
     </row>
     <row r="40">
@@ -2464,47 +2464,47 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>16713.77</v>
+        <v>16854.44</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>-0.0156</v>
+        <v>0.0011</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>-0.0213</v>
+        <v>-0.013</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>-0.03240000000000001</v>
+        <v>-0.0195</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>-0.0375</v>
+        <v>-0.0178</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>-0.0068</v>
+        <v>-0.0039</v>
       </c>
       <c r="I40" s="3" t="n">
-        <v>-0.1068</v>
+        <v>-0.0993</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>0.0104</v>
+        <v>0.0189</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>-0.0314</v>
+        <v>-0.0229</v>
       </c>
       <c r="L40" s="3" t="n">
-        <v>-0.06709999999999999</v>
+        <v>-0.0583</v>
       </c>
       <c r="M40" s="3" t="n">
-        <v>0.1158</v>
+        <v>0.1188</v>
       </c>
       <c r="N40" s="3" t="n">
-        <v>0.0915</v>
+        <v>0.09329999999999999</v>
       </c>
       <c r="O40" s="3" t="n">
-        <v>0.1416</v>
+        <v>0.1424</v>
       </c>
     </row>
     <row r="41">
@@ -2515,47 +2515,47 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>66188.71000000001</v>
+        <v>66882.39999999999</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>-0.022</v>
+        <v>-0.0043</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>-0.0125</v>
+        <v>-0.0022</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>-0.0285</v>
+        <v>-0.0067</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>-0.0712</v>
+        <v>-0.0636</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>0.0552</v>
+        <v>0.0583</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>0.06860000000000001</v>
+        <v>0.07980000000000001</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>0.0791</v>
+        <v>0.09039999999999999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>0.06320000000000001</v>
+        <v>0.07820000000000001</v>
       </c>
       <c r="L41" s="3" t="n">
-        <v>-0.0512</v>
+        <v>-0.0429</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>0.1224</v>
+        <v>0.1262</v>
       </c>
       <c r="N41" s="3" t="n">
-        <v>0.1348</v>
+        <v>0.1371</v>
       </c>
       <c r="O41" s="3" t="n">
-        <v>0.1668</v>
+        <v>0.1684</v>
       </c>
     </row>
     <row r="42">
@@ -2566,47 +2566,47 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>42106.33</v>
+        <v>41671.52</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>0.0092</v>
+        <v>-0.0023</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>-0.0653</v>
+        <v>-0.07490000000000001</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>-0.035</v>
+        <v>-0.0519</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>0.0275</v>
+        <v>0.0555</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>0.0291</v>
+        <v>-0.0031</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>-0.2199</v>
+        <v>-0.2279</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>0.012</v>
+        <v>0.0016</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>-0.1829</v>
+        <v>-0.198</v>
       </c>
       <c r="L42" s="3" t="n">
-        <v>-0.1626</v>
+        <v>-0.1539</v>
       </c>
       <c r="M42" s="3" t="n">
-        <v>-0.0211</v>
+        <v>-0.0245</v>
       </c>
       <c r="N42" s="3" t="n">
-        <v>-0.0198</v>
+        <v>-0.0218</v>
       </c>
       <c r="O42" s="3" t="n">
-        <v>0.1305</v>
+        <v>0.1298</v>
       </c>
     </row>
     <row r="43">
@@ -2974,47 +2974,47 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>4460.16</v>
+        <v>4507.39</v>
       </c>
       <c r="D50" s="3" t="n">
-        <v>-0.0194</v>
+        <v>-0.0005999999999999999</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>-0.0357</v>
+        <v>-0.0254</v>
       </c>
       <c r="F50" s="3" t="n">
-        <v>-0.0562</v>
+        <v>-0.0177</v>
       </c>
       <c r="G50" s="3" t="n">
-        <v>-0.0974</v>
+        <v>-0.08789999999999999</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>-0.0269</v>
+        <v>-0.0131</v>
       </c>
       <c r="I50" s="3" t="n">
-        <v>-0.0367</v>
+        <v>-0.0265</v>
       </c>
       <c r="J50" s="3" t="n">
-        <v>0.0023</v>
+        <v>0.0129</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>-0.02</v>
+        <v>0.0021</v>
       </c>
       <c r="L50" s="3" t="n">
-        <v>0.1872</v>
+        <v>0.1924</v>
       </c>
       <c r="M50" s="3" t="n">
-        <v>0.0617</v>
+        <v>0.06610000000000001</v>
       </c>
       <c r="N50" s="3" t="n">
-        <v>-0.0169</v>
+        <v>-0.0148</v>
       </c>
       <c r="O50" s="3" t="n">
-        <v>0.0318</v>
+        <v>0.033</v>
       </c>
     </row>
     <row r="51">

</xml_diff>

<commit_message>
Weekly indices update 2026-09-20
</commit_message>
<xml_diff>
--- a/tracker_auto.xlsx
+++ b/tracker_auto.xlsx
@@ -524,47 +524,47 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>23270.6</v>
+        <v>23346.4</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>-0.008800000000000001</v>
+        <v>-0.0022</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-0.0336</v>
+        <v>-0.0305</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>-0.0366</v>
+        <v>-0.0304</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>-0.0371</v>
+        <v>-0.0278</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>0.0117</v>
+        <v>0.01</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>-0.1094</v>
+        <v>-0.1065</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.0421</v>
+        <v>0.0455</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>-0.08130000000000001</v>
+        <v>-0.08169999999999999</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>-0.0432</v>
+        <v>-0.0409</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>0.0495</v>
+        <v>0.0506</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>0.0576</v>
+        <v>0.0583</v>
       </c>
       <c r="O2" s="3" t="n">
-        <v>0.1021</v>
+        <v>0.1029</v>
       </c>
     </row>
     <row r="3">
@@ -626,47 +626,47 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>71144</v>
+        <v>72025.39999999999</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>-0.0191</v>
+        <v>-0.0008</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>-0.0355</v>
+        <v>-0.0235</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>-0.0426</v>
+        <v>-0.0254</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>-0.02</v>
+        <v>-0.0046</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.1191</v>
+        <v>0.1278</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.0257</v>
+        <v>0.0384</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.1789</v>
+        <v>0.1935</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>0.0289</v>
+        <v>0.0388</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>-0.0277</v>
+        <v>-0.0196</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>0.1563</v>
+        <v>0.1609</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>0.1052</v>
+        <v>0.1078</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>0.12</v>
+        <v>0.1213</v>
       </c>
     </row>
     <row r="5">
@@ -677,47 +677,47 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>24377.75</v>
+        <v>24498.75</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>-0.0108</v>
+        <v>-0.0019</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>-0.034</v>
+        <v>-0.0292</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>-0.0377</v>
+        <v>-0.0295</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>-0.0339</v>
+        <v>-0.0234</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>0.0307</v>
+        <v>0.0308</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>-0.0866</v>
+        <v>-0.08210000000000001</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0.06570000000000001</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>-0.062</v>
+        <v>-0.0607</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>-0.0404</v>
+        <v>-0.0371</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>0.0673</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>0.06419999999999999</v>
+        <v>0.06519999999999999</v>
       </c>
       <c r="O5" s="3" t="n">
-        <v>0.1047</v>
+        <v>0.1056</v>
       </c>
     </row>
     <row r="6">
@@ -728,47 +728,47 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>31892.3</v>
+        <v>31943.2</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>-0.009000000000000001</v>
+        <v>-0.002</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-0.033</v>
+        <v>-0.0315</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-0.0339</v>
+        <v>-0.0305</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>-0.0269</v>
+        <v>-0.0227</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.0545</v>
+        <v>0.0481</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>-0.0432</v>
+        <v>-0.0416</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.079</v>
+        <v>0.08070000000000001</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>-0.0158</v>
+        <v>-0.0169</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>-0.0125</v>
+        <v>-0.0101</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>0.0998</v>
+        <v>0.1003</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>0.102</v>
+        <v>0.1023</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>0.113</v>
+        <v>0.1135</v>
       </c>
     </row>
     <row r="7">
@@ -779,47 +779,47 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>33705.7</v>
+        <v>33968</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>-0.0154</v>
+        <v>-0.0015</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-0.0368</v>
+        <v>-0.0293</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>-0.04019999999999999</v>
+        <v>-0.0291</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>-0.0257</v>
+        <v>-0.0153</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.0877</v>
+        <v>0.08939999999999999</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>-0.0074</v>
+        <v>0.0004</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>0.1315</v>
+        <v>0.1404</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>0.0044</v>
+        <v>0.0092</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>-0.0156</v>
+        <v>-0.009899999999999999</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>0.1261</v>
+        <v>0.1289</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>0.1004</v>
+        <v>0.1021</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>0.1124</v>
+        <v>0.1134</v>
       </c>
     </row>
     <row r="8">
@@ -881,47 +881,47 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>16224.6</v>
+        <v>16385.6</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>-0.0127</v>
+        <v>0.0002</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-0.03759999999999999</v>
+        <v>-0.0281</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-0.0359</v>
+        <v>-0.0233</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>-0.0241</v>
+        <v>-0.0134</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>0.0762</v>
+        <v>0.08109999999999999</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>-0.0374</v>
+        <v>-0.0278</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>0.1132</v>
+        <v>0.1243</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>-0.0146</v>
+        <v>-0.008100000000000001</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>-0.0158</v>
+        <v>-0.008699999999999999</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>0.105</v>
+        <v>0.1085</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>0.1074</v>
+        <v>0.1095</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>0.1334</v>
+        <v>0.135</v>
       </c>
     </row>
     <row r="10">
@@ -932,47 +932,47 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>22568.85</v>
+        <v>22901.85</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>-0.0146</v>
+        <v>0.0024</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>-0.0411</v>
+        <v>-0.027</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>-0.0341</v>
+        <v>-0.0173</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>-0.0142</v>
+        <v>-0.0031</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.1223</v>
+        <v>0.1322</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>0.0131</v>
+        <v>0.0281</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.1615</v>
+        <v>0.1786</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>0.0338</v>
+        <v>0.0458</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>0.0075</v>
+        <v>0.0185</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>0.1417</v>
+        <v>0.1472</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0.15</v>
+        <v>0.1532</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>0.1605</v>
+        <v>0.1627</v>
       </c>
     </row>
     <row r="11">
@@ -983,47 +983,47 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>18009.25</v>
+        <v>18287.4</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>-0.023</v>
+        <v>-0.0029</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>-0.0198</v>
+        <v>-0.0046</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>-0.0184</v>
+        <v>0.003</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>0.0225</v>
+        <v>0.03240000000000001</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0.2207</v>
+        <v>0.2363</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>0.0794</v>
+        <v>0.09609999999999999</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>0.2604</v>
+        <v>0.2799</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>0.0308</v>
+        <v>0.0461</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>-0.0144</v>
+        <v>-0.0051</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>0.1374</v>
+        <v>0.1431</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>0.1415</v>
+        <v>0.1449</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>0.1373</v>
+        <v>0.1391</v>
       </c>
     </row>
     <row r="12">
@@ -1034,47 +1034,47 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>20924.9</v>
+        <v>21238.65</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>-0.0176</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>-0.0338</v>
+        <v>-0.0194</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>-0.0287</v>
+        <v>-0.0104</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>-0.0017</v>
+        <v>0.0089</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.1547</v>
+        <v>0.1664</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>0.035</v>
+        <v>0.0505</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0.194</v>
+        <v>0.212</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>0.0319</v>
+        <v>0.0451</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>-0.0008</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0.1399</v>
+        <v>0.1454</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.1473</v>
+        <v>0.1506</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>0.1528</v>
+        <v>0.1549</v>
       </c>
     </row>
     <row r="13">
@@ -1085,47 +1085,47 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>22654.65</v>
+        <v>22840.55</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>-0.013</v>
+        <v>-0.0011</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>-0.0339</v>
+        <v>-0.026</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>-0.0348</v>
+        <v>-0.0233</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>-0.0238</v>
+        <v>-0.0131</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>0.0673</v>
+        <v>0.0709</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>-0.051</v>
+        <v>-0.0432</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>0.1036</v>
+        <v>0.1127</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>-0.0337</v>
+        <v>-0.0288</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>-0.0278</v>
+        <v>-0.0224</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>0.0876</v>
+        <v>0.09050000000000001</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>0.08560000000000001</v>
+        <v>0.0873</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>0.1168</v>
+        <v>0.118</v>
       </c>
     </row>
     <row r="14">
@@ -1136,47 +1136,47 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>35439.31</v>
+        <v>35625.23</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>-0.0132</v>
+        <v>-0.004099999999999999</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>-0.0321</v>
+        <v>-0.0271</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>-0.0356</v>
+        <v>-0.026</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>-0.0233</v>
+        <v>-0.0152</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0.06570000000000001</v>
+        <v>0.0659</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>-0.0535</v>
+        <v>-0.0486</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>0.1012</v>
+        <v>0.107</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>-0.0373</v>
+        <v>-0.0353</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>-0.0318</v>
+        <v>-0.0275</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0.0828</v>
+        <v>0.08460000000000001</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>0.08199999999999999</v>
+        <v>0.08310000000000001</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>0.1156</v>
+        <v>0.1165</v>
       </c>
     </row>
     <row r="15">
@@ -1187,47 +1187,47 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>19378.85</v>
+        <v>19359.85</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>-0.0064</v>
+        <v>-0.004</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>-0.0417</v>
+        <v>-0.0426</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>-0.0411</v>
+        <v>-0.0408</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>-0.0231</v>
+        <v>-0.0192</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>0.0362</v>
+        <v>0.0268</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>-0.08289999999999999</v>
+        <v>-0.08380000000000001</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>0.0585</v>
+        <v>0.0574</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>-0.0619</v>
+        <v>-0.06610000000000001</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>-0.0445</v>
+        <v>-0.0421</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>0.0795</v>
+        <v>0.0791</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>0.0735</v>
+        <v>0.0733</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>0.1078</v>
+        <v>0.1082</v>
       </c>
     </row>
     <row r="16">
@@ -1238,47 +1238,47 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>5457.8</v>
+        <v>5444.35</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>-0.0131</v>
+        <v>-0.0097</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>-0.0458</v>
+        <v>-0.0482</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>-0.0418</v>
+        <v>-0.0409</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>-0.0147</v>
+        <v>-0.0089</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>0.0565</v>
+        <v>0.0445</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>-0.06860000000000001</v>
+        <v>-0.0709</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>0.08439999999999999</v>
+        <v>0.08169999999999999</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>-0.0559</v>
+        <v>-0.0607</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>-0.06309999999999999</v>
+        <v>-0.05980000000000001</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0.0634</v>
+        <v>0.0625</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>0.0619</v>
+        <v>0.0613</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>0.0925</v>
+        <v>0.09269999999999999</v>
       </c>
     </row>
     <row r="17">
@@ -1442,47 +1442,47 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>30130.5</v>
+        <v>30425.85</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>-0.0251</v>
+        <v>-0.008699999999999999</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>-0.039</v>
+        <v>-0.0295</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>-0.0318</v>
+        <v>-0.0115</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>-0.0363</v>
+        <v>-0.0265</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>0.0643</v>
+        <v>0.0709</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>-0.0327</v>
+        <v>-0.0232</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>0.113</v>
+        <v>0.1239</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>-0.0264</v>
+        <v>-0.021</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>-0.0924</v>
+        <v>-0.0858</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>0.0935</v>
+        <v>0.0969</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>0.0861</v>
+        <v>0.0882</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>0.1516</v>
+        <v>0.1529</v>
       </c>
     </row>
     <row r="21">
@@ -1493,47 +1493,47 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>55090.4</v>
+        <v>56192.35</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>-0.0286</v>
+        <v>-0.0022</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>-0.0426</v>
+        <v>-0.0234</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>-0.0242</v>
+        <v>0.0074</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>0.0221</v>
+        <v>0.0328</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>0.1809</v>
+        <v>0.203</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>0.095</v>
+        <v>0.1169</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>0.2383</v>
+        <v>0.2631</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>0.0593</v>
+        <v>0.08019999999999999</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>-0.0442</v>
+        <v>-0.0351</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>0.1512</v>
+        <v>0.1587</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>0.1174</v>
+        <v>0.1218</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>0.1914</v>
+        <v>0.1941</v>
       </c>
     </row>
     <row r="22">
@@ -1544,38 +1544,38 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>26101</v>
+        <v>26110.95</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>-0.0131</v>
+        <v>-0.0048</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>-0.0398</v>
+        <v>-0.0394</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>-0.0411</v>
+        <v>-0.0387</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>-0.0091</v>
+        <v>-0.0071</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>0.0548</v>
+        <v>0.0498</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>-0.036</v>
+        <v>-0.0357</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>0.08929999999999999</v>
+        <v>0.0897</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>-0.0292</v>
+        <v>-0.0328</v>
       </c>
       <c r="L22" s="3" t="n">
-        <v>-0.07519999999999999</v>
+        <v>-0.07240000000000001</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0.09210000000000002</v>
@@ -1584,7 +1584,7 @@
         <v>0.0779</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>0.1174</v>
+        <v>0.1177</v>
       </c>
     </row>
     <row r="23">
@@ -2209,47 +2209,47 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>9818</v>
+        <v>9852.52</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>-0.0157</v>
+        <v>-0.0072</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>-0.0441</v>
+        <v>-0.0407</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>-0.04650000000000001</v>
+        <v>-0.0413</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>0.0285</v>
+        <v>0.0314</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>0.1603</v>
+        <v>0.1564</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>-0.004099999999999999</v>
+        <v>-0.0005999999999999999</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>0.2007</v>
+        <v>0.205</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>-0.0444</v>
+        <v>-0.0433</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>-0.0429</v>
+        <v>-0.0391</v>
       </c>
       <c r="M35" s="3" t="n">
-        <v>0.114</v>
+        <v>0.1152</v>
       </c>
       <c r="N35" s="3" t="n">
-        <v>0.1224</v>
+        <v>0.1232</v>
       </c>
       <c r="O35" s="3" t="n">
-        <v>0.1179</v>
+        <v>0.1187</v>
       </c>
     </row>
     <row r="36">
@@ -2362,47 +2362,47 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>5418.38</v>
+        <v>5480.88</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>-0.0243</v>
+        <v>-0.0031</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>0.0067</v>
+        <v>0.0183</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>-0.0308</v>
+        <v>-0.0073</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>-0.0969</v>
+        <v>-0.0901</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>0.0118</v>
+        <v>0.0137</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>0.0545</v>
+        <v>0.0667</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>0.0415</v>
+        <v>0.0535</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>0.0186</v>
+        <v>0.0282</v>
       </c>
       <c r="L38" s="3" t="n">
-        <v>-0.0885</v>
+        <v>-0.083</v>
       </c>
       <c r="M38" s="3" t="n">
-        <v>0.1334</v>
+        <v>0.1376</v>
       </c>
       <c r="N38" s="3" t="n">
-        <v>0.1401</v>
+        <v>0.1426</v>
       </c>
       <c r="O38" s="3" t="n">
-        <v>0.1201</v>
+        <v>0.1221</v>
       </c>
     </row>
     <row r="39">
@@ -2617,47 +2617,47 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>7637.76</v>
+        <v>7650.5</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>0.0061</v>
+        <v>-0.0008</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>-0.0063</v>
+        <v>-0.0046</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>-0.006999999999999999</v>
+        <v>-0.0075</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>0.0183</v>
+        <v>0.02</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>0.1561</v>
+        <v>0.1758</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>0.1157</v>
+        <v>0.1176</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>0.1699</v>
+        <v>0.1719</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>0.1572</v>
+        <v>0.1536</v>
       </c>
       <c r="L43" s="3" t="n">
-        <v>0.1644</v>
+        <v>0.1671</v>
       </c>
       <c r="M43" s="3" t="n">
-        <v>0.1971</v>
+        <v>0.1987</v>
       </c>
       <c r="N43" s="3" t="n">
-        <v>0.115</v>
+        <v>0.1153</v>
       </c>
       <c r="O43" s="3" t="n">
-        <v>0.1358</v>
+        <v>0.136</v>
       </c>
     </row>
     <row r="44">
@@ -2668,47 +2668,47 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>29446.98</v>
+        <v>29644.17</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>0.0118</v>
+        <v>0.009399999999999999</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>-0.0003</v>
+        <v>0.0064</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>-0.0015</v>
+        <v>0.0074</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>-0.0315</v>
+        <v>-0.0251</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>0.2091</v>
+        <v>0.2404</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>0.1662</v>
+        <v>0.174</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>0.2404</v>
+        <v>0.2487</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>0.2156</v>
+        <v>0.2122</v>
       </c>
       <c r="L44" s="3" t="n">
-        <v>0.2312</v>
+        <v>0.2381</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>0.2461</v>
+        <v>0.2498</v>
       </c>
       <c r="N44" s="3" t="n">
-        <v>0.1394</v>
+        <v>0.1409</v>
       </c>
       <c r="O44" s="3" t="n">
-        <v>0.1991</v>
+        <v>0.1997</v>
       </c>
     </row>
     <row r="45">
@@ -2774,43 +2774,43 @@
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>25532.82</v>
+        <v>25304.06</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>-0.0014</v>
+        <v>-0.0103</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>-0.0276</v>
+        <v>-0.0363</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>-0.0214</v>
+        <v>-0.0302</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>0.0219</v>
+        <v>0.0127</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>0.1409</v>
+        <v>0.1306</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>0.0426</v>
+        <v>0.0332</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>0.1258</v>
+        <v>0.1157</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>0.0785</v>
+        <v>0.0688</v>
       </c>
       <c r="L46" s="3" t="n">
-        <v>0.1683</v>
+        <v>0.163</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>0.177</v>
+        <v>0.1735</v>
       </c>
       <c r="N46" s="3" t="n">
-        <v>0.1051</v>
+        <v>0.1031</v>
       </c>
       <c r="O46" s="3" t="n">
-        <v>0.0941</v>
+        <v>0.0931</v>
       </c>
     </row>
     <row r="47">
@@ -2825,43 +2825,43 @@
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>8116.7</v>
+        <v>8065.02</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>-0.0077</v>
+        <v>-0.014</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>-0.0261</v>
+        <v>-0.0323</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>-0.0453</v>
+        <v>-0.05139999999999999</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>-0.0362</v>
+        <v>-0.0423</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>0.0588</v>
+        <v>0.0521</v>
       </c>
       <c r="I47" s="3" t="n">
-        <v>-0.004</v>
+        <v>-0.0104</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>0.0383</v>
+        <v>0.0317</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>0.0334</v>
+        <v>0.0268</v>
       </c>
       <c r="L47" s="3" t="n">
-        <v>0.0442</v>
+        <v>0.0408</v>
       </c>
       <c r="M47" s="3" t="n">
-        <v>0.0369</v>
+        <v>0.0346</v>
       </c>
       <c r="N47" s="3" t="n">
-        <v>0.0432</v>
+        <v>0.0418</v>
       </c>
       <c r="O47" s="3" t="n">
-        <v>0.0635</v>
+        <v>0.06280000000000001</v>
       </c>
     </row>
     <row r="48">
@@ -2876,43 +2876,43 @@
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>10726.4</v>
+        <v>10659.13</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>0.0071</v>
+        <v>0.0008</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>-0.009000000000000001</v>
+        <v>-0.0153</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>-0.0016</v>
+        <v>-0.007800000000000001</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>0.035</v>
+        <v>0.0285</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>0.0815</v>
+        <v>0.0747</v>
       </c>
       <c r="I48" s="3" t="n">
-        <v>0.08</v>
+        <v>0.0733</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>0.05400000000000001</v>
+        <v>0.0474</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>0.1624</v>
+        <v>0.1551</v>
       </c>
       <c r="L48" s="3" t="n">
-        <v>0.1401</v>
+        <v>0.1365</v>
       </c>
       <c r="M48" s="3" t="n">
-        <v>0.1188</v>
+        <v>0.1165</v>
       </c>
       <c r="N48" s="3" t="n">
-        <v>0.0902</v>
+        <v>0.0888</v>
       </c>
       <c r="O48" s="3" t="n">
-        <v>0.0462</v>
+        <v>0.0455</v>
       </c>
     </row>
     <row r="49">
@@ -3025,11 +3025,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>95.87</v>
+        <v>95.88</v>
       </c>
       <c r="D51" s="3" t="n">
         <v>0.0019</v>
@@ -3038,34 +3038,34 @@
         <v>0.0052</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0011</v>
       </c>
       <c r="G51" s="3" t="n">
+        <v>0.0163</v>
+      </c>
+      <c r="H51" s="3" t="n">
+        <v>0.0301</v>
+      </c>
+      <c r="I51" s="3" t="n">
+        <v>0.06809999999999999</v>
+      </c>
+      <c r="J51" s="3" t="n">
         <v>0.0162</v>
       </c>
-      <c r="H51" s="3" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="I51" s="3" t="n">
-        <v>0.068</v>
-      </c>
-      <c r="J51" s="3" t="n">
-        <v>0.0161</v>
-      </c>
       <c r="K51" s="3" t="n">
-        <v>0.0906</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="L51" s="3" t="n">
-        <v>0.0698</v>
+        <v>0.0709</v>
       </c>
       <c r="M51" s="3" t="n">
-        <v>0.0482</v>
+        <v>0.0489</v>
       </c>
       <c r="N51" s="3" t="n">
-        <v>0.0544</v>
+        <v>0.0542</v>
       </c>
       <c r="O51" s="3" t="n">
-        <v>0.0366</v>
+        <v>0.0369</v>
       </c>
     </row>
     <row r="52">
@@ -3080,43 +3080,43 @@
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>4421.4</v>
+        <v>4424.9</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>0.0028</v>
+        <v>0.0036</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>-0.0022</v>
+        <v>-0.0014</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>-0.0151</v>
+        <v>-0.0144</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>0.0467</v>
+        <v>0.0475</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>-0.0326</v>
+        <v>-0.0318</v>
       </c>
       <c r="I52" s="3" t="n">
-        <v>0.0221</v>
+        <v>0.023</v>
       </c>
       <c r="J52" s="3" t="n">
-        <v>-0.0487</v>
+        <v>-0.0479</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>0.2134</v>
+        <v>0.2144</v>
       </c>
       <c r="L52" s="3" t="n">
-        <v>0.3117</v>
+        <v>0.3122</v>
       </c>
       <c r="M52" s="3" t="n">
-        <v>0.3181</v>
+        <v>0.3184</v>
       </c>
       <c r="N52" s="3" t="n">
-        <v>0.2037</v>
+        <v>0.2038</v>
       </c>
       <c r="O52" s="3" t="n">
-        <v>0.1291</v>
+        <v>0.1292</v>
       </c>
     </row>
     <row r="53">
@@ -3131,43 +3131,43 @@
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>67.66</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>0.0481</v>
+        <v>0.04019999999999999</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>0.0217</v>
+        <v>0.014</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>0.0293</v>
+        <v>0.0215</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>0.0212</v>
+        <v>0.0135</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>-0.0245</v>
+        <v>-0.0319</v>
       </c>
       <c r="I53" s="3" t="n">
-        <v>-0.0353</v>
+        <v>-0.0426</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>-0.0941</v>
+        <v>-0.101</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>0.6223</v>
+        <v>0.61</v>
       </c>
       <c r="L53" s="3" t="n">
-        <v>0.4937</v>
+        <v>0.4881</v>
       </c>
       <c r="M53" s="3" t="n">
-        <v>0.4292</v>
+        <v>0.4256</v>
       </c>
       <c r="N53" s="3" t="n">
-        <v>0.2485</v>
+        <v>0.2466</v>
       </c>
       <c r="O53" s="3" t="n">
-        <v>0.1344</v>
+        <v>0.1335</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Weekly indices update 2026-09-27
</commit_message>
<xml_diff>
--- a/tracker_auto.xlsx
+++ b/tracker_auto.xlsx
@@ -524,47 +524,47 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>23346.4</v>
+        <v>23140.5</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>-0.0022</v>
+        <v>-0.008800000000000001</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-0.0305</v>
+        <v>-0.039</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>-0.0304</v>
+        <v>-0.0441</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>-0.0278</v>
+        <v>-0.0381</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>0.01</v>
+        <v>0.0141</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>-0.1065</v>
+        <v>-0.1144</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.0455</v>
+        <v>0.0362</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>-0.08169999999999999</v>
+        <v>-0.0703</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>-0.0409</v>
+        <v>-0.0567</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>0.0506</v>
+        <v>0.0558</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>0.0583</v>
+        <v>0.0532</v>
       </c>
       <c r="O2" s="3" t="n">
-        <v>0.1029</v>
+        <v>0.1028</v>
       </c>
     </row>
     <row r="3">
@@ -575,47 +575,47 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>74294.96000000001</v>
+        <v>73895.74000000001</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>-0.006500000000000001</v>
+        <v>-0.0054</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>-0.0346</v>
+        <v>-0.0398</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>-0.034</v>
+        <v>-0.0462</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>-0.0327</v>
+        <v>-0.0416</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>-0.0032</v>
+        <v>0.0042</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>-0.1282</v>
+        <v>-0.1329</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>0.0326</v>
+        <v>0.0271</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>-0.105</v>
+        <v>-0.0895</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>-0.0536</v>
+        <v>-0.06860000000000001</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>0.032</v>
+        <v>0.0387</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>0.0471</v>
+        <v>0.0424</v>
       </c>
       <c r="O3" s="3" t="n">
-        <v>0.1005</v>
+        <v>0.1011</v>
       </c>
     </row>
     <row r="4">
@@ -626,47 +626,47 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>72025.39999999999</v>
+        <v>71778.64999999999</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>-0.0008</v>
+        <v>-0.0034</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>-0.0235</v>
+        <v>-0.0269</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>-0.0254</v>
+        <v>-0.0365</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>-0.0046</v>
+        <v>-0.0058</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.1278</v>
+        <v>0.1569</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.0384</v>
+        <v>0.0348</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.1935</v>
+        <v>0.1894</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>0.0388</v>
+        <v>0.051</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>-0.0196</v>
+        <v>-0.0315</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>0.1609</v>
+        <v>0.1672</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>0.1078</v>
+        <v>0.1075</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>0.1213</v>
+        <v>0.1199</v>
       </c>
     </row>
     <row r="5">
@@ -677,47 +677,47 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>24498.75</v>
+        <v>24307.55</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>-0.0019</v>
+        <v>-0.007800000000000001</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>-0.0292</v>
+        <v>-0.0368</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>-0.0295</v>
+        <v>-0.04269999999999999</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>-0.0234</v>
+        <v>-0.0321</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>0.0308</v>
+        <v>0.0388</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>-0.08210000000000001</v>
+        <v>-0.0892</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.0626</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>-0.0607</v>
+        <v>-0.0491</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>-0.0371</v>
+        <v>-0.0521</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.07429999999999999</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>0.06519999999999999</v>
+        <v>0.0608</v>
       </c>
       <c r="O5" s="3" t="n">
-        <v>0.1056</v>
+        <v>0.1053</v>
       </c>
     </row>
     <row r="6">
@@ -728,47 +728,47 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>31943.2</v>
+        <v>31685.3</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>-0.002</v>
+        <v>-0.008100000000000001</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-0.0315</v>
+        <v>-0.0393</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-0.0305</v>
+        <v>-0.04190000000000001</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>-0.0227</v>
+        <v>-0.0273</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.0481</v>
+        <v>0.0506</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>-0.0416</v>
+        <v>-0.04940000000000001</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.08070000000000001</v>
+        <v>0.07200000000000001</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>-0.0169</v>
+        <v>-0.007800000000000001</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>-0.0101</v>
+        <v>-0.0232</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>0.1003</v>
+        <v>0.1035</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>0.1023</v>
+        <v>0.0987</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>0.1135</v>
+        <v>0.1132</v>
       </c>
     </row>
     <row r="7">
@@ -779,47 +779,47 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>33968</v>
+        <v>33776.85</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>-0.0015</v>
+        <v>-0.005600000000000001</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-0.0293</v>
+        <v>-0.0348</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>-0.0291</v>
+        <v>-0.04219999999999999</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>-0.0153</v>
+        <v>-0.0166</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.08939999999999999</v>
+        <v>0.1062</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>0.0004</v>
+        <v>-0.0053</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>0.1404</v>
+        <v>0.1339</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>0.0092</v>
+        <v>0.0192</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>-0.009899999999999999</v>
+        <v>-0.0218</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>0.1289</v>
+        <v>0.1332</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>0.1021</v>
+        <v>0.0998</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>0.1134</v>
+        <v>0.1127</v>
       </c>
     </row>
     <row r="8">
@@ -830,47 +830,47 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>18351.23</v>
+        <v>18160.19</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>-0.0016</v>
+        <v>-0.0104</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-0.0295</v>
+        <v>-0.0396</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-0.0271</v>
+        <v>-0.0438</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>-0.0164</v>
+        <v>-0.0255</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.0574</v>
+        <v>0.0622</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>-0.05400000000000001</v>
+        <v>-0.0638</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.0989</v>
+        <v>0.08749999999999999</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>-0.0304</v>
+        <v>-0.02</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>-0.0163</v>
+        <v>-0.032</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>0.0941</v>
+        <v>0.0978</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>0.09080000000000001</v>
+        <v>0.0859</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>0.1257</v>
+        <v>0.1249</v>
       </c>
     </row>
     <row r="9">
@@ -881,47 +881,47 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>16385.6</v>
+        <v>16153.55</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>0.0002</v>
+        <v>-0.0142</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-0.0281</v>
+        <v>-0.0418</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-0.0233</v>
+        <v>-0.0446</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>-0.0134</v>
+        <v>-0.0229</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>0.08109999999999999</v>
+        <v>0.0814</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>-0.0278</v>
+        <v>-0.0416</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>0.1243</v>
+        <v>0.1083</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>-0.008100000000000001</v>
+        <v>-0.0004</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>-0.008699999999999999</v>
+        <v>-0.0246</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>0.1085</v>
+        <v>0.1089</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>0.1095</v>
+        <v>0.1043</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>0.135</v>
+        <v>0.1331</v>
       </c>
     </row>
     <row r="10">
@@ -932,47 +932,47 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>22901.85</v>
+        <v>22437</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.0024</v>
+        <v>-0.0203</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>-0.027</v>
+        <v>-0.0467</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>-0.0173</v>
+        <v>-0.04650000000000001</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>-0.0031</v>
+        <v>-0.0138</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.1322</v>
+        <v>0.1245</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>0.0281</v>
+        <v>0.0072</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.1786</v>
+        <v>0.1547</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>0.0458</v>
+        <v>0.04940000000000001</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>0.0185</v>
+        <v>0.0018</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>0.1472</v>
+        <v>0.1426</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0.1532</v>
+        <v>0.1471</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>0.1627</v>
+        <v>0.1592</v>
       </c>
     </row>
     <row r="11">
@@ -983,47 +983,47 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>18287.4</v>
+        <v>18158.9</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>-0.0029</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>-0.0046</v>
+        <v>-0.0116</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.003</v>
+        <v>-0.0161</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>0.03240000000000001</v>
+        <v>0.0257</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0.2363</v>
+        <v>0.2391</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>0.09609999999999999</v>
+        <v>0.08839999999999999</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>0.2799</v>
+        <v>0.2709</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>0.0461</v>
+        <v>0.06509999999999999</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>-0.0051</v>
+        <v>-0.0098</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>0.1431</v>
+        <v>0.145</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>0.1449</v>
+        <v>0.143</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>0.1391</v>
+        <v>0.138</v>
       </c>
     </row>
     <row r="12">
@@ -1034,47 +1034,47 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>21238.65</v>
+        <v>20904.95</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0.0005999999999999999</v>
+        <v>-0.0157</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>-0.0194</v>
+        <v>-0.0348</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>-0.0104</v>
+        <v>-0.0361</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0.0089</v>
+        <v>-0.0004</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.1664</v>
+        <v>0.1621</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>0.0505</v>
+        <v>0.034</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0.212</v>
+        <v>0.1929</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>0.0451</v>
+        <v>0.05400000000000001</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>0.009599999999999999</v>
+        <v>-0.0028</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0.1454</v>
+        <v>0.143</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.1506</v>
+        <v>0.1459</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>0.1549</v>
+        <v>0.1522</v>
       </c>
     </row>
     <row r="13">
@@ -1085,47 +1085,47 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>22840.55</v>
+        <v>22603.5</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>-0.0011</v>
+        <v>-0.0104</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>-0.026</v>
+        <v>-0.0361</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>-0.0233</v>
+        <v>-0.0406</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>-0.0131</v>
+        <v>-0.0221</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>0.0709</v>
+        <v>0.07530000000000001</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>-0.0432</v>
+        <v>-0.05309999999999999</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>0.1127</v>
+        <v>0.1011</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>-0.0288</v>
+        <v>-0.0182</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>-0.0224</v>
+        <v>-0.03700000000000001</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>0.09050000000000001</v>
+        <v>0.09380000000000001</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>0.0873</v>
+        <v>0.0827</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>0.118</v>
+        <v>0.1172</v>
       </c>
     </row>
     <row r="14">
@@ -1136,47 +1136,47 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>35625.23</v>
+        <v>35353.29</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>-0.004099999999999999</v>
+        <v>-0.0076</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>-0.0271</v>
+        <v>-0.0345</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>-0.026</v>
+        <v>-0.0417</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>-0.0152</v>
+        <v>-0.0216</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0.0659</v>
+        <v>0.07339999999999999</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>-0.0486</v>
+        <v>-0.0558</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>0.107</v>
+        <v>0.09849999999999999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>-0.0353</v>
+        <v>-0.0222</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>-0.0275</v>
+        <v>-0.0407</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0.08460000000000001</v>
+        <v>0.0891</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>0.08310000000000001</v>
+        <v>0.0791</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>0.1165</v>
+        <v>0.1159</v>
       </c>
     </row>
     <row r="15">
@@ -1187,47 +1187,47 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>19359.85</v>
+        <v>19257.7</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>-0.004</v>
+        <v>-0.0053</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>-0.0426</v>
+        <v>-0.04769999999999999</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>-0.0408</v>
+        <v>-0.0463</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>-0.0192</v>
+        <v>-0.0284</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>0.0268</v>
+        <v>0.0299</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>-0.08380000000000001</v>
+        <v>-0.0886</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>0.0574</v>
+        <v>0.0519</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>-0.06610000000000001</v>
+        <v>-0.0462</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>-0.0421</v>
+        <v>-0.0533</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>0.0791</v>
+        <v>0.08470000000000001</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>0.0733</v>
+        <v>0.0699</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>0.1082</v>
+        <v>0.1081</v>
       </c>
     </row>
     <row r="16">
@@ -1238,47 +1238,47 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>5444.35</v>
+        <v>5443.15</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>-0.0097</v>
+        <v>-0.0002</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>-0.0482</v>
+        <v>-0.0484</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>-0.0409</v>
+        <v>-0.0454</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>-0.0089</v>
+        <v>0.0017</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>0.0445</v>
+        <v>0.06269999999999999</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>-0.0709</v>
+        <v>-0.0711</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>0.08169999999999999</v>
+        <v>0.0815</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>-0.0607</v>
+        <v>-0.0346</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>-0.05980000000000001</v>
+        <v>-0.0665</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0.0625</v>
+        <v>0.06660000000000001</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>0.0613</v>
+        <v>0.0578</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>0.09269999999999999</v>
+        <v>0.0935</v>
       </c>
     </row>
     <row r="17">
@@ -1289,47 +1289,47 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>25660.26</v>
+        <v>25572.12</v>
       </c>
       <c r="D17" s="3" t="n">
         <v>-0.0034</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>-0.0166</v>
+        <v>-0.02</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>-0.0191</v>
+        <v>-0.0298</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>-0.0539</v>
+        <v>-0.0413</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>0.0042</v>
+        <v>0.0221</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>0.0012</v>
+        <v>-0.0022</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>0.0438</v>
+        <v>0.04019999999999999</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>0.1197</v>
+        <v>0.1164</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>0.0461</v>
+        <v>0.0332</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>0.2293</v>
+        <v>0.2301</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>0.2465</v>
+        <v>0.2456</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>0.1682</v>
+        <v>0.1671</v>
       </c>
     </row>
     <row r="18">
@@ -1340,47 +1340,47 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>38277.74</v>
+        <v>38030.13</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>-0.008699999999999999</v>
+        <v>-0.006500000000000001</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>-0.0291</v>
+        <v>-0.0353</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>-0.0107</v>
+        <v>-0.0365</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>-0.0236</v>
+        <v>-0.0281</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>0.0762</v>
+        <v>0.08710000000000001</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>-0.0174</v>
+        <v>-0.0237</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>0.1293</v>
+        <v>0.122</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>-0.015</v>
+        <v>0.0033</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>-0.07969999999999999</v>
+        <v>-0.096</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>0.1059</v>
+        <v>0.1053</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>0.09789999999999999</v>
+        <v>0.0968</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>0.164</v>
+        <v>0.1611</v>
       </c>
     </row>
     <row r="19">
@@ -1391,47 +1391,47 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>28332.96</v>
+        <v>28178.09</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>-0.0073</v>
+        <v>-0.005500000000000001</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>-0.049</v>
+        <v>-0.0542</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>-0.0453</v>
+        <v>-0.05139999999999999</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>-0.0197</v>
+        <v>-0.0113</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>0.0475</v>
+        <v>0.0566</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>-0.0747</v>
+        <v>-0.07980000000000001</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>0.0839</v>
+        <v>0.078</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>-0.065</v>
+        <v>-0.0437</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>-0.0633</v>
+        <v>-0.0701</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>0.0711</v>
+        <v>0.07200000000000001</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>0.0683</v>
+        <v>0.06309999999999999</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>0.1183</v>
+        <v>0.1179</v>
       </c>
     </row>
     <row r="20">
@@ -1442,47 +1442,47 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>30425.85</v>
+        <v>30229</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>-0.008699999999999999</v>
+        <v>-0.006500000000000001</v>
       </c>
       <c r="E20" s="3" t="n">
+        <v>-0.0358</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>-0.0371</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>-0.0306</v>
+      </c>
+      <c r="H20" s="3" t="n">
+        <v>0.0818</v>
+      </c>
+      <c r="I20" s="3" t="n">
         <v>-0.0295</v>
       </c>
-      <c r="F20" s="3" t="n">
-        <v>-0.0115</v>
-      </c>
-      <c r="G20" s="3" t="n">
-        <v>-0.0265</v>
-      </c>
-      <c r="H20" s="3" t="n">
-        <v>0.0709</v>
-      </c>
-      <c r="I20" s="3" t="n">
-        <v>-0.0232</v>
-      </c>
       <c r="J20" s="3" t="n">
-        <v>0.1239</v>
+        <v>0.1166</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>-0.021</v>
+        <v>-0.0028</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>-0.0858</v>
+        <v>-0.102</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>0.0969</v>
+        <v>0.09630000000000001</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>0.0882</v>
+        <v>0.0872</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>0.1529</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="21">
@@ -1493,47 +1493,47 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>56192.35</v>
+        <v>55024.65</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>-0.0022</v>
+        <v>-0.0208</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>-0.0234</v>
+        <v>-0.0437</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>0.0074</v>
+        <v>-0.0437</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>0.0328</v>
+        <v>0.0275</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>0.203</v>
+        <v>0.199</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>0.1169</v>
+        <v>0.09369999999999999</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>0.2631</v>
+        <v>0.2368</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>0.08019999999999999</v>
+        <v>0.09080000000000001</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>-0.0351</v>
+        <v>-0.049</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>0.1587</v>
+        <v>0.1522</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>0.1218</v>
+        <v>0.1162</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>0.1941</v>
+        <v>0.1899</v>
       </c>
     </row>
     <row r="22">
@@ -1544,47 +1544,47 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>26110.95</v>
+        <v>25992.5</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>-0.0048</v>
+        <v>-0.004500000000000001</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>-0.0394</v>
+        <v>-0.0438</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>-0.0387</v>
+        <v>-0.0432</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>-0.0071</v>
+        <v>-0.017</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>0.0498</v>
+        <v>0.05690000000000001</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>-0.0357</v>
+        <v>-0.0401</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>0.0897</v>
+        <v>0.0848</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>-0.0328</v>
+        <v>-0.012</v>
       </c>
       <c r="L22" s="3" t="n">
-        <v>-0.07240000000000001</v>
+        <v>-0.08560000000000001</v>
       </c>
       <c r="M22" s="3" t="n">
-        <v>0.09210000000000002</v>
+        <v>0.09470000000000001</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>0.0779</v>
+        <v>0.07429999999999999</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>0.1177</v>
+        <v>0.1166</v>
       </c>
     </row>
     <row r="23">
@@ -1595,44 +1595,44 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>10363.48</v>
+        <v>10420.47</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>-0.0382</v>
+        <v>0.005500000000000001</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>-0.03759999999999999</v>
+        <v>-0.0323</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>-0.0474</v>
+        <v>-0.0349</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>-0.0231</v>
+        <v>0.0023</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>0.2108</v>
+        <v>0.2688</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>0.2128</v>
+        <v>0.2194</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>0.2983</v>
+        <v>0.3054</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>0.1363</v>
+        <v>0.1618</v>
       </c>
       <c r="L23" s="3" t="n">
-        <v>0.1952</v>
+        <v>0.1906</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>0.4257</v>
+        <v>0.4316</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>0.5146000000000001</v>
+        <v>0.5193</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -1648,47 +1648,47 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>11418.56</v>
+        <v>11386.9</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>-0.0039</v>
+        <v>-0.0028</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>-0.0339</v>
+        <v>-0.0366</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>-0.0348</v>
+        <v>-0.0433</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>-0.0457</v>
+        <v>-0.0395</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>-0.0245</v>
+        <v>0.0123</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>-0.018</v>
+        <v>-0.0208</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>0.0636</v>
+        <v>0.0607</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>0.1473</v>
+        <v>0.1303</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>0.1241</v>
+        <v>0.1176</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>0.1764</v>
+        <v>0.1776</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>0.2883</v>
+        <v>0.2993</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>0.1084</v>
+        <v>0.1099</v>
       </c>
     </row>
     <row r="25">
@@ -1699,47 +1699,47 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>79111.42</v>
+        <v>78018.91</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>-0.0044</v>
+        <v>-0.0138</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>-0.0287</v>
+        <v>-0.0421</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>-0.0154</v>
+        <v>-0.0381</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>-0.0211</v>
+        <v>-0.0428</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>0.06179999999999999</v>
+        <v>0.0702</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>-0.0479</v>
+        <v>-0.061</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>0.1284</v>
+        <v>0.1128</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>0.018</v>
+        <v>0.0176</v>
       </c>
       <c r="L25" s="3" t="n">
-        <v>0.0412</v>
+        <v>0.0209</v>
       </c>
       <c r="M25" s="3" t="n">
-        <v>0.0785</v>
+        <v>0.08439999999999999</v>
       </c>
       <c r="N25" s="3" t="n">
-        <v>0.0917</v>
+        <v>0.0886</v>
       </c>
       <c r="O25" s="3" t="n">
-        <v>0.1166</v>
+        <v>0.1169</v>
       </c>
     </row>
     <row r="26">
@@ -1750,47 +1750,47 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>32304.13</v>
+        <v>31822.57</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>-0.0053</v>
+        <v>-0.0149</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>-0.0256</v>
+        <v>-0.0401</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>0.003</v>
+        <v>-0.0306</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>-0.0188</v>
+        <v>-0.0482</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>0.08650000000000001</v>
+        <v>0.0824</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>-0.0441</v>
+        <v>-0.0584</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>0.1371</v>
+        <v>0.1201</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>0.0113</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="L26" s="3" t="n">
-        <v>0.0206</v>
+        <v>0.0012</v>
       </c>
       <c r="M26" s="3" t="n">
-        <v>0.0547</v>
+        <v>0.059</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>0.07400000000000001</v>
+        <v>0.0698</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>0.09970000000000001</v>
+        <v>0.1003</v>
       </c>
     </row>
     <row r="27">
@@ -1801,47 +1801,47 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>32642.69</v>
+        <v>32111.44</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>-0.0014</v>
+        <v>-0.0163</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>-0.0298</v>
+        <v>-0.04559999999999999</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>-0.0191</v>
+        <v>-0.0488</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>-0.0319</v>
+        <v>-0.0597</v>
       </c>
       <c r="H27" s="3" t="n">
         <v>0.0378</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>-0.0682</v>
+        <v>-0.0833</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>0.0931</v>
+        <v>0.07530000000000001</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>-0.0358</v>
+        <v>-0.0352</v>
       </c>
       <c r="L27" s="3" t="n">
-        <v>0.0338</v>
+        <v>0.0117</v>
       </c>
       <c r="M27" s="3" t="n">
-        <v>0.0876</v>
+        <v>0.09279999999999999</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>0.0767</v>
+        <v>0.07139999999999999</v>
       </c>
       <c r="O27" s="3" t="n">
-        <v>0.1294</v>
+        <v>0.1287</v>
       </c>
     </row>
     <row r="28">
@@ -1852,47 +1852,47 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>17385.42</v>
+        <v>17342.45</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>-0.009399999999999999</v>
+        <v>-0.0025</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>-0.008199999999999999</v>
+        <v>-0.0106</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>-0.0124</v>
+        <v>-0.0126</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>-0.0505</v>
+        <v>-0.0315</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>-0.0217</v>
+        <v>-0.0037</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>-0.0118</v>
+        <v>-0.0143</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>0.011</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>-0.0059</v>
+        <v>-0.0023</v>
       </c>
       <c r="L28" s="3" t="n">
-        <v>-0.0381</v>
+        <v>-0.0526</v>
       </c>
       <c r="M28" s="3" t="n">
-        <v>0.1993</v>
+        <v>0.2003</v>
       </c>
       <c r="N28" s="3" t="n">
-        <v>0.23</v>
+        <v>0.2309</v>
       </c>
       <c r="O28" s="3" t="n">
-        <v>0.1409</v>
+        <v>0.1404</v>
       </c>
     </row>
     <row r="29">
@@ -1903,47 +1903,47 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>940.97</v>
+        <v>968.98</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>-0.005</v>
+        <v>0.0298</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>-0.06610000000000001</v>
+        <v>-0.0383</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>-0.05690000000000001</v>
+        <v>-0.0446</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>0.0443</v>
+        <v>0.0567</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>0.2177</v>
+        <v>0.303</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>-0.034</v>
+        <v>-0.0053</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>0.3023</v>
+        <v>0.3411</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>-0.0765</v>
+        <v>-0.0028</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>-0.1056</v>
+        <v>-0.1195</v>
       </c>
       <c r="M29" s="3" t="n">
-        <v>0.138</v>
+        <v>0.1541</v>
       </c>
       <c r="N29" s="3" t="n">
-        <v>0.1574</v>
+        <v>0.1203</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>0.1566</v>
+        <v>0.1596</v>
       </c>
     </row>
     <row r="30">
@@ -1954,47 +1954,47 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>36314.06</v>
+        <v>36098.42</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>-0.0064</v>
+        <v>-0.0059</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>-0.0594</v>
+        <v>-0.065</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>-0.07049999999999999</v>
+        <v>-0.0701</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>0.0268</v>
+        <v>0.005699999999999999</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>0.1076</v>
+        <v>0.1174</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>-0.0276</v>
+        <v>-0.0334</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>0.1513</v>
+        <v>0.1444</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>0.0032</v>
+        <v>0.0185</v>
       </c>
       <c r="L30" s="3" t="n">
-        <v>0.0356</v>
+        <v>0.0115</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>0.1894</v>
+        <v>0.1942</v>
       </c>
       <c r="N30" s="3" t="n">
-        <v>0.2236</v>
+        <v>0.2203</v>
       </c>
       <c r="O30" s="3" t="n">
-        <v>0.1159</v>
+        <v>0.1161</v>
       </c>
     </row>
     <row r="31">
@@ -2005,47 +2005,47 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>20923.37</v>
+        <v>20860.87</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>-0.0024</v>
+        <v>-0.003</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>-0.0393</v>
+        <v>-0.04219999999999999</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>-0.0329</v>
+        <v>-0.0413</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>-0.0024</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>0.1002</v>
+        <v>0.1177</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>0.0416</v>
+        <v>0.0385</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>0.1418</v>
+        <v>0.1384</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>0.05400000000000001</v>
+        <v>0.0697</v>
       </c>
       <c r="L31" s="3" t="n">
-        <v>0.036</v>
+        <v>0.0215</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>0.1769</v>
+        <v>0.1846</v>
       </c>
       <c r="N31" s="3" t="n">
-        <v>0.1608</v>
+        <v>0.162</v>
       </c>
       <c r="O31" s="3" t="n">
-        <v>0.1392</v>
+        <v>0.1382</v>
       </c>
     </row>
     <row r="32">
@@ -2056,47 +2056,47 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>11982.33</v>
+        <v>11831.92</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>-0.0005999999999999999</v>
+        <v>-0.0126</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>-0.0112</v>
+        <v>-0.0236</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>-0.0246</v>
+        <v>-0.0351</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>-0.0429</v>
+        <v>-0.05</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>0.03700000000000001</v>
+        <v>0.0333</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>-0.05</v>
+        <v>-0.0619</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>0.0659</v>
+        <v>0.0525</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>-0.0091</v>
+        <v>-0.0052</v>
       </c>
       <c r="L32" s="3" t="n">
-        <v>-0.0059</v>
+        <v>-0.0269</v>
       </c>
       <c r="M32" s="3" t="n">
-        <v>0.1406</v>
+        <v>0.1414</v>
       </c>
       <c r="N32" s="3" t="n">
-        <v>0.1407</v>
+        <v>0.1347</v>
       </c>
       <c r="O32" s="3" t="n">
-        <v>0.1371</v>
+        <v>0.1374</v>
       </c>
     </row>
     <row r="33">
@@ -2107,47 +2107,47 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>19830.73</v>
+        <v>19907.91</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>0.0074</v>
+        <v>0.0039</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>-0.0193</v>
+        <v>-0.0155</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>0.0123</v>
+        <v>0.005600000000000001</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>0.0626</v>
+        <v>0.047</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>0.1585</v>
+        <v>0.159</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>0.1404</v>
+        <v>0.1448</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>0.1734</v>
+        <v>0.178</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>0.124</v>
+        <v>0.1597</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>0.0751</v>
+        <v>0.07200000000000001</v>
       </c>
       <c r="M33" s="3" t="n">
-        <v>0.2012</v>
+        <v>0.2152</v>
       </c>
       <c r="N33" s="3" t="n">
-        <v>0.135</v>
+        <v>0.1386</v>
       </c>
       <c r="O33" s="3" t="n">
-        <v>0.1073</v>
+        <v>0.1071</v>
       </c>
     </row>
     <row r="34">
@@ -2158,47 +2158,47 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>19918.59</v>
+        <v>19971.29</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>0.0042</v>
+        <v>0.0026</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>-0.0105</v>
+        <v>-0.007800000000000001</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>0.0028</v>
+        <v>-0.0333</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>0.0048</v>
+        <v>0.05400000000000001</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>0.154</v>
+        <v>0.1804</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>0.18</v>
+        <v>0.1831</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>0.1797</v>
+        <v>0.1828</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>0.3248</v>
+        <v>0.3111</v>
       </c>
       <c r="L34" s="3" t="n">
-        <v>0.1956</v>
+        <v>0.1679</v>
       </c>
       <c r="M34" s="3" t="n">
-        <v>0.2432</v>
+        <v>0.2555</v>
       </c>
       <c r="N34" s="3" t="n">
-        <v>0.1957</v>
+        <v>0.2041</v>
       </c>
       <c r="O34" s="3" t="n">
-        <v>0.2025</v>
+        <v>0.2014</v>
       </c>
     </row>
     <row r="35">
@@ -2209,47 +2209,47 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>9852.52</v>
+        <v>9858.870000000001</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>-0.0072</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>-0.0407</v>
+        <v>-0.0401</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>-0.0413</v>
+        <v>-0.0437</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>0.0314</v>
+        <v>0.0317</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>0.1564</v>
+        <v>0.1772</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>-0.0005999999999999999</v>
+        <v>0</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>0.205</v>
+        <v>0.2057</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>-0.0433</v>
+        <v>-0.0145</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>-0.0391</v>
+        <v>-0.0527</v>
       </c>
       <c r="M35" s="3" t="n">
-        <v>0.1152</v>
+        <v>0.1205</v>
       </c>
       <c r="N35" s="3" t="n">
-        <v>0.1232</v>
+        <v>0.1173</v>
       </c>
       <c r="O35" s="3" t="n">
-        <v>0.1187</v>
+        <v>0.1183</v>
       </c>
     </row>
     <row r="36">
@@ -2260,47 +2260,47 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>14258.59</v>
+        <v>14220.13</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>-0.0014</v>
+        <v>-0.0027</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>-0.0112</v>
+        <v>-0.0138</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>-0.0177</v>
+        <v>-0.03240000000000001</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>-0.04480000000000001</v>
+        <v>-0.0281</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>0.0259</v>
+        <v>0.0407</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>0.0146</v>
+        <v>0.0119</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>0.0545</v>
+        <v>0.0516</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>0.073</v>
+        <v>0.0699</v>
       </c>
       <c r="L36" s="3" t="n">
-        <v>0.023</v>
+        <v>0.006</v>
       </c>
       <c r="M36" s="3" t="n">
-        <v>0.1432</v>
+        <v>0.1493</v>
       </c>
       <c r="N36" s="3" t="n">
-        <v>0.1249</v>
+        <v>0.1269</v>
       </c>
       <c r="O36" s="3" t="n">
-        <v>0.1407</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="37">
@@ -2311,47 +2311,47 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>75444.25</v>
+        <v>76231.60000000001</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>0.0092</v>
+        <v>0.0104</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>-0.0121</v>
+        <v>-0.0018</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>-0.04219999999999999</v>
+        <v>-0.0278</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>-0.0781</v>
+        <v>-0.0677</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>-0.0268</v>
+        <v>-0.0044</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>-0.1746</v>
+        <v>-0.166</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>0.0046</v>
+        <v>0.0151</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>-0.1881</v>
+        <v>-0.1586</v>
       </c>
       <c r="L37" s="3" t="n">
-        <v>-0.1489</v>
+        <v>-0.1504</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>-0.0295</v>
+        <v>-0.0243</v>
       </c>
       <c r="N37" s="3" t="n">
-        <v>0.039</v>
+        <v>0.0397</v>
       </c>
       <c r="O37" s="3" t="n">
-        <v>0.09</v>
+        <v>0.09390000000000001</v>
       </c>
     </row>
     <row r="38">
@@ -2362,47 +2362,47 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>5480.88</v>
+        <v>5432.3</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>-0.0031</v>
+        <v>-0.0089</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>0.0183</v>
+        <v>0.009300000000000001</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>-0.0073</v>
+        <v>-0.0236</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>-0.0901</v>
+        <v>-0.08410000000000001</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>0.0137</v>
+        <v>0.0263</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>0.0667</v>
+        <v>0.0572</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>0.0535</v>
+        <v>0.0442</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>0.0282</v>
+        <v>0.005500000000000001</v>
       </c>
       <c r="L38" s="3" t="n">
-        <v>-0.083</v>
+        <v>-0.1094</v>
       </c>
       <c r="M38" s="3" t="n">
-        <v>0.1376</v>
+        <v>0.137</v>
       </c>
       <c r="N38" s="3" t="n">
-        <v>0.1426</v>
+        <v>0.1471</v>
       </c>
       <c r="O38" s="3" t="n">
-        <v>0.1221</v>
+        <v>0.1224</v>
       </c>
     </row>
     <row r="39">
@@ -2413,47 +2413,47 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>5950.87</v>
+        <v>5873.99</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>0.0027</v>
+        <v>-0.0129</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>-0.0309</v>
+        <v>-0.0434</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>-0.0322</v>
+        <v>-0.0486</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>-0.0012</v>
+        <v>-0.0127</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>0.06269999999999999</v>
+        <v>0.06280000000000001</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>-0.0522</v>
+        <v>-0.0644</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>0.103</v>
+        <v>0.08869999999999999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>-0.0269</v>
+        <v>-0.0181</v>
       </c>
       <c r="L39" s="3" t="n">
-        <v>-0.0132</v>
+        <v>-0.0278</v>
       </c>
       <c r="M39" s="3" t="n">
-        <v>0.0958</v>
+        <v>0.09789999999999999</v>
       </c>
       <c r="N39" s="3" t="n">
-        <v>0.0731</v>
+        <v>0.0672</v>
       </c>
       <c r="O39" s="3" t="n">
-        <v>0.1303</v>
+        <v>0.129</v>
       </c>
     </row>
     <row r="40">
@@ -2464,47 +2464,47 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>16854.44</v>
+        <v>16721.19</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>0.0011</v>
+        <v>-0.007900000000000001</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>-0.013</v>
+        <v>-0.0208</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>-0.0195</v>
+        <v>-0.0248</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>-0.0178</v>
+        <v>-0.0233</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>-0.0039</v>
+        <v>0.0069</v>
       </c>
       <c r="I40" s="3" t="n">
-        <v>-0.0993</v>
+        <v>-0.1064</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>0.0189</v>
+        <v>0.0108</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>-0.0229</v>
+        <v>-0.0243</v>
       </c>
       <c r="L40" s="3" t="n">
-        <v>-0.0583</v>
+        <v>-0.06950000000000001</v>
       </c>
       <c r="M40" s="3" t="n">
-        <v>0.1188</v>
+        <v>0.1231</v>
       </c>
       <c r="N40" s="3" t="n">
-        <v>0.09329999999999999</v>
+        <v>0.08929999999999999</v>
       </c>
       <c r="O40" s="3" t="n">
-        <v>0.1424</v>
+        <v>0.1397</v>
       </c>
     </row>
     <row r="41">
@@ -2515,47 +2515,47 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>66882.39999999999</v>
+        <v>66292.66</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>-0.0043</v>
+        <v>-0.008800000000000001</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>-0.0022</v>
+        <v>-0.011</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>-0.0067</v>
+        <v>-0.0149</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>-0.0636</v>
+        <v>-0.0507</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>0.0583</v>
+        <v>0.0696</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>0.07980000000000001</v>
+        <v>0.0703</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>0.09039999999999999</v>
+        <v>0.0808</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>0.07820000000000001</v>
+        <v>0.07429999999999999</v>
       </c>
       <c r="L41" s="3" t="n">
-        <v>-0.0429</v>
+        <v>-0.0658</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>0.1262</v>
+        <v>0.1286</v>
       </c>
       <c r="N41" s="3" t="n">
-        <v>0.1371</v>
+        <v>0.1322</v>
       </c>
       <c r="O41" s="3" t="n">
-        <v>0.1684</v>
+        <v>0.1657</v>
       </c>
     </row>
     <row r="42">
@@ -2566,47 +2566,47 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>41671.52</v>
+        <v>40669.75</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>-0.0023</v>
+        <v>-0.024</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>-0.07490000000000001</v>
+        <v>-0.09720000000000001</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>-0.0519</v>
+        <v>-0.0712</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>0.0555</v>
+        <v>0.0337</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>-0.0031</v>
+        <v>-0.0384</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>-0.2279</v>
+        <v>-0.2465</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>0.0016</v>
+        <v>-0.0225</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>-0.198</v>
+        <v>-0.1674</v>
       </c>
       <c r="L42" s="3" t="n">
-        <v>-0.1539</v>
+        <v>-0.1629</v>
       </c>
       <c r="M42" s="3" t="n">
-        <v>-0.0245</v>
+        <v>-0.0259</v>
       </c>
       <c r="N42" s="3" t="n">
-        <v>-0.0218</v>
+        <v>-0.0343</v>
       </c>
       <c r="O42" s="3" t="n">
-        <v>0.1298</v>
+        <v>0.1273</v>
       </c>
     </row>
     <row r="43">
@@ -2617,47 +2617,47 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>7650.5</v>
+        <v>7743.41</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>-0.0008</v>
+        <v>0.0121</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>-0.0046</v>
+        <v>0.0075</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>-0.0075</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>0.02</v>
+        <v>0.0529</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>0.1758</v>
+        <v>0.2158</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>0.1176</v>
+        <v>0.1312</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>0.1719</v>
+        <v>0.1861</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>0.1536</v>
+        <v>0.1724</v>
       </c>
       <c r="L43" s="3" t="n">
-        <v>0.1671</v>
+        <v>0.1634</v>
       </c>
       <c r="M43" s="3" t="n">
-        <v>0.1987</v>
+        <v>0.2193</v>
       </c>
       <c r="N43" s="3" t="n">
-        <v>0.1153</v>
+        <v>0.1168</v>
       </c>
       <c r="O43" s="3" t="n">
-        <v>0.136</v>
+        <v>0.1363</v>
       </c>
     </row>
     <row r="44">
@@ -2668,47 +2668,47 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>29644.17</v>
+        <v>30608.13</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>0.009399999999999999</v>
+        <v>0.0325</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>0.0064</v>
+        <v>0.0391</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>0.0074</v>
+        <v>0.0473</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>-0.0251</v>
+        <v>0.0512</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>0.2404</v>
+        <v>0.3232</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>0.174</v>
+        <v>0.2122</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>0.2487</v>
+        <v>0.2893</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>0.2122</v>
+        <v>0.2546</v>
       </c>
       <c r="L44" s="3" t="n">
         <v>0.2381</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>0.2498</v>
+        <v>0.2817</v>
       </c>
       <c r="N44" s="3" t="n">
-        <v>0.1409</v>
+        <v>0.1482</v>
       </c>
       <c r="O44" s="3" t="n">
-        <v>0.1997</v>
+        <v>0.202</v>
       </c>
     </row>
     <row r="45">
@@ -2719,47 +2719,47 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
-        <v>65018.95</v>
+        <v>66364.2</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>0.0157</v>
+        <v>0.0207</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>-0.0195</v>
+        <v>0.0008</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>-0.004699999999999999</v>
+        <v>0.0015</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>-0.08749999999999999</v>
+        <v>-0.0432</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>0.2182</v>
+        <v>0.2434</v>
       </c>
       <c r="I45" s="3" t="n">
-        <v>0.2916</v>
+        <v>0.3183</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>0.2733</v>
+        <v>0.2996</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>0.4352</v>
+        <v>0.4504</v>
       </c>
       <c r="L45" s="3" t="n">
-        <v>0.3371</v>
+        <v>0.324</v>
       </c>
       <c r="M45" s="3" t="n">
-        <v>0.2508</v>
+        <v>0.2713</v>
       </c>
       <c r="N45" s="3" t="n">
-        <v>0.1634</v>
+        <v>0.1701</v>
       </c>
       <c r="O45" s="3" t="n">
-        <v>0.1471</v>
+        <v>0.1482</v>
       </c>
     </row>
     <row r="46">
@@ -2770,47 +2770,47 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>25304.06</v>
+        <v>25408.64</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>-0.0103</v>
+        <v>0.004099999999999999</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>-0.0363</v>
+        <v>-0.03240000000000001</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>-0.0302</v>
+        <v>-0.0334</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>0.0127</v>
+        <v>0.0299</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>0.1306</v>
+        <v>0.1394</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>0.0332</v>
+        <v>0.0375</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>0.1157</v>
+        <v>0.1203</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>0.0688</v>
+        <v>0.0796</v>
       </c>
       <c r="L46" s="3" t="n">
-        <v>0.163</v>
+        <v>0.159</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>0.1735</v>
+        <v>0.1855</v>
       </c>
       <c r="N46" s="3" t="n">
-        <v>0.1031</v>
+        <v>0.1034</v>
       </c>
       <c r="O46" s="3" t="n">
-        <v>0.0931</v>
+        <v>0.09390000000000001</v>
       </c>
     </row>
     <row r="47">
@@ -2821,47 +2821,47 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>8065.02</v>
+        <v>8077.8</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>-0.014</v>
+        <v>0.0016</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>-0.0323</v>
+        <v>-0.0308</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>-0.05139999999999999</v>
+        <v>-0.0454</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>-0.0423</v>
+        <v>-0.0366</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>0.0521</v>
+        <v>0.0488</v>
       </c>
       <c r="I47" s="3" t="n">
-        <v>-0.0104</v>
+        <v>-0.008800000000000001</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>0.0317</v>
+        <v>0.0334</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>0.0268</v>
+        <v>0.0362</v>
       </c>
       <c r="L47" s="3" t="n">
-        <v>0.0408</v>
+        <v>0.0333</v>
       </c>
       <c r="M47" s="3" t="n">
-        <v>0.0346</v>
+        <v>0.0453</v>
       </c>
       <c r="N47" s="3" t="n">
-        <v>0.0418</v>
+        <v>0.04</v>
       </c>
       <c r="O47" s="3" t="n">
-        <v>0.06280000000000001</v>
+        <v>0.06269999999999999</v>
       </c>
     </row>
     <row r="48">
@@ -2872,47 +2872,47 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>10659.13</v>
+        <v>10695.3</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>0.0008</v>
+        <v>0.0034</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>-0.0153</v>
+        <v>-0.0119</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>-0.007800000000000001</v>
+        <v>-0.0168</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>0.0285</v>
+        <v>0.0178</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>0.0747</v>
+        <v>0.073</v>
       </c>
       <c r="I48" s="3" t="n">
-        <v>0.0733</v>
+        <v>0.07690000000000001</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>0.0474</v>
+        <v>0.051</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>0.1551</v>
+        <v>0.1608</v>
       </c>
       <c r="L48" s="3" t="n">
-        <v>0.1365</v>
+        <v>0.1374</v>
       </c>
       <c r="M48" s="3" t="n">
-        <v>0.1165</v>
+        <v>0.1194</v>
       </c>
       <c r="N48" s="3" t="n">
-        <v>0.0888</v>
+        <v>0.0868</v>
       </c>
       <c r="O48" s="3" t="n">
-        <v>0.0455</v>
+        <v>0.0462</v>
       </c>
     </row>
     <row r="49">
@@ -2923,47 +2923,47 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>24750.78</v>
+        <v>24510.09</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>-0.0022</v>
+        <v>-0.0097</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>-0.0319</v>
+        <v>-0.0413</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>-0.0292</v>
+        <v>-0.0446</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>0.0345</v>
+        <v>0.08109999999999999</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>-0.0208</v>
+        <v>-0.0177</v>
       </c>
       <c r="I49" s="3" t="n">
-        <v>-0.0343</v>
+        <v>-0.0437</v>
       </c>
       <c r="J49" s="3" t="n">
-        <v>-0.0015</v>
+        <v>-0.0112</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>-0.06759999999999999</v>
+        <v>-0.0746</v>
       </c>
       <c r="L49" s="3" t="n">
-        <v>0.1837</v>
+        <v>0.132</v>
       </c>
       <c r="M49" s="3" t="n">
-        <v>0.1121</v>
+        <v>0.1196</v>
       </c>
       <c r="N49" s="3" t="n">
-        <v>-0.0014</v>
+        <v>0.0026</v>
       </c>
       <c r="O49" s="3" t="n">
-        <v>0.0051</v>
+        <v>0.0039</v>
       </c>
     </row>
     <row r="50">
@@ -2974,47 +2974,47 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>4507.39</v>
+        <v>4439.14</v>
       </c>
       <c r="D50" s="3" t="n">
-        <v>-0.0005999999999999999</v>
+        <v>-0.004699999999999999</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>-0.0254</v>
+        <v>-0.04019999999999999</v>
       </c>
       <c r="F50" s="3" t="n">
-        <v>-0.0177</v>
+        <v>-0.0248</v>
       </c>
       <c r="G50" s="3" t="n">
-        <v>-0.08789999999999999</v>
+        <v>-0.1157</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>-0.0131</v>
+        <v>-0.0086</v>
       </c>
       <c r="I50" s="3" t="n">
-        <v>-0.0265</v>
+        <v>-0.0412</v>
       </c>
       <c r="J50" s="3" t="n">
-        <v>0.0129</v>
+        <v>-0.0025</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>0.0021</v>
+        <v>-0.0278</v>
       </c>
       <c r="L50" s="3" t="n">
-        <v>0.1924</v>
+        <v>0.1509</v>
       </c>
       <c r="M50" s="3" t="n">
-        <v>0.06610000000000001</v>
+        <v>0.0612</v>
       </c>
       <c r="N50" s="3" t="n">
-        <v>-0.0148</v>
+        <v>-0.0175</v>
       </c>
       <c r="O50" s="3" t="n">
-        <v>0.033</v>
+        <v>0.0326</v>
       </c>
     </row>
     <row r="51">
@@ -3025,47 +3025,47 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>95.88</v>
+        <v>95.81999999999999</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>0.0019</v>
+        <v>-0.0005999999999999999</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>0.0052</v>
+        <v>0.0046</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>0.0011</v>
+        <v>0.0037</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>0.0163</v>
+        <v>0.015</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>0.0301</v>
+        <v>0.016</v>
       </c>
       <c r="I51" s="3" t="n">
-        <v>0.06809999999999999</v>
+        <v>0.0674</v>
       </c>
       <c r="J51" s="3" t="n">
-        <v>0.0162</v>
+        <v>0.0155</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.0794</v>
       </c>
       <c r="L51" s="3" t="n">
-        <v>0.0709</v>
+        <v>0.07049999999999999</v>
       </c>
       <c r="M51" s="3" t="n">
-        <v>0.0489</v>
+        <v>0.0481</v>
       </c>
       <c r="N51" s="3" t="n">
-        <v>0.0542</v>
+        <v>0.0536</v>
       </c>
       <c r="O51" s="3" t="n">
-        <v>0.0369</v>
+        <v>0.0375</v>
       </c>
     </row>
     <row r="52">
@@ -3076,47 +3076,47 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>4424.9</v>
+        <v>4321.2</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>0.0036</v>
+        <v>-0.0234</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>-0.0014</v>
+        <v>-0.0248</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>-0.0144</v>
+        <v>-0.0602</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>0.0475</v>
+        <v>0.0595</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>-0.0318</v>
+        <v>-0.038</v>
       </c>
       <c r="I52" s="3" t="n">
-        <v>0.023</v>
+        <v>-0.001</v>
       </c>
       <c r="J52" s="3" t="n">
-        <v>-0.0479</v>
+        <v>-0.0702</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>0.2144</v>
+        <v>0.1564</v>
       </c>
       <c r="L52" s="3" t="n">
-        <v>0.3122</v>
+        <v>0.275</v>
       </c>
       <c r="M52" s="3" t="n">
-        <v>0.3184</v>
+        <v>0.3152</v>
       </c>
       <c r="N52" s="3" t="n">
-        <v>0.2038</v>
+        <v>0.1981</v>
       </c>
       <c r="O52" s="3" t="n">
-        <v>0.1292</v>
+        <v>0.1255</v>
       </c>
     </row>
     <row r="53">
@@ -3127,47 +3127,47 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>67.15000000000001</v>
+        <v>64.8</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>0.04019999999999999</v>
+        <v>-0.035</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>0.014</v>
+        <v>-0.0214</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>0.0215</v>
+        <v>-0.0469</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>0.0135</v>
+        <v>0.09429999999999999</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>-0.0319</v>
+        <v>-0.0682</v>
       </c>
       <c r="I53" s="3" t="n">
-        <v>-0.0426</v>
+        <v>-0.076</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>-0.101</v>
+        <v>-0.1324</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>0.61</v>
+        <v>0.4498</v>
       </c>
       <c r="L53" s="3" t="n">
-        <v>0.4881</v>
+        <v>0.4301</v>
       </c>
       <c r="M53" s="3" t="n">
-        <v>0.4256</v>
+        <v>0.4137</v>
       </c>
       <c r="N53" s="3" t="n">
-        <v>0.2466</v>
+        <v>0.2367</v>
       </c>
       <c r="O53" s="3" t="n">
-        <v>0.1335</v>
+        <v>0.1301</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Weekly indices update 2026-10-01
</commit_message>
<xml_diff>
--- a/tracker_auto.xlsx
+++ b/tracker_auto.xlsx
@@ -524,47 +524,47 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>23140.5</v>
+        <v>22620.45</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>-0.008800000000000001</v>
+        <v>-0.0352</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-0.039</v>
+        <v>-0.06059999999999999</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>-0.0441</v>
+        <v>-0.06059999999999999</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>-0.0381</v>
+        <v>-0.05769999999999999</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>0.0141</v>
+        <v>-0.0026</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>-0.1144</v>
+        <v>-0.1343</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.0362</v>
+        <v>0.0129</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>-0.0703</v>
+        <v>-0.0809</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>-0.0567</v>
+        <v>-0.0639</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>0.0558</v>
+        <v>0.0482</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>0.0532</v>
+        <v>0.05230000000000001</v>
       </c>
       <c r="O2" s="3" t="n">
-        <v>0.1028</v>
+        <v>0.1014</v>
       </c>
     </row>
     <row r="3">
@@ -575,47 +575,47 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>73895.74000000001</v>
+        <v>71748.7</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>-0.0054</v>
+        <v>-0.0249</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>-0.0398</v>
+        <v>-0.0101</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>-0.0462</v>
+        <v>-0.0675</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>-0.0416</v>
+        <v>-0.0742</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>0.0042</v>
+        <v>-0.0214</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>-0.1329</v>
+        <v>-0.1581</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>0.0271</v>
+        <v>-0.0028</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>-0.0895</v>
+        <v>-0.114</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>-0.06860000000000001</v>
+        <v>-0.07730000000000001</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>0.0387</v>
+        <v>0.0291</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>0.0424</v>
+        <v>0.0407</v>
       </c>
       <c r="O3" s="3" t="n">
-        <v>0.1011</v>
+        <v>0.0978</v>
       </c>
     </row>
     <row r="4">
@@ -626,47 +626,47 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>71778.64999999999</v>
+        <v>69746.95</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>-0.0034</v>
+        <v>-0.0375</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>-0.0269</v>
+        <v>-0.0544</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>-0.0365</v>
+        <v>-0.0544</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>-0.0058</v>
+        <v>-0.0326</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.1569</v>
+        <v>0.1265</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.0348</v>
+        <v>0.005500000000000001</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.1894</v>
+        <v>0.1557</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>0.051</v>
+        <v>0.028</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>-0.0315</v>
+        <v>-0.0489</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>0.1672</v>
+        <v>0.1568</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>0.1075</v>
+        <v>0.1042</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>0.1199</v>
+        <v>0.1178</v>
       </c>
     </row>
     <row r="5">
@@ -677,47 +677,47 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>24307.55</v>
+        <v>23734.7</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>-0.007800000000000001</v>
+        <v>-0.0357</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>-0.0368</v>
+        <v>-0.0595</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>-0.04269999999999999</v>
+        <v>-0.0595</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>-0.0321</v>
+        <v>-0.05309999999999999</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>0.0388</v>
+        <v>0.0198</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>-0.0892</v>
+        <v>-0.1107</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0.0626</v>
+        <v>0.03759999999999999</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>-0.0491</v>
+        <v>-0.0617</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>-0.0521</v>
+        <v>-0.0605</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>0.07429999999999999</v>
+        <v>0.06619999999999999</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>0.0608</v>
+        <v>0.0595</v>
       </c>
       <c r="O5" s="3" t="n">
-        <v>0.1053</v>
+        <v>0.1038</v>
       </c>
     </row>
     <row r="6">
@@ -728,47 +728,47 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>31685.3</v>
+        <v>30904.45</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>-0.008100000000000001</v>
+        <v>-0.0383</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-0.0393</v>
+        <v>-0.063</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-0.04190000000000001</v>
+        <v>-0.063</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>-0.0273</v>
+        <v>-0.0507</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.0506</v>
+        <v>0.03</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>-0.04940000000000001</v>
+        <v>-0.0728</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.07200000000000001</v>
+        <v>0.04559999999999999</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>-0.007800000000000001</v>
+        <v>-0.0206</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>-0.0232</v>
+        <v>-0.0374</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>0.1035</v>
+        <v>0.09449999999999999</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>0.0987</v>
+        <v>0.09429999999999999</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>0.1132</v>
+        <v>0.1113</v>
       </c>
     </row>
     <row r="7">
@@ -779,47 +779,47 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>33776.85</v>
+        <v>32860.75</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>-0.005600000000000001</v>
+        <v>-0.0379</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-0.0348</v>
+        <v>-0.061</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>-0.04219999999999999</v>
+        <v>-0.061</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>-0.0166</v>
+        <v>-0.0425</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.1062</v>
+        <v>0.08019999999999999</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>-0.0053</v>
+        <v>-0.0322</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>0.1339</v>
+        <v>0.1032</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>0.0192</v>
+        <v>0.0015</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>-0.0218</v>
+        <v>-0.0365</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>0.1332</v>
+        <v>0.1233</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>0.0998</v>
+        <v>0.0956</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>0.1127</v>
+        <v>0.1107</v>
       </c>
     </row>
     <row r="8">
@@ -830,47 +830,47 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>18160.19</v>
+        <v>17724.2</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>-0.0104</v>
+        <v>-0.0384</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-0.0396</v>
+        <v>-0.0626</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-0.0438</v>
+        <v>-0.0626</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>-0.0255</v>
+        <v>-0.0482</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.0622</v>
+        <v>0.0423</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>-0.0638</v>
+        <v>-0.0863</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.08749999999999999</v>
+        <v>0.0614</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>-0.02</v>
+        <v>-0.0323</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>-0.032</v>
+        <v>-0.0409</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>0.0978</v>
+        <v>0.08890000000000001</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>0.0859</v>
+        <v>0.0837</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>0.1249</v>
+        <v>0.1233</v>
       </c>
     </row>
     <row r="9">
@@ -881,47 +881,47 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>16153.55</v>
+        <v>15757.7</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>-0.0142</v>
+        <v>-0.0411</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-0.0418</v>
+        <v>-0.0653</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-0.0446</v>
+        <v>-0.0653</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>-0.0229</v>
+        <v>-0.0475</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>0.0814</v>
+        <v>0.06</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>-0.0416</v>
+        <v>-0.06509999999999999</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>0.1083</v>
+        <v>0.08119999999999999</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>-0.0004</v>
+        <v>-0.0118</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>-0.0246</v>
+        <v>-0.0347</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>0.1089</v>
+        <v>0.0987</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>0.1043</v>
+        <v>0.1001</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>0.1331</v>
+        <v>0.1311</v>
       </c>
     </row>
     <row r="10">
@@ -932,47 +932,47 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>22437</v>
+        <v>21867.5</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>-0.0203</v>
+        <v>-0.0463</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>-0.0467</v>
+        <v>-0.0709</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>-0.04650000000000001</v>
+        <v>-0.0709</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>-0.0138</v>
+        <v>-0.04190000000000001</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.1245</v>
+        <v>0.1006</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>0.0072</v>
+        <v>-0.0184</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.1547</v>
+        <v>0.1254</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>0.04940000000000001</v>
+        <v>0.0394</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>0.0018</v>
+        <v>-0.01</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>0.1426</v>
+        <v>0.1302</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0.1471</v>
+        <v>0.1398</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>0.1592</v>
+        <v>0.1567</v>
       </c>
     </row>
     <row r="11">
@@ -983,47 +983,47 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>18158.9</v>
+        <v>17798.8</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>-0.006999999999999999</v>
+        <v>-0.0333</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>-0.0116</v>
+        <v>-0.0312</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>-0.0161</v>
+        <v>-0.0312</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>0.0257</v>
+        <v>-0.0002</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0.2391</v>
+        <v>0.2068</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>0.08839999999999999</v>
+        <v>0.0668</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>0.2709</v>
+        <v>0.2457</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>0.06509999999999999</v>
+        <v>0.0663</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>-0.0098</v>
+        <v>-0.0168</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>0.145</v>
+        <v>0.1331</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>0.143</v>
+        <v>0.1365</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>0.138</v>
+        <v>0.1371</v>
       </c>
     </row>
     <row r="12">
@@ -1034,47 +1034,47 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>20904.95</v>
+        <v>20415</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>-0.0157</v>
+        <v>-0.0418</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>-0.0348</v>
+        <v>-0.0574</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>-0.0361</v>
+        <v>-0.0574</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>-0.0004</v>
+        <v>-0.0276</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.1621</v>
+        <v>0.1357</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>0.034</v>
+        <v>0.0098</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0.1929</v>
+        <v>0.165</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>0.05400000000000001</v>
+        <v>0.0479</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>-0.0028</v>
+        <v>-0.0129</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0.143</v>
+        <v>0.1308</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.1459</v>
+        <v>0.1389</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>0.1522</v>
+        <v>0.1502</v>
       </c>
     </row>
     <row r="13">
@@ -1085,47 +1085,47 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>22603.5</v>
+        <v>22072.1</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>-0.0104</v>
+        <v>-0.03759999999999999</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>-0.0361</v>
+        <v>-0.0588</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>-0.0406</v>
+        <v>-0.0588</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>-0.0221</v>
+        <v>-0.045</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>0.07530000000000001</v>
+        <v>0.05429999999999999</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>-0.05309999999999999</v>
+        <v>-0.07539999999999999</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>0.1011</v>
+        <v>0.07519999999999999</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>-0.0182</v>
+        <v>-0.0291</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>-0.03700000000000001</v>
+        <v>-0.0459</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>0.09380000000000001</v>
+        <v>0.08460000000000001</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>0.0827</v>
+        <v>0.08019999999999999</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>0.1172</v>
+        <v>0.1156</v>
       </c>
     </row>
     <row r="14">
@@ -1136,47 +1136,47 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>35353.29</v>
+        <v>34564.37</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>-0.0076</v>
+        <v>-0.0364</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>-0.0345</v>
+        <v>-0.05599999999999999</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>-0.0417</v>
+        <v>-0.05599999999999999</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>-0.0216</v>
+        <v>-0.043</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0.07339999999999999</v>
+        <v>0.0533</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>-0.0558</v>
+        <v>-0.07690000000000001</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>0.09849999999999999</v>
+        <v>0.07400000000000001</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>-0.0222</v>
+        <v>-0.0322</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>-0.0407</v>
+        <v>-0.0492</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0.0891</v>
+        <v>0.0803</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>0.0791</v>
+        <v>0.07690000000000001</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>0.1159</v>
+        <v>0.1144</v>
       </c>
     </row>
     <row r="15">
@@ -1187,47 +1187,47 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>19257.7</v>
+        <v>18785.65</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>-0.0053</v>
+        <v>-0.0342</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>-0.04769999999999999</v>
+        <v>-0.07099999999999999</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>-0.0463</v>
+        <v>-0.07099999999999999</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>-0.0284</v>
+        <v>-0.0518</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>0.0299</v>
+        <v>0.0167</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>-0.0886</v>
+        <v>-0.111</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>0.0519</v>
+        <v>0.0261</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>-0.0462</v>
+        <v>-0.057</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>-0.0533</v>
+        <v>-0.0638</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>0.08470000000000001</v>
+        <v>0.077</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>0.0699</v>
+        <v>0.0665</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>0.1081</v>
+        <v>0.1071</v>
       </c>
     </row>
     <row r="16">
@@ -1238,47 +1238,47 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>5443.15</v>
+        <v>5320.35</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>-0.0002</v>
+        <v>-0.0296</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>-0.0484</v>
+        <v>-0.0698</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>-0.0454</v>
+        <v>-0.0698</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>0.0017</v>
+        <v>-0.0178</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>0.06269999999999999</v>
+        <v>0.0363</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>-0.0711</v>
+        <v>-0.09210000000000002</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>0.0815</v>
+        <v>0.0571</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>-0.0346</v>
+        <v>-0.0444</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>-0.0665</v>
+        <v>-0.07870000000000001</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0.06660000000000001</v>
+        <v>0.0626</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>0.0578</v>
+        <v>0.0581</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>0.0935</v>
+        <v>0.09230000000000001</v>
       </c>
     </row>
     <row r="17">
@@ -1289,47 +1289,47 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>25572.12</v>
+        <v>24908.38</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>-0.0034</v>
+        <v>-0.038</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>-0.02</v>
+        <v>-0.0455</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>-0.0298</v>
+        <v>-0.0455</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>-0.0413</v>
+        <v>-0.0625</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>0.0221</v>
+        <v>-0.0063</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>-0.0022</v>
+        <v>-0.0281</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>0.04019999999999999</v>
+        <v>0.0132</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>0.1164</v>
+        <v>0.0789</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>0.0332</v>
+        <v>0.0048</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>0.2301</v>
+        <v>0.212</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>0.2456</v>
+        <v>0.2281</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>0.1671</v>
+        <v>0.1644</v>
       </c>
     </row>
     <row r="18">
@@ -1340,47 +1340,47 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>38030.13</v>
+        <v>37144.93</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>-0.006500000000000001</v>
+        <v>-0.0371</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>-0.0353</v>
+        <v>-0.0578</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>-0.0365</v>
+        <v>-0.0578</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>-0.0281</v>
+        <v>-0.0418</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>0.08710000000000001</v>
+        <v>0.0683</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>-0.0237</v>
+        <v>-0.04650000000000001</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>0.122</v>
+        <v>0.0959</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>0.0033</v>
+        <v>-0.004699999999999999</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>-0.096</v>
+        <v>-0.1079</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>0.1053</v>
+        <v>0.092</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>0.0968</v>
+        <v>0.09329999999999999</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>0.1611</v>
+        <v>0.1599</v>
       </c>
     </row>
     <row r="19">
@@ -1391,47 +1391,47 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>28178.09</v>
+        <v>27438.11</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>-0.005500000000000001</v>
+        <v>-0.0325</v>
       </c>
       <c r="E19" s="3" t="n">
+        <v>-0.079</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>-0.079</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>-0.0325</v>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>0.0253</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>-0.104</v>
+      </c>
+      <c r="J19" s="3" t="n">
+        <v>0.04969999999999999</v>
+      </c>
+      <c r="K19" s="3" t="n">
         <v>-0.0542</v>
       </c>
-      <c r="F19" s="3" t="n">
-        <v>-0.05139999999999999</v>
-      </c>
-      <c r="G19" s="3" t="n">
-        <v>-0.0113</v>
-      </c>
-      <c r="H19" s="3" t="n">
-        <v>0.0566</v>
-      </c>
-      <c r="I19" s="3" t="n">
-        <v>-0.07980000000000001</v>
-      </c>
-      <c r="J19" s="3" t="n">
-        <v>0.078</v>
-      </c>
-      <c r="K19" s="3" t="n">
-        <v>-0.0437</v>
-      </c>
       <c r="L19" s="3" t="n">
-        <v>-0.0701</v>
+        <v>-0.0843</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>0.07200000000000001</v>
+        <v>0.0664</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>0.06309999999999999</v>
+        <v>0.0638</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>0.1179</v>
+        <v>0.1167</v>
       </c>
     </row>
     <row r="20">
@@ -1442,47 +1442,47 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>30229</v>
+        <v>29518.95</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>-0.006500000000000001</v>
+        <v>-0.0373</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>-0.0358</v>
+        <v>-0.0585</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>-0.0371</v>
+        <v>-0.0585</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>-0.0306</v>
+        <v>-0.0445</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>0.0818</v>
+        <v>0.063</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>-0.0295</v>
+        <v>-0.05230000000000001</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>0.1166</v>
+        <v>0.09039999999999999</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>-0.0028</v>
+        <v>-0.0109</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>-0.102</v>
+        <v>-0.1139</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>0.09630000000000001</v>
+        <v>0.083</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>0.0872</v>
+        <v>0.0837</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>0.15</v>
+        <v>0.1488</v>
       </c>
     </row>
     <row r="21">
@@ -1493,47 +1493,47 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>55024.65</v>
+        <v>54079.15</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>-0.0208</v>
+        <v>-0.0333</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>-0.0437</v>
+        <v>-0.0601</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>-0.0437</v>
+        <v>-0.0601</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>0.0275</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>0.199</v>
+        <v>0.1813</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>0.09369999999999999</v>
+        <v>0.07490000000000001</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>0.2368</v>
+        <v>0.2156</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>0.09080000000000001</v>
+        <v>0.1099</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>-0.049</v>
+        <v>-0.0539</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>0.1522</v>
+        <v>0.1399</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>0.1162</v>
+        <v>0.1134</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>0.1899</v>
+        <v>0.1904</v>
       </c>
     </row>
     <row r="22">
@@ -1544,47 +1544,47 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>25992.5</v>
+        <v>25219.5</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>-0.004500000000000001</v>
+        <v>-0.0408</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>-0.0438</v>
+        <v>-0.0722</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>-0.0432</v>
+        <v>-0.0722</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>-0.017</v>
+        <v>-0.0476</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>0.05690000000000001</v>
+        <v>0.0438</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>-0.0401</v>
+        <v>-0.06860000000000001</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>0.0848</v>
+        <v>0.0525</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>-0.012</v>
+        <v>-0.0283</v>
       </c>
       <c r="L22" s="3" t="n">
-        <v>-0.08560000000000001</v>
+        <v>-0.0999</v>
       </c>
       <c r="M22" s="3" t="n">
-        <v>0.09470000000000001</v>
+        <v>0.0819</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>0.07429999999999999</v>
+        <v>0.0742</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>0.1166</v>
+        <v>0.1147</v>
       </c>
     </row>
     <row r="23">
@@ -1595,44 +1595,44 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>10420.47</v>
+        <v>10282</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>0.005500000000000001</v>
+        <v>-0.0195</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>-0.0323</v>
+        <v>-0.0452</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>-0.0349</v>
+        <v>-0.0452</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>0.0023</v>
+        <v>-0.0275</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>0.2688</v>
+        <v>0.2231</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>0.2194</v>
+        <v>0.2032</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>0.3054</v>
+        <v>0.2881</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>0.1618</v>
+        <v>0.1879</v>
       </c>
       <c r="L23" s="3" t="n">
-        <v>0.1906</v>
+        <v>0.1871</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>0.4316</v>
+        <v>0.423</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>0.5193</v>
+        <v>0.5108</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -1648,47 +1648,47 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>11386.9</v>
+        <v>11004.65</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>-0.0028</v>
+        <v>-0.0418</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>-0.0366</v>
+        <v>-0.0689</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>-0.0433</v>
+        <v>-0.0689</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>-0.0395</v>
+        <v>-0.0653</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>0.0123</v>
+        <v>-0.0115</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>-0.0208</v>
+        <v>-0.0536</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>0.0607</v>
+        <v>0.0251</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>0.1303</v>
+        <v>0.073</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>0.1176</v>
+        <v>0.09699999999999999</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>0.1776</v>
+        <v>0.1589</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>0.2993</v>
+        <v>0.2757</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>0.1099</v>
+        <v>0.1054</v>
       </c>
     </row>
     <row r="25">
@@ -1699,47 +1699,47 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>78018.91</v>
+        <v>76689.05</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>-0.0138</v>
+        <v>-0.0339</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>-0.0421</v>
+        <v>-0.0585</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>-0.0381</v>
+        <v>-0.0585</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>-0.0428</v>
+        <v>-0.0568</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>0.0702</v>
+        <v>0.0689</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>-0.061</v>
+        <v>-0.077</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>0.1128</v>
+        <v>0.09380000000000001</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>0.0176</v>
+        <v>0.006500000000000001</v>
       </c>
       <c r="L25" s="3" t="n">
-        <v>0.0209</v>
+        <v>0.0229</v>
       </c>
       <c r="M25" s="3" t="n">
-        <v>0.08439999999999999</v>
+        <v>0.0784</v>
       </c>
       <c r="N25" s="3" t="n">
-        <v>0.0886</v>
+        <v>0.08839999999999999</v>
       </c>
       <c r="O25" s="3" t="n">
-        <v>0.1169</v>
+        <v>0.1163</v>
       </c>
     </row>
     <row r="26">
@@ -1750,47 +1750,47 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>31822.57</v>
+        <v>31600.55</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>-0.0149</v>
+        <v>-0.0244</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>-0.0401</v>
+        <v>-0.04679999999999999</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>-0.0306</v>
+        <v>-0.04679999999999999</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>-0.0482</v>
+        <v>-0.05</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>0.0824</v>
+        <v>0.0931</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>-0.0584</v>
+        <v>-0.0649</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>0.1201</v>
+        <v>0.1123</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.0149</v>
       </c>
       <c r="L26" s="3" t="n">
-        <v>0.0012</v>
+        <v>0.0095</v>
       </c>
       <c r="M26" s="3" t="n">
-        <v>0.059</v>
+        <v>0.0561</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>0.0698</v>
+        <v>0.0738</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>0.1003</v>
+        <v>0.1011</v>
       </c>
     </row>
     <row r="27">
@@ -1801,47 +1801,47 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>32111.44</v>
+        <v>31541.58</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>-0.0163</v>
+        <v>-0.0358</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>-0.04559999999999999</v>
+        <v>-0.0625</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>-0.0488</v>
+        <v>-0.0625</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>-0.0597</v>
+        <v>-0.07780000000000001</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>0.0378</v>
+        <v>0.036</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>-0.0833</v>
+        <v>-0.09960000000000001</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>0.07530000000000001</v>
+        <v>0.0563</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>-0.0352</v>
+        <v>-0.0442</v>
       </c>
       <c r="L27" s="3" t="n">
-        <v>0.0117</v>
+        <v>0.013</v>
       </c>
       <c r="M27" s="3" t="n">
-        <v>0.09279999999999999</v>
+        <v>0.0859</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>0.07139999999999999</v>
+        <v>0.07339999999999999</v>
       </c>
       <c r="O27" s="3" t="n">
-        <v>0.1287</v>
+        <v>0.1283</v>
       </c>
     </row>
     <row r="28">
@@ -1852,47 +1852,47 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>17342.45</v>
+        <v>16962.36</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>-0.0025</v>
+        <v>-0.0285</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>-0.0106</v>
+        <v>-0.0323</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>-0.0126</v>
+        <v>-0.0323</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>-0.0315</v>
+        <v>-0.05860000000000001</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>-0.0037</v>
+        <v>-0.0279</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>-0.0143</v>
+        <v>-0.0359</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>0.008500000000000001</v>
+        <v>-0.0136</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>-0.0023</v>
+        <v>-0.0263</v>
       </c>
       <c r="L28" s="3" t="n">
-        <v>-0.0526</v>
+        <v>-0.0703</v>
       </c>
       <c r="M28" s="3" t="n">
-        <v>0.2003</v>
+        <v>0.1839</v>
       </c>
       <c r="N28" s="3" t="n">
-        <v>0.2309</v>
+        <v>0.2088</v>
       </c>
       <c r="O28" s="3" t="n">
-        <v>0.1404</v>
+        <v>0.1384</v>
       </c>
     </row>
     <row r="29">
@@ -1903,47 +1903,47 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>968.98</v>
+        <v>944.48</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>0.0298</v>
+        <v>-0.0272</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>-0.0383</v>
+        <v>-0.0626</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>-0.0446</v>
+        <v>-0.0626</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>0.0567</v>
+        <v>-0.009599999999999999</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>0.303</v>
+        <v>0.2799</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>-0.0053</v>
+        <v>-0.0304</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>0.3411</v>
+        <v>0.3071</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>-0.0028</v>
+        <v>-0.0188</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>-0.1195</v>
+        <v>-0.1185</v>
       </c>
       <c r="M29" s="3" t="n">
-        <v>0.1541</v>
+        <v>0.1415</v>
       </c>
       <c r="N29" s="3" t="n">
-        <v>0.1203</v>
+        <v>0.1126</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>0.1596</v>
+        <v>0.1585</v>
       </c>
     </row>
     <row r="30">
@@ -1954,47 +1954,47 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>36098.42</v>
+        <v>35196.26</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>-0.0059</v>
+        <v>-0.0318</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>-0.065</v>
+        <v>-0.0883</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>-0.0701</v>
+        <v>-0.0883</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>0.005699999999999999</v>
+        <v>-0.0123</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>0.1174</v>
+        <v>0.09420000000000001</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>-0.0334</v>
+        <v>-0.0576</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>0.1444</v>
+        <v>0.1158</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>0.0185</v>
+        <v>0.0012</v>
       </c>
       <c r="L30" s="3" t="n">
-        <v>0.0115</v>
+        <v>-0.0038</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>0.1942</v>
+        <v>0.186</v>
       </c>
       <c r="N30" s="3" t="n">
-        <v>0.2203</v>
+        <v>0.2106</v>
       </c>
       <c r="O30" s="3" t="n">
-        <v>0.1161</v>
+        <v>0.1128</v>
       </c>
     </row>
     <row r="31">
@@ -2005,47 +2005,47 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>20860.87</v>
+        <v>20299.36</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>-0.003</v>
+        <v>-0.0352</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>-0.04219999999999999</v>
+        <v>-0.068</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>-0.0413</v>
+        <v>-0.068</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>0.0005999999999999999</v>
+        <v>-0.0242</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>0.1177</v>
+        <v>0.09039999999999999</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>0.0385</v>
+        <v>0.0106</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>0.1384</v>
+        <v>0.1077</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>0.0697</v>
+        <v>0.0548</v>
       </c>
       <c r="L31" s="3" t="n">
-        <v>0.0215</v>
+        <v>0.0026</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>0.1846</v>
+        <v>0.1721</v>
       </c>
       <c r="N31" s="3" t="n">
-        <v>0.162</v>
+        <v>0.1534</v>
       </c>
       <c r="O31" s="3" t="n">
-        <v>0.1382</v>
+        <v>0.136</v>
       </c>
     </row>
     <row r="32">
@@ -2056,47 +2056,47 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>11831.92</v>
+        <v>11536.67</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>-0.0126</v>
+        <v>-0.0397</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>-0.0236</v>
+        <v>-0.048</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>-0.0351</v>
+        <v>-0.048</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>-0.05</v>
+        <v>-0.07190000000000001</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>0.0333</v>
+        <v>0.0135</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>-0.0619</v>
+        <v>-0.08529999999999999</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>0.0525</v>
+        <v>0.0263</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>-0.0052</v>
+        <v>-0.0223</v>
       </c>
       <c r="L32" s="3" t="n">
-        <v>-0.0269</v>
+        <v>-0.0367</v>
       </c>
       <c r="M32" s="3" t="n">
-        <v>0.1414</v>
+        <v>0.1277</v>
       </c>
       <c r="N32" s="3" t="n">
-        <v>0.1347</v>
+        <v>0.128</v>
       </c>
       <c r="O32" s="3" t="n">
-        <v>0.1374</v>
+        <v>0.1357</v>
       </c>
     </row>
     <row r="33">
@@ -2107,47 +2107,47 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>19907.91</v>
+        <v>19262.36</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>0.0039</v>
+        <v>-0.0433</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>-0.0155</v>
+        <v>-0.0474</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>0.005600000000000001</v>
+        <v>-0.0474</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>0.047</v>
+        <v>0.0069</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>0.159</v>
+        <v>0.1516</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>0.1448</v>
+        <v>0.1077</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>0.178</v>
+        <v>0.1398</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>0.1597</v>
+        <v>0.147</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>0.07200000000000001</v>
+        <v>0.0517</v>
       </c>
       <c r="M33" s="3" t="n">
-        <v>0.2152</v>
+        <v>0.1906</v>
       </c>
       <c r="N33" s="3" t="n">
-        <v>0.1386</v>
+        <v>0.1304</v>
       </c>
       <c r="O33" s="3" t="n">
-        <v>0.1071</v>
+        <v>0.1065</v>
       </c>
     </row>
     <row r="34">
@@ -2158,47 +2158,47 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>19971.29</v>
+        <v>19480.28</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>0.0026</v>
+        <v>-0.0404</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>-0.007800000000000001</v>
+        <v>-0.0322</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>-0.0333</v>
+        <v>-0.0322</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>0.05400000000000001</v>
+        <v>0.0322</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>0.1804</v>
+        <v>0.1261</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>0.1831</v>
+        <v>0.1541</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>0.1828</v>
+        <v>0.1538</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>0.3111</v>
+        <v>0.2845</v>
       </c>
       <c r="L34" s="3" t="n">
-        <v>0.1679</v>
+        <v>0.1293</v>
       </c>
       <c r="M34" s="3" t="n">
-        <v>0.2555</v>
+        <v>0.2408</v>
       </c>
       <c r="N34" s="3" t="n">
-        <v>0.2041</v>
+        <v>0.1923</v>
       </c>
       <c r="O34" s="3" t="n">
-        <v>0.2014</v>
+        <v>0.1984</v>
       </c>
     </row>
     <row r="35">
@@ -2209,47 +2209,47 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>9858.870000000001</v>
+        <v>9640.370000000001</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>0.0005999999999999999</v>
+        <v>-0.0322</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>-0.0401</v>
+        <v>-0.0614</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>-0.0437</v>
+        <v>-0.0614</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>0.0317</v>
+        <v>-0.0019</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>0.1772</v>
+        <v>0.147</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>0</v>
+        <v>-0.0221</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>0.2057</v>
+        <v>0.179</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>-0.0145</v>
+        <v>-0.0194</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>-0.0527</v>
+        <v>-0.0617</v>
       </c>
       <c r="M35" s="3" t="n">
-        <v>0.1205</v>
+        <v>0.1139</v>
       </c>
       <c r="N35" s="3" t="n">
-        <v>0.1173</v>
+        <v>0.1132</v>
       </c>
       <c r="O35" s="3" t="n">
-        <v>0.1183</v>
+        <v>0.1156</v>
       </c>
     </row>
     <row r="36">
@@ -2260,47 +2260,47 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>14220.13</v>
+        <v>13876.21</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>-0.0027</v>
+        <v>-0.0349</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>-0.0138</v>
+        <v>-0.0377</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>-0.03240000000000001</v>
+        <v>-0.0377</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>-0.0281</v>
+        <v>-0.0449</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>0.0407</v>
+        <v>0.0119</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>0.0119</v>
+        <v>-0.0126</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>0.0516</v>
+        <v>0.0262</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>0.0699</v>
+        <v>0.0466</v>
       </c>
       <c r="L36" s="3" t="n">
-        <v>0.006</v>
+        <v>-0.0163</v>
       </c>
       <c r="M36" s="3" t="n">
-        <v>0.1493</v>
+        <v>0.1387</v>
       </c>
       <c r="N36" s="3" t="n">
-        <v>0.1269</v>
+        <v>0.1153</v>
       </c>
       <c r="O36" s="3" t="n">
-        <v>0.14</v>
+        <v>0.1378</v>
       </c>
     </row>
     <row r="37">
@@ -2311,47 +2311,47 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>76231.60000000001</v>
+        <v>73854.08</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>0.0104</v>
+        <v>-0.0378</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>-0.0018</v>
+        <v>-0.033</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>-0.0278</v>
+        <v>-0.033</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>-0.0677</v>
+        <v>-0.1038</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>-0.0044</v>
+        <v>-0.0293</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>-0.166</v>
+        <v>-0.192</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>0.0151</v>
+        <v>-0.0166</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>-0.1586</v>
+        <v>-0.1789</v>
       </c>
       <c r="L37" s="3" t="n">
-        <v>-0.1504</v>
+        <v>-0.1639</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>-0.0243</v>
+        <v>-0.0326</v>
       </c>
       <c r="N37" s="3" t="n">
-        <v>0.0397</v>
+        <v>0.0367</v>
       </c>
       <c r="O37" s="3" t="n">
-        <v>0.09390000000000001</v>
+        <v>0.09230000000000001</v>
       </c>
     </row>
     <row r="38">
@@ -2362,47 +2362,47 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>5432.3</v>
+        <v>5339.56</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>-0.0089</v>
+        <v>-0.0254</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>0.009300000000000001</v>
+        <v>-0.007900000000000001</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>-0.0236</v>
+        <v>-0.007900000000000001</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>-0.08410000000000001</v>
+        <v>-0.1027</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>0.0263</v>
+        <v>0.0143</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>0.0572</v>
+        <v>0.0392</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>0.0442</v>
+        <v>0.0264</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>0.005500000000000001</v>
+        <v>0.0028</v>
       </c>
       <c r="L38" s="3" t="n">
-        <v>-0.1094</v>
+        <v>-0.1119</v>
       </c>
       <c r="M38" s="3" t="n">
-        <v>0.137</v>
+        <v>0.1273</v>
       </c>
       <c r="N38" s="3" t="n">
-        <v>0.1471</v>
+        <v>0.1275</v>
       </c>
       <c r="O38" s="3" t="n">
-        <v>0.1224</v>
+        <v>0.1219</v>
       </c>
     </row>
     <row r="39">
@@ -2413,47 +2413,47 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>5873.99</v>
+        <v>5728.1</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>-0.0129</v>
+        <v>-0.0379</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>-0.0434</v>
+        <v>-0.0672</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>-0.0486</v>
+        <v>-0.0672</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>-0.0127</v>
+        <v>-0.0361</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>0.06280000000000001</v>
+        <v>0.0428</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>-0.0644</v>
+        <v>-0.0876</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>0.08869999999999999</v>
+        <v>0.0617</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>-0.0181</v>
+        <v>-0.0299</v>
       </c>
       <c r="L39" s="3" t="n">
-        <v>-0.0278</v>
+        <v>-0.0386</v>
       </c>
       <c r="M39" s="3" t="n">
-        <v>0.09789999999999999</v>
+        <v>0.09089999999999999</v>
       </c>
       <c r="N39" s="3" t="n">
         <v>0.0672</v>
       </c>
       <c r="O39" s="3" t="n">
-        <v>0.129</v>
+        <v>0.1273</v>
       </c>
     </row>
     <row r="40">
@@ -2464,47 +2464,47 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>16721.19</v>
+        <v>16340.02</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>-0.007900000000000001</v>
+        <v>-0.0355</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>-0.0208</v>
+        <v>-0.0432</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>-0.0248</v>
+        <v>-0.0432</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>-0.0233</v>
+        <v>-0.0404</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>0.0069</v>
+        <v>-0.025</v>
       </c>
       <c r="I40" s="3" t="n">
-        <v>-0.1064</v>
+        <v>-0.1268</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>0.0108</v>
+        <v>-0.0122</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>-0.0243</v>
+        <v>-0.0522</v>
       </c>
       <c r="L40" s="3" t="n">
-        <v>-0.06950000000000001</v>
+        <v>-0.08900000000000001</v>
       </c>
       <c r="M40" s="3" t="n">
-        <v>0.1231</v>
+        <v>0.113</v>
       </c>
       <c r="N40" s="3" t="n">
-        <v>0.08929999999999999</v>
+        <v>0.0767</v>
       </c>
       <c r="O40" s="3" t="n">
-        <v>0.1397</v>
+        <v>0.1373</v>
       </c>
     </row>
     <row r="41">
@@ -2515,47 +2515,47 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>66292.66</v>
+        <v>64868.48</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>-0.008800000000000001</v>
+        <v>-0.0298</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>-0.011</v>
+        <v>-0.0322</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>-0.0149</v>
+        <v>-0.0322</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>-0.0507</v>
+        <v>-0.07400000000000001</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>0.0696</v>
+        <v>0.0411</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>0.0703</v>
+        <v>0.0473</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>0.0808</v>
+        <v>0.0576</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>0.07429999999999999</v>
+        <v>0.05889999999999999</v>
       </c>
       <c r="L41" s="3" t="n">
-        <v>-0.0658</v>
+        <v>-0.07539999999999999</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>0.1286</v>
+        <v>0.1176</v>
       </c>
       <c r="N41" s="3" t="n">
-        <v>0.1322</v>
+        <v>0.1146</v>
       </c>
       <c r="O41" s="3" t="n">
-        <v>0.1657</v>
+        <v>0.164</v>
       </c>
     </row>
     <row r="42">
@@ -2566,47 +2566,47 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>40669.75</v>
+        <v>40011.07</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>-0.024</v>
+        <v>-0.0222</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>-0.09720000000000001</v>
+        <v>-0.1118</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>-0.0712</v>
+        <v>-0.1118</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>0.0337</v>
+        <v>0.0786</v>
       </c>
       <c r="H42" s="3" t="n">
+        <v>-0.058</v>
+      </c>
+      <c r="I42" s="3" t="n">
+        <v>-0.2587</v>
+      </c>
+      <c r="J42" s="3" t="n">
         <v>-0.0384</v>
       </c>
-      <c r="I42" s="3" t="n">
-        <v>-0.2465</v>
-      </c>
-      <c r="J42" s="3" t="n">
-        <v>-0.0225</v>
-      </c>
       <c r="K42" s="3" t="n">
-        <v>-0.1674</v>
+        <v>-0.1592</v>
       </c>
       <c r="L42" s="3" t="n">
-        <v>-0.1629</v>
+        <v>-0.1696</v>
       </c>
       <c r="M42" s="3" t="n">
-        <v>-0.0259</v>
+        <v>-0.0242</v>
       </c>
       <c r="N42" s="3" t="n">
-        <v>-0.0343</v>
+        <v>-0.025</v>
       </c>
       <c r="O42" s="3" t="n">
-        <v>0.1273</v>
+        <v>0.1266</v>
       </c>
     </row>
     <row r="43">
@@ -2617,47 +2617,47 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>7743.41</v>
+        <v>7651.54</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>0.0121</v>
+        <v>-0.0071</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>0.0075</v>
+        <v>-0.004500000000000001</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>0.008800000000000001</v>
+        <v>-0.004500000000000001</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>0.0529</v>
+        <v>0.0225</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>0.2158</v>
+        <v>0.1637</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>0.1312</v>
+        <v>0.1177</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>0.1861</v>
+        <v>0.172</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>0.1724</v>
+        <v>0.144</v>
       </c>
       <c r="L43" s="3" t="n">
-        <v>0.1634</v>
+        <v>0.1524</v>
       </c>
       <c r="M43" s="3" t="n">
-        <v>0.2193</v>
+        <v>0.2126</v>
       </c>
       <c r="N43" s="3" t="n">
-        <v>0.1168</v>
+        <v>0.1193</v>
       </c>
       <c r="O43" s="3" t="n">
-        <v>0.1363</v>
+        <v>0.1344</v>
       </c>
     </row>
     <row r="44">
@@ -2668,47 +2668,47 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>30608.13</v>
+        <v>30408.5</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>0.0325</v>
+        <v>-0.002</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>0.0391</v>
+        <v>0.0323</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>0.0473</v>
+        <v>0.0323</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>0.0512</v>
+        <v>0.0201</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>0.3232</v>
+        <v>0.266</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>0.2122</v>
+        <v>0.2043</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>0.2893</v>
+        <v>0.2809</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>0.2546</v>
+        <v>0.2321</v>
       </c>
       <c r="L44" s="3" t="n">
-        <v>0.2381</v>
+        <v>0.2314</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>0.2817</v>
+        <v>0.2734</v>
       </c>
       <c r="N44" s="3" t="n">
-        <v>0.1482</v>
+        <v>0.1551</v>
       </c>
       <c r="O44" s="3" t="n">
-        <v>0.202</v>
+        <v>0.2009</v>
       </c>
     </row>
     <row r="45">
@@ -2719,47 +2719,47 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
-        <v>66364.2</v>
+        <v>68956.72</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>0.0207</v>
+        <v>0.0525</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>0.0008</v>
+        <v>0.033</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>0.0015</v>
+        <v>0.0414</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>-0.0432</v>
+        <v>0.0033</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>0.2434</v>
+        <v>0.3144</v>
       </c>
       <c r="I45" s="3" t="n">
-        <v>0.3183</v>
+        <v>0.3698</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>0.2996</v>
+        <v>0.3504</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>0.4504</v>
+        <v>0.5478000000000001</v>
       </c>
       <c r="L45" s="3" t="n">
-        <v>0.324</v>
+        <v>0.3359</v>
       </c>
       <c r="M45" s="3" t="n">
-        <v>0.2713</v>
+        <v>0.2951</v>
       </c>
       <c r="N45" s="3" t="n">
-        <v>0.1701</v>
+        <v>0.1911</v>
       </c>
       <c r="O45" s="3" t="n">
-        <v>0.1482</v>
+        <v>0.1532</v>
       </c>
     </row>
     <row r="46">
@@ -2770,47 +2770,47 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>25408.64</v>
+        <v>24996.89</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>0.004099999999999999</v>
+        <v>-0.0107</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>-0.03240000000000001</v>
+        <v>-0.008</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>-0.0334</v>
+        <v>-0.0375</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>0.0299</v>
+        <v>-0.0228</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>0.1394</v>
+        <v>0.0789</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>0.0375</v>
+        <v>0.0207</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>0.1203</v>
+        <v>0.1022</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>0.0796</v>
+        <v>0.0366</v>
       </c>
       <c r="L46" s="3" t="n">
-        <v>0.159</v>
+        <v>0.1407</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>0.1855</v>
+        <v>0.1793</v>
       </c>
       <c r="N46" s="3" t="n">
-        <v>0.1034</v>
+        <v>0.1053</v>
       </c>
       <c r="O46" s="3" t="n">
-        <v>0.09390000000000001</v>
+        <v>0.09050000000000001</v>
       </c>
     </row>
     <row r="47">
@@ -2821,47 +2821,47 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>8077.8</v>
+        <v>7863</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>0.0016</v>
+        <v>-0.027</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>-0.0308</v>
+        <v>-0.0127</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>-0.0454</v>
+        <v>-0.0529</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>-0.0366</v>
+        <v>-0.0722</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>0.0488</v>
+        <v>-0.0125</v>
       </c>
       <c r="I47" s="3" t="n">
-        <v>-0.008800000000000001</v>
+        <v>-0.0352</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>0.0334</v>
+        <v>0.0059</v>
       </c>
       <c r="K47" s="3" t="n">
+        <v>-0.013</v>
+      </c>
+      <c r="L47" s="3" t="n">
+        <v>0.0189</v>
+      </c>
+      <c r="M47" s="3" t="n">
         <v>0.0362</v>
       </c>
-      <c r="L47" s="3" t="n">
-        <v>0.0333</v>
-      </c>
-      <c r="M47" s="3" t="n">
-        <v>0.0453</v>
-      </c>
       <c r="N47" s="3" t="n">
-        <v>0.04</v>
+        <v>0.0382</v>
       </c>
       <c r="O47" s="3" t="n">
-        <v>0.06269999999999999</v>
+        <v>0.0585</v>
       </c>
     </row>
     <row r="48">
@@ -2872,47 +2872,47 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>10695.3</v>
+        <v>10441.72</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>0.0034</v>
+        <v>-0.0223</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>-0.0119</v>
+        <v>-0.0155</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>-0.0168</v>
+        <v>-0.0322</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>0.0178</v>
+        <v>-0.0198</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>0.073</v>
+        <v>0.0005</v>
       </c>
       <c r="I48" s="3" t="n">
-        <v>0.07690000000000001</v>
+        <v>0.05139999999999999</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>0.051</v>
+        <v>0.0261</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>0.1608</v>
+        <v>0.1054</v>
       </c>
       <c r="L48" s="3" t="n">
-        <v>0.1374</v>
+        <v>0.1233</v>
       </c>
       <c r="M48" s="3" t="n">
-        <v>0.1194</v>
+        <v>0.1162</v>
       </c>
       <c r="N48" s="3" t="n">
-        <v>0.0868</v>
+        <v>0.0824</v>
       </c>
       <c r="O48" s="3" t="n">
-        <v>0.0462</v>
+        <v>0.0411</v>
       </c>
     </row>
     <row r="49">
@@ -2923,47 +2923,47 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>24510.09</v>
+        <v>24613.27</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>-0.0097</v>
+        <v>-0.0089</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>-0.0413</v>
+        <v>-0.0373</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>-0.0446</v>
+        <v>-0.0373</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>0.08109999999999999</v>
+        <v>0.0757</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>-0.0177</v>
+        <v>-0.0269</v>
       </c>
       <c r="I49" s="3" t="n">
-        <v>-0.0437</v>
+        <v>-0.0397</v>
       </c>
       <c r="J49" s="3" t="n">
-        <v>-0.0112</v>
+        <v>-0.0071</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>-0.0746</v>
+        <v>-0.08349999999999999</v>
       </c>
       <c r="L49" s="3" t="n">
-        <v>0.132</v>
+        <v>0.07919999999999999</v>
       </c>
       <c r="M49" s="3" t="n">
-        <v>0.1196</v>
+        <v>0.1137</v>
       </c>
       <c r="N49" s="3" t="n">
-        <v>0.0026</v>
+        <v>0.0003</v>
       </c>
       <c r="O49" s="3" t="n">
-        <v>0.0039</v>
+        <v>0.005500000000000001</v>
       </c>
     </row>
     <row r="50">
@@ -2974,47 +2974,47 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>4439.14</v>
+        <v>4357.62</v>
       </c>
       <c r="D50" s="3" t="n">
-        <v>-0.004699999999999999</v>
+        <v>-0.0353</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>-0.04019999999999999</v>
+        <v>-0.0578</v>
       </c>
       <c r="F50" s="3" t="n">
-        <v>-0.0248</v>
+        <v>-0.0578</v>
       </c>
       <c r="G50" s="3" t="n">
-        <v>-0.1157</v>
+        <v>-0.1213</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>-0.0086</v>
+        <v>-0.0372</v>
       </c>
       <c r="I50" s="3" t="n">
-        <v>-0.0412</v>
+        <v>-0.0588</v>
       </c>
       <c r="J50" s="3" t="n">
-        <v>-0.0025</v>
+        <v>-0.0208</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>-0.0278</v>
+        <v>-0.061</v>
       </c>
       <c r="L50" s="3" t="n">
-        <v>0.1509</v>
+        <v>0.0415</v>
       </c>
       <c r="M50" s="3" t="n">
-        <v>0.0612</v>
+        <v>0.05690000000000001</v>
       </c>
       <c r="N50" s="3" t="n">
-        <v>-0.0175</v>
+        <v>-0.0218</v>
       </c>
       <c r="O50" s="3" t="n">
-        <v>0.0326</v>
+        <v>0.0297</v>
       </c>
     </row>
     <row r="51">
@@ -3025,47 +3025,47 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>95.81999999999999</v>
+        <v>96.2</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>-0.0005999999999999999</v>
+        <v>0.0048</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>0.0046</v>
+        <v>0.0016</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>0.0037</v>
+        <v>0.0114</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>0.015</v>
+        <v>0.008199999999999999</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>0.016</v>
+        <v>0.0384</v>
       </c>
       <c r="I51" s="3" t="n">
-        <v>0.0674</v>
+        <v>0.0716</v>
       </c>
       <c r="J51" s="3" t="n">
-        <v>0.0155</v>
+        <v>0.0195</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>0.0794</v>
+        <v>0.0828</v>
       </c>
       <c r="L51" s="3" t="n">
-        <v>0.07049999999999999</v>
+        <v>0.0713</v>
       </c>
       <c r="M51" s="3" t="n">
-        <v>0.0481</v>
+        <v>0.0503</v>
       </c>
       <c r="N51" s="3" t="n">
-        <v>0.0536</v>
+        <v>0.0532</v>
       </c>
       <c r="O51" s="3" t="n">
-        <v>0.0375</v>
+        <v>0.03759999999999999</v>
       </c>
     </row>
     <row r="52">
@@ -3076,47 +3076,47 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>4321.2</v>
+        <v>4190.1</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>-0.0234</v>
+        <v>-0.0251</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>-0.0248</v>
+        <v>0.0008</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>-0.0602</v>
+        <v>-0.0363</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>0.0595</v>
+        <v>0.0188</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>-0.038</v>
+        <v>-0.0992</v>
       </c>
       <c r="I52" s="3" t="n">
-        <v>-0.001</v>
+        <v>-0.0313</v>
       </c>
       <c r="J52" s="3" t="n">
-        <v>-0.0702</v>
+        <v>-0.0984</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>0.1564</v>
+        <v>0.0834</v>
       </c>
       <c r="L52" s="3" t="n">
-        <v>0.275</v>
+        <v>0.2536</v>
       </c>
       <c r="M52" s="3" t="n">
-        <v>0.3152</v>
+        <v>0.3183</v>
       </c>
       <c r="N52" s="3" t="n">
-        <v>0.1981</v>
+        <v>0.1899</v>
       </c>
       <c r="O52" s="3" t="n">
-        <v>0.1255</v>
+        <v>0.1235</v>
       </c>
     </row>
     <row r="53">
@@ -3127,47 +3127,47 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>64.8</v>
+        <v>60.76</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>-0.035</v>
+        <v>-0.0425</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>-0.0214</v>
+        <v>0.011</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>-0.0469</v>
+        <v>-0.0597</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>0.09429999999999999</v>
+        <v>0.0019</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>-0.0682</v>
+        <v>-0.1646</v>
       </c>
       <c r="I53" s="3" t="n">
-        <v>-0.076</v>
+        <v>-0.1337</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>-0.1324</v>
+        <v>-0.1865</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>0.4498</v>
+        <v>0.2848</v>
       </c>
       <c r="L53" s="3" t="n">
-        <v>0.4301</v>
+        <v>0.3904</v>
       </c>
       <c r="M53" s="3" t="n">
-        <v>0.4137</v>
+        <v>0.4204</v>
       </c>
       <c r="N53" s="3" t="n">
-        <v>0.2367</v>
+        <v>0.2197</v>
       </c>
       <c r="O53" s="3" t="n">
-        <v>0.1301</v>
+        <v>0.1246</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Weekly indices update 2026-10-04
</commit_message>
<xml_diff>
--- a/tracker_auto.xlsx
+++ b/tracker_auto.xlsx
@@ -524,47 +524,47 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>22620.45</v>
+        <v>22421.95</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>-0.0352</v>
+        <v>-0.0278</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-0.06059999999999999</v>
+        <v>-0.008800000000000001</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>-0.06059999999999999</v>
+        <v>-0.0679</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>-0.05769999999999999</v>
+        <v>-0.0725</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>-0.0026</v>
+        <v>-0.0128</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>-0.1343</v>
+        <v>-0.1419</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.0129</v>
+        <v>0.004099999999999999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>-0.0809</v>
+        <v>-0.09720000000000001</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>-0.0639</v>
+        <v>-0.0678</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>0.0482</v>
+        <v>0.0451</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>0.05230000000000001</v>
+        <v>0.0504</v>
       </c>
       <c r="O2" s="3" t="n">
-        <v>0.1014</v>
+        <v>0.0989</v>
       </c>
     </row>
     <row r="3">
@@ -579,43 +579,43 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>71748.7</v>
+        <v>71909.7</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>-0.0249</v>
+        <v>-0.0227</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>-0.0101</v>
+        <v>-0.007900000000000001</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>-0.0675</v>
+        <v>-0.0654</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>-0.0742</v>
+        <v>-0.0722</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>-0.0214</v>
+        <v>-0.0192</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>-0.1581</v>
+        <v>-0.1562</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>-0.0028</v>
+        <v>-0.0005</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>-0.114</v>
+        <v>-0.112</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>-0.07730000000000001</v>
+        <v>-0.07629999999999999</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>0.0291</v>
+        <v>0.0298</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>0.0407</v>
+        <v>0.0412</v>
       </c>
       <c r="O3" s="3" t="n">
-        <v>0.0978</v>
+        <v>0.098</v>
       </c>
     </row>
     <row r="4">
@@ -626,47 +626,47 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>69746.95</v>
+        <v>68981.35000000001</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>-0.0375</v>
+        <v>-0.0336</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>-0.0544</v>
+        <v>-0.011</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>-0.0544</v>
+        <v>-0.0534</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>-0.0326</v>
+        <v>-0.0475</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.1265</v>
+        <v>0.1134</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.005500000000000001</v>
+        <v>-0.005500000000000001</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.1557</v>
+        <v>0.143</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>0.028</v>
+        <v>0.0131</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>-0.0489</v>
+        <v>-0.0553</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>0.1568</v>
+        <v>0.1524</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>0.1042</v>
+        <v>0.1017</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>0.1178</v>
+        <v>0.1136</v>
       </c>
     </row>
     <row r="5">
@@ -677,47 +677,47 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>23734.7</v>
+        <v>23516.5</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>-0.0357</v>
+        <v>-0.0289</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>-0.0595</v>
+        <v>-0.0092</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>-0.0595</v>
+        <v>-0.06519999999999999</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>-0.05309999999999999</v>
+        <v>-0.0679</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>0.0198</v>
+        <v>0.0091</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>-0.1107</v>
+        <v>-0.1189</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0.03759999999999999</v>
+        <v>0.028</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>-0.0617</v>
+        <v>-0.0779</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>-0.0605</v>
+        <v>-0.06480000000000001</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>0.06619999999999999</v>
+        <v>0.0629</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>0.0595</v>
+        <v>0.0575</v>
       </c>
       <c r="O5" s="3" t="n">
-        <v>0.1038</v>
+        <v>0.101</v>
       </c>
     </row>
     <row r="6">
@@ -728,47 +728,47 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>30904.45</v>
+        <v>30532.4</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>-0.0383</v>
+        <v>-0.0339</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-0.063</v>
+        <v>-0.012</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-0.063</v>
+        <v>-0.0701</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>-0.0507</v>
+        <v>-0.0702</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.03</v>
+        <v>0.0176</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>-0.0728</v>
+        <v>-0.08400000000000001</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.04559999999999999</v>
+        <v>0.033</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>-0.0206</v>
+        <v>-0.0415</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>-0.0374</v>
+        <v>-0.043</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>0.09449999999999999</v>
+        <v>0.09</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>0.09429999999999999</v>
+        <v>0.0916</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>0.1113</v>
+        <v>0.1081</v>
       </c>
     </row>
     <row r="7">
@@ -779,47 +779,47 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>32860.75</v>
+        <v>32490.75</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>-0.0379</v>
+        <v>-0.0341</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-0.061</v>
+        <v>-0.0113</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>-0.061</v>
+        <v>-0.06419999999999999</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>-0.0425</v>
+        <v>-0.0596</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.08019999999999999</v>
+        <v>0.0674</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>-0.0322</v>
+        <v>-0.0431</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>0.1032</v>
+        <v>0.09080000000000001</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>0.0015</v>
+        <v>-0.0165</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>-0.0365</v>
+        <v>-0.042</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>0.1233</v>
+        <v>0.1189</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>0.0956</v>
+        <v>0.09300000000000001</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>0.1107</v>
+        <v>0.1071</v>
       </c>
     </row>
     <row r="8">
@@ -830,47 +830,47 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>17724.2</v>
+        <v>17557.98</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>-0.0384</v>
+        <v>-0.0305</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-0.0626</v>
+        <v>-0.009399999999999999</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-0.0626</v>
+        <v>-0.0665</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>-0.0482</v>
+        <v>-0.063</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.0423</v>
+        <v>0.0319</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>-0.0863</v>
+        <v>-0.0949</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.0614</v>
+        <v>0.05139999999999999</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>-0.0323</v>
+        <v>-0.0493</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>-0.0409</v>
+        <v>-0.04559999999999999</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>0.08890000000000001</v>
+        <v>0.08550000000000001</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>0.0837</v>
+        <v>0.08160000000000001</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>0.1233</v>
+        <v>0.1203</v>
       </c>
     </row>
     <row r="9">
@@ -881,47 +881,47 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>15757.7</v>
+        <v>15604.7</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>-0.0411</v>
+        <v>-0.0329</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-0.0653</v>
+        <v>-0.0097</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-0.0653</v>
+        <v>-0.0672</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>-0.0475</v>
+        <v>-0.0621</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>0.06</v>
+        <v>0.0507</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>-0.06509999999999999</v>
+        <v>-0.0742</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>0.08119999999999999</v>
+        <v>0.0707</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>-0.0118</v>
+        <v>-0.0296</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>-0.0347</v>
+        <v>-0.0401</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>0.0987</v>
+        <v>0.095</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>0.1001</v>
+        <v>0.09789999999999999</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>0.1311</v>
+        <v>0.1278</v>
       </c>
     </row>
     <row r="10">
@@ -932,47 +932,47 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>21867.5</v>
+        <v>21643.85</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>-0.0463</v>
+        <v>-0.0368</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>-0.0709</v>
+        <v>-0.0102</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>-0.0709</v>
+        <v>-0.0692</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>-0.04190000000000001</v>
+        <v>-0.0563</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.1006</v>
+        <v>0.09279999999999999</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>-0.0184</v>
+        <v>-0.0284</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.1254</v>
+        <v>0.1139</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>0.0394</v>
+        <v>0.02</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>-0.01</v>
+        <v>-0.0166</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>0.1302</v>
+        <v>0.1262</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0.1398</v>
+        <v>0.1374</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>0.1567</v>
+        <v>0.1528</v>
       </c>
     </row>
     <row r="11">
@@ -983,47 +983,47 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>17798.8</v>
+        <v>17589.05</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>-0.0333</v>
+        <v>-0.0312</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>-0.0312</v>
+        <v>-0.0118</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>-0.0312</v>
+        <v>-0.04219999999999999</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>-0.0002</v>
+        <v>-0.0219</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0.2068</v>
+        <v>0.1945</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>0.0668</v>
+        <v>0.0542</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>0.2457</v>
+        <v>0.231</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>0.0663</v>
+        <v>0.04269999999999999</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>-0.0168</v>
+        <v>-0.0258</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>0.1331</v>
+        <v>0.1285</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>0.1365</v>
+        <v>0.1337</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>0.1371</v>
+        <v>0.1326</v>
       </c>
     </row>
     <row r="12">
@@ -1034,47 +1034,47 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>20415</v>
+        <v>20194.95</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>-0.0418</v>
+        <v>-0.0348</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>-0.0574</v>
+        <v>-0.0108</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>-0.0574</v>
+        <v>-0.0599</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>-0.0276</v>
+        <v>-0.0445</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.1357</v>
+        <v>0.1265</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>0.0098</v>
+        <v>-0.0011</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0.165</v>
+        <v>0.1524</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>0.0479</v>
+        <v>0.027</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>-0.0129</v>
+        <v>-0.0204</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0.1308</v>
+        <v>0.1266</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.1389</v>
+        <v>0.1363</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>0.1502</v>
+        <v>0.1461</v>
       </c>
     </row>
     <row r="13">
@@ -1085,47 +1085,47 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>22072.1</v>
+        <v>21857.75</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>-0.03759999999999999</v>
+        <v>-0.0308</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>-0.0588</v>
+        <v>-0.0097</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>-0.0588</v>
+        <v>-0.0635</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>-0.045</v>
+        <v>-0.0605</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>0.05429999999999999</v>
+        <v>0.04389999999999999</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>-0.07539999999999999</v>
+        <v>-0.08439999999999999</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>0.07519999999999999</v>
+        <v>0.06480000000000001</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>-0.0291</v>
+        <v>-0.0467</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>-0.0459</v>
+        <v>-0.05110000000000001</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>0.08460000000000001</v>
+        <v>0.081</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>0.08019999999999999</v>
+        <v>0.078</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>0.1156</v>
+        <v>0.1125</v>
       </c>
     </row>
     <row r="14">
@@ -1136,47 +1136,47 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>34564.37</v>
+        <v>34221.41</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>-0.0364</v>
+        <v>-0.0303</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>-0.05599999999999999</v>
+        <v>-0.009899999999999999</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>-0.05599999999999999</v>
+        <v>-0.0626</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>-0.043</v>
+        <v>-0.0592</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0.0533</v>
+        <v>0.0421</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>-0.07690000000000001</v>
+        <v>-0.08599999999999999</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>0.07400000000000001</v>
+        <v>0.0634</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>-0.0322</v>
+        <v>-0.0498</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>-0.0492</v>
+        <v>-0.05429999999999999</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0.0803</v>
+        <v>0.0767</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>0.07690000000000001</v>
+        <v>0.0747</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>0.1144</v>
+        <v>0.1113</v>
       </c>
     </row>
     <row r="15">
@@ -1187,47 +1187,47 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>18785.65</v>
+        <v>18587.95</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>-0.0342</v>
+        <v>-0.0316</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>-0.07099999999999999</v>
+        <v>-0.0105</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>-0.07099999999999999</v>
+        <v>-0.07769999999999999</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>-0.0518</v>
+        <v>-0.07049999999999999</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>0.0167</v>
+        <v>0.005</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>-0.111</v>
+        <v>-0.1203</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>0.0261</v>
+        <v>0.0153</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>-0.057</v>
+        <v>-0.0721</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>-0.0638</v>
+        <v>-0.0683</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>0.077</v>
+        <v>0.0731</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>0.0665</v>
+        <v>0.06419999999999999</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>0.1071</v>
+        <v>0.1042</v>
       </c>
     </row>
     <row r="16">
@@ -1238,47 +1238,47 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>5320.35</v>
+        <v>5261.85</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>-0.0296</v>
+        <v>-0.0289</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>-0.0698</v>
+        <v>-0.011</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>-0.0698</v>
+        <v>-0.0762</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>-0.0178</v>
+        <v>-0.0413</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>0.0363</v>
+        <v>0.0208</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>-0.09210000000000002</v>
+        <v>-0.1021</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>0.0571</v>
+        <v>0.0454</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>-0.0444</v>
+        <v>-0.0583</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>-0.07870000000000001</v>
+        <v>-0.0843</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0.0626</v>
+        <v>0.0587</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>0.0581</v>
+        <v>0.0558</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>0.09230000000000001</v>
+        <v>0.0898</v>
       </c>
     </row>
     <row r="17">
@@ -1289,47 +1289,47 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>24908.38</v>
+        <v>24461.55</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>-0.038</v>
+        <v>-0.0442</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>-0.0455</v>
+        <v>-0.0179</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>-0.0455</v>
+        <v>-0.0581</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>-0.0625</v>
+        <v>-0.0825</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>-0.0063</v>
+        <v>-0.0219</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>-0.0281</v>
+        <v>-0.04559999999999999</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>0.0132</v>
+        <v>-0.005</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>0.0789</v>
+        <v>0.0575</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>0.0048</v>
+        <v>-0.004</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>0.212</v>
+        <v>0.2045</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>0.2281</v>
+        <v>0.2236</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>0.1644</v>
+        <v>0.1594</v>
       </c>
     </row>
     <row r="18">
@@ -1340,47 +1340,47 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>37144.93</v>
+        <v>36763.93</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>-0.0371</v>
+        <v>-0.0341</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>-0.0578</v>
+        <v>-0.0103</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>-0.0578</v>
+        <v>-0.04940000000000001</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>-0.0418</v>
+        <v>-0.0503</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>0.0683</v>
+        <v>0.06309999999999999</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>-0.04650000000000001</v>
+        <v>-0.0562</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>0.0959</v>
+        <v>0.08460000000000001</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>-0.004699999999999999</v>
+        <v>-0.0244</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>-0.1079</v>
+        <v>-0.1142</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>0.092</v>
+        <v>0.08810000000000001</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>0.09329999999999999</v>
+        <v>0.091</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>0.1599</v>
+        <v>0.1557</v>
       </c>
     </row>
     <row r="19">
@@ -1391,47 +1391,47 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>27438.11</v>
+        <v>27236.54</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>-0.0325</v>
+        <v>-0.0293</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>-0.079</v>
+        <v>-0.0073</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>-0.079</v>
+        <v>-0.0842</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>-0.0325</v>
+        <v>-0.05110000000000001</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>0.0253</v>
+        <v>0.0133</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>-0.104</v>
+        <v>-0.1105</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>0.04969999999999999</v>
+        <v>0.042</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>-0.0542</v>
+        <v>-0.0655</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>-0.0843</v>
+        <v>-0.08839999999999999</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>0.0664</v>
+        <v>0.06370000000000001</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>0.0638</v>
+        <v>0.0622</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>0.1167</v>
+        <v>0.114</v>
       </c>
     </row>
     <row r="20">
@@ -1442,47 +1442,47 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>29518.95</v>
+        <v>29216.2</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>-0.0373</v>
+        <v>-0.0343</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>-0.0585</v>
+        <v>-0.0103</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>-0.0585</v>
+        <v>-0.0501</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>-0.0445</v>
+        <v>-0.0529</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>0.063</v>
+        <v>0.0578</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>-0.05230000000000001</v>
+        <v>-0.062</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>0.09039999999999999</v>
+        <v>0.07919999999999999</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>-0.0109</v>
+        <v>-0.0305</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>-0.1139</v>
+        <v>-0.1202</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>0.083</v>
+        <v>0.07919999999999999</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>0.0837</v>
+        <v>0.0814</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>0.1488</v>
+        <v>0.1447</v>
       </c>
     </row>
     <row r="21">
@@ -1493,47 +1493,47 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>54079.15</v>
+        <v>53855.85</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>-0.0333</v>
+        <v>-0.022</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>-0.0601</v>
+        <v>-0.004099999999999999</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>-0.0601</v>
+        <v>-0.0498</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.0004</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>0.1813</v>
+        <v>0.1826</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>0.07490000000000001</v>
+        <v>0.07049999999999999</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>0.2156</v>
+        <v>0.2106</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>0.1099</v>
+        <v>0.0915</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>-0.0539</v>
+        <v>-0.0555</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>0.1399</v>
+        <v>0.1382</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>0.1134</v>
+        <v>0.1124</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>0.1904</v>
+        <v>0.1869</v>
       </c>
     </row>
     <row r="22">
@@ -1544,47 +1544,47 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>25219.5</v>
+        <v>24935.1</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>-0.0408</v>
+        <v>-0.03759999999999999</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>-0.0722</v>
+        <v>-0.0113</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>-0.0722</v>
+        <v>-0.07440000000000001</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>-0.0476</v>
+        <v>-0.06370000000000001</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>0.0438</v>
+        <v>0.0358</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>-0.06860000000000001</v>
+        <v>-0.0791</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>0.0525</v>
+        <v>0.0406</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>-0.0283</v>
+        <v>-0.0471</v>
       </c>
       <c r="L22" s="3" t="n">
-        <v>-0.0999</v>
+        <v>-0.1049</v>
       </c>
       <c r="M22" s="3" t="n">
-        <v>0.0819</v>
+        <v>0.07780000000000001</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>0.0742</v>
+        <v>0.0717</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>0.1147</v>
+        <v>0.111</v>
       </c>
     </row>
     <row r="23">
@@ -1595,44 +1595,44 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>10282</v>
+        <v>10133.27</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>-0.0195</v>
+        <v>-0.0234</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>-0.0452</v>
+        <v>-0.0145</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>-0.0452</v>
+        <v>-0.0521</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>-0.0275</v>
+        <v>-0.04650000000000001</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>0.2231</v>
+        <v>0.2049</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>0.2032</v>
+        <v>0.1858</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>0.2881</v>
+        <v>0.2695</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>0.1879</v>
+        <v>0.152</v>
       </c>
       <c r="L23" s="3" t="n">
-        <v>0.1871</v>
+        <v>0.1818</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>0.423</v>
+        <v>0.4156</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>0.5108</v>
+        <v>0.5061</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -1648,47 +1648,47 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>11004.65</v>
+        <v>10897.19</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>-0.0418</v>
+        <v>-0.0403</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>-0.0689</v>
+        <v>-0.0098</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>-0.0689</v>
+        <v>-0.0668</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>-0.0653</v>
+        <v>-0.0704</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>-0.0115</v>
+        <v>-0.0175</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>-0.0536</v>
+        <v>-0.0629</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>0.0251</v>
+        <v>0.0151</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>0.073</v>
+        <v>0.0664</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>0.09699999999999999</v>
+        <v>0.0911</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>0.1589</v>
+        <v>0.1549</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>0.2757</v>
+        <v>0.273</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>0.1054</v>
+        <v>0.1023</v>
       </c>
     </row>
     <row r="25">
@@ -1699,47 +1699,47 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>76689.05</v>
+        <v>76433.16</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>-0.0339</v>
+        <v>-0.0178</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>-0.0585</v>
+        <v>-0.0033</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>-0.0585</v>
+        <v>-0.0515</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>-0.0568</v>
+        <v>-0.06</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>0.0689</v>
+        <v>0.06320000000000001</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>-0.077</v>
+        <v>-0.0801</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>0.09380000000000001</v>
+        <v>0.0902</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>0.006500000000000001</v>
+        <v>-0.0097</v>
       </c>
       <c r="L25" s="3" t="n">
-        <v>0.0229</v>
+        <v>0.0217</v>
       </c>
       <c r="M25" s="3" t="n">
-        <v>0.0784</v>
+        <v>0.0771</v>
       </c>
       <c r="N25" s="3" t="n">
-        <v>0.08839999999999999</v>
+        <v>0.0877</v>
       </c>
       <c r="O25" s="3" t="n">
-        <v>0.1163</v>
+        <v>0.1142</v>
       </c>
     </row>
     <row r="26">
@@ -1750,38 +1750,38 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>31600.55</v>
+        <v>31602.51</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>-0.0244</v>
+        <v>-0.0025</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>-0.04679999999999999</v>
+        <v>0.0001</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>-0.04679999999999999</v>
+        <v>-0.0384</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>-0.05</v>
+        <v>-0.0512</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>0.0931</v>
+        <v>0.08890000000000001</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>-0.0649</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>0.1123</v>
+        <v>0.1124</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>0.0149</v>
+        <v>-0.004699999999999999</v>
       </c>
       <c r="L26" s="3" t="n">
-        <v>0.0095</v>
+        <v>0.0101</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0.0561</v>
@@ -1790,7 +1790,7 @@
         <v>0.0738</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>0.1011</v>
+        <v>0.09939999999999999</v>
       </c>
     </row>
     <row r="27">
@@ -1801,47 +1801,47 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>31541.58</v>
+        <v>31422.04</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>-0.0358</v>
+        <v>-0.016</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>-0.0625</v>
+        <v>-0.0038</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>-0.0625</v>
+        <v>-0.0557</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>-0.07780000000000001</v>
+        <v>-0.08349999999999999</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>0.036</v>
+        <v>0.0295</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>-0.09960000000000001</v>
+        <v>-0.103</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>0.0563</v>
+        <v>0.05230000000000001</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>-0.0442</v>
+        <v>-0.0608</v>
       </c>
       <c r="L27" s="3" t="n">
-        <v>0.013</v>
+        <v>0.0111</v>
       </c>
       <c r="M27" s="3" t="n">
-        <v>0.0859</v>
+        <v>0.08439999999999999</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>0.07339999999999999</v>
+        <v>0.0725</v>
       </c>
       <c r="O27" s="3" t="n">
-        <v>0.1283</v>
+        <v>0.1259</v>
       </c>
     </row>
     <row r="28">
@@ -1852,47 +1852,47 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>16962.36</v>
+        <v>16687.41</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>-0.0285</v>
+        <v>-0.036</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>-0.0323</v>
+        <v>-0.0162</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>-0.0323</v>
+        <v>-0.0436</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>-0.05860000000000001</v>
+        <v>-0.076</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>-0.0279</v>
+        <v>-0.0404</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>-0.0359</v>
+        <v>-0.0515</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>-0.0136</v>
+        <v>-0.0296</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>-0.0263</v>
+        <v>-0.0447</v>
       </c>
       <c r="L28" s="3" t="n">
-        <v>-0.0703</v>
+        <v>-0.076</v>
       </c>
       <c r="M28" s="3" t="n">
-        <v>0.1839</v>
+        <v>0.1773</v>
       </c>
       <c r="N28" s="3" t="n">
-        <v>0.2088</v>
+        <v>0.2048</v>
       </c>
       <c r="O28" s="3" t="n">
-        <v>0.1384</v>
+        <v>0.1342</v>
       </c>
     </row>
     <row r="29">
@@ -1903,47 +1903,47 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>944.48</v>
+        <v>930.72</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>-0.0272</v>
+        <v>-0.0306</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>-0.0626</v>
+        <v>-0.0146</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>-0.0626</v>
+        <v>-0.0629</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>-0.009599999999999999</v>
+        <v>-0.038</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>0.2799</v>
+        <v>0.248</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>-0.0304</v>
+        <v>-0.0445</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>0.3071</v>
+        <v>0.2881</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>-0.0188</v>
+        <v>-0.0436</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>-0.1185</v>
+        <v>-0.1241</v>
       </c>
       <c r="M29" s="3" t="n">
-        <v>0.1415</v>
+        <v>0.1358</v>
       </c>
       <c r="N29" s="3" t="n">
-        <v>0.1126</v>
+        <v>0.1093</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>0.1585</v>
+        <v>0.1534</v>
       </c>
     </row>
     <row r="30">
@@ -1954,47 +1954,47 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>35196.26</v>
+        <v>33979.49</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>-0.0318</v>
+        <v>-0.0503</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>-0.0883</v>
+        <v>-0.0346</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>-0.0883</v>
+        <v>-0.109</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>-0.0123</v>
+        <v>-0.0579</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>0.09420000000000001</v>
+        <v>0.0629</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>-0.0576</v>
+        <v>-0.0901</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>0.1158</v>
+        <v>0.07730000000000001</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>0.0012</v>
+        <v>-0.0416</v>
       </c>
       <c r="L30" s="3" t="n">
-        <v>-0.0038</v>
+        <v>-0.0222</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>0.186</v>
+        <v>0.172</v>
       </c>
       <c r="N30" s="3" t="n">
-        <v>0.2106</v>
+        <v>0.2019</v>
       </c>
       <c r="O30" s="3" t="n">
-        <v>0.1128</v>
+        <v>0.1063</v>
       </c>
     </row>
     <row r="31">
@@ -2005,47 +2005,47 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>20299.36</v>
+        <v>19959.81</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>-0.0352</v>
+        <v>-0.0388</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>-0.068</v>
+        <v>-0.0167</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>-0.068</v>
+        <v>-0.0735</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>-0.0242</v>
+        <v>-0.0459</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>0.09039999999999999</v>
+        <v>0.07769999999999999</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>0.0106</v>
+        <v>-0.0064</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>0.1077</v>
+        <v>0.0892</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>0.0548</v>
+        <v>0.0298</v>
       </c>
       <c r="L31" s="3" t="n">
-        <v>0.0026</v>
+        <v>-0.0068</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>0.1721</v>
+        <v>0.1653</v>
       </c>
       <c r="N31" s="3" t="n">
-        <v>0.1534</v>
+        <v>0.1494</v>
       </c>
       <c r="O31" s="3" t="n">
-        <v>0.136</v>
+        <v>0.1316</v>
       </c>
     </row>
     <row r="32">
@@ -2056,47 +2056,47 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>11536.67</v>
+        <v>11366.58</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>-0.0397</v>
+        <v>-0.038</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>-0.048</v>
+        <v>-0.0147</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>-0.048</v>
+        <v>-0.06509999999999999</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>-0.07190000000000001</v>
+        <v>-0.08689999999999999</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>0.0135</v>
+        <v>0.003</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>-0.08529999999999999</v>
+        <v>-0.09880000000000001</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>0.0263</v>
+        <v>0.0111</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>-0.0223</v>
+        <v>-0.0384</v>
       </c>
       <c r="L32" s="3" t="n">
-        <v>-0.0367</v>
+        <v>-0.0429</v>
       </c>
       <c r="M32" s="3" t="n">
-        <v>0.1277</v>
+        <v>0.122</v>
       </c>
       <c r="N32" s="3" t="n">
-        <v>0.128</v>
+        <v>0.1246</v>
       </c>
       <c r="O32" s="3" t="n">
-        <v>0.1357</v>
+        <v>0.1316</v>
       </c>
     </row>
     <row r="33">
@@ -2107,47 +2107,47 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>19262.36</v>
+        <v>19212.01</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>-0.0433</v>
+        <v>-0.0395</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>-0.0474</v>
+        <v>-0.0026</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>-0.0474</v>
+        <v>-0.0345</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>0.0069</v>
+        <v>-0.0013</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>0.1516</v>
+        <v>0.1586</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>0.1077</v>
+        <v>0.1048</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>0.1398</v>
+        <v>0.1368</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>0.147</v>
+        <v>0.1297</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>0.0517</v>
+        <v>0.0507</v>
       </c>
       <c r="M33" s="3" t="n">
-        <v>0.1906</v>
+        <v>0.1893</v>
       </c>
       <c r="N33" s="3" t="n">
-        <v>0.1304</v>
+        <v>0.1297</v>
       </c>
       <c r="O33" s="3" t="n">
-        <v>0.1065</v>
+        <v>0.1044</v>
       </c>
     </row>
     <row r="34">
@@ -2158,47 +2158,47 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>19480.28</v>
+        <v>19022.65</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>-0.0404</v>
+        <v>-0.0442</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>-0.0322</v>
+        <v>-0.0235</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>-0.0322</v>
+        <v>-0.0547</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>0.0322</v>
+        <v>-0.0008</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>0.1261</v>
+        <v>0.09539999999999998</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>0.1541</v>
+        <v>0.1269</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>0.1538</v>
+        <v>0.1266</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>0.2845</v>
+        <v>0.2475</v>
       </c>
       <c r="L34" s="3" t="n">
-        <v>0.1293</v>
+        <v>0.1146</v>
       </c>
       <c r="M34" s="3" t="n">
-        <v>0.2408</v>
+        <v>0.2308</v>
       </c>
       <c r="N34" s="3" t="n">
-        <v>0.1923</v>
+        <v>0.1866</v>
       </c>
       <c r="O34" s="3" t="n">
-        <v>0.1984</v>
+        <v>0.1927</v>
       </c>
     </row>
     <row r="35">
@@ -2209,47 +2209,47 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>9640.370000000001</v>
+        <v>9440.35</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>-0.0322</v>
+        <v>-0.039</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>-0.0614</v>
+        <v>-0.0207</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>-0.0614</v>
+        <v>-0.0726</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>-0.0019</v>
+        <v>-0.0333</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>0.147</v>
+        <v>0.1256</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>-0.0221</v>
+        <v>-0.0424</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>0.179</v>
+        <v>0.1545</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>-0.0194</v>
+        <v>-0.0487</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>-0.0617</v>
+        <v>-0.07200000000000001</v>
       </c>
       <c r="M35" s="3" t="n">
-        <v>0.1139</v>
+        <v>0.106</v>
       </c>
       <c r="N35" s="3" t="n">
-        <v>0.1132</v>
+        <v>0.1084</v>
       </c>
       <c r="O35" s="3" t="n">
-        <v>0.1156</v>
+        <v>0.1103</v>
       </c>
     </row>
     <row r="36">
@@ -2260,47 +2260,47 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>13876.21</v>
+        <v>13608.31</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>-0.0349</v>
+        <v>-0.0405</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>-0.0377</v>
+        <v>-0.0193</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>-0.0377</v>
+        <v>-0.0576</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>-0.0449</v>
+        <v>-0.0704</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>0.0119</v>
+        <v>-0.0033</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>-0.0126</v>
+        <v>-0.0317</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>0.0262</v>
+        <v>0.0064</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>0.0466</v>
+        <v>0.0218</v>
       </c>
       <c r="L36" s="3" t="n">
-        <v>-0.0163</v>
+        <v>-0.0247</v>
       </c>
       <c r="M36" s="3" t="n">
-        <v>0.1387</v>
+        <v>0.1312</v>
       </c>
       <c r="N36" s="3" t="n">
-        <v>0.1153</v>
+        <v>0.1109</v>
       </c>
       <c r="O36" s="3" t="n">
-        <v>0.1378</v>
+        <v>0.1332</v>
       </c>
     </row>
     <row r="37">
@@ -2311,47 +2311,47 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>73854.08</v>
+        <v>72661.67</v>
       </c>
       <c r="D37" s="3" t="n">
+        <v>-0.043</v>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="F37" s="3" t="n">
+        <v>-0.0574</v>
+      </c>
+      <c r="G37" s="3" t="n">
+        <v>-0.1232</v>
+      </c>
+      <c r="H37" s="3" t="n">
+        <v>-0.047</v>
+      </c>
+      <c r="I37" s="3" t="n">
+        <v>-0.205</v>
+      </c>
+      <c r="J37" s="3" t="n">
+        <v>-0.0325</v>
+      </c>
+      <c r="K37" s="3" t="n">
+        <v>-0.198</v>
+      </c>
+      <c r="L37" s="3" t="n">
+        <v>-0.1702</v>
+      </c>
+      <c r="M37" s="3" t="n">
         <v>-0.0378</v>
       </c>
-      <c r="E37" s="3" t="n">
-        <v>-0.033</v>
-      </c>
-      <c r="F37" s="3" t="n">
-        <v>-0.033</v>
-      </c>
-      <c r="G37" s="3" t="n">
-        <v>-0.1038</v>
-      </c>
-      <c r="H37" s="3" t="n">
-        <v>-0.0293</v>
-      </c>
-      <c r="I37" s="3" t="n">
-        <v>-0.192</v>
-      </c>
-      <c r="J37" s="3" t="n">
-        <v>-0.0166</v>
-      </c>
-      <c r="K37" s="3" t="n">
-        <v>-0.1789</v>
-      </c>
-      <c r="L37" s="3" t="n">
-        <v>-0.1639</v>
-      </c>
-      <c r="M37" s="3" t="n">
-        <v>-0.0326</v>
-      </c>
       <c r="N37" s="3" t="n">
-        <v>0.0367</v>
+        <v>0.0333</v>
       </c>
       <c r="O37" s="3" t="n">
-        <v>0.09230000000000001</v>
+        <v>0.08960000000000001</v>
       </c>
     </row>
     <row r="38">
@@ -2362,47 +2362,47 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>5339.56</v>
+        <v>5248.51</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>-0.0254</v>
+        <v>-0.0298</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>-0.007900000000000001</v>
+        <v>-0.0171</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>-0.007900000000000001</v>
+        <v>-0.027</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>-0.1027</v>
+        <v>-0.1206</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>0.0143</v>
+        <v>-0.0001</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>0.0392</v>
+        <v>0.0214</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>0.0264</v>
+        <v>0.0089</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>0.0028</v>
+        <v>-0.0244</v>
       </c>
       <c r="L38" s="3" t="n">
-        <v>-0.1119</v>
+        <v>-0.118</v>
       </c>
       <c r="M38" s="3" t="n">
-        <v>0.1273</v>
+        <v>0.1207</v>
       </c>
       <c r="N38" s="3" t="n">
-        <v>0.1275</v>
+        <v>0.1236</v>
       </c>
       <c r="O38" s="3" t="n">
-        <v>0.1219</v>
+        <v>0.1174</v>
       </c>
     </row>
     <row r="39">
@@ -2413,47 +2413,47 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>5728.1</v>
+        <v>5681.28</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>-0.0379</v>
+        <v>-0.0288</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>-0.0672</v>
+        <v>-0.008199999999999999</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>-0.0672</v>
+        <v>-0.0698</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>-0.0361</v>
+        <v>-0.0541</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>0.0428</v>
+        <v>0.0303</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>-0.0876</v>
+        <v>-0.0951</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>0.0617</v>
+        <v>0.053</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>-0.0299</v>
+        <v>-0.0461</v>
       </c>
       <c r="L39" s="3" t="n">
-        <v>-0.0386</v>
+        <v>-0.0428</v>
       </c>
       <c r="M39" s="3" t="n">
-        <v>0.09089999999999999</v>
+        <v>0.08779999999999999</v>
       </c>
       <c r="N39" s="3" t="n">
-        <v>0.0672</v>
+        <v>0.0654</v>
       </c>
       <c r="O39" s="3" t="n">
-        <v>0.1273</v>
+        <v>0.1246</v>
       </c>
     </row>
     <row r="40">
@@ -2464,47 +2464,47 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>16340.02</v>
+        <v>16127.94</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>-0.0355</v>
+        <v>-0.0362</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>-0.0432</v>
+        <v>-0.013</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>-0.0432</v>
+        <v>-0.0588</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>-0.0404</v>
+        <v>-0.057</v>
       </c>
       <c r="H40" s="3" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="I40" s="3" t="n">
+        <v>-0.1381</v>
+      </c>
+      <c r="J40" s="3" t="n">
         <v>-0.025</v>
       </c>
-      <c r="I40" s="3" t="n">
-        <v>-0.1268</v>
-      </c>
-      <c r="J40" s="3" t="n">
-        <v>-0.0122</v>
-      </c>
       <c r="K40" s="3" t="n">
-        <v>-0.0522</v>
+        <v>-0.0665</v>
       </c>
       <c r="L40" s="3" t="n">
-        <v>-0.08900000000000001</v>
+        <v>-0.0919</v>
       </c>
       <c r="M40" s="3" t="n">
-        <v>0.113</v>
+        <v>0.1081</v>
       </c>
       <c r="N40" s="3" t="n">
-        <v>0.0767</v>
+        <v>0.0738</v>
       </c>
       <c r="O40" s="3" t="n">
-        <v>0.1373</v>
+        <v>0.1339</v>
       </c>
     </row>
     <row r="41">
@@ -2515,47 +2515,47 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>64868.48</v>
+        <v>64436.87</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>-0.0298</v>
+        <v>-0.0259</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>-0.0322</v>
+        <v>-0.0067</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>-0.0322</v>
+        <v>-0.035</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>-0.07400000000000001</v>
+        <v>-0.0789</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>0.0411</v>
+        <v>0.0372</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>0.0473</v>
+        <v>0.0404</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>0.0576</v>
+        <v>0.0506</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>0.05889999999999999</v>
+        <v>0.0464</v>
       </c>
       <c r="L41" s="3" t="n">
-        <v>-0.07539999999999999</v>
+        <v>-0.0751</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>0.1176</v>
+        <v>0.115</v>
       </c>
       <c r="N41" s="3" t="n">
-        <v>0.1146</v>
+        <v>0.1131</v>
       </c>
       <c r="O41" s="3" t="n">
-        <v>0.164</v>
+        <v>0.1614</v>
       </c>
     </row>
     <row r="42">
@@ -2566,47 +2566,47 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>40011.07</v>
+        <v>40877.44</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>-0.0222</v>
+        <v>0.0034</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>-0.1118</v>
+        <v>0.0217</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>-0.1118</v>
+        <v>-0.1013</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>0.0786</v>
+        <v>0.05309999999999999</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>-0.058</v>
+        <v>-0.062</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>-0.2587</v>
+        <v>-0.2426</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>-0.0384</v>
+        <v>-0.0175</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>-0.1592</v>
+        <v>-0.1473</v>
       </c>
       <c r="L42" s="3" t="n">
-        <v>-0.1696</v>
+        <v>-0.1655</v>
       </c>
       <c r="M42" s="3" t="n">
-        <v>-0.0242</v>
+        <v>-0.0172</v>
       </c>
       <c r="N42" s="3" t="n">
-        <v>-0.025</v>
+        <v>-0.0208</v>
       </c>
       <c r="O42" s="3" t="n">
-        <v>0.1266</v>
+        <v>0.1288</v>
       </c>
     </row>
     <row r="43">
@@ -2617,47 +2617,47 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>7651.54</v>
+        <v>7722.72</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>-0.0071</v>
+        <v>-0.0027</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>-0.004500000000000001</v>
+        <v>0.009300000000000001</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>-0.004500000000000001</v>
+        <v>0.0073</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>0.0225</v>
+        <v>0.032</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>0.1637</v>
+        <v>0.1732</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>0.1177</v>
+        <v>0.1281</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>0.172</v>
+        <v>0.1829</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>0.144</v>
+        <v>0.15</v>
       </c>
       <c r="L43" s="3" t="n">
-        <v>0.1524</v>
+        <v>0.1631</v>
       </c>
       <c r="M43" s="3" t="n">
-        <v>0.2126</v>
+        <v>0.2224</v>
       </c>
       <c r="N43" s="3" t="n">
-        <v>0.1193</v>
+        <v>0.1212</v>
       </c>
       <c r="O43" s="3" t="n">
-        <v>0.1344</v>
+        <v>0.1365</v>
       </c>
     </row>
     <row r="44">
@@ -2668,47 +2668,47 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>30408.5</v>
+        <v>30807.93</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>-0.002</v>
+        <v>0.006500000000000001</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>0.0323</v>
+        <v>0.0131</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>0.0323</v>
+        <v>0.0571</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>0.0201</v>
+        <v>0.0504</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>0.266</v>
+        <v>0.2812</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>0.2043</v>
+        <v>0.2201</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>0.2809</v>
+        <v>0.2977</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>0.2321</v>
+        <v>0.2376</v>
       </c>
       <c r="L44" s="3" t="n">
-        <v>0.2314</v>
+        <v>0.2475</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>0.2734</v>
+        <v>0.2839</v>
       </c>
       <c r="N44" s="3" t="n">
-        <v>0.1551</v>
+        <v>0.158</v>
       </c>
       <c r="O44" s="3" t="n">
-        <v>0.2009</v>
+        <v>0.203</v>
       </c>
     </row>
     <row r="45">
@@ -2719,47 +2719,47 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
-        <v>68956.72</v>
+        <v>68309.46000000001</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>0.0525</v>
+        <v>0.0293</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>0.033</v>
+        <v>0.0233</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>0.0414</v>
+        <v>0.0619</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>0.0033</v>
+        <v>-0.0206</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>0.3144</v>
+        <v>0.2859</v>
       </c>
       <c r="I45" s="3" t="n">
-        <v>0.3698</v>
+        <v>0.357</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>0.3504</v>
+        <v>0.3377000000000001</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>0.5478000000000001</v>
+        <v>0.5201</v>
       </c>
       <c r="L45" s="3" t="n">
-        <v>0.3359</v>
+        <v>0.3444</v>
       </c>
       <c r="M45" s="3" t="n">
-        <v>0.2951</v>
+        <v>0.2982</v>
       </c>
       <c r="N45" s="3" t="n">
-        <v>0.1911</v>
+        <v>0.1887</v>
       </c>
       <c r="O45" s="3" t="n">
-        <v>0.1532</v>
+        <v>0.1511</v>
       </c>
     </row>
     <row r="46">
@@ -2770,44 +2770,44 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>24996.89</v>
+        <v>25231.2</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>-0.0107</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>-0.008</v>
+        <v>0.0013</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>-0.0375</v>
+        <v>-0.0235</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>-0.0228</v>
+        <v>-0.0213</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>0.0789</v>
+        <v>0.0891</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>0.0207</v>
+        <v>0.0302</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>0.1022</v>
+        <v>0.1125</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>0.0366</v>
+        <v>0.0331</v>
       </c>
       <c r="L46" s="3" t="n">
-        <v>0.1407</v>
+        <v>0.1475</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>0.1793</v>
+        <v>0.1872</v>
       </c>
       <c r="N46" s="3" t="n">
-        <v>0.1053</v>
+        <v>0.1073</v>
       </c>
       <c r="O46" s="3" t="n">
         <v>0.09050000000000001</v>
@@ -2821,47 +2821,47 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>7863</v>
+        <v>7897.19</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>-0.027</v>
+        <v>-0.0224</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>-0.0127</v>
+        <v>-0.008500000000000001</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>-0.0529</v>
+        <v>-0.0463</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>-0.0722</v>
+        <v>-0.0718</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>-0.0125</v>
+        <v>-0.008199999999999999</v>
       </c>
       <c r="I47" s="3" t="n">
-        <v>-0.0352</v>
+        <v>-0.031</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>0.0059</v>
+        <v>0.0103</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>-0.013</v>
+        <v>-0.0198</v>
       </c>
       <c r="L47" s="3" t="n">
-        <v>0.0189</v>
+        <v>0.0209</v>
       </c>
       <c r="M47" s="3" t="n">
-        <v>0.0362</v>
+        <v>0.0412</v>
       </c>
       <c r="N47" s="3" t="n">
-        <v>0.0382</v>
+        <v>0.0391</v>
       </c>
       <c r="O47" s="3" t="n">
-        <v>0.0585</v>
+        <v>0.0578</v>
       </c>
     </row>
     <row r="48">
@@ -2872,47 +2872,47 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>10441.72</v>
+        <v>10462</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>-0.0223</v>
+        <v>-0.0218</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>-0.0155</v>
+        <v>-0.0136</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>-0.0322</v>
+        <v>-0.0274</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>-0.0198</v>
+        <v>-0.0203</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>0.0005</v>
+        <v>0.0025</v>
       </c>
       <c r="I48" s="3" t="n">
-        <v>0.05139999999999999</v>
+        <v>0.0534</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>0.0261</v>
+        <v>0.0281</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>0.1054</v>
+        <v>0.1097</v>
       </c>
       <c r="L48" s="3" t="n">
-        <v>0.1233</v>
+        <v>0.1234</v>
       </c>
       <c r="M48" s="3" t="n">
-        <v>0.1162</v>
+        <v>0.1189</v>
       </c>
       <c r="N48" s="3" t="n">
-        <v>0.0824</v>
+        <v>0.0828</v>
       </c>
       <c r="O48" s="3" t="n">
-        <v>0.0411</v>
+        <v>0.0399</v>
       </c>
     </row>
     <row r="49">
@@ -2923,47 +2923,47 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>24613.27</v>
+        <v>23972.29</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>-0.0089</v>
+        <v>-0.0219</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>-0.0373</v>
+        <v>-0.026</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>-0.0373</v>
+        <v>-0.0529</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>0.0757</v>
+        <v>0.0266</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>-0.0269</v>
+        <v>-0.04559999999999999</v>
       </c>
       <c r="I49" s="3" t="n">
-        <v>-0.0397</v>
+        <v>-0.06469999999999999</v>
       </c>
       <c r="J49" s="3" t="n">
-        <v>-0.0071</v>
+        <v>-0.0329</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>-0.08349999999999999</v>
+        <v>-0.1215</v>
       </c>
       <c r="L49" s="3" t="n">
-        <v>0.07919999999999999</v>
+        <v>0.0335</v>
       </c>
       <c r="M49" s="3" t="n">
-        <v>0.1137</v>
+        <v>0.1143</v>
       </c>
       <c r="N49" s="3" t="n">
-        <v>0.0003</v>
+        <v>-0.005</v>
       </c>
       <c r="O49" s="3" t="n">
-        <v>0.005500000000000001</v>
+        <v>0.0012</v>
       </c>
     </row>
     <row r="50">
@@ -3025,44 +3025,44 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>96.2</v>
+        <v>96.3</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>0.0048</v>
+        <v>0.005</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>0.0016</v>
+        <v>0.0026</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>0.0114</v>
+        <v>0.0191</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>0.008199999999999999</v>
+        <v>0.008100000000000001</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>0.0384</v>
+        <v>0.0358</v>
       </c>
       <c r="I51" s="3" t="n">
-        <v>0.0716</v>
+        <v>0.0727</v>
       </c>
       <c r="J51" s="3" t="n">
-        <v>0.0195</v>
+        <v>0.0206</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>0.0828</v>
+        <v>0.08539999999999999</v>
       </c>
       <c r="L51" s="3" t="n">
-        <v>0.0713</v>
+        <v>0.0707</v>
       </c>
       <c r="M51" s="3" t="n">
-        <v>0.0503</v>
+        <v>0.0489</v>
       </c>
       <c r="N51" s="3" t="n">
-        <v>0.0532</v>
+        <v>0.0525</v>
       </c>
       <c r="O51" s="3" t="n">
         <v>0.03759999999999999</v>
@@ -3076,47 +3076,47 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>4190.1</v>
+        <v>4162.3</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>-0.0251</v>
+        <v>-0.0368</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>0.0008</v>
+        <v>-0.0058</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>-0.0363</v>
+        <v>-0.0467</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>0.0188</v>
+        <v>0.0121</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>-0.0992</v>
+        <v>-0.1052</v>
       </c>
       <c r="I52" s="3" t="n">
-        <v>-0.0313</v>
+        <v>-0.0378</v>
       </c>
       <c r="J52" s="3" t="n">
-        <v>-0.0984</v>
+        <v>-0.1044</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>0.0834</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="L52" s="3" t="n">
-        <v>0.2536</v>
+        <v>0.2541</v>
       </c>
       <c r="M52" s="3" t="n">
-        <v>0.3183</v>
+        <v>0.3166</v>
       </c>
       <c r="N52" s="3" t="n">
-        <v>0.1899</v>
+        <v>0.1882</v>
       </c>
       <c r="O52" s="3" t="n">
-        <v>0.1235</v>
+        <v>0.1265</v>
       </c>
     </row>
     <row r="53">
@@ -3127,47 +3127,47 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>60.76</v>
+        <v>60.42</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>-0.0425</v>
+        <v>-0.0677</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>0.011</v>
+        <v>0.0053</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>-0.0597</v>
+        <v>-0.06660000000000001</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>0.0019</v>
+        <v>-0.0038</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>-0.1646</v>
+        <v>-0.1694</v>
       </c>
       <c r="I53" s="3" t="n">
-        <v>-0.1337</v>
+        <v>-0.1386</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>-0.1865</v>
+        <v>-0.1911</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>0.2848</v>
+        <v>0.3134</v>
       </c>
       <c r="L53" s="3" t="n">
-        <v>0.3904</v>
+        <v>0.3824</v>
       </c>
       <c r="M53" s="3" t="n">
-        <v>0.4204</v>
+        <v>0.4186</v>
       </c>
       <c r="N53" s="3" t="n">
-        <v>0.2197</v>
+        <v>0.2182</v>
       </c>
       <c r="O53" s="3" t="n">
-        <v>0.1246</v>
+        <v>0.1306</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Weekly indices update 2026-10-06
</commit_message>
<xml_diff>
--- a/tracker_auto.xlsx
+++ b/tracker_auto.xlsx
@@ -524,47 +524,47 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>22421.95</v>
+        <v>22555.75</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>-0.0278</v>
+        <v>-0.009899999999999999</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-0.008800000000000001</v>
+        <v>-0.0029</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>-0.0679</v>
+        <v>-0.0562</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>-0.0725</v>
+        <v>-0.0767</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>-0.0128</v>
+        <v>-0.018</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>-0.1419</v>
+        <v>-0.1368</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.004099999999999999</v>
+        <v>0.01</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>-0.09720000000000001</v>
+        <v>-0.09390000000000001</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>-0.0678</v>
+        <v>-0.0504</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>0.0451</v>
+        <v>0.047</v>
       </c>
       <c r="N2" s="3" t="n">
         <v>0.0504</v>
       </c>
       <c r="O2" s="3" t="n">
-        <v>0.0989</v>
+        <v>0.1001</v>
       </c>
     </row>
     <row r="3">
@@ -575,47 +575,47 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>71909.7</v>
+        <v>72789.24000000001</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>-0.0227</v>
+        <v>0.0036</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>-0.007900000000000001</v>
+        <v>0.0043</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>-0.0654</v>
+        <v>-0.0487</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>-0.0722</v>
+        <v>-0.06900000000000001</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>-0.0192</v>
+        <v>-0.0245</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>-0.1562</v>
+        <v>-0.1459</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>-0.0005</v>
+        <v>0.0117</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>-0.112</v>
+        <v>-0.11</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>-0.07629999999999999</v>
+        <v>-0.0559</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>0.0298</v>
+        <v>0.0332</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>0.0412</v>
+        <v>0.0405</v>
       </c>
       <c r="O3" s="3" t="n">
-        <v>0.098</v>
+        <v>0.1001</v>
       </c>
     </row>
     <row r="4">
@@ -626,47 +626,47 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>68981.35000000001</v>
+        <v>69213.75</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>-0.0336</v>
+        <v>-0.0156</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>-0.011</v>
+        <v>-0.0076</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>-0.0534</v>
+        <v>-0.0503</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>-0.0475</v>
+        <v>-0.0478</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.1134</v>
+        <v>0.1011</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>-0.005500000000000001</v>
+        <v>-0.0022</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.143</v>
+        <v>0.1469</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>0.0131</v>
+        <v>0.0125</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>-0.0553</v>
+        <v>-0.0369</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>0.1524</v>
+        <v>0.1549</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>0.1017</v>
+        <v>0.1004</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>0.1136</v>
+        <v>0.1135</v>
       </c>
     </row>
     <row r="5">
@@ -677,47 +677,47 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>23516.5</v>
+        <v>23645.3</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>-0.0289</v>
+        <v>-0.0109</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>-0.0092</v>
+        <v>-0.0038</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>-0.06519999999999999</v>
+        <v>-0.0551</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>-0.0679</v>
+        <v>-0.07139999999999999</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>0.0091</v>
+        <v>0.0028</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>-0.1189</v>
+        <v>-0.1141</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0.028</v>
+        <v>0.0337</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>-0.0779</v>
+        <v>-0.07519999999999999</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>-0.06480000000000001</v>
+        <v>-0.0474</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>0.0629</v>
+        <v>0.0649</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>0.0575</v>
+        <v>0.0572</v>
       </c>
       <c r="O5" s="3" t="n">
-        <v>0.101</v>
+        <v>0.1019</v>
       </c>
     </row>
     <row r="6">
@@ -728,47 +728,47 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>30532.4</v>
+        <v>30700.05</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>-0.0339</v>
+        <v>-0.0173</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-0.012</v>
+        <v>-0.0066</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-0.0701</v>
+        <v>-0.0579</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>-0.0702</v>
+        <v>-0.07240000000000001</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.0176</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>-0.08400000000000001</v>
+        <v>-0.0789</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.033</v>
+        <v>0.0387</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>-0.0415</v>
+        <v>-0.0383</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>-0.043</v>
+        <v>-0.0257</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>0.09</v>
+        <v>0.09359999999999999</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>0.0916</v>
+        <v>0.09210000000000002</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>0.1081</v>
+        <v>0.1087</v>
       </c>
     </row>
     <row r="7">
@@ -779,47 +779,47 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>32490.75</v>
+        <v>32626.5</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>-0.0341</v>
+        <v>-0.0165</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-0.0113</v>
+        <v>-0.0071</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>-0.06419999999999999</v>
+        <v>-0.0571</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>-0.0596</v>
+        <v>-0.0624</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.0674</v>
+        <v>0.0562</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>-0.0431</v>
+        <v>-0.0391</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>0.09080000000000001</v>
+        <v>0.0953</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>-0.0165</v>
+        <v>-0.0155</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>-0.042</v>
+        <v>-0.0245</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>0.1189</v>
+        <v>0.1219</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>0.09300000000000001</v>
+        <v>0.0926</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>0.1071</v>
+        <v>0.1072</v>
       </c>
     </row>
     <row r="8">
@@ -830,47 +830,47 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>17557.98</v>
+        <v>17658.75</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>-0.0305</v>
+        <v>-0.0113</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-0.009399999999999999</v>
+        <v>-0.0037</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-0.0665</v>
+        <v>-0.0565</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>-0.063</v>
+        <v>-0.0653</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.0319</v>
+        <v>0.0251</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>-0.0949</v>
+        <v>-0.0897</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.05139999999999999</v>
+        <v>0.0574</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>-0.0493</v>
+        <v>-0.0472</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>-0.04559999999999999</v>
+        <v>-0.0277</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>0.08550000000000001</v>
+        <v>0.08800000000000001</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>0.08160000000000001</v>
+        <v>0.08130000000000001</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>0.1203</v>
+        <v>0.1211</v>
       </c>
     </row>
     <row r="9">
@@ -881,47 +881,47 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>15604.7</v>
+        <v>15687.65</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>-0.0329</v>
+        <v>-0.0127</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-0.0097</v>
+        <v>-0.0044</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-0.0672</v>
+        <v>-0.0581</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>-0.0621</v>
+        <v>-0.0623</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>0.0507</v>
+        <v>0.0426</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>-0.0742</v>
+        <v>-0.0693</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>0.0707</v>
+        <v>0.0764</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>-0.0296</v>
+        <v>-0.0298</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>-0.0401</v>
+        <v>-0.0225</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>0.095</v>
+        <v>0.09810000000000001</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>0.09789999999999999</v>
+        <v>0.09710000000000001</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>0.1278</v>
+        <v>0.1281</v>
       </c>
     </row>
     <row r="10">
@@ -932,47 +932,47 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>21643.85</v>
+        <v>21755.3</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>-0.0368</v>
+        <v>-0.0143</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>-0.0102</v>
+        <v>-0.0051</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>-0.0692</v>
+        <v>-0.061</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>-0.0563</v>
+        <v>-0.053</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.09279999999999999</v>
+        <v>0.08289999999999999</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>-0.0284</v>
+        <v>-0.0234</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.1139</v>
+        <v>0.1196</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>0.02</v>
+        <v>0.0166</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>-0.0166</v>
+        <v>0.001</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>0.1262</v>
+        <v>0.1304</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0.1374</v>
+        <v>0.1361</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>0.1528</v>
+        <v>0.1524</v>
       </c>
     </row>
     <row r="11">
@@ -983,47 +983,47 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>17589.05</v>
+        <v>17655.35</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>-0.0312</v>
+        <v>-0.0116</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>-0.0118</v>
+        <v>-0.008100000000000001</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>-0.04219999999999999</v>
+        <v>-0.0447</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>-0.0219</v>
+        <v>-0.0234</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0.1945</v>
+        <v>0.1864</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>0.0542</v>
+        <v>0.0582</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>0.231</v>
+        <v>0.2356</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>0.04269999999999999</v>
+        <v>0.03759999999999999</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>-0.0258</v>
+        <v>-0.0102</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>0.1285</v>
+        <v>0.1276</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>0.1337</v>
+        <v>0.1321</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>0.1326</v>
+        <v>0.1321</v>
       </c>
     </row>
     <row r="12">
@@ -1034,47 +1034,47 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>20194.95</v>
+        <v>20289.05</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>-0.0348</v>
+        <v>-0.0134</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>-0.0108</v>
+        <v>-0.0062</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>-0.0599</v>
+        <v>-0.0554</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>-0.0445</v>
+        <v>-0.0429</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.1265</v>
+        <v>0.1171</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>-0.0011</v>
+        <v>0.0035</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0.1524</v>
+        <v>0.1578</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>0.027</v>
+        <v>0.0231</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>-0.0204</v>
+        <v>-0.0035</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0.1266</v>
+        <v>0.1291</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.1363</v>
+        <v>0.1349</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>0.1461</v>
+        <v>0.1457</v>
       </c>
     </row>
     <row r="13">
@@ -1085,47 +1085,47 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>21857.75</v>
+        <v>21971.6</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>-0.0308</v>
+        <v>-0.0117</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>-0.0097</v>
+        <v>-0.0046</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>-0.0635</v>
+        <v>-0.0552</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>-0.0605</v>
+        <v>-0.0624</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>0.04389999999999999</v>
+        <v>0.0367</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>-0.08439999999999999</v>
+        <v>-0.0796</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>0.06480000000000001</v>
+        <v>0.0703</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>-0.0467</v>
+        <v>-0.0459</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>-0.05110000000000001</v>
+        <v>-0.0338</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>0.081</v>
+        <v>0.08310000000000001</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>0.078</v>
+        <v>0.0775</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>0.1125</v>
+        <v>0.1132</v>
       </c>
     </row>
     <row r="14">
@@ -1136,47 +1136,47 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>34221.41</v>
+        <v>34387.91</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>-0.0303</v>
+        <v>-0.0115</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>-0.009899999999999999</v>
+        <v>-0.0051</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>-0.0626</v>
+        <v>-0.0549</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>-0.0592</v>
+        <v>-0.06150000000000001</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0.0421</v>
+        <v>0.0348</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>-0.08599999999999999</v>
+        <v>-0.08160000000000001</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>0.0634</v>
+        <v>0.06849999999999999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>-0.0498</v>
+        <v>-0.0491</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>-0.05429999999999999</v>
+        <v>-0.0371</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0.0767</v>
+        <v>0.07870000000000001</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>0.0747</v>
+        <v>0.07400000000000001</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>0.1113</v>
+        <v>0.112</v>
       </c>
     </row>
     <row r="15">
@@ -1187,47 +1187,47 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>18587.95</v>
+        <v>18677.6</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>-0.0316</v>
+        <v>-0.0183</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>-0.0105</v>
+        <v>-0.0058</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>-0.07769999999999999</v>
+        <v>-0.0621</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>-0.07049999999999999</v>
+        <v>-0.075</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>0.005</v>
+        <v>-0.0038</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>-0.1203</v>
+        <v>-0.1161</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>0.0153</v>
+        <v>0.0202</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>-0.0721</v>
+        <v>-0.0692</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>-0.0683</v>
+        <v>-0.05110000000000001</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>0.0731</v>
+        <v>0.07690000000000001</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>0.06419999999999999</v>
+        <v>0.0658</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>0.1042</v>
+        <v>0.1052</v>
       </c>
     </row>
     <row r="16">
@@ -1238,47 +1238,47 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>5261.85</v>
+        <v>5286.75</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>-0.0289</v>
+        <v>-0.0172</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>-0.011</v>
+        <v>-0.0063</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>-0.0762</v>
+        <v>-0.0585</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>-0.0413</v>
+        <v>-0.0473</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>0.0208</v>
+        <v>0.0151</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>-0.1021</v>
+        <v>-0.0978</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>0.0454</v>
+        <v>0.0504</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>-0.0583</v>
+        <v>-0.05599999999999999</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>-0.0843</v>
+        <v>-0.0683</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0.0587</v>
+        <v>0.0601</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>0.0558</v>
+        <v>0.0559</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>0.0898</v>
+        <v>0.0907</v>
       </c>
     </row>
     <row r="17">
@@ -1289,47 +1289,47 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>24461.55</v>
+        <v>24684.71</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>-0.0442</v>
+        <v>-0.0144</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>-0.0179</v>
+        <v>-0.009000000000000001</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>-0.0581</v>
+        <v>-0.0557</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>-0.0825</v>
+        <v>-0.07389999999999999</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>-0.0219</v>
+        <v>-0.0258</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>-0.04559999999999999</v>
+        <v>-0.0369</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>-0.005</v>
+        <v>0.004099999999999999</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>0.0575</v>
+        <v>0.0565</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>-0.004</v>
+        <v>0.0159</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>0.2045</v>
+        <v>0.2163</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>0.2236</v>
+        <v>0.2229</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>0.1594</v>
+        <v>0.1579</v>
       </c>
     </row>
     <row r="18">
@@ -1340,47 +1340,47 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>36763.93</v>
+        <v>37055.49</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>-0.0341</v>
+        <v>-0.0054</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>-0.0103</v>
+        <v>-0.0024</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>-0.04940000000000001</v>
+        <v>-0.0411</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>-0.0503</v>
+        <v>-0.0393</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>0.06309999999999999</v>
+        <v>0.0483</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>-0.0562</v>
+        <v>-0.0487</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>0.08460000000000001</v>
+        <v>0.09320000000000001</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>-0.0244</v>
+        <v>-0.02</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>-0.1142</v>
+        <v>-0.09449999999999999</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>0.08810000000000001</v>
+        <v>0.09420000000000001</v>
       </c>
       <c r="N18" s="3" t="n">
         <v>0.091</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>0.1557</v>
+        <v>0.1556</v>
       </c>
     </row>
     <row r="19">
@@ -1391,47 +1391,47 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>27236.54</v>
+        <v>27383.55</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>-0.0293</v>
+        <v>-0.0177</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>-0.0073</v>
+        <v>-0.002</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>-0.0842</v>
+        <v>-0.065</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>-0.05110000000000001</v>
+        <v>-0.0544</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>0.0133</v>
+        <v>0.0069</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>-0.1105</v>
+        <v>-0.1057</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>0.042</v>
+        <v>0.0476</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>-0.0655</v>
+        <v>-0.0665</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>-0.08839999999999999</v>
+        <v>-0.07200000000000001</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>0.06370000000000001</v>
+        <v>0.06509999999999999</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>0.0622</v>
+        <v>0.0623</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>0.114</v>
+        <v>0.1156</v>
       </c>
     </row>
     <row r="20">
@@ -1442,47 +1442,47 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>29216.2</v>
+        <v>29447.9</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>-0.0343</v>
+        <v>-0.005600000000000001</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>-0.0103</v>
+        <v>-0.0024</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>-0.0501</v>
+        <v>-0.0414</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>-0.0529</v>
+        <v>-0.0416</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>0.0578</v>
+        <v>0.0431</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>-0.062</v>
+        <v>-0.0546</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>0.07919999999999999</v>
+        <v>0.08779999999999999</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>-0.0305</v>
+        <v>-0.0261</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>-0.1202</v>
+        <v>-0.1006</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>0.07919999999999999</v>
+        <v>0.08529999999999999</v>
       </c>
       <c r="N20" s="3" t="n">
         <v>0.0814</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>0.1447</v>
+        <v>0.1445</v>
       </c>
     </row>
     <row r="21">
@@ -1493,47 +1493,47 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>53855.85</v>
+        <v>54448.6</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>-0.022</v>
+        <v>0.0125</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>-0.004099999999999999</v>
+        <v>0.0068</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>-0.0498</v>
+        <v>-0.0347</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>0.0004</v>
+        <v>0.0101</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>0.1826</v>
+        <v>0.1737</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>0.07049999999999999</v>
+        <v>0.0823</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>0.2106</v>
+        <v>0.2239</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>0.0915</v>
+        <v>0.0968</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>-0.0555</v>
+        <v>-0.0353</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>0.1382</v>
+        <v>0.1445</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>0.1124</v>
+        <v>0.1099</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>0.1869</v>
+        <v>0.1882</v>
       </c>
     </row>
     <row r="22">
@@ -1544,47 +1544,47 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>24935.1</v>
+        <v>25011.5</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>-0.03759999999999999</v>
+        <v>-0.0257</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>-0.0113</v>
+        <v>-0.008199999999999999</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>-0.07440000000000001</v>
+        <v>-0.0612</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>-0.06370000000000001</v>
+        <v>-0.0718</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>0.0358</v>
+        <v>0.0254</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>-0.0791</v>
+        <v>-0.07629999999999999</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>0.0406</v>
+        <v>0.0438</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>-0.0471</v>
+        <v>-0.0461</v>
       </c>
       <c r="L22" s="3" t="n">
-        <v>-0.1049</v>
+        <v>-0.0907</v>
       </c>
       <c r="M22" s="3" t="n">
-        <v>0.07780000000000001</v>
+        <v>0.08210000000000001</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>0.0717</v>
+        <v>0.0721</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>0.111</v>
+        <v>0.1111</v>
       </c>
     </row>
     <row r="23">
@@ -1595,44 +1595,44 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>10133.27</v>
+        <v>10175.33</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>-0.0234</v>
+        <v>-0.005500000000000001</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>-0.0145</v>
+        <v>-0.0104</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>-0.0521</v>
+        <v>-0.0541</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>-0.04650000000000001</v>
+        <v>-0.0466</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>0.2049</v>
+        <v>0.1912</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>0.1858</v>
+        <v>0.1908</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>0.2695</v>
+        <v>0.2747</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>0.152</v>
+        <v>0.1346</v>
       </c>
       <c r="L23" s="3" t="n">
-        <v>0.1818</v>
+        <v>0.2017</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>0.4156</v>
+        <v>0.4135</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>0.5061</v>
+        <v>0.5022</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -1648,47 +1648,47 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>10897.19</v>
+        <v>11002.99</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>-0.0403</v>
+        <v>-0.0014</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>-0.0098</v>
+        <v>-0.0002</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>-0.0668</v>
+        <v>-0.0587</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>-0.0704</v>
+        <v>-0.0382</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>-0.0175</v>
+        <v>-0.0305</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>-0.0629</v>
+        <v>-0.0538</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>0.0151</v>
+        <v>0.0249</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>0.0664</v>
+        <v>0.06480000000000001</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>0.0911</v>
+        <v>0.1001</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>0.1549</v>
+        <v>0.1621</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>0.273</v>
+        <v>0.2765</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>0.1023</v>
+        <v>0.1026</v>
       </c>
     </row>
     <row r="25">
@@ -1699,47 +1699,47 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>76433.16</v>
+        <v>76802.85000000001</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>-0.0178</v>
+        <v>0.004500000000000001</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>-0.0033</v>
+        <v>0.0015</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>-0.0515</v>
+        <v>-0.0463</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>-0.06</v>
+        <v>-0.0596</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>0.06320000000000001</v>
+        <v>0.04679999999999999</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>-0.0801</v>
+        <v>-0.0757</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>0.0902</v>
+        <v>0.09539999999999998</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>-0.0097</v>
+        <v>-0.009300000000000001</v>
       </c>
       <c r="L25" s="3" t="n">
-        <v>0.0217</v>
+        <v>0.0386</v>
       </c>
       <c r="M25" s="3" t="n">
-        <v>0.0771</v>
+        <v>0.0809</v>
       </c>
       <c r="N25" s="3" t="n">
-        <v>0.0877</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="O25" s="3" t="n">
-        <v>0.1142</v>
+        <v>0.1158</v>
       </c>
     </row>
     <row r="26">
@@ -1750,47 +1750,47 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>31602.51</v>
+        <v>31627.25</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>-0.0025</v>
+        <v>0.0091</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.0001</v>
+        <v>0.0008</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>-0.0384</v>
+        <v>-0.0398</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>-0.0512</v>
+        <v>-0.0549</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>0.08890000000000001</v>
+        <v>0.0667</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>-0.0649</v>
+        <v>-0.0641</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>0.1124</v>
+        <v>0.1132</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>-0.004699999999999999</v>
+        <v>-0.0103</v>
       </c>
       <c r="L26" s="3" t="n">
-        <v>0.0101</v>
+        <v>0.0278</v>
       </c>
       <c r="M26" s="3" t="n">
-        <v>0.0561</v>
+        <v>0.0585</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>0.0738</v>
+        <v>0.0722</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>0.09939999999999999</v>
+        <v>0.101</v>
       </c>
     </row>
     <row r="27">
@@ -1801,47 +1801,47 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>31422.04</v>
+        <v>31550.39</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>-0.016</v>
+        <v>-0.0005999999999999999</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>-0.0038</v>
+        <v>0.0003</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>-0.0557</v>
+        <v>-0.0535</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>-0.08349999999999999</v>
+        <v>-0.08449999999999999</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>0.0295</v>
+        <v>0.0101</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>-0.103</v>
+        <v>-0.0993</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>0.05230000000000001</v>
+        <v>0.0566</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>-0.0608</v>
+        <v>-0.0585</v>
       </c>
       <c r="L27" s="3" t="n">
-        <v>0.0111</v>
+        <v>0.0313</v>
       </c>
       <c r="M27" s="3" t="n">
-        <v>0.08439999999999999</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>0.0725</v>
+        <v>0.07139999999999999</v>
       </c>
       <c r="O27" s="3" t="n">
-        <v>0.1259</v>
+        <v>0.1274</v>
       </c>
     </row>
     <row r="28">
@@ -1852,47 +1852,47 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>16687.41</v>
+        <v>16828.03</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>-0.036</v>
+        <v>-0.0108</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>-0.0162</v>
+        <v>-0.007900000000000001</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>-0.0436</v>
+        <v>-0.0433</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>-0.076</v>
+        <v>-0.0673</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>-0.0404</v>
+        <v>-0.0418</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>-0.0515</v>
+        <v>-0.0435</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>-0.0296</v>
+        <v>-0.0214</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>-0.0447</v>
+        <v>-0.0463</v>
       </c>
       <c r="L28" s="3" t="n">
-        <v>-0.076</v>
+        <v>-0.0558</v>
       </c>
       <c r="M28" s="3" t="n">
-        <v>0.1773</v>
+        <v>0.1876</v>
       </c>
       <c r="N28" s="3" t="n">
-        <v>0.2048</v>
+        <v>0.1997</v>
       </c>
       <c r="O28" s="3" t="n">
-        <v>0.1342</v>
+        <v>0.1332</v>
       </c>
     </row>
     <row r="29">
@@ -1903,47 +1903,47 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>930.72</v>
+        <v>935.95</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>-0.0306</v>
+        <v>-0.0131</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>-0.0146</v>
+        <v>-0.009000000000000001</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>-0.0629</v>
+        <v>-0.07490000000000001</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>-0.038</v>
+        <v>-0.0701</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>0.248</v>
+        <v>0.2275</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>-0.0445</v>
+        <v>-0.0392</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>0.2881</v>
+        <v>0.2953</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>-0.0436</v>
+        <v>-0.0371</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>-0.1241</v>
+        <v>-0.09420000000000001</v>
       </c>
       <c r="M29" s="3" t="n">
-        <v>0.1358</v>
+        <v>0.1306</v>
       </c>
       <c r="N29" s="3" t="n">
-        <v>0.1093</v>
+        <v>0.1125</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>0.1534</v>
+        <v>0.1528</v>
       </c>
     </row>
     <row r="30">
@@ -1954,47 +1954,47 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>33979.49</v>
+        <v>34028.98</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>-0.0503</v>
+        <v>-0.0416</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>-0.0346</v>
+        <v>-0.0332</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>-0.109</v>
+        <v>-0.08259999999999999</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>-0.0579</v>
+        <v>-0.0675</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>0.0629</v>
+        <v>0.05309999999999999</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>-0.0901</v>
+        <v>-0.0888</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>0.07730000000000001</v>
+        <v>0.0788</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>-0.0416</v>
+        <v>-0.0397</v>
       </c>
       <c r="L30" s="3" t="n">
-        <v>-0.0222</v>
+        <v>0.0001</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>0.172</v>
+        <v>0.1779</v>
       </c>
       <c r="N30" s="3" t="n">
-        <v>0.2019</v>
+        <v>0.2031</v>
       </c>
       <c r="O30" s="3" t="n">
-        <v>0.1063</v>
+        <v>0.1057</v>
       </c>
     </row>
     <row r="31">
@@ -2005,47 +2005,47 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>19959.81</v>
+        <v>19992.22</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>-0.0388</v>
+        <v>-0.0269</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>-0.0167</v>
+        <v>-0.0151</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>-0.0735</v>
+        <v>-0.0616</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>-0.0459</v>
+        <v>-0.0537</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>0.07769999999999999</v>
+        <v>0.0731</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>-0.0064</v>
+        <v>-0.004699999999999999</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>0.0892</v>
+        <v>0.091</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>0.0298</v>
+        <v>0.0259</v>
       </c>
       <c r="L31" s="3" t="n">
-        <v>-0.0068</v>
+        <v>0.0104</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>0.1653</v>
+        <v>0.1715</v>
       </c>
       <c r="N31" s="3" t="n">
-        <v>0.1494</v>
+        <v>0.1486</v>
       </c>
       <c r="O31" s="3" t="n">
-        <v>0.1316</v>
+        <v>0.1314</v>
       </c>
     </row>
     <row r="32">
@@ -2056,47 +2056,47 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>11366.58</v>
+        <v>11482.55</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>-0.038</v>
+        <v>-0.0102</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>-0.0147</v>
+        <v>-0.004699999999999999</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>-0.06509999999999999</v>
+        <v>-0.0549</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>-0.08689999999999999</v>
+        <v>-0.0839</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>0.003</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>-0.09880000000000001</v>
+        <v>-0.08960000000000001</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>0.0111</v>
+        <v>0.0215</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>-0.0384</v>
+        <v>-0.0339</v>
       </c>
       <c r="L32" s="3" t="n">
-        <v>-0.0429</v>
+        <v>-0.0171</v>
       </c>
       <c r="M32" s="3" t="n">
-        <v>0.122</v>
+        <v>0.127</v>
       </c>
       <c r="N32" s="3" t="n">
-        <v>0.1246</v>
+        <v>0.1253</v>
       </c>
       <c r="O32" s="3" t="n">
-        <v>0.1316</v>
+        <v>0.1331</v>
       </c>
     </row>
     <row r="33">
@@ -2107,47 +2107,47 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>19212.01</v>
+        <v>19019.93</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>-0.0395</v>
+        <v>-0.0364</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>-0.0026</v>
+        <v>-0.0126</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>-0.0345</v>
+        <v>-0.0289</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>-0.0013</v>
+        <v>-0.0313</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>0.1586</v>
+        <v>0.1446</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>0.1048</v>
+        <v>0.09380000000000001</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>0.1368</v>
+        <v>0.1254</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>0.1297</v>
+        <v>0.1208</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>0.0507</v>
+        <v>0.0532</v>
       </c>
       <c r="M33" s="3" t="n">
-        <v>0.1893</v>
+        <v>0.1937</v>
       </c>
       <c r="N33" s="3" t="n">
-        <v>0.1297</v>
+        <v>0.1301</v>
       </c>
       <c r="O33" s="3" t="n">
-        <v>0.1044</v>
+        <v>0.1049</v>
       </c>
     </row>
     <row r="34">
@@ -2158,47 +2158,47 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>19022.65</v>
+        <v>19087.15</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>-0.0442</v>
+        <v>-0.027</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>-0.0235</v>
+        <v>-0.0202</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>-0.0547</v>
+        <v>-0.06059999999999999</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>-0.0008</v>
+        <v>-0.0146</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>0.09539999999999998</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>0.1269</v>
+        <v>0.1308</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>0.1266</v>
+        <v>0.1305</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>0.2475</v>
+        <v>0.2293</v>
       </c>
       <c r="L34" s="3" t="n">
-        <v>0.1146</v>
+        <v>0.1224</v>
       </c>
       <c r="M34" s="3" t="n">
-        <v>0.2308</v>
+        <v>0.2386</v>
       </c>
       <c r="N34" s="3" t="n">
-        <v>0.1866</v>
+        <v>0.188</v>
       </c>
       <c r="O34" s="3" t="n">
-        <v>0.1927</v>
+        <v>0.1894</v>
       </c>
     </row>
     <row r="35">
@@ -2209,47 +2209,47 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>9440.35</v>
+        <v>9470.719999999999</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>-0.039</v>
+        <v>-0.0253</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>-0.0207</v>
+        <v>-0.0176</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>-0.0726</v>
+        <v>-0.0587</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>-0.0333</v>
+        <v>-0.0368</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>0.1256</v>
+        <v>0.1114</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>-0.0424</v>
+        <v>-0.0393</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>0.1545</v>
+        <v>0.1583</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>-0.0487</v>
+        <v>-0.0493</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>-0.07200000000000001</v>
+        <v>-0.053</v>
       </c>
       <c r="M35" s="3" t="n">
-        <v>0.106</v>
+        <v>0.1056</v>
       </c>
       <c r="N35" s="3" t="n">
-        <v>0.1084</v>
+        <v>0.1081</v>
       </c>
       <c r="O35" s="3" t="n">
-        <v>0.1103</v>
+        <v>0.1106</v>
       </c>
     </row>
     <row r="36">
@@ -2260,47 +2260,47 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>13608.31</v>
+        <v>13688.59</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>-0.0405</v>
+        <v>-0.0195</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>-0.0193</v>
+        <v>-0.0135</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>-0.0576</v>
+        <v>-0.06309999999999999</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>-0.0704</v>
+        <v>-0.0733</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>-0.0033</v>
+        <v>-0.005500000000000001</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>-0.0317</v>
+        <v>-0.026</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>0.0064</v>
+        <v>0.0123</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>0.0218</v>
+        <v>0.0216</v>
       </c>
       <c r="L36" s="3" t="n">
-        <v>-0.0247</v>
+        <v>-0.007800000000000001</v>
       </c>
       <c r="M36" s="3" t="n">
-        <v>0.1312</v>
+        <v>0.1411</v>
       </c>
       <c r="N36" s="3" t="n">
-        <v>0.1109</v>
+        <v>0.1095</v>
       </c>
       <c r="O36" s="3" t="n">
-        <v>0.1332</v>
+        <v>0.1317</v>
       </c>
     </row>
     <row r="37">
@@ -2311,47 +2311,47 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>72661.67</v>
+        <v>73972.19</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>-0.043</v>
+        <v>-0.0151</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>-0.0161</v>
+        <v>0.0016</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>-0.0574</v>
+        <v>-0.0286</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>-0.1232</v>
+        <v>-0.1093</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>-0.047</v>
+        <v>-0.0375</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>-0.205</v>
+        <v>-0.1907</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>-0.0325</v>
+        <v>-0.015</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>-0.198</v>
+        <v>-0.1845</v>
       </c>
       <c r="L37" s="3" t="n">
-        <v>-0.1702</v>
+        <v>-0.1489</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>-0.0378</v>
+        <v>-0.032</v>
       </c>
       <c r="N37" s="3" t="n">
-        <v>0.0333</v>
+        <v>0.0382</v>
       </c>
       <c r="O37" s="3" t="n">
-        <v>0.08960000000000001</v>
+        <v>0.092</v>
       </c>
     </row>
     <row r="38">
@@ -2362,47 +2362,47 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>5248.51</v>
+        <v>5289.21</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>-0.0298</v>
+        <v>-0.0037</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>-0.0171</v>
+        <v>-0.009399999999999999</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>-0.027</v>
+        <v>-0.0381</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>-0.1206</v>
+        <v>-0.1068</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>-0.0001</v>
+        <v>-0.0115</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>0.0214</v>
+        <v>0.0294</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>0.0089</v>
+        <v>0.0167</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>-0.0244</v>
+        <v>-0.0261</v>
       </c>
       <c r="L38" s="3" t="n">
-        <v>-0.118</v>
+        <v>-0.1011</v>
       </c>
       <c r="M38" s="3" t="n">
-        <v>0.1207</v>
+        <v>0.1323</v>
       </c>
       <c r="N38" s="3" t="n">
-        <v>0.1236</v>
+        <v>0.1201</v>
       </c>
       <c r="O38" s="3" t="n">
-        <v>0.1174</v>
+        <v>0.1178</v>
       </c>
     </row>
     <row r="39">
@@ -2413,47 +2413,47 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>5681.28</v>
+        <v>5697.3</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>-0.0288</v>
+        <v>-0.0145</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>-0.008199999999999999</v>
+        <v>-0.0054</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>-0.0698</v>
+        <v>-0.0597</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>-0.0541</v>
+        <v>-0.0607</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>0.0303</v>
+        <v>0.0185</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>-0.0951</v>
+        <v>-0.0926</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>0.053</v>
+        <v>0.05599999999999999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>-0.0461</v>
+        <v>-0.0449</v>
       </c>
       <c r="L39" s="3" t="n">
-        <v>-0.0428</v>
+        <v>-0.0268</v>
       </c>
       <c r="M39" s="3" t="n">
-        <v>0.08779999999999999</v>
+        <v>0.0876</v>
       </c>
       <c r="N39" s="3" t="n">
-        <v>0.0654</v>
+        <v>0.0646</v>
       </c>
       <c r="O39" s="3" t="n">
-        <v>0.1246</v>
+        <v>0.1254</v>
       </c>
     </row>
     <row r="40">
@@ -2464,47 +2464,47 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>16127.94</v>
+        <v>16183.18</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>-0.0362</v>
+        <v>-0.0139</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>-0.013</v>
+        <v>-0.009599999999999999</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>-0.0588</v>
+        <v>-0.0603</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>-0.057</v>
+        <v>-0.0646</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>-0.03</v>
+        <v>-0.0132</v>
       </c>
       <c r="I40" s="3" t="n">
-        <v>-0.1381</v>
+        <v>-0.1351</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>-0.025</v>
+        <v>-0.0217</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>-0.0665</v>
+        <v>-0.06900000000000001</v>
       </c>
       <c r="L40" s="3" t="n">
-        <v>-0.0919</v>
+        <v>-0.0727</v>
       </c>
       <c r="M40" s="3" t="n">
-        <v>0.1081</v>
+        <v>0.115</v>
       </c>
       <c r="N40" s="3" t="n">
-        <v>0.0738</v>
+        <v>0.06860000000000001</v>
       </c>
       <c r="O40" s="3" t="n">
-        <v>0.1339</v>
+        <v>0.1306</v>
       </c>
     </row>
     <row r="41">
@@ -2515,47 +2515,47 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>64436.87</v>
+        <v>64802.57</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>-0.0259</v>
+        <v>-0.0026</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>-0.0067</v>
+        <v>-0.001</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>-0.035</v>
+        <v>-0.0386</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>-0.0789</v>
+        <v>-0.0684</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>0.0372</v>
+        <v>0.0404</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>0.0404</v>
+        <v>0.0463</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>0.0506</v>
+        <v>0.0565</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>0.0464</v>
+        <v>0.0466</v>
       </c>
       <c r="L41" s="3" t="n">
-        <v>-0.0751</v>
+        <v>-0.0548</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>0.115</v>
+        <v>0.1256</v>
       </c>
       <c r="N41" s="3" t="n">
-        <v>0.1131</v>
+        <v>0.1059</v>
       </c>
       <c r="O41" s="3" t="n">
-        <v>0.1614</v>
+        <v>0.1594</v>
       </c>
     </row>
     <row r="42">
@@ -2566,47 +2566,47 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>40877.44</v>
+        <v>40873.08</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>0.0034</v>
+        <v>0.0077</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>0.0217</v>
+        <v>0.0215</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>-0.1013</v>
+        <v>-0.078</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>0.05309999999999999</v>
+        <v>0.0409</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>-0.062</v>
+        <v>-0.06809999999999999</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>-0.2426</v>
+        <v>-0.2427</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>-0.0175</v>
+        <v>-0.0176</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>-0.1473</v>
+        <v>-0.1485</v>
       </c>
       <c r="L42" s="3" t="n">
-        <v>-0.1655</v>
+        <v>-0.1601</v>
       </c>
       <c r="M42" s="3" t="n">
-        <v>-0.0172</v>
+        <v>-0.023</v>
       </c>
       <c r="N42" s="3" t="n">
-        <v>-0.0208</v>
+        <v>-0.0225</v>
       </c>
       <c r="O42" s="3" t="n">
-        <v>0.1288</v>
+        <v>0.1302</v>
       </c>
     </row>
     <row r="43">
@@ -2617,47 +2617,47 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>7722.72</v>
+        <v>7773.95</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>-0.0027</v>
+        <v>0.0117</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>0.009300000000000001</v>
+        <v>0.016</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>0.0073</v>
+        <v>0.0072</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>0.032</v>
+        <v>0.0314</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>0.1732</v>
+        <v>0.1758</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>0.1281</v>
+        <v>0.1356</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>0.1829</v>
+        <v>0.1908</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>0.15</v>
+        <v>0.1576</v>
       </c>
       <c r="L43" s="3" t="n">
-        <v>0.1631</v>
+        <v>0.1625</v>
       </c>
       <c r="M43" s="3" t="n">
-        <v>0.2224</v>
+        <v>0.2176</v>
       </c>
       <c r="N43" s="3" t="n">
-        <v>0.1212</v>
+        <v>0.1225</v>
       </c>
       <c r="O43" s="3" t="n">
-        <v>0.1365</v>
+        <v>0.1371</v>
       </c>
     </row>
     <row r="44">
@@ -2668,47 +2668,47 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>30807.93</v>
+        <v>31076.44</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>0.006500000000000001</v>
+        <v>0.0264</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>0.0131</v>
+        <v>0.022</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>0.0571</v>
+        <v>0.0519</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>0.0504</v>
+        <v>0.0464</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>0.2812</v>
+        <v>0.2846</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>0.2201</v>
+        <v>0.2308</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>0.2977</v>
+        <v>0.309</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>0.2376</v>
+        <v>0.2538</v>
       </c>
       <c r="L44" s="3" t="n">
-        <v>0.2475</v>
+        <v>0.2452</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>0.2839</v>
+        <v>0.2758</v>
       </c>
       <c r="N44" s="3" t="n">
-        <v>0.158</v>
+        <v>0.1606</v>
       </c>
       <c r="O44" s="3" t="n">
-        <v>0.203</v>
+        <v>0.2039</v>
       </c>
     </row>
     <row r="45">
@@ -2719,47 +2719,47 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
-        <v>68309.46000000001</v>
+        <v>70772.67</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>0.0293</v>
+        <v>0.0808</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>0.0233</v>
+        <v>0.0602</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>0.0619</v>
+        <v>0.0885</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>-0.0206</v>
+        <v>0.0369</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>0.2859</v>
+        <v>0.3246</v>
       </c>
       <c r="I45" s="3" t="n">
-        <v>0.357</v>
+        <v>0.4059</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>0.3377000000000001</v>
+        <v>0.386</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>0.5201</v>
+        <v>0.4761</v>
       </c>
       <c r="L45" s="3" t="n">
-        <v>0.3444</v>
+        <v>0.3526</v>
       </c>
       <c r="M45" s="3" t="n">
-        <v>0.2982</v>
+        <v>0.3167</v>
       </c>
       <c r="N45" s="3" t="n">
-        <v>0.1887</v>
+        <v>0.2067</v>
       </c>
       <c r="O45" s="3" t="n">
-        <v>0.1511</v>
+        <v>0.1543</v>
       </c>
     </row>
     <row r="46">
@@ -2770,47 +2770,47 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>25231.2</v>
+        <v>25254.21</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>-0.006999999999999999</v>
+        <v>-0.004699999999999999</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>0.0013</v>
+        <v>0.0022</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>-0.0235</v>
+        <v>-0.0304</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>-0.0213</v>
+        <v>-0.0218</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>0.0891</v>
+        <v>0.09</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>0.0302</v>
+        <v>0.0312</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>0.1125</v>
+        <v>0.1135</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>0.0331</v>
+        <v>0.0359</v>
       </c>
       <c r="L46" s="3" t="n">
-        <v>0.1475</v>
+        <v>0.1491</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>0.1872</v>
+        <v>0.1838</v>
       </c>
       <c r="N46" s="3" t="n">
-        <v>0.1073</v>
+        <v>0.1103</v>
       </c>
       <c r="O46" s="3" t="n">
-        <v>0.09050000000000001</v>
+        <v>0.0919</v>
       </c>
     </row>
     <row r="47">
@@ -2821,47 +2821,47 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>7897.19</v>
+        <v>7834.1</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>-0.0224</v>
+        <v>-0.0303</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>-0.008500000000000001</v>
+        <v>-0.0164</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>-0.0463</v>
+        <v>-0.0537</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>-0.0718</v>
+        <v>-0.0762</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>-0.008199999999999999</v>
+        <v>-0.0161</v>
       </c>
       <c r="I47" s="3" t="n">
-        <v>-0.031</v>
+        <v>-0.0387</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>0.0103</v>
+        <v>0.0022</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>-0.0198</v>
+        <v>-0.0306</v>
       </c>
       <c r="L47" s="3" t="n">
-        <v>0.0209</v>
+        <v>0.0192</v>
       </c>
       <c r="M47" s="3" t="n">
-        <v>0.0412</v>
+        <v>0.0353</v>
       </c>
       <c r="N47" s="3" t="n">
-        <v>0.0391</v>
+        <v>0.0383</v>
       </c>
       <c r="O47" s="3" t="n">
-        <v>0.0578</v>
+        <v>0.0582</v>
       </c>
     </row>
     <row r="48">
@@ -2872,47 +2872,47 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>10462</v>
+        <v>10497.9</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>-0.0218</v>
+        <v>-0.0175</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>-0.0136</v>
+        <v>-0.0102</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>-0.0274</v>
+        <v>-0.0308</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>-0.0203</v>
+        <v>-0.0144</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>0.0025</v>
+        <v>0.0059</v>
       </c>
       <c r="I48" s="3" t="n">
-        <v>0.0534</v>
+        <v>0.057</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>0.0281</v>
+        <v>0.0316</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>0.1097</v>
+        <v>0.1061</v>
       </c>
       <c r="L48" s="3" t="n">
-        <v>0.1234</v>
+        <v>0.1259</v>
       </c>
       <c r="M48" s="3" t="n">
-        <v>0.1189</v>
+        <v>0.119</v>
       </c>
       <c r="N48" s="3" t="n">
-        <v>0.0828</v>
+        <v>0.08460000000000001</v>
       </c>
       <c r="O48" s="3" t="n">
-        <v>0.0399</v>
+        <v>0.0407</v>
       </c>
     </row>
     <row r="49">
@@ -2923,47 +2923,47 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>23972.29</v>
+        <v>24187.73</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>-0.0219</v>
+        <v>-0.0137</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>-0.026</v>
+        <v>-0.0173</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>-0.0529</v>
+        <v>-0.057</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>0.0266</v>
+        <v>0.0294</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>-0.04559999999999999</v>
+        <v>-0.03700000000000001</v>
       </c>
       <c r="I49" s="3" t="n">
-        <v>-0.06469999999999999</v>
+        <v>-0.0563</v>
       </c>
       <c r="J49" s="3" t="n">
-        <v>-0.0329</v>
+        <v>-0.0242</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>-0.1215</v>
+        <v>-0.1028</v>
       </c>
       <c r="L49" s="3" t="n">
-        <v>0.0335</v>
+        <v>0.0313</v>
       </c>
       <c r="M49" s="3" t="n">
-        <v>0.1143</v>
+        <v>0.1142</v>
       </c>
       <c r="N49" s="3" t="n">
-        <v>-0.005</v>
+        <v>-0.0042</v>
       </c>
       <c r="O49" s="3" t="n">
-        <v>0.0012</v>
+        <v>0.0014</v>
       </c>
     </row>
     <row r="50">
@@ -3025,44 +3025,44 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>96.3</v>
+        <v>96.44</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>0.005</v>
+        <v>0.004699999999999999</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>0.0026</v>
+        <v>0.004</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>0.0191</v>
+        <v>0.0206</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>0.008100000000000001</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>0.0358</v>
+        <v>0.039</v>
       </c>
       <c r="I51" s="3" t="n">
-        <v>0.0727</v>
+        <v>0.07429999999999999</v>
       </c>
       <c r="J51" s="3" t="n">
-        <v>0.0206</v>
+        <v>0.0221</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>0.08539999999999999</v>
+        <v>0.0868</v>
       </c>
       <c r="L51" s="3" t="n">
-        <v>0.0707</v>
+        <v>0.0713</v>
       </c>
       <c r="M51" s="3" t="n">
-        <v>0.0489</v>
+        <v>0.0503</v>
       </c>
       <c r="N51" s="3" t="n">
-        <v>0.0525</v>
+        <v>0.05230000000000001</v>
       </c>
       <c r="O51" s="3" t="n">
         <v>0.03759999999999999</v>
@@ -3076,47 +3076,47 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>4162.3</v>
+        <v>4145.1</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>-0.0368</v>
+        <v>-0.0083</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>-0.0058</v>
+        <v>-0.009899999999999999</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>-0.0467</v>
+        <v>-0.0643</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>0.0121</v>
+        <v>-0</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>-0.1052</v>
+        <v>-0.1099</v>
       </c>
       <c r="I52" s="3" t="n">
-        <v>-0.0378</v>
+        <v>-0.0417</v>
       </c>
       <c r="J52" s="3" t="n">
-        <v>-0.1044</v>
+        <v>-0.1081</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.0498</v>
       </c>
       <c r="L52" s="3" t="n">
-        <v>0.2541</v>
+        <v>0.2511</v>
       </c>
       <c r="M52" s="3" t="n">
-        <v>0.3166</v>
+        <v>0.3132</v>
       </c>
       <c r="N52" s="3" t="n">
-        <v>0.1882</v>
+        <v>0.1873</v>
       </c>
       <c r="O52" s="3" t="n">
-        <v>0.1265</v>
+        <v>0.1275</v>
       </c>
     </row>
     <row r="53">
@@ -3127,47 +3127,47 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>60.42</v>
+        <v>60.72</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>-0.0677</v>
+        <v>0.0009</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>0.0053</v>
+        <v>0.0103</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.08070000000000001</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>-0.0038</v>
+        <v>-0.0035</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>-0.1694</v>
+        <v>-0.1546</v>
       </c>
       <c r="I53" s="3" t="n">
-        <v>-0.1386</v>
+        <v>-0.1342</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>-0.1911</v>
+        <v>-0.187</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>0.3134</v>
+        <v>0.2628</v>
       </c>
       <c r="L53" s="3" t="n">
-        <v>0.3824</v>
+        <v>0.3739</v>
       </c>
       <c r="M53" s="3" t="n">
-        <v>0.4186</v>
+        <v>0.4125</v>
       </c>
       <c r="N53" s="3" t="n">
-        <v>0.2182</v>
+        <v>0.2184</v>
       </c>
       <c r="O53" s="3" t="n">
-        <v>0.1306</v>
+        <v>0.1337</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Weekly indices update 2026-10-11
</commit_message>
<xml_diff>
--- a/tracker_auto.xlsx
+++ b/tracker_auto.xlsx
@@ -524,47 +524,47 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>22555.75</v>
+        <v>22520.45</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>-0.009899999999999999</v>
+        <v>0.0044</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-0.0029</v>
+        <v>-0.0044</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>-0.0562</v>
+        <v>-0.0389</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>-0.0767</v>
+        <v>-0.0697</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>-0.018</v>
+        <v>-0.0636</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>-0.1368</v>
+        <v>-0.1381</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.01</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>-0.09390000000000001</v>
+        <v>-0.1057</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>-0.0504</v>
+        <v>-0.0506</v>
       </c>
       <c r="M2" s="3" t="n">
+        <v>0.0458</v>
+      </c>
+      <c r="N2" s="3" t="n">
         <v>0.047</v>
       </c>
-      <c r="N2" s="3" t="n">
-        <v>0.0504</v>
-      </c>
       <c r="O2" s="3" t="n">
-        <v>0.1001</v>
+        <v>0.09970000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -575,47 +575,47 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>72789.24000000001</v>
+        <v>72472.33</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.0036</v>
+        <v>0.007800000000000001</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.0043</v>
+        <v>-0.0001</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>-0.0487</v>
+        <v>-0.0307</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>-0.06900000000000001</v>
+        <v>-0.06570000000000001</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>-0.0245</v>
+        <v>-0.0655</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>-0.1459</v>
+        <v>-0.1496</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>0.0117</v>
+        <v>0.0073</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>-0.11</v>
+        <v>-0.118</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>-0.0559</v>
+        <v>-0.05690000000000001</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>0.0332</v>
+        <v>0.0313</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>0.0405</v>
+        <v>0.0383</v>
       </c>
       <c r="O3" s="3" t="n">
-        <v>0.1001</v>
+        <v>0.09949999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -626,47 +626,47 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>69213.75</v>
+        <v>68166.7</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>-0.0156</v>
+        <v>-0.0118</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>-0.0076</v>
+        <v>-0.0227</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>-0.0503</v>
+        <v>-0.0643</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>-0.0478</v>
+        <v>-0.0584</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.1011</v>
+        <v>0.007800000000000001</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>-0.0022</v>
+        <v>-0.0173</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.1469</v>
+        <v>0.1295</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>0.0125</v>
+        <v>-0.0052</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>-0.0369</v>
+        <v>-0.0493</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>0.1549</v>
+        <v>0.1485</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>0.1004</v>
+        <v>0.0951</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>0.1135</v>
+        <v>0.112</v>
       </c>
     </row>
     <row r="5">
@@ -677,47 +677,47 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>23645.3</v>
+        <v>23547.9</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>-0.0109</v>
+        <v>0.0013</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>-0.0038</v>
+        <v>-0.007900000000000001</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>-0.0551</v>
+        <v>-0.0437</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>-0.07139999999999999</v>
+        <v>-0.06759999999999999</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>0.0028</v>
+        <v>-0.0509</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>-0.1141</v>
+        <v>-0.1177</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0.0337</v>
+        <v>0.0294</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>-0.07519999999999999</v>
+        <v>-0.0882</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>-0.0474</v>
+        <v>-0.0498</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>0.0649</v>
+        <v>0.06280000000000001</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>0.0572</v>
+        <v>0.0535</v>
       </c>
       <c r="O5" s="3" t="n">
-        <v>0.1019</v>
+        <v>0.1013</v>
       </c>
     </row>
     <row r="6">
@@ -728,47 +728,47 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>30700.05</v>
+        <v>30516.35</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>-0.0173</v>
+        <v>-0.0005</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-0.0066</v>
+        <v>-0.0126</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-0.0579</v>
+        <v>-0.0508</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>-0.07240000000000001</v>
+        <v>-0.0693</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.008699999999999999</v>
+        <v>-0.0424</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>-0.0789</v>
+        <v>-0.08439999999999999</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.0387</v>
+        <v>0.0325</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>-0.0383</v>
+        <v>-0.05309999999999999</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>-0.0257</v>
+        <v>-0.0279</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>0.09359999999999999</v>
+        <v>0.09029999999999999</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>0.09210000000000002</v>
+        <v>0.08810000000000001</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>0.1087</v>
+        <v>0.1077</v>
       </c>
     </row>
     <row r="7">
@@ -779,47 +779,47 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>32626.5</v>
+        <v>32292.15</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>-0.0165</v>
+        <v>-0.0061</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-0.0071</v>
+        <v>-0.0173</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>-0.0571</v>
+        <v>-0.0583</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>-0.0624</v>
+        <v>-0.0667</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.0562</v>
+        <v>-0.0157</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>-0.0391</v>
+        <v>-0.049</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>0.0953</v>
+        <v>0.08410000000000001</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>-0.0155</v>
+        <v>-0.0309</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>-0.0245</v>
+        <v>-0.031</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>0.1219</v>
+        <v>0.1177</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>0.0926</v>
+        <v>0.08789999999999999</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>0.1072</v>
+        <v>0.1059</v>
       </c>
     </row>
     <row r="8">
@@ -830,47 +830,47 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>17658.75</v>
+        <v>17580.4</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>-0.0113</v>
+        <v>0.0013</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-0.0037</v>
+        <v>-0.008100000000000001</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-0.0565</v>
+        <v>-0.0471</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>-0.0653</v>
+        <v>-0.06519999999999999</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.0251</v>
+        <v>-0.0317</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>-0.0897</v>
+        <v>-0.09369999999999999</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.0574</v>
+        <v>0.0528</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>-0.0472</v>
+        <v>-0.0619</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>-0.0277</v>
+        <v>-0.0311</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>0.08800000000000001</v>
+        <v>0.0859</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>0.08130000000000001</v>
+        <v>0.0771</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>0.1211</v>
+        <v>0.1205</v>
       </c>
     </row>
     <row r="9">
@@ -881,47 +881,47 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>15687.65</v>
+        <v>15600.55</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>-0.0127</v>
+        <v>-0.0003</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-0.0044</v>
+        <v>-0.01</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-0.0581</v>
+        <v>-0.0522</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>-0.0623</v>
+        <v>-0.0675</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>0.0426</v>
+        <v>-0.0183</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>-0.0693</v>
+        <v>-0.07440000000000001</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>0.0764</v>
+        <v>0.0704</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>-0.0298</v>
+        <v>-0.0457</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>-0.0225</v>
+        <v>-0.0278</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>0.09810000000000001</v>
+        <v>0.096</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>0.09710000000000001</v>
+        <v>0.09179999999999999</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>0.1281</v>
+        <v>0.1273</v>
       </c>
     </row>
     <row r="10">
@@ -932,47 +932,47 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>21755.3</v>
+        <v>21603.25</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>-0.0143</v>
+        <v>-0.0019</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>-0.0051</v>
+        <v>-0.0121</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>-0.061</v>
+        <v>-0.0604</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>-0.053</v>
+        <v>-0.0675</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.08289999999999999</v>
+        <v>0.0142</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>-0.0234</v>
+        <v>-0.0302</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.1196</v>
+        <v>0.1118</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>0.0166</v>
+        <v>-0.0024</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>0.001</v>
+        <v>-0.0072</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>0.1304</v>
+        <v>0.1282</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0.1361</v>
+        <v>0.1291</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>0.1524</v>
+        <v>0.1515</v>
       </c>
     </row>
     <row r="11">
@@ -983,47 +983,47 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>17655.35</v>
+        <v>17574.85</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>-0.0116</v>
+        <v>-0.0008</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>-0.008100000000000001</v>
+        <v>-0.0126</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>-0.0447</v>
+        <v>-0.04650000000000001</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>-0.0234</v>
+        <v>-0.03</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0.1864</v>
+        <v>0.1156</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>0.0582</v>
+        <v>0.0533</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>0.2356</v>
+        <v>0.23</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>0.03759999999999999</v>
+        <v>0.0333</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>-0.0102</v>
+        <v>-0.0147</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>0.1276</v>
+        <v>0.1279</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>0.1321</v>
+        <v>0.1265</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>0.1321</v>
+        <v>0.1314</v>
       </c>
     </row>
     <row r="12">
@@ -1034,47 +1034,47 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>20289.05</v>
+        <v>20164.7</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>-0.0134</v>
+        <v>-0.0015</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>-0.0062</v>
+        <v>-0.0123</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>-0.0554</v>
+        <v>-0.0556</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>-0.0429</v>
+        <v>-0.0547</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.1171</v>
+        <v>0.04769999999999999</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>0.0035</v>
+        <v>-0.0026</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0.1578</v>
+        <v>0.1507</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>0.0231</v>
+        <v>0.0092</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>-0.0035</v>
+        <v>-0.0104</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0.1291</v>
+        <v>0.1277</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.1349</v>
+        <v>0.1284</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>0.1457</v>
+        <v>0.1449</v>
       </c>
     </row>
     <row r="13">
@@ -1085,47 +1085,47 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>21971.6</v>
+        <v>21866.65</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>-0.0117</v>
+        <v>0.0004</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>-0.0046</v>
+        <v>-0.009300000000000001</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>-0.0552</v>
+        <v>-0.0476</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>-0.0624</v>
+        <v>-0.0635</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>0.0367</v>
+        <v>-0.0215</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>-0.0796</v>
+        <v>-0.08400000000000001</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>0.0703</v>
+        <v>0.06519999999999999</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>-0.0459</v>
+        <v>-0.0592</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>-0.0338</v>
+        <v>-0.0374</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>0.08310000000000001</v>
+        <v>0.08119999999999999</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>0.0775</v>
+        <v>0.0731</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>0.1132</v>
+        <v>0.1125</v>
       </c>
     </row>
     <row r="14">
@@ -1136,47 +1136,47 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>34387.91</v>
+        <v>34192.47</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>-0.0115</v>
+        <v>-0.0008</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>-0.0051</v>
+        <v>-0.0108</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>-0.0549</v>
+        <v>-0.0481</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>-0.06150000000000001</v>
+        <v>-0.0634</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0.0348</v>
+        <v>-0.0232</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>-0.08160000000000001</v>
+        <v>-0.0868</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>0.06849999999999999</v>
+        <v>0.0625</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>-0.0491</v>
+        <v>-0.0629</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>-0.0371</v>
+        <v>-0.0413</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0.07870000000000001</v>
+        <v>0.0765</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>0.07400000000000001</v>
+        <v>0.06950000000000001</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>0.112</v>
+        <v>0.1112</v>
       </c>
     </row>
     <row r="15">
@@ -1187,47 +1187,47 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>18677.6</v>
+        <v>18625.4</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>-0.0183</v>
+        <v>0.002</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>-0.0058</v>
+        <v>-0.008500000000000001</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>-0.0621</v>
+        <v>-0.045</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>-0.075</v>
+        <v>-0.07150000000000001</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>-0.0038</v>
+        <v>-0.04769999999999999</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>-0.1161</v>
+        <v>-0.1185</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>0.0202</v>
+        <v>0.0173</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>-0.0692</v>
+        <v>-0.0832</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>-0.05110000000000001</v>
+        <v>-0.052</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>0.07690000000000001</v>
+        <v>0.0757</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>0.0658</v>
+        <v>0.0639</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>0.1052</v>
+        <v>0.1045</v>
       </c>
     </row>
     <row r="16">
@@ -1238,47 +1238,47 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>5286.75</v>
+        <v>5264.7</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>-0.0172</v>
+        <v>0.0005</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>-0.0063</v>
+        <v>-0.0105</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>-0.0585</v>
+        <v>-0.052</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>-0.0473</v>
+        <v>-0.0417</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>0.0151</v>
+        <v>-0.0323</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>-0.0978</v>
+        <v>-0.1016</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>0.0504</v>
+        <v>0.046</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>-0.05599999999999999</v>
+        <v>-0.0687</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>-0.0683</v>
+        <v>-0.0722</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0.0601</v>
+        <v>0.0567</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>0.0559</v>
+        <v>0.052</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>0.0907</v>
+        <v>0.08960000000000001</v>
       </c>
     </row>
     <row r="17">
@@ -1289,47 +1289,47 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>24684.71</v>
+        <v>24413.16</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>-0.0144</v>
+        <v>-0.002</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>-0.009000000000000001</v>
+        <v>-0.0199</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>-0.0557</v>
+        <v>-0.0596</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>-0.07389999999999999</v>
+        <v>-0.0771</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>-0.0258</v>
+        <v>-0.08550000000000001</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>-0.0369</v>
+        <v>-0.0475</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>0.004099999999999999</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>0.0565</v>
+        <v>0.0392</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>0.0159</v>
+        <v>0.0199</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>0.2163</v>
+        <v>0.2102</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>0.2229</v>
+        <v>0.2198</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>0.1579</v>
+        <v>0.1566</v>
       </c>
     </row>
     <row r="18">
@@ -1340,47 +1340,47 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>37055.49</v>
+        <v>36740.35</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>-0.0054</v>
+        <v>-0.0005999999999999999</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>-0.0024</v>
+        <v>-0.0109</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>-0.0411</v>
+        <v>-0.0622</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>-0.0393</v>
+        <v>-0.0441</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>0.0483</v>
+        <v>-0.0384</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>-0.0487</v>
+        <v>-0.0568</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>0.09320000000000001</v>
+        <v>0.0839</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>-0.02</v>
+        <v>-0.0525</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>-0.09449999999999999</v>
+        <v>-0.1082</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>0.09420000000000001</v>
+        <v>0.0897</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>0.091</v>
+        <v>0.0843</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>0.1556</v>
+        <v>0.154</v>
       </c>
     </row>
     <row r="19">
@@ -1391,47 +1391,47 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>27383.55</v>
+        <v>27322.67</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>-0.0177</v>
+        <v>0.0032</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>-0.002</v>
+        <v>-0.0042</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>-0.065</v>
+        <v>-0.0525</v>
       </c>
       <c r="G19" s="3" t="n">
         <v>-0.0544</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>0.0069</v>
+        <v>-0.0366</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>-0.1057</v>
+        <v>-0.1077</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>0.0476</v>
+        <v>0.0453</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>-0.0665</v>
+        <v>-0.07919999999999999</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>-0.07200000000000001</v>
+        <v>-0.0767</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>0.06509999999999999</v>
+        <v>0.0621</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>0.0623</v>
+        <v>0.05860000000000001</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>0.1156</v>
+        <v>0.1149</v>
       </c>
     </row>
     <row r="20">
@@ -1442,47 +1442,47 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>29447.9</v>
+        <v>29197.45</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>-0.005600000000000001</v>
+        <v>-0.0005999999999999999</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>-0.0024</v>
+        <v>-0.0109</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>-0.0414</v>
+        <v>-0.0624</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>-0.0416</v>
+        <v>-0.046</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>0.0431</v>
+        <v>-0.0432</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>-0.0546</v>
+        <v>-0.0626</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>0.08779999999999999</v>
+        <v>0.0785</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>-0.0261</v>
+        <v>-0.0585</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>-0.1006</v>
+        <v>-0.1142</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>0.08529999999999999</v>
+        <v>0.0808</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>0.0814</v>
+        <v>0.07480000000000001</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>0.1445</v>
+        <v>0.1429</v>
       </c>
     </row>
     <row r="21">
@@ -1493,47 +1493,47 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>54448.6</v>
+        <v>55339.9</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>0.0125</v>
+        <v>0.0276</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0.0068</v>
+        <v>0.0233</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>-0.0347</v>
+        <v>-0.0245</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>0.0101</v>
+        <v>0.0198</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>0.1737</v>
+        <v>0.1106</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>0.0823</v>
+        <v>0.1</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>0.2239</v>
+        <v>0.2439</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>0.0968</v>
+        <v>0.09539999999999998</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>-0.0353</v>
+        <v>-0.0384</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>0.1445</v>
+        <v>0.1521</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>0.1099</v>
+        <v>0.1084</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>0.1882</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="22">
@@ -1544,47 +1544,47 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>25011.5</v>
+        <v>24692.85</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>-0.0257</v>
+        <v>-0.0097</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>-0.008199999999999999</v>
+        <v>-0.0209</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>-0.0612</v>
+        <v>-0.0679</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>-0.0718</v>
+        <v>-0.0815</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>0.0254</v>
+        <v>-0.03700000000000001</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>-0.07629999999999999</v>
+        <v>-0.08800000000000001</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>0.0438</v>
+        <v>0.0305</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>-0.0461</v>
+        <v>-0.0704</v>
       </c>
       <c r="L22" s="3" t="n">
-        <v>-0.0907</v>
+        <v>-0.09759999999999999</v>
       </c>
       <c r="M22" s="3" t="n">
-        <v>0.08210000000000001</v>
+        <v>0.0764</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>0.0721</v>
+        <v>0.0665</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>0.1111</v>
+        <v>0.1093</v>
       </c>
     </row>
     <row r="23">
@@ -1595,44 +1595,44 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>10175.33</v>
+        <v>9982.65</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>-0.005500000000000001</v>
+        <v>-0.0149</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>-0.0104</v>
+        <v>-0.0291</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>-0.0541</v>
+        <v>-0.0892</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>-0.0466</v>
+        <v>-0.0493</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>0.1912</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>0.1908</v>
+        <v>0.1682</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>0.2747</v>
+        <v>0.2506</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>0.1346</v>
+        <v>0.1162</v>
       </c>
       <c r="L23" s="3" t="n">
-        <v>0.2017</v>
+        <v>0.1776</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>0.4135</v>
+        <v>0.4035</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>0.5022</v>
+        <v>0.4908</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -1648,47 +1648,47 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>11002.99</v>
+        <v>11156.08</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>-0.0014</v>
+        <v>0.0238</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>-0.0002</v>
+        <v>0.0138</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>-0.0587</v>
+        <v>-0.029</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>-0.0382</v>
+        <v>-0.0384</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>-0.0305</v>
+        <v>-0.0679</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>-0.0538</v>
+        <v>-0.0406</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>0.0249</v>
+        <v>0.0392</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>0.06480000000000001</v>
+        <v>0.08160000000000001</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>0.1001</v>
+        <v>0.1155</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>0.1621</v>
+        <v>0.1716</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>0.2765</v>
+        <v>0.2739</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>0.1026</v>
+        <v>0.105</v>
       </c>
     </row>
     <row r="25">
@@ -1699,47 +1699,47 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>76802.85000000001</v>
+        <v>77564.42</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>0.004500000000000001</v>
+        <v>0.0148</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>0.0015</v>
+        <v>0.0114</v>
       </c>
       <c r="F25" s="3" t="n">
+        <v>-0.0185</v>
+      </c>
+      <c r="G25" s="3" t="n">
         <v>-0.0463</v>
       </c>
-      <c r="G25" s="3" t="n">
-        <v>-0.0596</v>
-      </c>
       <c r="H25" s="3" t="n">
-        <v>0.04679999999999999</v>
+        <v>-0.0052</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>-0.0757</v>
+        <v>-0.0665</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>0.09539999999999998</v>
+        <v>0.1063</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>-0.009300000000000001</v>
+        <v>-0.0102</v>
       </c>
       <c r="L25" s="3" t="n">
-        <v>0.0386</v>
+        <v>0.0484</v>
       </c>
       <c r="M25" s="3" t="n">
-        <v>0.0809</v>
+        <v>0.08439999999999999</v>
       </c>
       <c r="N25" s="3" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.0876</v>
       </c>
       <c r="O25" s="3" t="n">
-        <v>0.1158</v>
+        <v>0.117</v>
       </c>
     </row>
     <row r="26">
@@ -1750,47 +1750,47 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>31627.25</v>
+        <v>32224.3</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>0.0091</v>
+        <v>0.0197</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.0008</v>
+        <v>0.0197</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>-0.0398</v>
+        <v>0.0003</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>-0.0549</v>
+        <v>-0.0282</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>0.0667</v>
+        <v>0.0226</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>-0.0641</v>
+        <v>-0.04650000000000001</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>0.1132</v>
+        <v>0.1343</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>-0.0103</v>
+        <v>-0.0048</v>
       </c>
       <c r="L26" s="3" t="n">
-        <v>0.0278</v>
+        <v>0.042</v>
       </c>
       <c r="M26" s="3" t="n">
-        <v>0.0585</v>
+        <v>0.0646</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>0.0722</v>
+        <v>0.0733</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>0.101</v>
+        <v>0.1031</v>
       </c>
     </row>
     <row r="27">
@@ -1801,47 +1801,47 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>31550.39</v>
+        <v>31949.76</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>-0.0005999999999999999</v>
+        <v>0.0168</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>0.0003</v>
+        <v>0.0129</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>-0.0535</v>
+        <v>-0.0161</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>-0.08449999999999999</v>
+        <v>-0.0675</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>0.0101</v>
+        <v>-0.04</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>-0.0993</v>
+        <v>-0.08789999999999999</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>0.0566</v>
+        <v>0.0699</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>-0.0585</v>
+        <v>-0.0572</v>
       </c>
       <c r="L27" s="3" t="n">
-        <v>0.0313</v>
+        <v>0.0396</v>
       </c>
       <c r="M27" s="3" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.09029999999999999</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>0.07139999999999999</v>
+        <v>0.07440000000000001</v>
       </c>
       <c r="O27" s="3" t="n">
-        <v>0.1274</v>
+        <v>0.1292</v>
       </c>
     </row>
     <row r="28">
@@ -1852,47 +1852,47 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>16828.03</v>
+        <v>16454.98</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>-0.0108</v>
+        <v>-0.0139</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>-0.007900000000000001</v>
+        <v>-0.0299</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>-0.0433</v>
+        <v>-0.06709999999999999</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>-0.0673</v>
+        <v>-0.0771</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>-0.0418</v>
+        <v>-0.1009</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>-0.0435</v>
+        <v>-0.06469999999999999</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>-0.0214</v>
+        <v>-0.0431</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>-0.0463</v>
+        <v>-0.0634</v>
       </c>
       <c r="L28" s="3" t="n">
-        <v>-0.0558</v>
+        <v>-0.0609</v>
       </c>
       <c r="M28" s="3" t="n">
-        <v>0.1876</v>
+        <v>0.1762</v>
       </c>
       <c r="N28" s="3" t="n">
-        <v>0.1997</v>
+        <v>0.1952</v>
       </c>
       <c r="O28" s="3" t="n">
-        <v>0.1332</v>
+        <v>0.1309</v>
       </c>
     </row>
     <row r="29">
@@ -1903,47 +1903,47 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>935.95</v>
+        <v>896.1</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>-0.0131</v>
+        <v>-0.0372</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>-0.009000000000000001</v>
+        <v>-0.0512</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>-0.07490000000000001</v>
+        <v>-0.0781</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>-0.0701</v>
+        <v>-0.1398</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>0.2275</v>
+        <v>0.0636</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>-0.0392</v>
+        <v>-0.0801</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>0.2953</v>
+        <v>0.2402</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>-0.0371</v>
+        <v>-0.08410000000000001</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>-0.09420000000000001</v>
+        <v>-0.1224</v>
       </c>
       <c r="M29" s="3" t="n">
-        <v>0.1306</v>
+        <v>0.1027</v>
       </c>
       <c r="N29" s="3" t="n">
-        <v>0.1125</v>
+        <v>0.09449999999999999</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>0.1528</v>
+        <v>0.1492</v>
       </c>
     </row>
     <row r="30">
@@ -1954,47 +1954,47 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>34028.98</v>
+        <v>33276.66</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>-0.0416</v>
+        <v>-0.0207</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>-0.0332</v>
+        <v>-0.0545</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>-0.08259999999999999</v>
+        <v>-0.101</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>-0.0675</v>
+        <v>-0.07139999999999999</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>0.05309999999999999</v>
+        <v>-0.0587</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>-0.0888</v>
+        <v>-0.109</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>0.0788</v>
+        <v>0.055</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>-0.0397</v>
+        <v>-0.055</v>
       </c>
       <c r="L30" s="3" t="n">
-        <v>0.0001</v>
+        <v>-0.0209</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>0.1779</v>
+        <v>0.1682</v>
       </c>
       <c r="N30" s="3" t="n">
-        <v>0.2031</v>
+        <v>0.1862</v>
       </c>
       <c r="O30" s="3" t="n">
-        <v>0.1057</v>
+        <v>0.1033</v>
       </c>
     </row>
     <row r="31">
@@ -2005,47 +2005,47 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>19992.22</v>
+        <v>19640.86</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>-0.0269</v>
+        <v>-0.016</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>-0.0151</v>
+        <v>-0.03240000000000001</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>-0.0616</v>
+        <v>-0.0775</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>-0.0537</v>
+        <v>-0.0599</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>0.0731</v>
+        <v>-0.0109</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>-0.004699999999999999</v>
+        <v>-0.0222</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>0.091</v>
+        <v>0.0718</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>0.0259</v>
+        <v>0.005600000000000001</v>
       </c>
       <c r="L31" s="3" t="n">
-        <v>0.0104</v>
+        <v>-0.0043</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>0.1715</v>
+        <v>0.1643</v>
       </c>
       <c r="N31" s="3" t="n">
-        <v>0.1486</v>
+        <v>0.1391</v>
       </c>
       <c r="O31" s="3" t="n">
-        <v>0.1314</v>
+        <v>0.1293</v>
       </c>
     </row>
     <row r="32">
@@ -2056,47 +2056,47 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>11482.55</v>
+        <v>11326.02</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>-0.0102</v>
+        <v>-0.0036</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>-0.004699999999999999</v>
+        <v>-0.0183</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>-0.0549</v>
+        <v>-0.05980000000000001</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>-0.0839</v>
+        <v>-0.0877</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>0.008800000000000001</v>
+        <v>-0.0539</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>-0.08960000000000001</v>
+        <v>-0.102</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>0.0215</v>
+        <v>0.0075</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>-0.0339</v>
+        <v>-0.0554</v>
       </c>
       <c r="L32" s="3" t="n">
-        <v>-0.0171</v>
+        <v>-0.0234</v>
       </c>
       <c r="M32" s="3" t="n">
-        <v>0.127</v>
+        <v>0.1218</v>
       </c>
       <c r="N32" s="3" t="n">
-        <v>0.1253</v>
+        <v>0.1193</v>
       </c>
       <c r="O32" s="3" t="n">
-        <v>0.1331</v>
+        <v>0.1319</v>
       </c>
     </row>
     <row r="33">
@@ -2107,47 +2107,47 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>19019.93</v>
+        <v>18925.52</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>-0.0364</v>
+        <v>-0.0149</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>-0.0126</v>
+        <v>-0.0175</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>-0.0289</v>
+        <v>-0.0438</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>-0.0313</v>
+        <v>-0.0285</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>0.1446</v>
+        <v>0.1203</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>0.09380000000000001</v>
+        <v>0.0883</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>0.1254</v>
+        <v>0.1199</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>0.1208</v>
+        <v>0.09179999999999999</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>0.0532</v>
+        <v>0.0347</v>
       </c>
       <c r="M33" s="3" t="n">
-        <v>0.1937</v>
+        <v>0.1922</v>
       </c>
       <c r="N33" s="3" t="n">
-        <v>0.1301</v>
+        <v>0.1279</v>
       </c>
       <c r="O33" s="3" t="n">
-        <v>0.1049</v>
+        <v>0.1037</v>
       </c>
     </row>
     <row r="34">
@@ -2158,47 +2158,47 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>19087.15</v>
+        <v>18327.77</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>-0.027</v>
+        <v>-0.0365</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>-0.0202</v>
+        <v>-0.0592</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>-0.06059999999999999</v>
+        <v>-0.1031</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>-0.0146</v>
+        <v>-0.053</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>0.08699999999999999</v>
+        <v>-0.0215</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>0.1308</v>
+        <v>0.0858</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>0.1305</v>
+        <v>0.08550000000000001</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>0.2293</v>
+        <v>0.1714</v>
       </c>
       <c r="L34" s="3" t="n">
-        <v>0.1224</v>
+        <v>0.1174</v>
       </c>
       <c r="M34" s="3" t="n">
-        <v>0.2386</v>
+        <v>0.2196</v>
       </c>
       <c r="N34" s="3" t="n">
-        <v>0.188</v>
+        <v>0.1759</v>
       </c>
       <c r="O34" s="3" t="n">
-        <v>0.1894</v>
+        <v>0.1826</v>
       </c>
     </row>
     <row r="35">
@@ -2209,47 +2209,47 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>9470.719999999999</v>
+        <v>9360.940000000001</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>-0.0253</v>
+        <v>-0.008399999999999999</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>-0.0176</v>
+        <v>-0.029</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>-0.0587</v>
+        <v>-0.063</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>-0.0368</v>
+        <v>-0.04679999999999999</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>0.1114</v>
+        <v>0.0283</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>-0.0393</v>
+        <v>-0.0505</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>0.1583</v>
+        <v>0.1448</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>-0.0493</v>
+        <v>-0.0595</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>-0.053</v>
+        <v>-0.0664</v>
       </c>
       <c r="M35" s="3" t="n">
-        <v>0.1056</v>
+        <v>0.1021</v>
       </c>
       <c r="N35" s="3" t="n">
-        <v>0.1081</v>
+        <v>0.0973</v>
       </c>
       <c r="O35" s="3" t="n">
-        <v>0.1106</v>
+        <v>0.1089</v>
       </c>
     </row>
     <row r="36">
@@ -2260,47 +2260,47 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>13688.59</v>
+        <v>13302.26</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>-0.0195</v>
+        <v>-0.0225</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>-0.0135</v>
+        <v>-0.0414</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>-0.06309999999999999</v>
+        <v>-0.08359999999999999</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>-0.0733</v>
+        <v>-0.09480000000000001</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>-0.005500000000000001</v>
+        <v>-0.0795</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>-0.026</v>
+        <v>-0.0534</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>0.0123</v>
+        <v>-0.0162</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>0.0216</v>
+        <v>-0.0124</v>
       </c>
       <c r="L36" s="3" t="n">
-        <v>-0.007800000000000001</v>
+        <v>-0.0122</v>
       </c>
       <c r="M36" s="3" t="n">
-        <v>0.1411</v>
+        <v>0.1296</v>
       </c>
       <c r="N36" s="3" t="n">
-        <v>0.1095</v>
+        <v>0.1014</v>
       </c>
       <c r="O36" s="3" t="n">
-        <v>0.1317</v>
+        <v>0.1281</v>
       </c>
     </row>
     <row r="37">
@@ -2311,47 +2311,47 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>73972.19</v>
+        <v>74444.39999999999</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>-0.0151</v>
+        <v>0.0245</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>0.0016</v>
+        <v>0.008</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>-0.0286</v>
+        <v>-0.0098</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>-0.1093</v>
+        <v>-0.0883</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>-0.0375</v>
+        <v>-0.0634</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>-0.1907</v>
+        <v>-0.1855</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>-0.015</v>
+        <v>-0.008699999999999999</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>-0.1845</v>
+        <v>-0.1723</v>
       </c>
       <c r="L37" s="3" t="n">
-        <v>-0.1489</v>
+        <v>-0.1392</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>-0.032</v>
+        <v>-0.0314</v>
       </c>
       <c r="N37" s="3" t="n">
-        <v>0.0382</v>
+        <v>0.0404</v>
       </c>
       <c r="O37" s="3" t="n">
-        <v>0.092</v>
+        <v>0.0925</v>
       </c>
     </row>
     <row r="38">
@@ -2362,47 +2362,47 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>5289.21</v>
+        <v>5118.36</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>-0.0037</v>
+        <v>-0.0248</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>-0.009399999999999999</v>
+        <v>-0.0414</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>-0.0381</v>
+        <v>-0.07580000000000001</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>-0.1068</v>
+        <v>-0.1307</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>-0.0115</v>
+        <v>-0.09050000000000001</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>0.0294</v>
+        <v>-0.0039</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>0.0167</v>
+        <v>-0.0162</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>-0.0261</v>
+        <v>-0.0475</v>
       </c>
       <c r="L38" s="3" t="n">
-        <v>-0.1011</v>
+        <v>-0.1106</v>
       </c>
       <c r="M38" s="3" t="n">
-        <v>0.1323</v>
+        <v>0.1241</v>
       </c>
       <c r="N38" s="3" t="n">
-        <v>0.1201</v>
+        <v>0.1134</v>
       </c>
       <c r="O38" s="3" t="n">
-        <v>0.1178</v>
+        <v>0.114</v>
       </c>
     </row>
     <row r="39">
@@ -2413,47 +2413,47 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>5697.3</v>
+        <v>5671.99</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>-0.0145</v>
+        <v>-0.0016</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>-0.0054</v>
+        <v>-0.0098</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>-0.0597</v>
+        <v>-0.0483</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>-0.0607</v>
+        <v>-0.0614</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>0.0185</v>
+        <v>-0.0385</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>-0.0926</v>
+        <v>-0.09660000000000001</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>0.05599999999999999</v>
+        <v>0.0513</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>-0.0449</v>
+        <v>-0.0603</v>
       </c>
       <c r="L39" s="3" t="n">
-        <v>-0.0268</v>
+        <v>-0.0312</v>
       </c>
       <c r="M39" s="3" t="n">
-        <v>0.0876</v>
+        <v>0.08529999999999999</v>
       </c>
       <c r="N39" s="3" t="n">
-        <v>0.0646</v>
+        <v>0.06059999999999999</v>
       </c>
       <c r="O39" s="3" t="n">
-        <v>0.1254</v>
+        <v>0.1248</v>
       </c>
     </row>
     <row r="40">
@@ -2464,47 +2464,47 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>16183.18</v>
+        <v>15928.44</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>-0.0139</v>
+        <v>-0.0124</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>-0.009599999999999999</v>
+        <v>-0.0252</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>-0.0603</v>
+        <v>-0.06179999999999999</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>-0.0646</v>
+        <v>-0.0725</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>-0.0132</v>
+        <v>-0.07200000000000001</v>
       </c>
       <c r="I40" s="3" t="n">
-        <v>-0.1351</v>
+        <v>-0.1488</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>-0.0217</v>
+        <v>-0.0371</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>-0.06900000000000001</v>
+        <v>-0.0911</v>
       </c>
       <c r="L40" s="3" t="n">
-        <v>-0.0727</v>
+        <v>-0.0723</v>
       </c>
       <c r="M40" s="3" t="n">
-        <v>0.115</v>
+        <v>0.1104</v>
       </c>
       <c r="N40" s="3" t="n">
-        <v>0.06860000000000001</v>
+        <v>0.064</v>
       </c>
       <c r="O40" s="3" t="n">
-        <v>0.1306</v>
+        <v>0.1295</v>
       </c>
     </row>
     <row r="41">
@@ -2515,47 +2515,47 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>64802.57</v>
+        <v>63371.48</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>-0.0026</v>
+        <v>-0.0165</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>-0.001</v>
+        <v>-0.0231</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>-0.0386</v>
+        <v>-0.0663</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>-0.0684</v>
+        <v>-0.08349999999999999</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>0.0404</v>
+        <v>-0.0314</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>0.0463</v>
+        <v>0.0232</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>0.0565</v>
+        <v>0.0332</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>0.0466</v>
+        <v>0.0273</v>
       </c>
       <c r="L41" s="3" t="n">
-        <v>-0.0548</v>
+        <v>-0.0575</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>0.1256</v>
+        <v>0.117</v>
       </c>
       <c r="N41" s="3" t="n">
-        <v>0.1059</v>
+        <v>0.1008</v>
       </c>
       <c r="O41" s="3" t="n">
-        <v>0.1594</v>
+        <v>0.1575</v>
       </c>
     </row>
     <row r="42">
@@ -2566,47 +2566,47 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>40873.08</v>
+        <v>41267.69</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>0.0077</v>
+        <v>0.0095</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>0.0215</v>
+        <v>0.0314</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>-0.078</v>
+        <v>-0.0117</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>0.0409</v>
+        <v>0.0234</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>-0.06809999999999999</v>
+        <v>-0.0711</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>-0.2427</v>
+        <v>-0.2354</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>-0.0176</v>
+        <v>-0.008199999999999999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>-0.1485</v>
+        <v>-0.1808</v>
       </c>
       <c r="L42" s="3" t="n">
-        <v>-0.1601</v>
+        <v>-0.1633</v>
       </c>
       <c r="M42" s="3" t="n">
-        <v>-0.023</v>
+        <v>-0.0221</v>
       </c>
       <c r="N42" s="3" t="n">
-        <v>-0.0225</v>
+        <v>-0.0278</v>
       </c>
       <c r="O42" s="3" t="n">
-        <v>0.1302</v>
+        <v>0.1303</v>
       </c>
     </row>
     <row r="43">
@@ -2617,47 +2617,47 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>7773.95</v>
+        <v>7811.54</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>0.0117</v>
+        <v>0.0115</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>0.016</v>
+        <v>0.0209</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>0.0072</v>
+        <v>0.0229</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>0.0314</v>
+        <v>0.0312</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>0.1758</v>
+        <v>0.1459</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>0.1356</v>
+        <v>0.1411</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>0.1908</v>
+        <v>0.1965</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>0.1576</v>
+        <v>0.1598</v>
       </c>
       <c r="L43" s="3" t="n">
-        <v>0.1625</v>
+        <v>0.1614</v>
       </c>
       <c r="M43" s="3" t="n">
-        <v>0.2176</v>
+        <v>0.2149</v>
       </c>
       <c r="N43" s="3" t="n">
-        <v>0.1225</v>
+        <v>0.122</v>
       </c>
       <c r="O43" s="3" t="n">
-        <v>0.1371</v>
+        <v>0.1385</v>
       </c>
     </row>
     <row r="44">
@@ -2668,47 +2668,47 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>31076.44</v>
+        <v>30883.15</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>0.0264</v>
+        <v>0.0024</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>0.022</v>
+        <v>0.0156</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>0.0519</v>
+        <v>0.04969999999999999</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>0.0464</v>
+        <v>0.0355</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>0.2846</v>
+        <v>0.2296</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>0.2308</v>
+        <v>0.2231</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>0.309</v>
+        <v>0.3009</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>0.2538</v>
+        <v>0.2305</v>
       </c>
       <c r="L44" s="3" t="n">
-        <v>0.2452</v>
+        <v>0.2346</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>0.2758</v>
+        <v>0.2687</v>
       </c>
       <c r="N44" s="3" t="n">
-        <v>0.1606</v>
+        <v>0.1581</v>
       </c>
       <c r="O44" s="3" t="n">
-        <v>0.2039</v>
+        <v>0.2042</v>
       </c>
     </row>
     <row r="45">
@@ -2719,47 +2719,47 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
-        <v>70772.67</v>
+        <v>69030.92</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>0.0808</v>
+        <v>0.0106</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>0.0602</v>
+        <v>0.0341</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>0.0885</v>
+        <v>0.0597</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>0.0369</v>
+        <v>0.0069</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>0.3246</v>
+        <v>0.2127</v>
       </c>
       <c r="I45" s="3" t="n">
-        <v>0.4059</v>
+        <v>0.3713</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>0.386</v>
+        <v>0.3519</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>0.4761</v>
+        <v>0.421</v>
       </c>
       <c r="L45" s="3" t="n">
-        <v>0.3526</v>
+        <v>0.326</v>
       </c>
       <c r="M45" s="3" t="n">
-        <v>0.3167</v>
+        <v>0.2958</v>
       </c>
       <c r="N45" s="3" t="n">
-        <v>0.2067</v>
+        <v>0.1973</v>
       </c>
       <c r="O45" s="3" t="n">
-        <v>0.1543</v>
+        <v>0.1504</v>
       </c>
     </row>
     <row r="46">
@@ -2770,47 +2770,47 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>25254.21</v>
+        <v>25087.27</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>-0.004699999999999999</v>
+        <v>-0.005699999999999999</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>0.0022</v>
+        <v>-0.0044</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>-0.0304</v>
+        <v>-0.0191</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>-0.0218</v>
+        <v>0.0008</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>0.09</v>
+        <v>0.0539</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>0.0312</v>
+        <v>0.0244</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>0.1135</v>
+        <v>0.1061</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>0.0359</v>
+        <v>0.0193</v>
       </c>
       <c r="L46" s="3" t="n">
-        <v>0.1491</v>
+        <v>0.1416</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>0.1838</v>
+        <v>0.1762</v>
       </c>
       <c r="N46" s="3" t="n">
-        <v>0.1103</v>
+        <v>0.1053</v>
       </c>
       <c r="O46" s="3" t="n">
-        <v>0.0919</v>
+        <v>0.09029999999999999</v>
       </c>
     </row>
     <row r="47">
@@ -2821,47 +2821,47 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>7834.1</v>
+        <v>7803.33</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>-0.0303</v>
+        <v>-0.0119</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>-0.0164</v>
+        <v>-0.0202</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>-0.0537</v>
+        <v>-0.0433</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>-0.0762</v>
+        <v>-0.06419999999999999</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>-0.0161</v>
+        <v>-0.0552</v>
       </c>
       <c r="I47" s="3" t="n">
-        <v>-0.0387</v>
+        <v>-0.0425</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>0.0022</v>
+        <v>-0.0017</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>-0.0306</v>
+        <v>-0.0296</v>
       </c>
       <c r="L47" s="3" t="n">
-        <v>0.0192</v>
+        <v>0.016</v>
       </c>
       <c r="M47" s="3" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="N47" s="3" t="n">
         <v>0.0353</v>
       </c>
-      <c r="N47" s="3" t="n">
-        <v>0.0383</v>
-      </c>
       <c r="O47" s="3" t="n">
-        <v>0.0582</v>
+        <v>0.0573</v>
       </c>
     </row>
     <row r="48">
@@ -2872,47 +2872,47 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>10497.9</v>
+        <v>10552.1</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>-0.0175</v>
+        <v>0.0086</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>-0.0102</v>
+        <v>-0.0051</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>-0.0308</v>
+        <v>-0.0111</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>-0.0144</v>
+        <v>0.0052</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>0.0059</v>
+        <v>-0.0046</v>
       </c>
       <c r="I48" s="3" t="n">
-        <v>0.057</v>
+        <v>0.0625</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>0.0316</v>
+        <v>0.0369</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>0.1061</v>
+        <v>0.1096</v>
       </c>
       <c r="L48" s="3" t="n">
-        <v>0.1259</v>
+        <v>0.1315</v>
       </c>
       <c r="M48" s="3" t="n">
-        <v>0.119</v>
+        <v>0.1143</v>
       </c>
       <c r="N48" s="3" t="n">
-        <v>0.08460000000000001</v>
+        <v>0.08259999999999999</v>
       </c>
       <c r="O48" s="3" t="n">
-        <v>0.0407</v>
+        <v>0.0409</v>
       </c>
     </row>
     <row r="49">
@@ -2923,47 +2923,47 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>24187.73</v>
+        <v>24211.35</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>-0.0137</v>
+        <v>0.01</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>-0.0173</v>
+        <v>-0.0163</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>-0.057</v>
+        <v>-0.0421</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>0.0294</v>
+        <v>0.0015</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>-0.03700000000000001</v>
+        <v>-0.065</v>
       </c>
       <c r="I49" s="3" t="n">
-        <v>-0.0563</v>
+        <v>-0.0554</v>
       </c>
       <c r="J49" s="3" t="n">
-        <v>-0.0242</v>
+        <v>-0.0233</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>-0.1028</v>
+        <v>-0.095</v>
       </c>
       <c r="L49" s="3" t="n">
-        <v>0.0313</v>
+        <v>0.0832</v>
       </c>
       <c r="M49" s="3" t="n">
-        <v>0.1142</v>
+        <v>0.1109</v>
       </c>
       <c r="N49" s="3" t="n">
-        <v>-0.0042</v>
+        <v>-0.0051</v>
       </c>
       <c r="O49" s="3" t="n">
-        <v>0.0014</v>
+        <v>0.0028</v>
       </c>
     </row>
     <row r="50">
@@ -3025,47 +3025,47 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>96.44</v>
+        <v>96.73</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>0.004699999999999999</v>
+        <v>0.004500000000000001</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>0.004</v>
+        <v>0.0071</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>0.0206</v>
+        <v>0.0108</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>0.008699999999999999</v>
+        <v>0.014</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>0.039</v>
+        <v>0.0461</v>
       </c>
       <c r="I51" s="3" t="n">
-        <v>0.07429999999999999</v>
+        <v>0.0775</v>
       </c>
       <c r="J51" s="3" t="n">
-        <v>0.0221</v>
+        <v>0.0252</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>0.0868</v>
+        <v>0.0885</v>
       </c>
       <c r="L51" s="3" t="n">
-        <v>0.0713</v>
+        <v>0.0735</v>
       </c>
       <c r="M51" s="3" t="n">
-        <v>0.0503</v>
+        <v>0.0515</v>
       </c>
       <c r="N51" s="3" t="n">
-        <v>0.05230000000000001</v>
+        <v>0.05110000000000001</v>
       </c>
       <c r="O51" s="3" t="n">
-        <v>0.03759999999999999</v>
+        <v>0.0377</v>
       </c>
     </row>
     <row r="52">
@@ -3076,47 +3076,47 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>4145.1</v>
+        <v>4216.3</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>-0.0083</v>
+        <v>0.013</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>-0.009899999999999999</v>
+        <v>0.0071</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>-0.0643</v>
+        <v>-0.0452</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>-0</v>
+        <v>0.0273</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>-0.1099</v>
+        <v>-0.1146</v>
       </c>
       <c r="I52" s="3" t="n">
-        <v>-0.0417</v>
+        <v>-0.0253</v>
       </c>
       <c r="J52" s="3" t="n">
-        <v>-0.1081</v>
+        <v>-0.09279999999999999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>0.0498</v>
+        <v>0.0684</v>
       </c>
       <c r="L52" s="3" t="n">
-        <v>0.2511</v>
+        <v>0.2722</v>
       </c>
       <c r="M52" s="3" t="n">
-        <v>0.3132</v>
+        <v>0.3136</v>
       </c>
       <c r="N52" s="3" t="n">
-        <v>0.1873</v>
+        <v>0.1913</v>
       </c>
       <c r="O52" s="3" t="n">
-        <v>0.1275</v>
+        <v>0.1291</v>
       </c>
     </row>
     <row r="53">
@@ -3127,47 +3127,47 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>60.72</v>
+        <v>61.05</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>0.0009</v>
+        <v>0.0105</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>0.0103</v>
+        <v>0.0158</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>-0.08070000000000001</v>
+        <v>-0.1015</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>-0.0035</v>
+        <v>0.0207</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>-0.1546</v>
+        <v>-0.2001</v>
       </c>
       <c r="I53" s="3" t="n">
-        <v>-0.1342</v>
+        <v>-0.1296</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>-0.187</v>
+        <v>-0.1826</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>0.2628</v>
+        <v>0.3031</v>
       </c>
       <c r="L53" s="3" t="n">
-        <v>0.3739</v>
+        <v>0.4169</v>
       </c>
       <c r="M53" s="3" t="n">
-        <v>0.4125</v>
+        <v>0.4104</v>
       </c>
       <c r="N53" s="3" t="n">
-        <v>0.2184</v>
+        <v>0.2189</v>
       </c>
       <c r="O53" s="3" t="n">
-        <v>0.1337</v>
+        <v>0.1335</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Weekly indices update 2026-10-16
</commit_message>
<xml_diff>
--- a/tracker_auto.xlsx
+++ b/tracker_auto.xlsx
@@ -524,47 +524,47 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>22520.45</v>
+        <v>22997.35</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.0044</v>
+        <v>0.0344</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-0.0044</v>
+        <v>0.0167</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>-0.0389</v>
+        <v>-0.0052</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>-0.0697</v>
+        <v>-0.0447</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>-0.0636</v>
+        <v>-0.0496</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>-0.1381</v>
+        <v>-0.1199</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.0298</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>-0.1057</v>
+        <v>-0.0919</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>-0.0506</v>
+        <v>-0.042</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>0.0458</v>
+        <v>0.0524</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>0.047</v>
+        <v>0.0463</v>
       </c>
       <c r="O2" s="3" t="n">
-        <v>0.09970000000000001</v>
+        <v>0.1045</v>
       </c>
     </row>
     <row r="3">
@@ -575,47 +575,47 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>72472.33</v>
+        <v>74600.67999999999</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.007800000000000001</v>
+        <v>0.0294</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>-0.0001</v>
+        <v>0.0293</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>-0.0307</v>
+        <v>0.0036</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>-0.06570000000000001</v>
+        <v>-0.0454</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>-0.0655</v>
+        <v>-0.0496</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>-0.1496</v>
+        <v>-0.1246</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>0.0073</v>
+        <v>0.0369</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>-0.118</v>
+        <v>-0.1062</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>-0.05690000000000001</v>
+        <v>-0.0433</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>0.0313</v>
+        <v>0.0395</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>0.0383</v>
+        <v>0.04</v>
       </c>
       <c r="O3" s="3" t="n">
-        <v>0.09949999999999999</v>
+        <v>0.1028</v>
       </c>
     </row>
     <row r="4">
@@ -626,47 +626,47 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>68166.7</v>
+        <v>68671.60000000001</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>-0.0118</v>
+        <v>0.0156</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>-0.0227</v>
+        <v>-0.0154</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>-0.0643</v>
+        <v>-0.0229</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>-0.0584</v>
+        <v>-0.0449</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.007800000000000001</v>
+        <v>-0.0091</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>-0.0173</v>
+        <v>-0.01</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.1295</v>
+        <v>0.1379</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>-0.0052</v>
+        <v>-0.0064</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>-0.0493</v>
+        <v>-0.0486</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>0.1485</v>
+        <v>0.1478</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>0.0951</v>
+        <v>0.0901</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>0.112</v>
+        <v>0.1148</v>
       </c>
     </row>
     <row r="5">
@@ -677,47 +677,47 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>23547.9</v>
+        <v>23986.1</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>0.0013</v>
+        <v>0.0309</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>-0.007900000000000001</v>
+        <v>0.0106</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>-0.0437</v>
+        <v>-0.0086</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>-0.06759999999999999</v>
+        <v>-0.0447</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>-0.0509</v>
+        <v>-0.04219999999999999</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>-0.1177</v>
+        <v>-0.1013</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0.0294</v>
+        <v>0.04849999999999999</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>-0.0882</v>
+        <v>-0.07690000000000001</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>-0.0498</v>
+        <v>-0.0423</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>0.06280000000000001</v>
+        <v>0.0682</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>0.0535</v>
+        <v>0.052</v>
       </c>
       <c r="O5" s="3" t="n">
-        <v>0.1013</v>
+        <v>0.1057</v>
       </c>
     </row>
     <row r="6">
@@ -728,47 +728,47 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>30516.35</v>
+        <v>31051.1</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>-0.0005</v>
+        <v>0.0318</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-0.0126</v>
+        <v>0.004699999999999999</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-0.0508</v>
+        <v>-0.016</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>-0.0693</v>
+        <v>-0.0478</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>-0.0424</v>
+        <v>-0.0372</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>-0.08439999999999999</v>
+        <v>-0.0684</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.0325</v>
+        <v>0.0506</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>-0.05309999999999999</v>
+        <v>-0.0433</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>-0.0279</v>
+        <v>-0.0192</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>0.09029999999999999</v>
+        <v>0.0941</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>0.08810000000000001</v>
+        <v>0.08470000000000001</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>0.1077</v>
+        <v>0.1126</v>
       </c>
     </row>
     <row r="7">
@@ -779,47 +779,47 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>32292.15</v>
+        <v>32701.95</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>-0.0061</v>
+        <v>0.0245</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-0.0173</v>
+        <v>-0.0048</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>-0.0583</v>
+        <v>-0.0191</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>-0.0667</v>
+        <v>-0.0488</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>-0.0157</v>
+        <v>-0.0217</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>-0.049</v>
+        <v>-0.0369</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>0.08410000000000001</v>
+        <v>0.09789999999999999</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>-0.0309</v>
+        <v>-0.0251</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>-0.031</v>
+        <v>-0.0249</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>0.1177</v>
+        <v>0.1193</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>0.08789999999999999</v>
+        <v>0.08439999999999999</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>0.1059</v>
+        <v>0.1099</v>
       </c>
     </row>
     <row r="8">
@@ -830,47 +830,47 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>17580.4</v>
+        <v>17868.66</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>0.0013</v>
+        <v>0.0294</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-0.008100000000000001</v>
+        <v>0.008199999999999999</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-0.0471</v>
+        <v>-0.0122</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>-0.06519999999999999</v>
+        <v>-0.0445</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>-0.0317</v>
+        <v>-0.0273</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>-0.09369999999999999</v>
+        <v>-0.0789</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.0528</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>-0.0619</v>
+        <v>-0.0529</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>-0.0311</v>
+        <v>-0.025</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>0.0859</v>
+        <v>0.09039999999999999</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>0.0771</v>
+        <v>0.07490000000000001</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>0.1205</v>
+        <v>0.1247</v>
       </c>
     </row>
     <row r="9">
@@ -881,47 +881,47 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>15600.55</v>
+        <v>15801.35</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>-0.0003</v>
+        <v>0.0259</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-0.01</v>
+        <v>0.0028</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-0.0522</v>
+        <v>-0.0178</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>-0.0675</v>
+        <v>-0.0506</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>-0.0183</v>
+        <v>-0.0213</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>-0.07440000000000001</v>
+        <v>-0.0625</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>0.0704</v>
+        <v>0.0842</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>-0.0457</v>
+        <v>-0.0395</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>-0.0278</v>
+        <v>-0.0246</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>0.096</v>
+        <v>0.09859999999999999</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>0.09179999999999999</v>
+        <v>0.0888</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>0.1273</v>
+        <v>0.1309</v>
       </c>
     </row>
     <row r="10">
@@ -932,47 +932,47 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>21603.25</v>
+        <v>21756.35</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>-0.0019</v>
+        <v>0.0209</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>-0.0121</v>
+        <v>-0.0051</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>-0.0604</v>
+        <v>-0.0269</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>-0.0675</v>
+        <v>-0.0565</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.0142</v>
+        <v>-0.0011</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>-0.0302</v>
+        <v>-0.0234</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.1118</v>
+        <v>0.1197</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>-0.0024</v>
+        <v>-0.0018</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>-0.0072</v>
+        <v>-0.008500000000000001</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>0.1282</v>
+        <v>0.1279</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0.1291</v>
+        <v>0.1245</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>0.1515</v>
+        <v>0.1541</v>
       </c>
     </row>
     <row r="11">
@@ -983,47 +983,47 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>17574.85</v>
+        <v>17627.05</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>-0.0008</v>
+        <v>0.007900000000000001</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>-0.0126</v>
+        <v>-0.009599999999999999</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>-0.04650000000000001</v>
+        <v>-0.0149</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>-0.03</v>
+        <v>-0.0266</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0.1156</v>
+        <v>0.08810000000000001</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>0.0533</v>
+        <v>0.0565</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>0.23</v>
+        <v>0.2337</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>0.0333</v>
+        <v>0.0337</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>-0.0147</v>
+        <v>-0.023</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>0.1279</v>
+        <v>0.1231</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>0.1265</v>
+        <v>0.1215</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>0.1314</v>
+        <v>0.1334</v>
       </c>
     </row>
     <row r="12">
@@ -1034,47 +1034,47 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>20164.7</v>
+        <v>20278.15</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>-0.0015</v>
+        <v>0.0163</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>-0.0123</v>
+        <v>-0.0067</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>-0.0556</v>
+        <v>-0.0228</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>-0.0547</v>
+        <v>-0.0463</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.04769999999999999</v>
+        <v>0.0284</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>-0.0026</v>
+        <v>0.003</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0.1507</v>
+        <v>0.1571</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>0.0092</v>
+        <v>0.0097</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>-0.0104</v>
+        <v>-0.0142</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0.1277</v>
+        <v>0.1258</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.1284</v>
+        <v>0.1237</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>0.1449</v>
+        <v>0.1473</v>
       </c>
     </row>
     <row r="13">
@@ -1085,47 +1085,47 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>21866.65</v>
+        <v>22180.8</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0.0004</v>
+        <v>0.0261</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>-0.009300000000000001</v>
+        <v>0.0049</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>-0.0476</v>
+        <v>-0.0132</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>-0.0635</v>
+        <v>-0.0453</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>-0.0215</v>
+        <v>-0.021</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>-0.08400000000000001</v>
+        <v>-0.0708</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>0.06519999999999999</v>
+        <v>0.0805</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>-0.0592</v>
+        <v>-0.0512</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>-0.0374</v>
+        <v>-0.0333</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>0.08119999999999999</v>
+        <v>0.08449999999999999</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>0.0731</v>
+        <v>0.0706</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>0.1125</v>
+        <v>0.1163</v>
       </c>
     </row>
     <row r="14">
@@ -1136,47 +1136,47 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>34192.47</v>
+        <v>34738.24</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>-0.0008</v>
+        <v>0.0267</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>-0.0108</v>
+        <v>0.005</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>-0.0481</v>
+        <v>-0.0123</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>-0.0634</v>
+        <v>-0.04389999999999999</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>-0.0232</v>
+        <v>-0.0211</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>-0.0868</v>
+        <v>-0.0722</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>0.0625</v>
+        <v>0.0794</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>-0.0629</v>
+        <v>-0.0533</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>-0.0413</v>
+        <v>-0.0362</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0.0765</v>
+        <v>0.0803</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>0.06950000000000001</v>
+        <v>0.0673</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>0.1112</v>
+        <v>0.1152</v>
       </c>
     </row>
     <row r="15">
@@ -1187,47 +1187,47 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>18625.4</v>
+        <v>18843.45</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>0.002</v>
+        <v>0.0268</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>-0.008500000000000001</v>
+        <v>0.0031</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>-0.045</v>
+        <v>-0.0203</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>-0.07150000000000001</v>
+        <v>-0.0584</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>-0.04769999999999999</v>
+        <v>-0.0423</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>-0.1185</v>
+        <v>-0.1082</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>0.0173</v>
+        <v>0.0292</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>-0.0832</v>
+        <v>-0.0789</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>-0.052</v>
+        <v>-0.046</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>0.0757</v>
+        <v>0.076</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>0.0639</v>
+        <v>0.0633</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>0.1045</v>
+        <v>0.1087</v>
       </c>
     </row>
     <row r="16">
@@ -1238,47 +1238,47 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>5264.7</v>
+        <v>5412.85</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>0.0005</v>
+        <v>0.0457</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>-0.0105</v>
+        <v>0.0174</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>-0.052</v>
+        <v>-0.0024</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>-0.0417</v>
+        <v>-0.016</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>-0.0323</v>
+        <v>-0.0179</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>-0.1016</v>
+        <v>-0.07629999999999999</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>0.046</v>
+        <v>0.0755</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>-0.0687</v>
+        <v>-0.0455</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>-0.0722</v>
+        <v>-0.06</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0.0567</v>
+        <v>0.0653</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>0.052</v>
+        <v>0.0552</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>0.08960000000000001</v>
+        <v>0.0949</v>
       </c>
     </row>
     <row r="17">
@@ -1289,47 +1289,47 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>24413.16</v>
+        <v>24594.34</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>-0.002</v>
+        <v>0.0217</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>-0.0199</v>
+        <v>-0.0126</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>-0.0596</v>
+        <v>-0.0294</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>-0.0771</v>
+        <v>-0.0619</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>-0.08550000000000001</v>
+        <v>-0.0955</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>-0.0475</v>
+        <v>-0.0404</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>-0.006999999999999999</v>
+        <v>0.0004</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>0.0392</v>
+        <v>0.045</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>0.0199</v>
+        <v>0.0179</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>0.2102</v>
+        <v>0.2072</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>0.2198</v>
+        <v>0.2088</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>0.1566</v>
+        <v>0.1599</v>
       </c>
     </row>
     <row r="18">
@@ -1340,47 +1340,47 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>36740.35</v>
+        <v>36610.48</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>-0.0005999999999999999</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>-0.0109</v>
+        <v>-0.0144</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>-0.0622</v>
+        <v>-0.0212</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>-0.0441</v>
+        <v>-0.0462</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>-0.0384</v>
+        <v>-0.0424</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>-0.0568</v>
+        <v>-0.0602</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>0.0839</v>
+        <v>0.0801</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>-0.0525</v>
+        <v>-0.07290000000000001</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>-0.1082</v>
+        <v>-0.1137</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>0.0897</v>
+        <v>0.08539999999999999</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>0.0843</v>
+        <v>0.0689</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>0.154</v>
+        <v>0.1559</v>
       </c>
     </row>
     <row r="19">
@@ -1391,47 +1391,47 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>27322.67</v>
+        <v>28062.77</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>0.0032</v>
+        <v>0.0469</v>
       </c>
       <c r="E19" s="3" t="n">
+        <v>0.0228</v>
+      </c>
+      <c r="F19" s="3" t="n">
         <v>-0.0042</v>
       </c>
-      <c r="F19" s="3" t="n">
-        <v>-0.0525</v>
-      </c>
       <c r="G19" s="3" t="n">
-        <v>-0.0544</v>
+        <v>-0.0272</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>-0.0366</v>
+        <v>-0.0238</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>-0.1077</v>
+        <v>-0.08359999999999999</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>0.0453</v>
+        <v>0.0736</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>-0.07919999999999999</v>
+        <v>-0.05599999999999999</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>-0.0767</v>
+        <v>-0.0664</v>
       </c>
       <c r="M19" s="3" t="n">
+        <v>0.0709</v>
+      </c>
+      <c r="N19" s="3" t="n">
         <v>0.0621</v>
       </c>
-      <c r="N19" s="3" t="n">
-        <v>0.05860000000000001</v>
-      </c>
       <c r="O19" s="3" t="n">
-        <v>0.1149</v>
+        <v>0.1206</v>
       </c>
     </row>
     <row r="20">
@@ -1442,47 +1442,47 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>29197.45</v>
+        <v>29070.25</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>-0.0005999999999999999</v>
+        <v>0.007900000000000001</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>-0.0109</v>
+        <v>-0.0152</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>-0.0624</v>
+        <v>-0.0222</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>-0.046</v>
+        <v>-0.0489</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>-0.0432</v>
+        <v>-0.0479</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>-0.0626</v>
+        <v>-0.0667</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>0.0785</v>
+        <v>0.0738</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>-0.0585</v>
+        <v>-0.0795</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>-0.1142</v>
+        <v>-0.12</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>0.0808</v>
+        <v>0.0762</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>0.07480000000000001</v>
+        <v>0.0593</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>0.1429</v>
+        <v>0.1447</v>
       </c>
     </row>
     <row r="21">
@@ -1493,47 +1493,47 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>55339.9</v>
+        <v>53751.45</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>0.0276</v>
+        <v>-0.0155</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0.0233</v>
+        <v>-0.0061</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>-0.0245</v>
+        <v>-0.0135</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>0.0198</v>
+        <v>-0.0044</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>0.1106</v>
+        <v>0.0645</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>0.1</v>
+        <v>0.0684</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>0.2439</v>
+        <v>0.2082</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>0.09539999999999998</v>
+        <v>0.0499</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>-0.0384</v>
+        <v>-0.0594</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>0.1521</v>
+        <v>0.1371</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>0.1084</v>
+        <v>0.0964</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>0.19</v>
+        <v>0.187</v>
       </c>
     </row>
     <row r="22">
@@ -1544,47 +1544,47 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>24692.85</v>
+        <v>24880.6</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>-0.0097</v>
+        <v>0.0193</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>-0.0209</v>
+        <v>-0.0134</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>-0.0679</v>
+        <v>-0.0335</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>-0.0815</v>
+        <v>-0.06900000000000001</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>-0.03700000000000001</v>
+        <v>-0.0299</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>-0.08800000000000001</v>
+        <v>-0.08109999999999999</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>0.0305</v>
+        <v>0.0384</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>-0.0704</v>
+        <v>-0.0716</v>
       </c>
       <c r="L22" s="3" t="n">
-        <v>-0.09759999999999999</v>
+        <v>-0.09210000000000002</v>
       </c>
       <c r="M22" s="3" t="n">
-        <v>0.0764</v>
+        <v>0.0756</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>0.0665</v>
+        <v>0.06469999999999999</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>0.1093</v>
+        <v>0.1124</v>
       </c>
     </row>
     <row r="23">
@@ -1595,44 +1595,44 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>9982.65</v>
+        <v>10192.78</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>-0.0149</v>
+        <v>0.0262</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>-0.0291</v>
+        <v>-0.008699999999999999</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>-0.0892</v>
+        <v>0.0059</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>-0.0493</v>
+        <v>-0.008500000000000001</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.0605</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>0.1682</v>
+        <v>0.1928</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>0.2506</v>
+        <v>0.2769</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>0.1162</v>
+        <v>0.1453</v>
       </c>
       <c r="L23" s="3" t="n">
-        <v>0.1776</v>
+        <v>0.1703</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>0.4035</v>
+        <v>0.4141</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>0.4908</v>
+        <v>0.4801</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -1648,47 +1648,47 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>11156.08</v>
+        <v>11039.18</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>0.0238</v>
+        <v>0.005699999999999999</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>0.0138</v>
+        <v>0.0031</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>-0.029</v>
+        <v>-0.0144</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>-0.0384</v>
+        <v>-0.0367</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>-0.0679</v>
+        <v>-0.07969999999999999</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>-0.0406</v>
+        <v>-0.0507</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>0.0392</v>
+        <v>0.0283</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>0.08160000000000001</v>
+        <v>0.049</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>0.1155</v>
+        <v>0.1101</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>0.1716</v>
+        <v>0.1734</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>0.2739</v>
+        <v>0.2552</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>0.105</v>
+        <v>0.1072</v>
       </c>
     </row>
     <row r="25">
@@ -1699,47 +1699,47 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>77564.42</v>
+        <v>78341.89</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>0.0148</v>
+        <v>0.0238</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>0.0114</v>
+        <v>0.0216</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>-0.0185</v>
+        <v>0.0003</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>-0.0463</v>
+        <v>-0.029</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>-0.0052</v>
+        <v>0.0016</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>-0.0665</v>
+        <v>-0.0571</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>0.1063</v>
+        <v>0.1174</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>-0.0102</v>
+        <v>-0.011</v>
       </c>
       <c r="L25" s="3" t="n">
-        <v>0.0484</v>
+        <v>0.0445</v>
       </c>
       <c r="M25" s="3" t="n">
-        <v>0.08439999999999999</v>
+        <v>0.0891</v>
       </c>
       <c r="N25" s="3" t="n">
-        <v>0.0876</v>
+        <v>0.081</v>
       </c>
       <c r="O25" s="3" t="n">
-        <v>0.117</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="26">
@@ -1750,47 +1750,47 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>32224.3</v>
+        <v>32764.99</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>0.0197</v>
+        <v>0.0302</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.0197</v>
+        <v>0.0368</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>0.0003</v>
+        <v>0.0225</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>-0.0282</v>
+        <v>-0.0059</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>0.0226</v>
+        <v>0.036</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>-0.04650000000000001</v>
+        <v>-0.0305</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>0.1343</v>
+        <v>0.1533</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>-0.0048</v>
+        <v>0.0043</v>
       </c>
       <c r="L26" s="3" t="n">
-        <v>0.042</v>
+        <v>0.0398</v>
       </c>
       <c r="M26" s="3" t="n">
-        <v>0.0646</v>
+        <v>0.0701</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>0.0733</v>
+        <v>0.06950000000000001</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>0.1031</v>
+        <v>0.106</v>
       </c>
     </row>
     <row r="27">
@@ -1801,47 +1801,47 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>31949.76</v>
+        <v>32456.11</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>0.0168</v>
+        <v>0.0294</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>0.0129</v>
+        <v>0.029</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>-0.0161</v>
+        <v>0.0115</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>-0.0675</v>
+        <v>-0.0429</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>-0.04</v>
+        <v>-0.0295</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>-0.08789999999999999</v>
+        <v>-0.0735</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>0.0699</v>
+        <v>0.08689999999999999</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>-0.0572</v>
+        <v>-0.0546</v>
       </c>
       <c r="L27" s="3" t="n">
-        <v>0.0396</v>
+        <v>0.0408</v>
       </c>
       <c r="M27" s="3" t="n">
-        <v>0.09029999999999999</v>
+        <v>0.0964</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>0.07440000000000001</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="O27" s="3" t="n">
-        <v>0.1292</v>
+        <v>0.1337</v>
       </c>
     </row>
     <row r="28">
@@ -1852,47 +1852,47 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>16454.98</v>
+        <v>16780.16</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>-0.0139</v>
+        <v>0.0274</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>-0.0299</v>
+        <v>-0.0107</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>-0.06709999999999999</v>
+        <v>-0.0216</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>-0.0771</v>
+        <v>-0.0588</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>-0.1009</v>
+        <v>-0.1078</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>-0.06469999999999999</v>
+        <v>-0.0462</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>-0.0431</v>
+        <v>-0.0242</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>-0.0634</v>
+        <v>-0.04650000000000001</v>
       </c>
       <c r="L28" s="3" t="n">
-        <v>-0.0609</v>
+        <v>-0.059</v>
       </c>
       <c r="M28" s="3" t="n">
-        <v>0.1762</v>
+        <v>0.1761</v>
       </c>
       <c r="N28" s="3" t="n">
-        <v>0.1952</v>
+        <v>0.1904</v>
       </c>
       <c r="O28" s="3" t="n">
-        <v>0.1309</v>
+        <v>0.1331</v>
       </c>
     </row>
     <row r="29">
@@ -1903,47 +1903,47 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>896.1</v>
+        <v>923.65</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>-0.0372</v>
+        <v>0.0403</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>-0.0512</v>
+        <v>-0.0221</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>-0.0781</v>
+        <v>0.0177</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>-0.1398</v>
+        <v>-0.08169999999999999</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>0.0636</v>
+        <v>0.0677</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>-0.0801</v>
+        <v>-0.0518</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>0.2402</v>
+        <v>0.2783</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>-0.08410000000000001</v>
+        <v>-0.09050000000000001</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>-0.1224</v>
+        <v>-0.1202</v>
       </c>
       <c r="M29" s="3" t="n">
-        <v>0.1027</v>
+        <v>0.1111</v>
       </c>
       <c r="N29" s="3" t="n">
-        <v>0.09449999999999999</v>
+        <v>0.0935</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>0.1492</v>
+        <v>0.1557</v>
       </c>
     </row>
     <row r="30">
@@ -1954,47 +1954,47 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>33276.66</v>
+        <v>34235.76</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>-0.0207</v>
+        <v>0.0434</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>-0.0545</v>
+        <v>-0.0273</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>-0.101</v>
+        <v>-0.0441</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>-0.07139999999999999</v>
+        <v>-0.0414</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>-0.0587</v>
+        <v>-0.0221</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>-0.109</v>
+        <v>-0.0833</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>0.055</v>
+        <v>0.08539999999999999</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>-0.055</v>
+        <v>-0.0322</v>
       </c>
       <c r="L30" s="3" t="n">
-        <v>-0.0209</v>
+        <v>-0.003</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>0.1682</v>
+        <v>0.1675</v>
       </c>
       <c r="N30" s="3" t="n">
-        <v>0.1862</v>
+        <v>0.178</v>
       </c>
       <c r="O30" s="3" t="n">
-        <v>0.1033</v>
+        <v>0.1101</v>
       </c>
     </row>
     <row r="31">
@@ -2005,47 +2005,47 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>19640.86</v>
+        <v>19865.84</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>-0.016</v>
+        <v>0.0188</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>-0.03240000000000001</v>
+        <v>-0.0214</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>-0.0775</v>
+        <v>-0.0295</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>-0.0599</v>
+        <v>-0.05</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>-0.0109</v>
+        <v>-0.0146</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>-0.0222</v>
+        <v>-0.011</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>0.0718</v>
+        <v>0.08410000000000001</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>0.005600000000000001</v>
+        <v>0.0173</v>
       </c>
       <c r="L31" s="3" t="n">
-        <v>-0.0043</v>
+        <v>0.0023</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>0.1643</v>
+        <v>0.1622</v>
       </c>
       <c r="N31" s="3" t="n">
-        <v>0.1391</v>
+        <v>0.1333</v>
       </c>
       <c r="O31" s="3" t="n">
-        <v>0.1293</v>
+        <v>0.1334</v>
       </c>
     </row>
     <row r="32">
@@ -2056,47 +2056,47 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>11326.02</v>
+        <v>11473.21</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>-0.0036</v>
+        <v>0.0214</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>-0.0183</v>
+        <v>-0.005500000000000001</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>-0.05980000000000001</v>
+        <v>-0.0252</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>-0.0877</v>
+        <v>-0.06610000000000001</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>-0.0539</v>
+        <v>-0.0537</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>-0.102</v>
+        <v>-0.09029999999999999</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>0.0075</v>
+        <v>0.0206</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>-0.0554</v>
+        <v>-0.0509</v>
       </c>
       <c r="L32" s="3" t="n">
-        <v>-0.0234</v>
+        <v>-0.0209</v>
       </c>
       <c r="M32" s="3" t="n">
-        <v>0.1218</v>
+        <v>0.1219</v>
       </c>
       <c r="N32" s="3" t="n">
-        <v>0.1193</v>
+        <v>0.1159</v>
       </c>
       <c r="O32" s="3" t="n">
-        <v>0.1319</v>
+        <v>0.1358</v>
       </c>
     </row>
     <row r="33">
@@ -2107,47 +2107,47 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>18925.52</v>
+        <v>18769.01</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>-0.0149</v>
+        <v>0.0025</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>-0.0175</v>
+        <v>-0.0256</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>-0.0438</v>
+        <v>-0.0353</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>-0.0285</v>
+        <v>-0.04559999999999999</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>0.1203</v>
+        <v>0.0926</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>0.0883</v>
+        <v>0.0793</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>0.1199</v>
+        <v>0.1106</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>0.09179999999999999</v>
+        <v>0.075</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>0.0347</v>
+        <v>0.0342</v>
       </c>
       <c r="M33" s="3" t="n">
-        <v>0.1922</v>
+        <v>0.1864</v>
       </c>
       <c r="N33" s="3" t="n">
-        <v>0.1279</v>
+        <v>0.123</v>
       </c>
       <c r="O33" s="3" t="n">
-        <v>0.1037</v>
+        <v>0.1051</v>
       </c>
     </row>
     <row r="34">
@@ -2158,47 +2158,47 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>18327.77</v>
+        <v>18374.29</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>-0.0365</v>
+        <v>0.0136</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>-0.0592</v>
+        <v>-0.0568</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>-0.1031</v>
+        <v>-0.0495</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>-0.053</v>
+        <v>-0.0359</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>-0.0215</v>
+        <v>-0.0486</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>0.0858</v>
+        <v>0.0885</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>0.08550000000000001</v>
+        <v>0.0882</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>0.1714</v>
+        <v>0.1903</v>
       </c>
       <c r="L34" s="3" t="n">
-        <v>0.1174</v>
+        <v>0.121</v>
       </c>
       <c r="M34" s="3" t="n">
-        <v>0.2196</v>
+        <v>0.2147</v>
       </c>
       <c r="N34" s="3" t="n">
-        <v>0.1759</v>
+        <v>0.163</v>
       </c>
       <c r="O34" s="3" t="n">
-        <v>0.1826</v>
+        <v>0.1874</v>
       </c>
     </row>
     <row r="35">
@@ -2209,47 +2209,47 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>9360.940000000001</v>
+        <v>9470.780000000001</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>-0.008399999999999999</v>
+        <v>0.0194</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>-0.029</v>
+        <v>-0.0176</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>-0.063</v>
+        <v>-0.024</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>-0.04679999999999999</v>
+        <v>-0.03240000000000001</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>0.0283</v>
+        <v>0.0275</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>-0.0505</v>
+        <v>-0.0393</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>0.1448</v>
+        <v>0.1583</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>-0.0595</v>
+        <v>-0.05309999999999999</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>-0.0664</v>
+        <v>-0.061</v>
       </c>
       <c r="M35" s="3" t="n">
-        <v>0.1021</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="N35" s="3" t="n">
-        <v>0.0973</v>
+        <v>0.09050000000000001</v>
       </c>
       <c r="O35" s="3" t="n">
-        <v>0.1089</v>
+        <v>0.1137</v>
       </c>
     </row>
     <row r="36">
@@ -2260,47 +2260,47 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>13302.26</v>
+        <v>13525.92</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>-0.0225</v>
+        <v>0.0251</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>-0.0414</v>
+        <v>-0.0252</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>-0.08359999999999999</v>
+        <v>-0.0354</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>-0.09480000000000001</v>
+        <v>-0.0727</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>-0.0795</v>
+        <v>-0.0842</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>-0.0534</v>
+        <v>-0.0375</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>-0.0162</v>
+        <v>0.0003</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>-0.0124</v>
+        <v>0.0027</v>
       </c>
       <c r="L36" s="3" t="n">
-        <v>-0.0122</v>
+        <v>-0.0036</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0.1296</v>
       </c>
       <c r="N36" s="3" t="n">
-        <v>0.1014</v>
+        <v>0.0969</v>
       </c>
       <c r="O36" s="3" t="n">
-        <v>0.1281</v>
+        <v>0.1317</v>
       </c>
     </row>
     <row r="37">
@@ -2311,47 +2311,47 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>74444.39999999999</v>
+        <v>74323.97</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>0.0245</v>
+        <v>0.0204</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>0.008</v>
+        <v>0.0064</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>-0.0098</v>
+        <v>-0.0009</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>-0.0883</v>
+        <v>-0.0728</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>-0.0634</v>
+        <v>-0.06849999999999999</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>-0.1855</v>
+        <v>-0.1868</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>-0.008699999999999999</v>
+        <v>-0.0103</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>-0.1723</v>
+        <v>-0.1743</v>
       </c>
       <c r="L37" s="3" t="n">
-        <v>-0.1392</v>
+        <v>-0.1418</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>-0.0314</v>
+        <v>-0.0356</v>
       </c>
       <c r="N37" s="3" t="n">
-        <v>0.0404</v>
+        <v>0.033</v>
       </c>
       <c r="O37" s="3" t="n">
-        <v>0.0925</v>
+        <v>0.09369999999999999</v>
       </c>
     </row>
     <row r="38">
@@ -2362,47 +2362,47 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>5118.36</v>
+        <v>5211.33</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>-0.0248</v>
+        <v>0.027</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>-0.0414</v>
+        <v>-0.024</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>-0.07580000000000001</v>
+        <v>-0.0349</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>-0.1307</v>
+        <v>-0.1087</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>-0.09050000000000001</v>
+        <v>-0.1211</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>-0.0039</v>
+        <v>0.0142</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>-0.0162</v>
+        <v>0.0017</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>-0.0475</v>
+        <v>-0.0466</v>
       </c>
       <c r="L38" s="3" t="n">
-        <v>-0.1106</v>
+        <v>-0.104</v>
       </c>
       <c r="M38" s="3" t="n">
-        <v>0.1241</v>
+        <v>0.1267</v>
       </c>
       <c r="N38" s="3" t="n">
-        <v>0.1134</v>
+        <v>0.1038</v>
       </c>
       <c r="O38" s="3" t="n">
-        <v>0.114</v>
+        <v>0.1174</v>
       </c>
     </row>
     <row r="39">
@@ -2413,47 +2413,47 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>5671.99</v>
+        <v>5801.18</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>-0.0016</v>
+        <v>0.0363</v>
       </c>
       <c r="E39" s="3" t="n">
+        <v>0.0128</v>
+      </c>
+      <c r="F39" s="3" t="n">
         <v>-0.0098</v>
       </c>
-      <c r="F39" s="3" t="n">
-        <v>-0.0483</v>
-      </c>
       <c r="G39" s="3" t="n">
-        <v>-0.0614</v>
+        <v>-0.0395</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>-0.0385</v>
+        <v>-0.0287</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>-0.09660000000000001</v>
+        <v>-0.076</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>0.0513</v>
+        <v>0.07519999999999999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>-0.0603</v>
+        <v>-0.0458</v>
       </c>
       <c r="L39" s="3" t="n">
-        <v>-0.0312</v>
+        <v>-0.0207</v>
       </c>
       <c r="M39" s="3" t="n">
-        <v>0.08529999999999999</v>
+        <v>0.0929</v>
       </c>
       <c r="N39" s="3" t="n">
-        <v>0.06059999999999999</v>
+        <v>0.061</v>
       </c>
       <c r="O39" s="3" t="n">
-        <v>0.1248</v>
+        <v>0.1302</v>
       </c>
     </row>
     <row r="40">
@@ -2464,47 +2464,47 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>15928.44</v>
+        <v>16327.65</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>-0.0124</v>
+        <v>0.0241</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>-0.0252</v>
+        <v>-0.0008</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>-0.06179999999999999</v>
+        <v>-0.0176</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>-0.0725</v>
+        <v>-0.05019999999999999</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>-0.07200000000000001</v>
+        <v>-0.05400000000000001</v>
       </c>
       <c r="I40" s="3" t="n">
-        <v>-0.1488</v>
+        <v>-0.1274</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>-0.0371</v>
+        <v>-0.013</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>-0.0911</v>
+        <v>-0.0654</v>
       </c>
       <c r="L40" s="3" t="n">
-        <v>-0.0723</v>
+        <v>-0.0608</v>
       </c>
       <c r="M40" s="3" t="n">
-        <v>0.1104</v>
+        <v>0.112</v>
       </c>
       <c r="N40" s="3" t="n">
-        <v>0.064</v>
+        <v>0.0668</v>
       </c>
       <c r="O40" s="3" t="n">
-        <v>0.1295</v>
+        <v>0.1323</v>
       </c>
     </row>
     <row r="41">
@@ -2515,47 +2515,47 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>63371.48</v>
+        <v>64127.92</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>-0.0165</v>
+        <v>0.0158</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>-0.0231</v>
+        <v>-0.0114</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>-0.0663</v>
+        <v>-0.025</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>-0.08349999999999999</v>
+        <v>-0.075</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>-0.0314</v>
+        <v>-0.0458</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>0.0232</v>
+        <v>0.0354</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>0.0332</v>
+        <v>0.0455</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>0.0273</v>
+        <v>0.0373</v>
       </c>
       <c r="L41" s="3" t="n">
-        <v>-0.0575</v>
+        <v>-0.0508</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>0.117</v>
+        <v>0.1144</v>
       </c>
       <c r="N41" s="3" t="n">
-        <v>0.1008</v>
+        <v>0.0956</v>
       </c>
       <c r="O41" s="3" t="n">
-        <v>0.1575</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="42">
@@ -2566,47 +2566,47 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>41267.69</v>
+        <v>44410.82</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>0.0095</v>
+        <v>0.1087</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>0.0314</v>
+        <v>0.11</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>-0.0117</v>
+        <v>0.0405</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>0.0234</v>
+        <v>0.07290000000000001</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>-0.0711</v>
+        <v>-0.025</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>-0.2354</v>
+        <v>-0.1772</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>-0.008199999999999999</v>
+        <v>0.0674</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>-0.1808</v>
+        <v>-0.1135</v>
       </c>
       <c r="L42" s="3" t="n">
-        <v>-0.1633</v>
+        <v>-0.1332</v>
       </c>
       <c r="M42" s="3" t="n">
-        <v>-0.0221</v>
+        <v>0.0107</v>
       </c>
       <c r="N42" s="3" t="n">
-        <v>-0.0278</v>
+        <v>-0.009899999999999999</v>
       </c>
       <c r="O42" s="3" t="n">
-        <v>0.1303</v>
+        <v>0.1399</v>
       </c>
     </row>
     <row r="43">
@@ -2617,47 +2617,47 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>7811.54</v>
+        <v>7744.06</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>0.0115</v>
+        <v>-0.0027</v>
       </c>
       <c r="E43" s="3" t="n">
+        <v>0.0121</v>
+      </c>
+      <c r="F43" s="3" t="n">
         <v>0.0209</v>
       </c>
-      <c r="F43" s="3" t="n">
-        <v>0.0229</v>
-      </c>
       <c r="G43" s="3" t="n">
-        <v>0.0312</v>
+        <v>0.0279</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>0.1459</v>
+        <v>0.0998</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>0.1411</v>
+        <v>0.1313</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>0.1965</v>
+        <v>0.1862</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>0.1598</v>
+        <v>0.1608</v>
       </c>
       <c r="L43" s="3" t="n">
-        <v>0.1614</v>
+        <v>0.1541</v>
       </c>
       <c r="M43" s="3" t="n">
-        <v>0.2149</v>
+        <v>0.2099</v>
       </c>
       <c r="N43" s="3" t="n">
-        <v>0.122</v>
+        <v>0.1161</v>
       </c>
       <c r="O43" s="3" t="n">
-        <v>0.1385</v>
+        <v>0.1381</v>
       </c>
     </row>
     <row r="44">
@@ -2668,47 +2668,47 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>30883.15</v>
+        <v>29935.6</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>0.0024</v>
+        <v>-0.0257</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>0.0156</v>
+        <v>-0.0156</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>0.04969999999999999</v>
+        <v>0.0345</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>0.0355</v>
+        <v>0.0313</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>0.2296</v>
+        <v>0.1368</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>0.2231</v>
+        <v>0.1856</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>0.3009</v>
+        <v>0.261</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>0.2305</v>
+        <v>0.2097</v>
       </c>
       <c r="L44" s="3" t="n">
-        <v>0.2346</v>
+        <v>0.2187</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>0.2687</v>
+        <v>0.2544</v>
       </c>
       <c r="N44" s="3" t="n">
-        <v>0.1581</v>
+        <v>0.146</v>
       </c>
       <c r="O44" s="3" t="n">
-        <v>0.2042</v>
+        <v>0.2011</v>
       </c>
     </row>
     <row r="45">
@@ -2719,47 +2719,47 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
-        <v>69030.92</v>
+        <v>65324.29</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>0.0106</v>
+        <v>-0.0537</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>0.0341</v>
+        <v>-0.0214</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>0.0597</v>
+        <v>0.0261</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>0.0069</v>
+        <v>0.0184</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>0.2127</v>
+        <v>0.1171</v>
       </c>
       <c r="I45" s="3" t="n">
-        <v>0.3713</v>
+        <v>0.2977</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>0.3519</v>
+        <v>0.2793</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>0.421</v>
+        <v>0.3531</v>
       </c>
       <c r="L45" s="3" t="n">
-        <v>0.326</v>
+        <v>0.2915</v>
       </c>
       <c r="M45" s="3" t="n">
-        <v>0.2958</v>
+        <v>0.2682</v>
       </c>
       <c r="N45" s="3" t="n">
-        <v>0.1973</v>
+        <v>0.1757</v>
       </c>
       <c r="O45" s="3" t="n">
-        <v>0.1504</v>
+        <v>0.1444</v>
       </c>
     </row>
     <row r="46">
@@ -2770,47 +2770,47 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>25087.27</v>
+        <v>25382.62</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>-0.005699999999999999</v>
+        <v>0.0232</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>-0.0044</v>
+        <v>0.0073</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>-0.0191</v>
+        <v>-0.0008</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>0.0008</v>
+        <v>0.0187</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>0.0539</v>
+        <v>0.0508</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>0.0244</v>
+        <v>0.0364</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>0.1061</v>
+        <v>0.1192</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>0.0193</v>
+        <v>0.04969999999999999</v>
       </c>
       <c r="L46" s="3" t="n">
-        <v>0.1416</v>
+        <v>0.1414</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>0.1762</v>
+        <v>0.1856</v>
       </c>
       <c r="N46" s="3" t="n">
-        <v>0.1053</v>
+        <v>0.1024</v>
       </c>
       <c r="O46" s="3" t="n">
-        <v>0.09029999999999999</v>
+        <v>0.09230000000000001</v>
       </c>
     </row>
     <row r="47">
@@ -2821,47 +2821,47 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>7803.33</v>
+        <v>7934.7</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>-0.0119</v>
+        <v>0.0265</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>-0.0202</v>
+        <v>-0.0037</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>-0.0433</v>
+        <v>-0.0192</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>-0.06419999999999999</v>
+        <v>-0.0529</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>-0.0552</v>
+        <v>-0.0397</v>
       </c>
       <c r="I47" s="3" t="n">
-        <v>-0.0425</v>
+        <v>-0.0264</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>-0.0017</v>
+        <v>0.0151</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>-0.0296</v>
+        <v>-0.0176</v>
       </c>
       <c r="L47" s="3" t="n">
-        <v>0.016</v>
+        <v>0.0271</v>
       </c>
       <c r="M47" s="3" t="n">
-        <v>0.029</v>
+        <v>0.0416</v>
       </c>
       <c r="N47" s="3" t="n">
-        <v>0.0353</v>
+        <v>0.0336</v>
       </c>
       <c r="O47" s="3" t="n">
-        <v>0.0573</v>
+        <v>0.0596</v>
       </c>
     </row>
     <row r="48">
@@ -2872,47 +2872,47 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>10552.1</v>
+        <v>10840.4</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>0.0086</v>
+        <v>0.0382</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>-0.0051</v>
+        <v>0.0221</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>-0.0111</v>
+        <v>0.0171</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>0.0052</v>
+        <v>0.0254</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>-0.0046</v>
+        <v>0.0236</v>
       </c>
       <c r="I48" s="3" t="n">
-        <v>0.0625</v>
+        <v>0.0915</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>0.0369</v>
+        <v>0.06519999999999999</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>0.1096</v>
+        <v>0.1502</v>
       </c>
       <c r="L48" s="3" t="n">
-        <v>0.1315</v>
+        <v>0.1464</v>
       </c>
       <c r="M48" s="3" t="n">
-        <v>0.1143</v>
+        <v>0.1243</v>
       </c>
       <c r="N48" s="3" t="n">
-        <v>0.08259999999999999</v>
+        <v>0.0843</v>
       </c>
       <c r="O48" s="3" t="n">
-        <v>0.0409</v>
+        <v>0.0455</v>
       </c>
     </row>
     <row r="49">
@@ -2923,47 +2923,47 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>24211.35</v>
+        <v>24134.57</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>0.01</v>
+        <v>-0.0032</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>-0.0163</v>
+        <v>-0.0194</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>-0.0421</v>
+        <v>-0.0228</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>0.0015</v>
+        <v>-0.0174</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>-0.065</v>
+        <v>-0.0774</v>
       </c>
       <c r="I49" s="3" t="n">
-        <v>-0.0554</v>
+        <v>-0.0584</v>
       </c>
       <c r="J49" s="3" t="n">
-        <v>-0.0233</v>
+        <v>-0.0264</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>-0.095</v>
+        <v>-0.0677</v>
       </c>
       <c r="L49" s="3" t="n">
-        <v>0.0832</v>
+        <v>0.09080000000000001</v>
       </c>
       <c r="M49" s="3" t="n">
-        <v>0.1109</v>
+        <v>0.1074</v>
       </c>
       <c r="N49" s="3" t="n">
-        <v>-0.0051</v>
+        <v>-0.009599999999999999</v>
       </c>
       <c r="O49" s="3" t="n">
-        <v>0.0028</v>
+        <v>0.0031</v>
       </c>
     </row>
     <row r="50">
@@ -2974,47 +2974,47 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>4357.62</v>
+        <v>4160.37</v>
       </c>
       <c r="D50" s="3" t="n">
-        <v>-0.0353</v>
+        <v>-0.0363</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>-0.0578</v>
+        <v>-0.0453</v>
       </c>
       <c r="F50" s="3" t="n">
-        <v>-0.0578</v>
+        <v>-0.07099999999999999</v>
       </c>
       <c r="G50" s="3" t="n">
-        <v>-0.1213</v>
+        <v>-0.0814</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>-0.0372</v>
+        <v>-0.1202</v>
       </c>
       <c r="I50" s="3" t="n">
-        <v>-0.0588</v>
+        <v>-0.1014</v>
       </c>
       <c r="J50" s="3" t="n">
-        <v>-0.0208</v>
+        <v>-0.06509999999999999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>-0.061</v>
+        <v>-0.0992</v>
       </c>
       <c r="L50" s="3" t="n">
-        <v>0.0415</v>
+        <v>0.0421</v>
       </c>
       <c r="M50" s="3" t="n">
-        <v>0.05690000000000001</v>
+        <v>0.04559999999999999</v>
       </c>
       <c r="N50" s="3" t="n">
-        <v>-0.0218</v>
+        <v>-0.0334</v>
       </c>
       <c r="O50" s="3" t="n">
-        <v>0.0297</v>
+        <v>0.0228</v>
       </c>
     </row>
     <row r="51">
@@ -3025,47 +3025,47 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>96.73</v>
+        <v>95.05</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>0.004500000000000001</v>
+        <v>-0.0183</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>0.0071</v>
+        <v>-0.0104</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>0.0108</v>
+        <v>-0.0092</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>0.014</v>
+        <v>-0.0166</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>0.0461</v>
+        <v>0.0215</v>
       </c>
       <c r="I51" s="3" t="n">
-        <v>0.0775</v>
+        <v>0.0588</v>
       </c>
       <c r="J51" s="3" t="n">
-        <v>0.0252</v>
+        <v>0.0073</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>0.0885</v>
+        <v>0.0824</v>
       </c>
       <c r="L51" s="3" t="n">
-        <v>0.0735</v>
+        <v>0.0634</v>
       </c>
       <c r="M51" s="3" t="n">
-        <v>0.0515</v>
+        <v>0.0454</v>
       </c>
       <c r="N51" s="3" t="n">
-        <v>0.05110000000000001</v>
+        <v>0.04849999999999999</v>
       </c>
       <c r="O51" s="3" t="n">
-        <v>0.0377</v>
+        <v>0.0359</v>
       </c>
     </row>
     <row r="52">
@@ -3076,47 +3076,47 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>4216.3</v>
+        <v>4200.6</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>0.013</v>
+        <v>-0.0037</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>0.0071</v>
+        <v>0.0033</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>-0.0452</v>
+        <v>-0.0372</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>0.0273</v>
+        <v>0.04679999999999999</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>-0.1146</v>
+        <v>-0.1353</v>
       </c>
       <c r="I52" s="3" t="n">
-        <v>-0.0253</v>
+        <v>-0.0289</v>
       </c>
       <c r="J52" s="3" t="n">
-        <v>-0.09279999999999999</v>
+        <v>-0.09619999999999999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>0.0684</v>
+        <v>-0.0186</v>
       </c>
       <c r="L52" s="3" t="n">
-        <v>0.2722</v>
+        <v>0.2536</v>
       </c>
       <c r="M52" s="3" t="n">
-        <v>0.3136</v>
+        <v>0.2978</v>
       </c>
       <c r="N52" s="3" t="n">
-        <v>0.1913</v>
+        <v>0.189</v>
       </c>
       <c r="O52" s="3" t="n">
-        <v>0.1291</v>
+        <v>0.128</v>
       </c>
     </row>
     <row r="53">
@@ -3127,47 +3127,47 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>61.05</v>
+        <v>57.92</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>0.0105</v>
+        <v>-0.0512</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>0.0158</v>
+        <v>-0.0362</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>-0.1015</v>
+        <v>-0.11</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>0.0207</v>
+        <v>0.0336</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>-0.2001</v>
+        <v>-0.2914</v>
       </c>
       <c r="I53" s="3" t="n">
-        <v>-0.1296</v>
+        <v>-0.1742</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>-0.1826</v>
+        <v>-0.2245</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>0.3031</v>
+        <v>0.0924</v>
       </c>
       <c r="L53" s="3" t="n">
-        <v>0.4169</v>
+        <v>0.3507</v>
       </c>
       <c r="M53" s="3" t="n">
-        <v>0.4104</v>
+        <v>0.3635</v>
       </c>
       <c r="N53" s="3" t="n">
-        <v>0.2189</v>
+        <v>0.1994</v>
       </c>
       <c r="O53" s="3" t="n">
-        <v>0.1335</v>
+        <v>0.1267</v>
       </c>
     </row>
   </sheetData>

</xml_diff>